<commit_message>
Count the level 110 gold orb from a promo code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1104,10 +1104,10 @@
     <t xml:space="preserve">Training Day run</t>
   </si>
   <si>
-    <t xml:space="preserve">Level 110 gold orb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">825K + 825K + 1.65M per orb. Copy the row for each orb</t>
+    <t xml:space="preserve">Level 110 gold orb, promo code Oct 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">825K + 825K + 1.65M. Copy the row for each new orb</t>
   </si>
   <si>
     <t xml:space="preserve">Gold orbs</t>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>510273450.9648</v>
+        <v>515399959.520418</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="B6" s="27" t="n">
         <f aca="false">SUMIFS(B13:B51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
-        <v>13900000</v>
+        <v>17200000</v>
       </c>
       <c r="C6" s="27" t="n">
         <f aca="false">SUMIFS(C13:C51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>16720000</v>
+        <v>20020000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -7113,7 +7113,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>16720000</v>
+        <v>20020000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8128,7 +8128,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J40" s="11" t="s">
         <v>253</v>
@@ -9854,7 +9854,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19258179.4743865</v>
+        <v>19451658.5188738</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Breaker of Nature rewards and pending orbs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="528">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1108,6 +1108,24 @@
   </si>
   <si>
     <t xml:space="preserve">825K + 825K + 1.65M. Copy the row for each new orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level 110 gold orb, Breaker of Nature level 120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending claim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature level 110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending claim. Also gives the level 110 training orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level 110 training orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending claim. Enter amounts once opened</t>
   </si>
   <si>
     <t xml:space="preserve">Gold orbs</t>
@@ -4103,7 +4121,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>515399959.520418</v>
+        <v>515448478.906659</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6935,7 +6953,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K78"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -7013,31 +7031,31 @@
         <v>315</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
-        <v>17200000</v>
+        <f aca="false">SUMIFS(B13:B54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
+        <v>20500000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
-        <v>3750000</v>
+        <f aca="false">SUMIFS(C13:C54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
+        <v>4000000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
+        <f aca="false">SUMIFS(D13:D54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
         <v>3000000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
+        <f aca="false">SUMIFS(E13:E54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
         <v>2600000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
+        <f aca="false">SUMIFS(F13:F54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
+        <f aca="false">SUMIFS(G13:G54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H51,$I$13:$I$51,"Yes",$J$13:$J$51,"No")</f>
+        <f aca="false">SUMIFS(H13:H54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
         <v>225</v>
       </c>
     </row>
@@ -7047,11 +7065,11 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>20020000</v>
+        <v>23320000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>4455800</v>
+        <v>4705800</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
@@ -7079,31 +7097,31 @@
         <v>317</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$55:$J$73,"Planned",B55:B73)</f>
+        <f aca="false">SUMIF($J$58:$J$76,"Planned",B58:B76)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$55:$J$73,"Planned",C55:C73)</f>
+        <f aca="false">SUMIF($J$58:$J$76,"Planned",C58:C76)</f>
         <v>1710000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$55:$J$73,"Planned",D55:D73)</f>
+        <f aca="false">SUMIF($J$58:$J$76,"Planned",D58:D76)</f>
         <v>2640000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$55:$J$73,"Planned",E55:E73)</f>
+        <f aca="false">SUMIF($J$58:$J$76,"Planned",E58:E76)</f>
         <v>1710000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$55:$J$73,"Planned",F55:F73)</f>
+        <f aca="false">SUMIF($J$58:$J$76,"Planned",F58:F76)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$55:$J$73,"Planned",G55:G73)</f>
+        <f aca="false">SUMIF($J$58:$J$76,"Planned",G58:G76)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$55:$J$73,"Planned",H55:H73)</f>
+        <f aca="false">SUMIF($J$58:$J$76,"Planned",H58:H76)</f>
         <v>0</v>
       </c>
     </row>
@@ -7113,11 +7131,11 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>20020000</v>
+        <v>23320000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>2745800</v>
+        <v>2995800</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
@@ -8142,7 +8160,7 @@
         <v>359</v>
       </c>
       <c r="B41" s="30" t="n">
-        <v>0</v>
+        <v>3300000</v>
       </c>
       <c r="C41" s="30" t="n">
         <v>0</v>
@@ -8163,7 +8181,7 @@
         <v>0</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J41" s="11" t="s">
         <v>253</v>
@@ -8173,43 +8191,103 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12"/>
-      <c r="B42" s="30"/>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
-      <c r="E42" s="30"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="30"/>
-      <c r="H42" s="30"/>
-      <c r="I42" s="11"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="12"/>
+      <c r="A42" s="12" t="s">
+        <v>361</v>
+      </c>
+      <c r="B42" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="30" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D42" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J42" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K42" s="15" t="s">
+        <v>362</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="12"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
-      <c r="E43" s="30"/>
+      <c r="A43" s="12" t="s">
+        <v>363</v>
+      </c>
+      <c r="B43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="F43" s="30"/>
       <c r="G43" s="30"/>
       <c r="H43" s="30"/>
-      <c r="I43" s="11"/>
-      <c r="J43" s="11"/>
-      <c r="K43" s="12"/>
+      <c r="I43" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J43" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K43" s="15" t="s">
+        <v>364</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12"/>
-      <c r="B44" s="30"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
-      <c r="F44" s="30"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="30"/>
-      <c r="I44" s="11"/>
-      <c r="J44" s="11"/>
-      <c r="K44" s="12"/>
+      <c r="A44" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="B44" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J44" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K44" s="15" t="s">
+        <v>366</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12"/>
@@ -8302,175 +8380,129 @@
       <c r="J51" s="11"/>
       <c r="K51" s="12"/>
     </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="12"/>
+      <c r="B52" s="30"/>
+      <c r="C52" s="30"/>
+      <c r="D52" s="30"/>
+      <c r="E52" s="30"/>
+      <c r="F52" s="30"/>
+      <c r="G52" s="30"/>
+      <c r="H52" s="30"/>
+      <c r="I52" s="11"/>
+      <c r="J52" s="11"/>
+      <c r="K52" s="12"/>
+    </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="29" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
-        <v>362</v>
-      </c>
-      <c r="B54" s="3" t="s">
+      <c r="A53" s="12"/>
+      <c r="B53" s="30"/>
+      <c r="C53" s="30"/>
+      <c r="D53" s="30"/>
+      <c r="E53" s="30"/>
+      <c r="F53" s="30"/>
+      <c r="G53" s="30"/>
+      <c r="H53" s="30"/>
+      <c r="I53" s="11"/>
+      <c r="J53" s="11"/>
+      <c r="K53" s="12"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="12"/>
+      <c r="B54" s="30"/>
+      <c r="C54" s="30"/>
+      <c r="D54" s="30"/>
+      <c r="E54" s="30"/>
+      <c r="F54" s="30"/>
+      <c r="G54" s="30"/>
+      <c r="H54" s="30"/>
+      <c r="I54" s="11"/>
+      <c r="J54" s="11"/>
+      <c r="K54" s="12"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="29" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="B57" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C57" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="D57" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="E57" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="F54" s="3" t="s">
+      <c r="F57" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="G54" s="3" t="s">
+      <c r="G57" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="H54" s="3" t="s">
+      <c r="H57" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="I54" s="3" t="s">
+      <c r="I57" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J54" s="3" t="s">
+      <c r="J57" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K54" s="3" t="s">
+      <c r="K57" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12" t="s">
-        <v>363</v>
-      </c>
-      <c r="B55" s="30" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C55" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G55" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" s="30" t="n">
-        <v>183</v>
-      </c>
-      <c r="I55" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="11" t="s">
-        <v>364</v>
-      </c>
-      <c r="K55" s="15" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="12" t="s">
-        <v>366</v>
-      </c>
-      <c r="B56" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C56" s="30" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D56" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E56" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="11" t="s">
-        <v>364</v>
-      </c>
-      <c r="K56" s="15"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="12" t="s">
-        <v>367</v>
-      </c>
-      <c r="B57" s="26"/>
-      <c r="C57" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E57" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F57" s="26"/>
-      <c r="G57" s="26"/>
-      <c r="H57" s="26"/>
-      <c r="I57" s="30" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J57" s="11" t="s">
-        <v>368</v>
-      </c>
-      <c r="K57" s="15" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="B58" s="30" t="n">
+        <v>1837500</v>
+      </c>
+      <c r="C58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G58" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="30" t="n">
+        <v>183</v>
+      </c>
+      <c r="I58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="11" t="s">
         <v>370</v>
       </c>
-      <c r="B58" s="26"/>
-      <c r="C58" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E58" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="26"/>
-      <c r="G58" s="26"/>
-      <c r="H58" s="26"/>
-      <c r="I58" s="30" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J58" s="11" t="s">
-        <v>368</v>
-      </c>
       <c r="K58" s="15" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>371</v>
-      </c>
-      <c r="B59" s="26"/>
+        <v>372</v>
+      </c>
+      <c r="B59" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="C59" s="30" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D59" s="30" t="n">
         <v>0</v>
@@ -8478,22 +8510,26 @@
       <c r="E59" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F59" s="26"/>
-      <c r="G59" s="26"/>
-      <c r="H59" s="26"/>
+      <c r="F59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I59" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>368</v>
-      </c>
-      <c r="K59" s="15" t="s">
-        <v>369</v>
-      </c>
+        <v>370</v>
+      </c>
+      <c r="K59" s="15"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B60" s="26"/>
       <c r="C60" s="30" t="n">
@@ -8512,15 +8548,15 @@
         <v>3000000</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="K60" s="15" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B61" s="26"/>
       <c r="C61" s="30" t="n">
@@ -8532,55 +8568,41 @@
       <c r="E61" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F61" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F61" s="26"/>
+      <c r="G61" s="26"/>
+      <c r="H61" s="26"/>
       <c r="I61" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="K61" s="15" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
+        <v>377</v>
+      </c>
+      <c r="B62" s="26"/>
+      <c r="C62" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="26"/>
+      <c r="G62" s="26"/>
+      <c r="H62" s="26"/>
+      <c r="I62" s="30" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J62" s="11" t="s">
         <v>374</v>
-      </c>
-      <c r="B62" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C62" s="30" t="n">
-        <v>1710000</v>
-      </c>
-      <c r="D62" s="30" t="n">
-        <v>2640000</v>
-      </c>
-      <c r="E62" s="30" t="n">
-        <v>1710000</v>
-      </c>
-      <c r="F62" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G62" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H62" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I62" s="30" t="n">
-        <v>17000000</v>
-      </c>
-      <c r="J62" s="11" t="s">
-        <v>368</v>
       </c>
       <c r="K62" s="15" t="s">
         <v>375</v>
@@ -8588,43 +8610,45 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>376</v>
-      </c>
-      <c r="B63" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C63" s="26"/>
-      <c r="D63" s="26"/>
-      <c r="E63" s="26"/>
-      <c r="F63" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G63" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H63" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>378</v>
+      </c>
+      <c r="B63" s="26"/>
+      <c r="C63" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="26"/>
+      <c r="G63" s="26"/>
+      <c r="H63" s="26"/>
       <c r="I63" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="K63" s="15" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>377</v>
-      </c>
-      <c r="B64" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C64" s="26"/>
-      <c r="D64" s="26"/>
-      <c r="E64" s="26"/>
+        <v>379</v>
+      </c>
+      <c r="B64" s="26"/>
+      <c r="C64" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="F64" s="30" t="n">
         <v>0</v>
       </c>
@@ -8638,22 +8662,28 @@
         <v>17000000</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="K64" s="15" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B65" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C65" s="26"/>
-      <c r="D65" s="26"/>
-      <c r="E65" s="26"/>
+      <c r="C65" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D65" s="30" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="E65" s="30" t="n">
+        <v>1710000</v>
+      </c>
       <c r="F65" s="30" t="n">
         <v>0</v>
       </c>
@@ -8667,15 +8697,15 @@
         <v>17000000</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="K65" s="15" t="s">
-        <v>369</v>
+        <v>381</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="12" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B66" s="30" t="n">
         <v>0</v>
@@ -8696,79 +8726,127 @@
         <v>17000000</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="K66" s="15" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="12" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B67" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" s="26"/>
+      <c r="D67" s="26"/>
+      <c r="E67" s="26"/>
+      <c r="F67" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J67" s="11" t="s">
+        <v>384</v>
+      </c>
+      <c r="K67" s="15" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="B68" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" s="26"/>
+      <c r="D68" s="26"/>
+      <c r="E68" s="26"/>
+      <c r="F68" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J68" s="11" t="s">
+        <v>384</v>
+      </c>
+      <c r="K68" s="15" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="B69" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" s="26"/>
+      <c r="D69" s="26"/>
+      <c r="E69" s="26"/>
+      <c r="F69" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J69" s="11" t="s">
+        <v>384</v>
+      </c>
+      <c r="K69" s="15" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="B70" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C67" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D67" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E67" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F67" s="26"/>
-      <c r="G67" s="26"/>
-      <c r="H67" s="26"/>
-      <c r="I67" s="30" t="n">
+      <c r="C70" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="26"/>
+      <c r="G70" s="26"/>
+      <c r="H70" s="26"/>
+      <c r="I70" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J67" s="11" t="s">
-        <v>378</v>
-      </c>
-      <c r="K67" s="15" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="12"/>
-      <c r="B68" s="30"/>
-      <c r="C68" s="30"/>
-      <c r="D68" s="30"/>
-      <c r="E68" s="30"/>
-      <c r="F68" s="30"/>
-      <c r="G68" s="30"/>
-      <c r="H68" s="30"/>
-      <c r="I68" s="30"/>
-      <c r="J68" s="11"/>
-      <c r="K68" s="12"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="12"/>
-      <c r="B69" s="30"/>
-      <c r="C69" s="30"/>
-      <c r="D69" s="30"/>
-      <c r="E69" s="30"/>
-      <c r="F69" s="30"/>
-      <c r="G69" s="30"/>
-      <c r="H69" s="30"/>
-      <c r="I69" s="30"/>
-      <c r="J69" s="11"/>
-      <c r="K69" s="12"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="12"/>
-      <c r="B70" s="30"/>
-      <c r="C70" s="30"/>
-      <c r="D70" s="30"/>
-      <c r="E70" s="30"/>
-      <c r="F70" s="30"/>
-      <c r="G70" s="30"/>
-      <c r="H70" s="30"/>
-      <c r="I70" s="30"/>
-      <c r="J70" s="11"/>
-      <c r="K70" s="12"/>
+      <c r="J70" s="11" t="s">
+        <v>384</v>
+      </c>
+      <c r="K70" s="15" t="s">
+        <v>388</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="12"/>
@@ -8809,12 +8887,51 @@
       <c r="J73" s="11"/>
       <c r="K73" s="12"/>
     </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="12"/>
+      <c r="B74" s="30"/>
+      <c r="C74" s="30"/>
+      <c r="D74" s="30"/>
+      <c r="E74" s="30"/>
+      <c r="F74" s="30"/>
+      <c r="G74" s="30"/>
+      <c r="H74" s="30"/>
+      <c r="I74" s="30"/>
+      <c r="J74" s="11"/>
+      <c r="K74" s="12"/>
+    </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="16" t="s">
-        <v>383</v>
-      </c>
-      <c r="I75" s="20" t="n">
-        <f aca="false">SUMIF(J55:J73,"Planned",I55:I73)</f>
+      <c r="A75" s="12"/>
+      <c r="B75" s="30"/>
+      <c r="C75" s="30"/>
+      <c r="D75" s="30"/>
+      <c r="E75" s="30"/>
+      <c r="F75" s="30"/>
+      <c r="G75" s="30"/>
+      <c r="H75" s="30"/>
+      <c r="I75" s="30"/>
+      <c r="J75" s="11"/>
+      <c r="K75" s="12"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="12"/>
+      <c r="B76" s="30"/>
+      <c r="C76" s="30"/>
+      <c r="D76" s="30"/>
+      <c r="E76" s="30"/>
+      <c r="F76" s="30"/>
+      <c r="G76" s="30"/>
+      <c r="H76" s="30"/>
+      <c r="I76" s="30"/>
+      <c r="J76" s="11"/>
+      <c r="K76" s="12"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="16" t="s">
+        <v>389</v>
+      </c>
+      <c r="I78" s="20" t="n">
+        <f aca="false">SUMIF(J58:J76,"Planned",I58:I76)</f>
         <v>63000000</v>
       </c>
     </row>
@@ -8824,22 +8941,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J55:J73">
+  <conditionalFormatting sqref="J58:J76">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J51">
+  <conditionalFormatting sqref="J13:J54">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J51" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J54" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J55:J73" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J58:J76" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -8870,12 +8987,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8889,53 +9006,53 @@
         <v>307</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -8947,19 +9064,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -8971,19 +9088,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -8995,19 +9112,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
+        <v>409</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>403</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>397</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9019,19 +9136,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9043,19 +9160,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9067,19 +9184,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9091,19 +9208,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9115,19 +9232,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9139,19 +9256,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -9163,19 +9280,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -9187,16 +9304,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -9209,16 +9326,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="E18" s="32"/>
       <c r="F18" s="32"/>
@@ -9231,16 +9348,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="E19" s="32"/>
       <c r="F19" s="32"/>
@@ -9253,19 +9370,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
+        <v>428</v>
+      </c>
+      <c r="B20" s="13" t="s">
         <v>422</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>416</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -9277,21 +9394,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="E22" s="32"/>
       <c r="F22" s="32"/>
@@ -9304,16 +9421,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -9326,16 +9443,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -9348,19 +9465,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -9372,19 +9489,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -9396,16 +9513,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -9418,16 +9535,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -9440,21 +9557,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -9467,16 +9584,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -9489,16 +9606,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -9511,16 +9628,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="E33" s="32"/>
       <c r="F33" s="32"/>
@@ -9533,16 +9650,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -9555,16 +9672,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -9577,16 +9694,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -9599,16 +9716,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -9621,7 +9738,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -9658,7 +9775,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -9695,7 +9812,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
     </row>
   </sheetData>
@@ -9739,12 +9856,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9752,10 +9869,10 @@
         <v>155</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9766,13 +9883,13 @@
         <v>46313.6875</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9783,7 +9900,7 @@
         <v>285372765</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -9833,7 +9950,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -9841,7 +9958,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -9850,11 +9967,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19451658.5188738</v>
+        <v>19453489.6871156</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9865,19 +9982,19 @@
         <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>473</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>466</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>467</v>
-      </c>
       <c r="G12" s="3" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -9893,7 +10010,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -9919,7 +10036,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -9945,7 +10062,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -9971,7 +10088,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -9996,10 +10113,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10024,10 +10141,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10052,10 +10169,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10080,10 +10197,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10108,10 +10225,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10136,10 +10253,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -10165,7 +10282,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -10190,10 +10307,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -10218,10 +10335,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -10246,10 +10363,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -10277,7 +10394,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -10304,10 +10421,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -10334,10 +10451,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -10364,10 +10481,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -10388,10 +10505,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -10418,7 +10535,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -10446,10 +10563,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -10476,7 +10593,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -10504,10 +10621,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -10534,7 +10651,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -10562,10 +10679,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -10592,7 +10709,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -10620,10 +10737,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -10650,7 +10767,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -10678,10 +10795,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -10708,7 +10825,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -10736,10 +10853,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -10766,7 +10883,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -10794,7 +10911,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -10822,7 +10939,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -10850,7 +10967,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -10878,7 +10995,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -10906,7 +11023,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -10934,7 +11051,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -10962,7 +11079,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -10990,7 +11107,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11018,7 +11135,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11046,7 +11163,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11068,7 +11185,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update stock after midday energy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -4121,7 +4121,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>515448478.906659</v>
+        <v>515935161.064989</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7005,7 +7005,7 @@
         <v>314</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>2820000</v>
+        <v>2864000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>705800</v>
@@ -7017,10 +7017,10 @@
         <v>14390000</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>647</v>
+        <v>667</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>244</v>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>23320000</v>
+        <v>23364000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -7081,11 +7081,11 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>747</v>
+        <v>767</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
@@ -7131,7 +7131,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>23320000</v>
+        <v>23364000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -7147,11 +7147,11 @@
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>747</v>
+        <v>767</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
@@ -9971,7 +9971,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19453489.6871156</v>
+        <v>19471857.5178847</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Update gold and today's dailies
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="528">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1008,7 +1008,7 @@
     <t xml:space="preserve">Today's remaining optional objectives</t>
   </si>
   <si>
-    <t xml:space="preserve">Raids plus the two energy objectives</t>
+    <t xml:space="preserve">Raid battles objective</t>
   </si>
   <si>
     <t xml:space="preserve">Daily objectives, Oct 12</t>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>515935161.064989</v>
+        <v>515957718.978309</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7005,7 +7005,7 @@
         <v>314</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>2864000</v>
+        <v>2920000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>705800</v>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="B6" s="27" t="n">
         <f aca="false">SUMIFS(B13:B54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
-        <v>20500000</v>
+        <v>20450000</v>
       </c>
       <c r="C6" s="27" t="n">
         <f aca="false">SUMIFS(C13:C54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>23364000</v>
+        <v>23370000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -7131,7 +7131,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>23364000</v>
+        <v>23370000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -7208,7 +7208,7 @@
         <v>324</v>
       </c>
       <c r="B13" s="30" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="C13" s="30" t="n">
         <v>0</v>
@@ -9337,7 +9337,9 @@
       <c r="D18" s="15" t="s">
         <v>425</v>
       </c>
-      <c r="E18" s="32"/>
+      <c r="E18" s="32" t="s">
+        <v>370</v>
+      </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
       <c r="H18" s="32"/>
@@ -9359,7 +9361,9 @@
       <c r="D19" s="15" t="s">
         <v>427</v>
       </c>
-      <c r="E19" s="32"/>
+      <c r="E19" s="32" t="s">
+        <v>370</v>
+      </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
       <c r="H19" s="32"/>
@@ -9410,7 +9414,9 @@
       <c r="D22" s="15" t="s">
         <v>433</v>
       </c>
-      <c r="E22" s="32"/>
+      <c r="E22" s="32" t="s">
+        <v>370</v>
+      </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
       <c r="H22" s="32"/>
@@ -9639,7 +9645,9 @@
       <c r="D33" s="15" t="s">
         <v>457</v>
       </c>
-      <c r="E33" s="32"/>
+      <c r="E33" s="32" t="s">
+        <v>370</v>
+      </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
       <c r="H33" s="32"/>
@@ -9742,7 +9750,7 @@
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
-        <v>2350000</v>
+        <v>2400000</v>
       </c>
       <c r="F39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(F5:F37="Done"))</f>
@@ -9971,7 +9979,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19471857.5178847</v>
+        <v>19472708.8645584</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Alliance War ions and update gold after opening orb
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="530">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1126,6 +1126,12 @@
   </si>
   <si>
     <t xml:space="preserve">Pending claim. Enter amounts once opened</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alliance War, Oct 13 to 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defeat reward counted. A win doubles it to 272K each</t>
   </si>
   <si>
     <t xml:space="preserve">Gold orbs</t>
@@ -4121,7 +4127,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>520352529.035002</v>
+        <v>520600173.007745</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6953,7 +6959,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K78"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -7005,7 +7011,7 @@
         <v>314</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>3070000</v>
+        <v>6370000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>705800</v>
@@ -7031,31 +7037,31 @@
         <v>315</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
-        <v>20150000</v>
+        <f aca="false">SUMIFS(B13:B55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
+        <v>16850000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
+        <f aca="false">SUMIFS(C13:C55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
         <v>4000000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
-        <v>3000000</v>
+        <f aca="false">SUMIFS(D13:D55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
+        <v>3136000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
-        <v>2600000</v>
+        <f aca="false">SUMIFS(E13:E55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
+        <v>2736000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
+        <f aca="false">SUMIFS(F13:F55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
+        <f aca="false">SUMIFS(G13:G55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H54,$I$13:$I$54,"Yes",$J$13:$J$54,"No")</f>
+        <f aca="false">SUMIFS(H13:H55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
         <v>190</v>
       </c>
     </row>
@@ -7073,11 +7079,11 @@
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>7370000</v>
+        <v>7506000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>16990000</v>
+        <v>17126000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -7097,31 +7103,31 @@
         <v>317</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$58:$J$76,"Planned",B58:B76)</f>
+        <f aca="false">SUMIF($J$59:$J$77,"Planned",B59:B77)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$58:$J$76,"Planned",C58:C76)</f>
+        <f aca="false">SUMIF($J$59:$J$77,"Planned",C59:C77)</f>
         <v>1710000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$58:$J$76,"Planned",D58:D76)</f>
+        <f aca="false">SUMIF($J$59:$J$77,"Planned",D59:D77)</f>
         <v>2640000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$58:$J$76,"Planned",E58:E76)</f>
+        <f aca="false">SUMIF($J$59:$J$77,"Planned",E59:E77)</f>
         <v>1710000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$58:$J$76,"Planned",F58:F76)</f>
+        <f aca="false">SUMIF($J$59:$J$77,"Planned",F59:F77)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$58:$J$76,"Planned",G58:G76)</f>
+        <f aca="false">SUMIF($J$59:$J$77,"Planned",G59:G77)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$58:$J$76,"Planned",H58:H76)</f>
+        <f aca="false">SUMIF($J$59:$J$77,"Planned",H59:H77)</f>
         <v>0</v>
       </c>
     </row>
@@ -7139,11 +7145,11 @@
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>4730000</v>
+        <v>4866000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>15280000</v>
+        <v>15416000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -8149,7 +8155,7 @@
         <v>249</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K40" s="15" t="s">
         <v>358</v>
@@ -8265,10 +8271,10 @@
         <v>0</v>
       </c>
       <c r="D44" s="30" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="E44" s="30" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="F44" s="30" t="n">
         <v>0</v>
@@ -8280,7 +8286,7 @@
         <v>0</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J44" s="11" t="s">
         <v>253</v>
@@ -8290,17 +8296,39 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="12"/>
-      <c r="B45" s="30"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
-      <c r="F45" s="30"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="30"/>
-      <c r="I45" s="11"/>
-      <c r="J45" s="11"/>
-      <c r="K45" s="12"/>
+      <c r="A45" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="B45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J45" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K45" s="15" t="s">
+        <v>368</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12"/>
@@ -8419,121 +8447,103 @@
       <c r="J54" s="11"/>
       <c r="K54" s="12"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="29" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
-        <v>368</v>
-      </c>
-      <c r="B57" s="3" t="s">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="12"/>
+      <c r="B55" s="30"/>
+      <c r="C55" s="30"/>
+      <c r="D55" s="30"/>
+      <c r="E55" s="30"/>
+      <c r="F55" s="30"/>
+      <c r="G55" s="30"/>
+      <c r="H55" s="30"/>
+      <c r="I55" s="11"/>
+      <c r="J55" s="11"/>
+      <c r="K55" s="12"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="29" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="B58" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C58" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="D57" s="3" t="s">
+      <c r="D58" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="E57" s="3" t="s">
+      <c r="E58" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="F57" s="3" t="s">
+      <c r="F58" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="G57" s="3" t="s">
+      <c r="G58" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="H57" s="3" t="s">
+      <c r="H58" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="I57" s="3" t="s">
+      <c r="I58" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J57" s="3" t="s">
+      <c r="J58" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K57" s="3" t="s">
+      <c r="K58" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12" t="s">
-        <v>369</v>
-      </c>
-      <c r="B58" s="30" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C58" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E58" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G58" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H58" s="30" t="n">
-        <v>183</v>
-      </c>
-      <c r="I58" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="11" t="s">
-        <v>370</v>
-      </c>
-      <c r="K58" s="15" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="B59" s="30" t="n">
+        <v>1837500</v>
+      </c>
+      <c r="C59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" s="30" t="n">
+        <v>183</v>
+      </c>
+      <c r="I59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="11" t="s">
         <v>372</v>
       </c>
-      <c r="B59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C59" s="30" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" s="11" t="s">
-        <v>370</v>
-      </c>
-      <c r="K59" s="15"/>
+      <c r="K59" s="15" t="s">
+        <v>373</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>373</v>
-      </c>
-      <c r="B60" s="26"/>
+        <v>374</v>
+      </c>
+      <c r="B60" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="C60" s="30" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D60" s="30" t="n">
         <v>0</v>
@@ -8541,22 +8551,26 @@
       <c r="E60" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F60" s="26"/>
-      <c r="G60" s="26"/>
-      <c r="H60" s="26"/>
+      <c r="F60" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I60" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>374</v>
-      </c>
-      <c r="K60" s="15" t="s">
-        <v>375</v>
-      </c>
+        <v>372</v>
+      </c>
+      <c r="K60" s="15"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B61" s="26"/>
       <c r="C61" s="30" t="n">
@@ -8575,15 +8589,15 @@
         <v>3000000</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K61" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B62" s="26"/>
       <c r="C62" s="30" t="n">
@@ -8602,15 +8616,15 @@
         <v>3000000</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K62" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B63" s="26"/>
       <c r="C63" s="30" t="n">
@@ -8629,15 +8643,15 @@
         <v>3000000</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K63" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B64" s="26"/>
       <c r="C64" s="30" t="n">
@@ -8649,40 +8663,32 @@
       <c r="E64" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F64" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G64" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H64" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F64" s="26"/>
+      <c r="G64" s="26"/>
+      <c r="H64" s="26"/>
       <c r="I64" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K64" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>380</v>
-      </c>
-      <c r="B65" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>381</v>
+      </c>
+      <c r="B65" s="26"/>
       <c r="C65" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="D65" s="30" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="E65" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="F65" s="30" t="n">
         <v>0</v>
@@ -8697,10 +8703,10 @@
         <v>17000000</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K65" s="15" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8710,9 +8716,15 @@
       <c r="B66" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C66" s="26"/>
-      <c r="D66" s="26"/>
-      <c r="E66" s="26"/>
+      <c r="C66" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D66" s="30" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="E66" s="30" t="n">
+        <v>1710000</v>
+      </c>
       <c r="F66" s="30" t="n">
         <v>0</v>
       </c>
@@ -8726,15 +8738,15 @@
         <v>17000000</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K66" s="15" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="12" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B67" s="30" t="n">
         <v>0</v>
@@ -8755,10 +8767,10 @@
         <v>17000000</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="K67" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8784,15 +8796,15 @@
         <v>17000000</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="K68" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="12" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B69" s="30" t="n">
         <v>0</v>
@@ -8813,53 +8825,69 @@
         <v>17000000</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="K69" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="12" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B70" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C70" s="26"/>
+      <c r="D70" s="26"/>
+      <c r="E70" s="26"/>
+      <c r="F70" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J70" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="K70" s="15" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="B71" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F70" s="26"/>
-      <c r="G70" s="26"/>
-      <c r="H70" s="26"/>
-      <c r="I70" s="30" t="n">
+      <c r="C71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="26"/>
+      <c r="G71" s="26"/>
+      <c r="H71" s="26"/>
+      <c r="I71" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J70" s="11" t="s">
-        <v>384</v>
-      </c>
-      <c r="K70" s="15" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="12"/>
-      <c r="B71" s="30"/>
-      <c r="C71" s="30"/>
-      <c r="D71" s="30"/>
-      <c r="E71" s="30"/>
-      <c r="F71" s="30"/>
-      <c r="G71" s="30"/>
-      <c r="H71" s="30"/>
-      <c r="I71" s="30"/>
-      <c r="J71" s="11"/>
-      <c r="K71" s="12"/>
+      <c r="J71" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="K71" s="15" t="s">
+        <v>390</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12"/>
@@ -8926,12 +8954,25 @@
       <c r="J76" s="11"/>
       <c r="K76" s="12"/>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="16" t="s">
-        <v>389</v>
-      </c>
-      <c r="I78" s="20" t="n">
-        <f aca="false">SUMIF(J58:J76,"Planned",I58:I76)</f>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="12"/>
+      <c r="B77" s="30"/>
+      <c r="C77" s="30"/>
+      <c r="D77" s="30"/>
+      <c r="E77" s="30"/>
+      <c r="F77" s="30"/>
+      <c r="G77" s="30"/>
+      <c r="H77" s="30"/>
+      <c r="I77" s="30"/>
+      <c r="J77" s="11"/>
+      <c r="K77" s="12"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="16" t="s">
+        <v>391</v>
+      </c>
+      <c r="I79" s="20" t="n">
+        <f aca="false">SUMIF(J59:J77,"Planned",I59:I77)</f>
         <v>63000000</v>
       </c>
     </row>
@@ -8941,22 +8982,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J58:J76">
+  <conditionalFormatting sqref="J59:J77">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J54">
+  <conditionalFormatting sqref="J13:J55">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J54" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J55" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J58:J76" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J59:J77" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -8987,12 +9028,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9006,53 +9047,53 @@
         <v>307</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -9064,19 +9105,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
+        <v>407</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>405</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>403</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -9088,19 +9129,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -9112,19 +9153,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9136,19 +9177,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9160,19 +9201,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9184,19 +9225,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9208,19 +9249,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9232,19 +9273,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9256,19 +9297,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -9280,19 +9321,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -9304,16 +9345,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -9326,19 +9367,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
+        <v>426</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>424</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>422</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -9350,19 +9391,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -9374,19 +9415,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -9398,24 +9439,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -9427,16 +9468,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
+        <v>436</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>434</v>
       </c>
-      <c r="B23" s="13" t="s">
-        <v>432</v>
-      </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -9449,16 +9490,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
+        <v>437</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>434</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="15" t="s">
         <v>435</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>432</v>
-      </c>
-      <c r="C24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>433</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -9471,19 +9512,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -9495,19 +9536,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
+        <v>441</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>439</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>437</v>
-      </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -9519,16 +9560,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -9541,16 +9582,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -9563,21 +9604,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -9590,16 +9631,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
+        <v>453</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>451</v>
       </c>
-      <c r="B31" s="13" t="s">
-        <v>449</v>
-      </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -9612,16 +9653,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -9634,19 +9675,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -9658,16 +9699,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
+        <v>460</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>458</v>
       </c>
-      <c r="B34" s="13" t="s">
-        <v>456</v>
-      </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -9680,16 +9721,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -9702,16 +9743,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -9724,16 +9765,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -9746,7 +9787,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -9783,7 +9824,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -9820,7 +9861,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -9864,12 +9905,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9877,10 +9918,10 @@
         <v>155</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9891,13 +9932,13 @@
         <v>46313.6875</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9908,7 +9949,7 @@
         <v>285372765</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -9958,7 +9999,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -9966,7 +10007,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -9975,11 +10016,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19638572.9888335</v>
+        <v>19647919.2607567</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9990,19 +10031,19 @@
         <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10018,7 +10059,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10044,7 +10085,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10070,7 +10111,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10096,7 +10137,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10121,10 +10162,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10149,10 +10190,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10177,10 +10218,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10205,10 +10246,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10233,10 +10274,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10261,10 +10302,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -10290,7 +10331,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -10315,10 +10356,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -10343,10 +10384,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -10371,10 +10412,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
+        <v>501</v>
+      </c>
+      <c r="D26" s="12" t="s">
         <v>499</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>497</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -10402,7 +10443,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -10429,10 +10470,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -10459,10 +10500,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -10489,10 +10530,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -10513,10 +10554,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -10543,7 +10584,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -10571,10 +10612,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -10601,7 +10642,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -10629,10 +10670,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -10659,7 +10700,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -10687,10 +10728,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -10717,7 +10758,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -10745,10 +10786,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -10775,7 +10816,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -10803,10 +10844,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -10833,7 +10874,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -10861,10 +10902,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -10891,7 +10932,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -10919,7 +10960,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -10947,7 +10988,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -10975,7 +11016,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11003,7 +11044,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11031,7 +11072,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11059,7 +11100,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11087,7 +11128,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11115,7 +11156,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11143,7 +11184,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11171,7 +11212,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11193,7 +11234,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update event points and end times
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -4127,7 +4127,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>520600173.007745</v>
+        <v>520681298.996326</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9929,7 +9929,7 @@
         <v>157</v>
       </c>
       <c r="B5" s="18" t="n">
-        <v>46313.6875</v>
+        <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
         <v>474</v>
@@ -9946,7 +9946,7 @@
         <v>158</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>285372765</v>
+        <v>285572765</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>477</v>
@@ -9994,7 +9994,7 @@
       </c>
       <c r="B8" s="20" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>14627235</v>
+        <v>14427235</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10011,7 +10011,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>139627235</v>
+        <v>139427235</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19647919.2607567</v>
+        <v>19565466.1322062</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10459,7 +10459,7 @@
       </c>
       <c r="I27" s="23" t="n">
         <f aca="false">IF(B27="","",MAX(0,B27-$B$6))</f>
-        <v>14627235</v>
+        <v>14427235</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10489,7 +10489,7 @@
       </c>
       <c r="I28" s="23" t="n">
         <f aca="false">IF(B28="","",MAX(0,B28-$B$6))</f>
-        <v>39627235</v>
+        <v>39427235</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10519,7 +10519,7 @@
       </c>
       <c r="I29" s="23" t="n">
         <f aca="false">IF(B29="","",MAX(0,B29-$B$6))</f>
-        <v>64627235</v>
+        <v>64427235</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10543,7 +10543,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>89627235</v>
+        <v>89427235</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10573,7 +10573,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>114627235</v>
+        <v>114427235</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>139627235</v>
+        <v>139427235</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10631,7 +10631,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>164627235</v>
+        <v>164427235</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10659,7 +10659,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>189627235</v>
+        <v>189427235</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>214627235</v>
+        <v>214427235</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10717,7 +10717,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>239627235</v>
+        <v>239427235</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10747,7 +10747,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>264627235</v>
+        <v>264427235</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>314627235</v>
+        <v>314427235</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10805,7 +10805,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>364627235</v>
+        <v>364427235</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10833,7 +10833,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>464627235</v>
+        <v>464427235</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>614627235</v>
+        <v>614427235</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10891,7 +10891,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>814627235</v>
+        <v>814427235</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10921,7 +10921,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>1014627235</v>
+        <v>1014427235</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10949,7 +10949,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1214627235</v>
+        <v>1214427235</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10977,7 +10977,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1414627235</v>
+        <v>1414427235</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11005,7 +11005,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1614627235</v>
+        <v>1614427235</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1814627235</v>
+        <v>1814427235</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>2014627235</v>
+        <v>2014427235</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11089,7 +11089,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2214627235</v>
+        <v>2214427235</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11117,7 +11117,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2414627235</v>
+        <v>2414427235</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2614627235</v>
+        <v>2614427235</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11173,7 +11173,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2814627235</v>
+        <v>2814427235</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11201,7 +11201,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>3014627235</v>
+        <v>3014427235</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11229,7 +11229,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3214627235</v>
+        <v>3214427235</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Fix Iron Vengeance current points
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -4053,7 +4053,7 @@
         <v>157</v>
       </c>
       <c r="B5" s="18" t="n">
-        <v>46313.6875</v>
+        <v>46313.7083333333</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4061,14 +4061,14 @@
         <v>158</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>425373500</v>
+        <v>432211000</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>159</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F50</f>
-        <v>5945373500</v>
+        <v>5952211000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="B9" s="20" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>9626500</v>
+        <v>2789000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3699626500</v>
+        <v>3692789000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>520681298.996326</v>
+        <v>518211012.409315</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4792,7 +4792,7 @@
       <c r="D50" s="12"/>
       <c r="E50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>9626500</v>
+        <v>2789000</v>
       </c>
       <c r="F50" s="11" t="s">
         <v>207</v>
@@ -4811,7 +4811,7 @@
       <c r="D51" s="12"/>
       <c r="E51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>24626500</v>
+        <v>17789000</v>
       </c>
       <c r="F51" s="11" t="s">
         <v>207</v>
@@ -4830,7 +4830,7 @@
       <c r="D52" s="12"/>
       <c r="E52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>54626500</v>
+        <v>47789000</v>
       </c>
       <c r="F52" s="11" t="s">
         <v>207</v>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="E53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>84626500</v>
+        <v>77789000</v>
       </c>
       <c r="F53" s="11" t="s">
         <v>207</v>
@@ -4870,7 +4870,7 @@
       <c r="D54" s="12"/>
       <c r="E54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>114626500</v>
+        <v>107789000</v>
       </c>
       <c r="F54" s="11" t="s">
         <v>207</v>
@@ -4889,7 +4889,7 @@
       <c r="D55" s="12"/>
       <c r="E55" s="23" t="n">
         <f aca="false">IF(B55="","",MAX(0,B55-$B$6))</f>
-        <v>144626500</v>
+        <v>137789000</v>
       </c>
       <c r="F55" s="11" t="s">
         <v>207</v>
@@ -4908,7 +4908,7 @@
       <c r="D56" s="12"/>
       <c r="E56" s="23" t="n">
         <f aca="false">IF(B56="","",MAX(0,B56-$B$6))</f>
-        <v>174626500</v>
+        <v>167789000</v>
       </c>
       <c r="F56" s="11" t="s">
         <v>207</v>
@@ -4927,7 +4927,7 @@
       <c r="D57" s="12"/>
       <c r="E57" s="23" t="n">
         <f aca="false">IF(B57="","",MAX(0,B57-$B$6))</f>
-        <v>204626500</v>
+        <v>197789000</v>
       </c>
       <c r="F57" s="11" t="s">
         <v>207</v>
@@ -4946,7 +4946,7 @@
       <c r="D58" s="12"/>
       <c r="E58" s="23" t="n">
         <f aca="false">IF(B58="","",MAX(0,B58-$B$6))</f>
-        <v>234626500</v>
+        <v>227789000</v>
       </c>
       <c r="F58" s="11" t="s">
         <v>207</v>
@@ -4965,7 +4965,7 @@
       <c r="D59" s="12"/>
       <c r="E59" s="23" t="n">
         <f aca="false">IF(B59="","",MAX(0,B59-$B$6))</f>
-        <v>264626500</v>
+        <v>257789000</v>
       </c>
       <c r="F59" s="11" t="s">
         <v>207</v>
@@ -4984,7 +4984,7 @@
       <c r="D60" s="12"/>
       <c r="E60" s="23" t="n">
         <f aca="false">IF(B60="","",MAX(0,B60-$B$6))</f>
-        <v>324626500</v>
+        <v>317789000</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>207</v>
@@ -5003,7 +5003,7 @@
       <c r="D61" s="12"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>399626500</v>
+        <v>392789000</v>
       </c>
       <c r="F61" s="11" t="s">
         <v>207</v>
@@ -5022,7 +5022,7 @@
       <c r="D62" s="12"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>474626500</v>
+        <v>467789000</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>207</v>
@@ -5041,7 +5041,7 @@
       <c r="D63" s="12"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>549626500</v>
+        <v>542789000</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>207</v>
@@ -5060,7 +5060,7 @@
       <c r="D64" s="12"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>624626500</v>
+        <v>617789000</v>
       </c>
       <c r="F64" s="11" t="s">
         <v>207</v>
@@ -5079,7 +5079,7 @@
       <c r="D65" s="12"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>699626500</v>
+        <v>692789000</v>
       </c>
       <c r="F65" s="11" t="s">
         <v>207</v>
@@ -5098,7 +5098,7 @@
       <c r="D66" s="12"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>774626500</v>
+        <v>767789000</v>
       </c>
       <c r="F66" s="11" t="s">
         <v>207</v>
@@ -5117,7 +5117,7 @@
       <c r="D67" s="12"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>924626500</v>
+        <v>917789000</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>207</v>
@@ -5136,7 +5136,7 @@
       <c r="D68" s="12"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>1074626500</v>
+        <v>1067789000</v>
       </c>
       <c r="F68" s="11" t="s">
         <v>207</v>
@@ -5155,7 +5155,7 @@
       <c r="D69" s="12"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>1224626500</v>
+        <v>1217789000</v>
       </c>
       <c r="F69" s="11" t="s">
         <v>207</v>
@@ -5174,7 +5174,7 @@
       <c r="D70" s="12"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1449626500</v>
+        <v>1442789000</v>
       </c>
       <c r="F70" s="11" t="s">
         <v>207</v>
@@ -5193,7 +5193,7 @@
       <c r="D71" s="12"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1824626500</v>
+        <v>1817789000</v>
       </c>
       <c r="F71" s="11" t="s">
         <v>207</v>
@@ -5212,7 +5212,7 @@
       <c r="D72" s="12"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>2199626500</v>
+        <v>2192789000</v>
       </c>
       <c r="F72" s="11" t="s">
         <v>207</v>
@@ -5231,7 +5231,7 @@
       <c r="D73" s="12"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2574626500</v>
+        <v>2567789000</v>
       </c>
       <c r="F73" s="11" t="s">
         <v>207</v>
@@ -5250,7 +5250,7 @@
       <c r="D74" s="12"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2949626500</v>
+        <v>2942789000</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>207</v>
@@ -5269,7 +5269,7 @@
       <c r="D75" s="12"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>3324626500</v>
+        <v>3317789000</v>
       </c>
       <c r="F75" s="11" t="s">
         <v>207</v>
@@ -5288,7 +5288,7 @@
       <c r="D76" s="12"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3699626500</v>
+        <v>3692789000</v>
       </c>
       <c r="F76" s="11" t="s">
         <v>207</v>
@@ -10020,7 +10020,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19565466.1322062</v>
+        <v>19565896.8550835</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Update training material stock
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -4127,7 +4127,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>518211012.409315</v>
+        <v>518546916.466447</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7026,10 +7026,10 @@
         <v>217</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>667</v>
+        <v>715</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>264</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7091,11 +7091,11 @@
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>767</v>
+        <v>815</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>454</v>
+        <v>469</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7157,11 +7157,11 @@
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>767</v>
+        <v>815</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>454</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19565896.8550835</v>
+        <v>19578579.4664557</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Update stock after allied supply orb
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -4130,7 +4130,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>527985465.944581</v>
+        <v>528657281.043092</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7050,10 +7050,10 @@
         <v>315</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>6370000</v>
+        <v>6570000</v>
       </c>
       <c r="C5" s="26" t="n">
-        <v>705800</v>
+        <v>755800</v>
       </c>
       <c r="D5" s="26" t="n">
         <v>4370000</v>
@@ -7068,7 +7068,7 @@
         <v>715</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>279</v>
+        <v>429</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7110,11 +7110,11 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>23220000</v>
+        <v>23420000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>4705800</v>
+        <v>4755800</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
@@ -7134,7 +7134,7 @@
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>469</v>
+        <v>619</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7176,11 +7176,11 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>23220000</v>
+        <v>23420000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>2995800</v>
+        <v>3045800</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>469</v>
+        <v>619</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19934947.2004886</v>
+        <v>19960312.6844277</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Breaker of Nature daily gold and upcoming levels
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="531">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="545">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1135,6 +1135,48 @@
   </si>
   <si>
     <t xml:space="preserve">Defeat reward counted. A win doubles it to 272K each</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature dailies, today</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log in, play any battle, collect essence. 250K gold each</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature dailies, Oct 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">250K gold each, plus 3 levels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature dailies, Oct 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature dailies, Oct 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature dailies, Oct 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature dailies, Oct 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature dailies, Oct 17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature dailies, Oct 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature level 130</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected Oct 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature level 140</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected about Oct 15. Gives 2,000 gold orb fragments, one orb</t>
   </si>
   <si>
     <t xml:space="preserve">Gold orbs</t>
@@ -4130,7 +4172,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>528657281.043092</v>
+        <v>528818361.289085</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6998,7 +7040,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -7076,31 +7118,31 @@
         <v>316</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
-        <v>16850000</v>
+        <f aca="false">SUMIFS(B13:B65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
+        <v>22850000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
-        <v>4000000</v>
+        <f aca="false">SUMIFS(C13:C65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
+        <v>4250000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
+        <f aca="false">SUMIFS(D13:D65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
         <v>3136000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
+        <f aca="false">SUMIFS(E13:E65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
         <v>2736000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
+        <f aca="false">SUMIFS(F13:F65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
+        <f aca="false">SUMIFS(G13:G65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H55,$I$13:$I$55,"Yes",$J$13:$J$55,"No")</f>
+        <f aca="false">SUMIFS(H13:H65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
         <v>190</v>
       </c>
     </row>
@@ -7110,11 +7152,11 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>23420000</v>
+        <v>29420000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>4755800</v>
+        <v>5005800</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
@@ -7142,31 +7184,31 @@
         <v>318</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$59:$J$77,"Planned",B59:B77)</f>
+        <f aca="false">SUMIF($J$69:$J$87,"Planned",B69:B87)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$59:$J$77,"Planned",C59:C77)</f>
+        <f aca="false">SUMIF($J$69:$J$87,"Planned",C69:C87)</f>
         <v>1710000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$59:$J$77,"Planned",D59:D77)</f>
+        <f aca="false">SUMIF($J$69:$J$87,"Planned",D69:D87)</f>
         <v>2640000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$59:$J$77,"Planned",E59:E77)</f>
+        <f aca="false">SUMIF($J$69:$J$87,"Planned",E69:E87)</f>
         <v>1710000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$59:$J$77,"Planned",F59:F77)</f>
+        <f aca="false">SUMIF($J$69:$J$87,"Planned",F69:F87)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$59:$J$77,"Planned",G59:G77)</f>
+        <f aca="false">SUMIF($J$69:$J$87,"Planned",G69:G87)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$59:$J$77,"Planned",H59:H77)</f>
+        <f aca="false">SUMIF($J$69:$J$87,"Planned",H69:H87)</f>
         <v>0</v>
       </c>
     </row>
@@ -7176,11 +7218,11 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>23420000</v>
+        <v>29420000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>3045800</v>
+        <v>3295800</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
@@ -8339,7 +8381,7 @@
         <v>368</v>
       </c>
       <c r="B45" s="30" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C45" s="30" t="n">
         <v>0</v>
@@ -8360,7 +8402,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J45" s="11" t="s">
         <v>253</v>
@@ -8370,504 +8412,558 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="12"/>
-      <c r="B46" s="30"/>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="30"/>
-      <c r="F46" s="30"/>
-      <c r="G46" s="30"/>
-      <c r="H46" s="30"/>
-      <c r="I46" s="11"/>
-      <c r="J46" s="11"/>
-      <c r="K46" s="12"/>
+      <c r="A46" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="B46" s="30" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C46" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J46" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K46" s="15" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="12"/>
-      <c r="B47" s="30"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
-      <c r="F47" s="30"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="30"/>
-      <c r="I47" s="11"/>
-      <c r="J47" s="11"/>
-      <c r="K47" s="12"/>
+      <c r="A47" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="B47" s="30" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C47" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J47" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K47" s="15" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="12"/>
-      <c r="B48" s="30"/>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="30"/>
-      <c r="F48" s="30"/>
-      <c r="G48" s="30"/>
-      <c r="H48" s="30"/>
-      <c r="I48" s="11"/>
-      <c r="J48" s="11"/>
-      <c r="K48" s="12"/>
+      <c r="A48" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="B48" s="30" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C48" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J48" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K48" s="15" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="12"/>
-      <c r="B49" s="30"/>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="30"/>
-      <c r="F49" s="30"/>
-      <c r="G49" s="30"/>
-      <c r="H49" s="30"/>
-      <c r="I49" s="11"/>
-      <c r="J49" s="11"/>
-      <c r="K49" s="12"/>
+      <c r="A49" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B49" s="30" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C49" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J49" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K49" s="15" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="12"/>
-      <c r="B50" s="30"/>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
-      <c r="E50" s="30"/>
-      <c r="F50" s="30"/>
-      <c r="G50" s="30"/>
-      <c r="H50" s="30"/>
-      <c r="I50" s="11"/>
-      <c r="J50" s="11"/>
-      <c r="K50" s="12"/>
+      <c r="A50" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="B50" s="30" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C50" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J50" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K50" s="15" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="12"/>
-      <c r="B51" s="30"/>
-      <c r="C51" s="30"/>
-      <c r="D51" s="30"/>
-      <c r="E51" s="30"/>
-      <c r="F51" s="30"/>
-      <c r="G51" s="30"/>
-      <c r="H51" s="30"/>
-      <c r="I51" s="11"/>
-      <c r="J51" s="11"/>
-      <c r="K51" s="12"/>
+      <c r="A51" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="B51" s="30" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C51" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J51" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K51" s="15" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="12"/>
-      <c r="B52" s="30"/>
-      <c r="C52" s="30"/>
-      <c r="D52" s="30"/>
-      <c r="E52" s="30"/>
-      <c r="F52" s="30"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="30"/>
-      <c r="I52" s="11"/>
-      <c r="J52" s="11"/>
-      <c r="K52" s="12"/>
+      <c r="A52" s="12" t="s">
+        <v>377</v>
+      </c>
+      <c r="B52" s="30" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C52" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J52" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K52" s="15" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="12"/>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
-      <c r="F53" s="30"/>
-      <c r="G53" s="30"/>
-      <c r="H53" s="30"/>
-      <c r="I53" s="11"/>
-      <c r="J53" s="11"/>
-      <c r="K53" s="12"/>
+      <c r="A53" s="12" t="s">
+        <v>378</v>
+      </c>
+      <c r="B53" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="30" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D53" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J53" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K53" s="15" t="s">
+        <v>379</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="12"/>
-      <c r="B54" s="30"/>
-      <c r="C54" s="30"/>
-      <c r="D54" s="30"/>
-      <c r="E54" s="30"/>
-      <c r="F54" s="30"/>
-      <c r="G54" s="30"/>
-      <c r="H54" s="30"/>
-      <c r="I54" s="11"/>
-      <c r="J54" s="11"/>
-      <c r="K54" s="12"/>
+      <c r="A54" s="12" t="s">
+        <v>380</v>
+      </c>
+      <c r="B54" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J54" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K54" s="15" t="s">
+        <v>381</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12"/>
-      <c r="B55" s="30"/>
-      <c r="C55" s="30"/>
-      <c r="D55" s="30"/>
-      <c r="E55" s="30"/>
-      <c r="F55" s="30"/>
-      <c r="G55" s="30"/>
-      <c r="H55" s="30"/>
-      <c r="I55" s="11"/>
-      <c r="J55" s="11"/>
-      <c r="K55" s="12"/>
+      <c r="A55" s="12" t="s">
+        <v>382</v>
+      </c>
+      <c r="B55" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J55" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K55" s="15" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="12"/>
+      <c r="B56" s="30"/>
+      <c r="C56" s="30"/>
+      <c r="D56" s="30"/>
+      <c r="E56" s="30"/>
+      <c r="F56" s="30"/>
+      <c r="G56" s="30"/>
+      <c r="H56" s="30"/>
+      <c r="I56" s="11"/>
+      <c r="J56" s="11"/>
+      <c r="K56" s="12"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="29" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="B58" s="3" t="s">
+      <c r="A57" s="12"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="30"/>
+      <c r="D57" s="30"/>
+      <c r="E57" s="30"/>
+      <c r="F57" s="30"/>
+      <c r="G57" s="30"/>
+      <c r="H57" s="30"/>
+      <c r="I57" s="11"/>
+      <c r="J57" s="11"/>
+      <c r="K57" s="12"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12"/>
+      <c r="B58" s="30"/>
+      <c r="C58" s="30"/>
+      <c r="D58" s="30"/>
+      <c r="E58" s="30"/>
+      <c r="F58" s="30"/>
+      <c r="G58" s="30"/>
+      <c r="H58" s="30"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="11"/>
+      <c r="K58" s="12"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="12"/>
+      <c r="B59" s="30"/>
+      <c r="C59" s="30"/>
+      <c r="D59" s="30"/>
+      <c r="E59" s="30"/>
+      <c r="F59" s="30"/>
+      <c r="G59" s="30"/>
+      <c r="H59" s="30"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="11"/>
+      <c r="K59" s="12"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="12"/>
+      <c r="B60" s="30"/>
+      <c r="C60" s="30"/>
+      <c r="D60" s="30"/>
+      <c r="E60" s="30"/>
+      <c r="F60" s="30"/>
+      <c r="G60" s="30"/>
+      <c r="H60" s="30"/>
+      <c r="I60" s="11"/>
+      <c r="J60" s="11"/>
+      <c r="K60" s="12"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="12"/>
+      <c r="B61" s="30"/>
+      <c r="C61" s="30"/>
+      <c r="D61" s="30"/>
+      <c r="E61" s="30"/>
+      <c r="F61" s="30"/>
+      <c r="G61" s="30"/>
+      <c r="H61" s="30"/>
+      <c r="I61" s="11"/>
+      <c r="J61" s="11"/>
+      <c r="K61" s="12"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="12"/>
+      <c r="B62" s="30"/>
+      <c r="C62" s="30"/>
+      <c r="D62" s="30"/>
+      <c r="E62" s="30"/>
+      <c r="F62" s="30"/>
+      <c r="G62" s="30"/>
+      <c r="H62" s="30"/>
+      <c r="I62" s="11"/>
+      <c r="J62" s="11"/>
+      <c r="K62" s="12"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="12"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="30"/>
+      <c r="D63" s="30"/>
+      <c r="E63" s="30"/>
+      <c r="F63" s="30"/>
+      <c r="G63" s="30"/>
+      <c r="H63" s="30"/>
+      <c r="I63" s="11"/>
+      <c r="J63" s="11"/>
+      <c r="K63" s="12"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="12"/>
+      <c r="B64" s="30"/>
+      <c r="C64" s="30"/>
+      <c r="D64" s="30"/>
+      <c r="E64" s="30"/>
+      <c r="F64" s="30"/>
+      <c r="G64" s="30"/>
+      <c r="H64" s="30"/>
+      <c r="I64" s="11"/>
+      <c r="J64" s="11"/>
+      <c r="K64" s="12"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="12"/>
+      <c r="B65" s="30"/>
+      <c r="C65" s="30"/>
+      <c r="D65" s="30"/>
+      <c r="E65" s="30"/>
+      <c r="F65" s="30"/>
+      <c r="G65" s="30"/>
+      <c r="H65" s="30"/>
+      <c r="I65" s="11"/>
+      <c r="J65" s="11"/>
+      <c r="K65" s="12"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="29" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="B68" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C68" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="D58" s="3" t="s">
+      <c r="D68" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="E68" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="F58" s="3" t="s">
+      <c r="F68" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="G58" s="3" t="s">
+      <c r="G68" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="H58" s="3" t="s">
+      <c r="H68" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="I58" s="3" t="s">
+      <c r="I68" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J58" s="3" t="s">
+      <c r="J68" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K58" s="3" t="s">
+      <c r="K68" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12" t="s">
-        <v>372</v>
-      </c>
-      <c r="B59" s="30" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G59" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H59" s="30" t="n">
-        <v>183</v>
-      </c>
-      <c r="I59" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" s="11" t="s">
-        <v>373</v>
-      </c>
-      <c r="K59" s="15" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="12" t="s">
-        <v>375</v>
-      </c>
-      <c r="B60" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C60" s="30" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D60" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E60" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F60" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" s="11" t="s">
-        <v>373</v>
-      </c>
-      <c r="K60" s="15"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="12" t="s">
-        <v>376</v>
-      </c>
-      <c r="B61" s="26"/>
-      <c r="C61" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D61" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E61" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F61" s="26"/>
-      <c r="G61" s="26"/>
-      <c r="H61" s="26"/>
-      <c r="I61" s="30" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J61" s="11" t="s">
-        <v>377</v>
-      </c>
-      <c r="K61" s="15" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="12" t="s">
-        <v>379</v>
-      </c>
-      <c r="B62" s="26"/>
-      <c r="C62" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E62" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" s="26"/>
-      <c r="G62" s="26"/>
-      <c r="H62" s="26"/>
-      <c r="I62" s="30" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J62" s="11" t="s">
-        <v>377</v>
-      </c>
-      <c r="K62" s="15" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="12" t="s">
-        <v>380</v>
-      </c>
-      <c r="B63" s="26"/>
-      <c r="C63" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E63" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F63" s="26"/>
-      <c r="G63" s="26"/>
-      <c r="H63" s="26"/>
-      <c r="I63" s="30" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J63" s="11" t="s">
-        <v>377</v>
-      </c>
-      <c r="K63" s="15" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="12" t="s">
-        <v>381</v>
-      </c>
-      <c r="B64" s="26"/>
-      <c r="C64" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E64" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F64" s="26"/>
-      <c r="G64" s="26"/>
-      <c r="H64" s="26"/>
-      <c r="I64" s="30" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J64" s="11" t="s">
-        <v>377</v>
-      </c>
-      <c r="K64" s="15" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="12" t="s">
-        <v>382</v>
-      </c>
-      <c r="B65" s="26"/>
-      <c r="C65" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D65" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E65" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F65" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G65" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I65" s="30" t="n">
-        <v>17000000</v>
-      </c>
-      <c r="J65" s="11" t="s">
-        <v>377</v>
-      </c>
-      <c r="K65" s="15" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="12" t="s">
-        <v>383</v>
-      </c>
-      <c r="B66" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C66" s="30" t="n">
-        <v>1710000</v>
-      </c>
-      <c r="D66" s="30" t="n">
-        <v>2640000</v>
-      </c>
-      <c r="E66" s="30" t="n">
-        <v>1710000</v>
-      </c>
-      <c r="F66" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G66" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H66" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I66" s="30" t="n">
-        <v>17000000</v>
-      </c>
-      <c r="J66" s="11" t="s">
-        <v>377</v>
-      </c>
-      <c r="K66" s="15" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="12" t="s">
-        <v>385</v>
-      </c>
-      <c r="B67" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C67" s="26"/>
-      <c r="D67" s="26"/>
-      <c r="E67" s="26"/>
-      <c r="F67" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G67" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H67" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I67" s="30" t="n">
-        <v>17000000</v>
-      </c>
-      <c r="J67" s="11" t="s">
-        <v>377</v>
-      </c>
-      <c r="K67" s="15" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="B68" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C68" s="26"/>
-      <c r="D68" s="26"/>
-      <c r="E68" s="26"/>
-      <c r="F68" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H68" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" s="30" t="n">
-        <v>17000000</v>
-      </c>
-      <c r="J68" s="11" t="s">
-        <v>387</v>
-      </c>
-      <c r="K68" s="15" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="12" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B69" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C69" s="26"/>
-      <c r="D69" s="26"/>
-      <c r="E69" s="26"/>
+        <v>1837500</v>
+      </c>
+      <c r="C69" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="F69" s="30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G69" s="30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H69" s="30" t="n">
-        <v>0</v>
+        <v>183</v>
       </c>
       <c r="I69" s="30" t="n">
-        <v>17000000</v>
+        <v>0</v>
       </c>
       <c r="J69" s="11" t="s">
         <v>387</v>
       </c>
       <c r="K69" s="15" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8877,9 +8973,15 @@
       <c r="B70" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C70" s="26"/>
-      <c r="D70" s="26"/>
-      <c r="E70" s="26"/>
+      <c r="C70" s="30" t="n">
+        <v>359800</v>
+      </c>
+      <c r="D70" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="F70" s="30" t="n">
         <v>0</v>
       </c>
@@ -8890,22 +8992,18 @@
         <v>0</v>
       </c>
       <c r="I70" s="30" t="n">
-        <v>17000000</v>
+        <v>0</v>
       </c>
       <c r="J70" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="K70" s="15" t="s">
-        <v>378</v>
-      </c>
+      <c r="K70" s="15"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="12" t="s">
         <v>390</v>
       </c>
-      <c r="B71" s="30" t="n">
-        <v>13000000</v>
-      </c>
+      <c r="B71" s="26"/>
       <c r="C71" s="30" t="n">
         <v>0</v>
       </c>
@@ -8919,99 +9017,393 @@
       <c r="G71" s="26"/>
       <c r="H71" s="26"/>
       <c r="I71" s="30" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J71" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="K71" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="B72" s="26"/>
+      <c r="C72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="26"/>
+      <c r="G72" s="26"/>
+      <c r="H72" s="26"/>
+      <c r="I72" s="30" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J72" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="K72" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="12" t="s">
+        <v>394</v>
+      </c>
+      <c r="B73" s="26"/>
+      <c r="C73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="26"/>
+      <c r="G73" s="26"/>
+      <c r="H73" s="26"/>
+      <c r="I73" s="30" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J73" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="K73" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="B74" s="26"/>
+      <c r="C74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="26"/>
+      <c r="G74" s="26"/>
+      <c r="H74" s="26"/>
+      <c r="I74" s="30" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J74" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="K74" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="B75" s="26"/>
+      <c r="C75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J75" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="K75" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="12" t="s">
+        <v>397</v>
+      </c>
+      <c r="B76" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C76" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D76" s="30" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="E76" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="F76" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J76" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="K76" s="15" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="12" t="s">
+        <v>399</v>
+      </c>
+      <c r="B77" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77" s="26"/>
+      <c r="D77" s="26"/>
+      <c r="E77" s="26"/>
+      <c r="F77" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J77" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="K77" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="12" t="s">
+        <v>400</v>
+      </c>
+      <c r="B78" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C78" s="26"/>
+      <c r="D78" s="26"/>
+      <c r="E78" s="26"/>
+      <c r="F78" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J78" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="K78" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="12" t="s">
+        <v>402</v>
+      </c>
+      <c r="B79" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C79" s="26"/>
+      <c r="D79" s="26"/>
+      <c r="E79" s="26"/>
+      <c r="F79" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J79" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="K79" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="12" t="s">
+        <v>403</v>
+      </c>
+      <c r="B80" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" s="26"/>
+      <c r="D80" s="26"/>
+      <c r="E80" s="26"/>
+      <c r="F80" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J80" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="K80" s="15" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="12" t="s">
+        <v>404</v>
+      </c>
+      <c r="B81" s="30" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="C81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="26"/>
+      <c r="G81" s="26"/>
+      <c r="H81" s="26"/>
+      <c r="I81" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J71" s="11" t="s">
-        <v>387</v>
-      </c>
-      <c r="K71" s="15" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="12"/>
-      <c r="B72" s="30"/>
-      <c r="C72" s="30"/>
-      <c r="D72" s="30"/>
-      <c r="E72" s="30"/>
-      <c r="F72" s="30"/>
-      <c r="G72" s="30"/>
-      <c r="H72" s="30"/>
-      <c r="I72" s="30"/>
-      <c r="J72" s="11"/>
-      <c r="K72" s="12"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="12"/>
-      <c r="B73" s="30"/>
-      <c r="C73" s="30"/>
-      <c r="D73" s="30"/>
-      <c r="E73" s="30"/>
-      <c r="F73" s="30"/>
-      <c r="G73" s="30"/>
-      <c r="H73" s="30"/>
-      <c r="I73" s="30"/>
-      <c r="J73" s="11"/>
-      <c r="K73" s="12"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="12"/>
-      <c r="B74" s="30"/>
-      <c r="C74" s="30"/>
-      <c r="D74" s="30"/>
-      <c r="E74" s="30"/>
-      <c r="F74" s="30"/>
-      <c r="G74" s="30"/>
-      <c r="H74" s="30"/>
-      <c r="I74" s="30"/>
-      <c r="J74" s="11"/>
-      <c r="K74" s="12"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="12"/>
-      <c r="B75" s="30"/>
-      <c r="C75" s="30"/>
-      <c r="D75" s="30"/>
-      <c r="E75" s="30"/>
-      <c r="F75" s="30"/>
-      <c r="G75" s="30"/>
-      <c r="H75" s="30"/>
-      <c r="I75" s="30"/>
-      <c r="J75" s="11"/>
-      <c r="K75" s="12"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="12"/>
-      <c r="B76" s="30"/>
-      <c r="C76" s="30"/>
-      <c r="D76" s="30"/>
-      <c r="E76" s="30"/>
-      <c r="F76" s="30"/>
-      <c r="G76" s="30"/>
-      <c r="H76" s="30"/>
-      <c r="I76" s="30"/>
-      <c r="J76" s="11"/>
-      <c r="K76" s="12"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="12"/>
-      <c r="B77" s="30"/>
-      <c r="C77" s="30"/>
-      <c r="D77" s="30"/>
-      <c r="E77" s="30"/>
-      <c r="F77" s="30"/>
-      <c r="G77" s="30"/>
-      <c r="H77" s="30"/>
-      <c r="I77" s="30"/>
-      <c r="J77" s="11"/>
-      <c r="K77" s="12"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="16" t="s">
-        <v>392</v>
-      </c>
-      <c r="I79" s="20" t="n">
-        <f aca="false">SUMIF(J59:J77,"Planned",I59:I77)</f>
+      <c r="J81" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="K81" s="15" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="12"/>
+      <c r="B82" s="30"/>
+      <c r="C82" s="30"/>
+      <c r="D82" s="30"/>
+      <c r="E82" s="30"/>
+      <c r="F82" s="30"/>
+      <c r="G82" s="30"/>
+      <c r="H82" s="30"/>
+      <c r="I82" s="30"/>
+      <c r="J82" s="11"/>
+      <c r="K82" s="12"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="12"/>
+      <c r="B83" s="30"/>
+      <c r="C83" s="30"/>
+      <c r="D83" s="30"/>
+      <c r="E83" s="30"/>
+      <c r="F83" s="30"/>
+      <c r="G83" s="30"/>
+      <c r="H83" s="30"/>
+      <c r="I83" s="30"/>
+      <c r="J83" s="11"/>
+      <c r="K83" s="12"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="12"/>
+      <c r="B84" s="30"/>
+      <c r="C84" s="30"/>
+      <c r="D84" s="30"/>
+      <c r="E84" s="30"/>
+      <c r="F84" s="30"/>
+      <c r="G84" s="30"/>
+      <c r="H84" s="30"/>
+      <c r="I84" s="30"/>
+      <c r="J84" s="11"/>
+      <c r="K84" s="12"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="12"/>
+      <c r="B85" s="30"/>
+      <c r="C85" s="30"/>
+      <c r="D85" s="30"/>
+      <c r="E85" s="30"/>
+      <c r="F85" s="30"/>
+      <c r="G85" s="30"/>
+      <c r="H85" s="30"/>
+      <c r="I85" s="30"/>
+      <c r="J85" s="11"/>
+      <c r="K85" s="12"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="12"/>
+      <c r="B86" s="30"/>
+      <c r="C86" s="30"/>
+      <c r="D86" s="30"/>
+      <c r="E86" s="30"/>
+      <c r="F86" s="30"/>
+      <c r="G86" s="30"/>
+      <c r="H86" s="30"/>
+      <c r="I86" s="30"/>
+      <c r="J86" s="11"/>
+      <c r="K86" s="12"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="12"/>
+      <c r="B87" s="30"/>
+      <c r="C87" s="30"/>
+      <c r="D87" s="30"/>
+      <c r="E87" s="30"/>
+      <c r="F87" s="30"/>
+      <c r="G87" s="30"/>
+      <c r="H87" s="30"/>
+      <c r="I87" s="30"/>
+      <c r="J87" s="11"/>
+      <c r="K87" s="12"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="16" t="s">
+        <v>406</v>
+      </c>
+      <c r="I89" s="20" t="n">
+        <f aca="false">SUMIF(J69:J87,"Planned",I69:I87)</f>
         <v>63000000</v>
       </c>
     </row>
@@ -9021,22 +9413,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J59:J77">
+  <conditionalFormatting sqref="J69:J87">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J55">
+  <conditionalFormatting sqref="J13:J65">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J55" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J65" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J59:J77" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J69:J87" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9067,12 +9459,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>393</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>394</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9086,53 +9478,53 @@
         <v>308</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>395</v>
+        <v>409</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>396</v>
+        <v>410</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>397</v>
+        <v>411</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>398</v>
+        <v>412</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>399</v>
+        <v>413</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>400</v>
+        <v>414</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>401</v>
+        <v>415</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>402</v>
+        <v>416</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>403</v>
+        <v>417</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>404</v>
+        <v>418</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>405</v>
+        <v>419</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>407</v>
+        <v>421</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -9144,19 +9536,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>408</v>
+        <v>422</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>409</v>
+        <v>423</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -9168,19 +9560,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>410</v>
+        <v>424</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>411</v>
+        <v>425</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -9192,19 +9584,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>412</v>
+        <v>426</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>413</v>
+        <v>427</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9216,19 +9608,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>414</v>
+        <v>428</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>411</v>
+        <v>425</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9240,19 +9632,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>415</v>
+        <v>429</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>411</v>
+        <v>425</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9264,19 +9656,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>416</v>
+        <v>430</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>417</v>
+        <v>431</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9288,19 +9680,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>418</v>
+        <v>432</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>411</v>
+        <v>425</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9312,19 +9704,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>419</v>
+        <v>433</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>420</v>
+        <v>434</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9336,19 +9728,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>421</v>
+        <v>435</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>411</v>
+        <v>425</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -9360,19 +9752,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>422</v>
+        <v>436</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>423</v>
+        <v>437</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -9384,16 +9776,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>424</v>
+        <v>438</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>425</v>
+        <v>439</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>426</v>
+        <v>440</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -9406,19 +9798,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>427</v>
+        <v>441</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>425</v>
+        <v>439</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>428</v>
+        <v>442</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -9430,19 +9822,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>429</v>
+        <v>443</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>425</v>
+        <v>439</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>430</v>
+        <v>444</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -9454,19 +9846,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>431</v>
+        <v>445</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>425</v>
+        <v>439</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>432</v>
+        <v>446</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -9478,24 +9870,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>433</v>
+        <v>447</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>434</v>
+        <v>448</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>435</v>
+        <v>449</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>436</v>
+        <v>450</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -9507,16 +9899,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>437</v>
+        <v>451</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>435</v>
+        <v>449</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>436</v>
+        <v>450</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -9529,16 +9921,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>438</v>
+        <v>452</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>435</v>
+        <v>449</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>436</v>
+        <v>450</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -9551,19 +9943,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>439</v>
+        <v>453</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>440</v>
+        <v>454</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>441</v>
+        <v>455</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -9575,19 +9967,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>442</v>
+        <v>456</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>440</v>
+        <v>454</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>443</v>
+        <v>457</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -9599,16 +9991,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>444</v>
+        <v>458</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>445</v>
+        <v>459</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>446</v>
+        <v>460</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -9621,16 +10013,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>447</v>
+        <v>461</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>448</v>
+        <v>462</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>449</v>
+        <v>463</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -9643,21 +10035,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>450</v>
+        <v>464</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>451</v>
+        <v>465</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>452</v>
+        <v>466</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>453</v>
+        <v>467</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -9670,16 +10062,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>454</v>
+        <v>468</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>452</v>
+        <v>466</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>455</v>
+        <v>469</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -9692,16 +10084,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>456</v>
+        <v>470</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>452</v>
+        <v>466</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>457</v>
+        <v>471</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -9714,19 +10106,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>458</v>
+        <v>472</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>459</v>
+        <v>473</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>460</v>
+        <v>474</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -9738,16 +10130,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>461</v>
+        <v>475</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>459</v>
+        <v>473</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>462</v>
+        <v>476</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -9760,16 +10152,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>463</v>
+        <v>477</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>459</v>
+        <v>473</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>462</v>
+        <v>476</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -9782,16 +10174,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>464</v>
+        <v>478</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>452</v>
+        <v>466</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>465</v>
+        <v>479</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -9804,16 +10196,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
+        <v>480</v>
+      </c>
+      <c r="B37" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="B37" s="13" t="s">
-        <v>452</v>
-      </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>467</v>
+        <v>481</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -9826,7 +10218,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>468</v>
+        <v>482</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -9863,7 +10255,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>469</v>
+        <v>483</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -9900,7 +10292,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>470</v>
+        <v>484</v>
       </c>
     </row>
   </sheetData>
@@ -9944,12 +10336,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>471</v>
+        <v>485</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>472</v>
+        <v>486</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9957,10 +10349,10 @@
         <v>155</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>473</v>
+        <v>487</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>474</v>
+        <v>488</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9971,13 +10363,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>475</v>
+        <v>489</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>476</v>
+        <v>490</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>477</v>
+        <v>491</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9988,7 +10380,7 @@
         <v>285572765</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>478</v>
+        <v>492</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -10038,7 +10430,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>479</v>
+        <v>493</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -10046,7 +10438,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>480</v>
+        <v>494</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -10055,11 +10447,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>481</v>
+        <v>495</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19960312.6844277</v>
+        <v>19966394.5132271</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10070,19 +10462,19 @@
         <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>482</v>
+        <v>496</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>395</v>
+        <v>409</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>475</v>
+        <v>489</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>476</v>
+        <v>490</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>477</v>
+        <v>491</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10098,7 +10490,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>483</v>
+        <v>497</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10124,7 +10516,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>484</v>
+        <v>498</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10150,7 +10542,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>485</v>
+        <v>499</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10176,7 +10568,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>485</v>
+        <v>499</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10201,10 +10593,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>487</v>
+        <v>501</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10229,10 +10621,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>488</v>
+        <v>502</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>489</v>
+        <v>503</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10257,10 +10649,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>490</v>
+        <v>504</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>491</v>
+        <v>505</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10285,10 +10677,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>492</v>
+        <v>506</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>493</v>
+        <v>507</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10313,10 +10705,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>494</v>
+        <v>508</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>495</v>
+        <v>509</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10341,10 +10733,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>496</v>
+        <v>510</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>497</v>
+        <v>511</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -10370,7 +10762,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>498</v>
+        <v>512</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -10395,10 +10787,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>499</v>
+        <v>513</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -10423,10 +10815,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -10451,10 +10843,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
-        <v>502</v>
+        <v>516</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -10482,7 +10874,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -10509,10 +10901,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>503</v>
+        <v>517</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -10539,10 +10931,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>504</v>
+        <v>518</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -10569,10 +10961,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>505</v>
+        <v>519</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>506</v>
+        <v>520</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -10593,10 +10985,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>507</v>
+        <v>521</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -10623,7 +11015,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>508</v>
+        <v>522</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -10651,10 +11043,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>509</v>
+        <v>523</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -10681,7 +11073,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>510</v>
+        <v>524</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -10709,10 +11101,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>511</v>
+        <v>525</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -10739,7 +11131,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>512</v>
+        <v>526</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -10767,10 +11159,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>513</v>
+        <v>527</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -10797,7 +11189,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>514</v>
+        <v>528</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -10825,10 +11217,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>515</v>
+        <v>529</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -10855,7 +11247,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>516</v>
+        <v>530</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -10883,10 +11275,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>517</v>
+        <v>531</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -10913,7 +11305,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>518</v>
+        <v>532</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -10941,10 +11333,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>519</v>
+        <v>533</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>500</v>
+        <v>514</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -10971,7 +11363,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>520</v>
+        <v>534</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -10999,7 +11391,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>521</v>
+        <v>535</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -11027,7 +11419,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>519</v>
+        <v>533</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -11055,7 +11447,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>522</v>
+        <v>536</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11083,7 +11475,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>523</v>
+        <v>537</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11111,7 +11503,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>524</v>
+        <v>538</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11139,7 +11531,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>525</v>
+        <v>539</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11167,7 +11559,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>526</v>
+        <v>540</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11195,7 +11587,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>527</v>
+        <v>541</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11223,7 +11615,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>528</v>
+        <v>542</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11251,7 +11643,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>529</v>
+        <v>543</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11273,7 +11665,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>530</v>
+        <v>544</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Iron Vengeance points
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -4106,14 +4106,14 @@
         <v>158</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>432211000</v>
+        <v>440711000</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>159</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>5979211000</v>
+        <v>5987711000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6))+SUMPRODUCT((B13:B76="")*(F13:F76="Claimed"))</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>161</v>
@@ -4138,14 +4138,14 @@
       </c>
       <c r="B8" s="16" t="n">
         <f aca="false">IFERROR(INDEX(A13:A76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),"All done")</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>163</v>
       </c>
       <c r="E8" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6)*(F13:F76&lt;&gt;"Claimed"))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="B9" s="20" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>2789000</v>
+        <v>9289000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3692789000</v>
+        <v>3684289000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>528818361.289085</v>
+        <v>528126531.296779</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4837,7 +4837,7 @@
       <c r="D50" s="12"/>
       <c r="E50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2789000</v>
+        <v>0</v>
       </c>
       <c r="F50" s="11" t="s">
         <v>207</v>
@@ -4856,7 +4856,7 @@
       <c r="D51" s="12"/>
       <c r="E51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>17789000</v>
+        <v>9289000</v>
       </c>
       <c r="F51" s="11" t="s">
         <v>207</v>
@@ -4875,7 +4875,7 @@
       <c r="D52" s="12"/>
       <c r="E52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>47789000</v>
+        <v>39289000</v>
       </c>
       <c r="F52" s="11" t="s">
         <v>207</v>
@@ -4896,7 +4896,7 @@
       </c>
       <c r="E53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>77789000</v>
+        <v>69289000</v>
       </c>
       <c r="F53" s="11" t="s">
         <v>207</v>
@@ -4915,7 +4915,7 @@
       <c r="D54" s="12"/>
       <c r="E54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>107789000</v>
+        <v>99289000</v>
       </c>
       <c r="F54" s="11" t="s">
         <v>207</v>
@@ -4934,7 +4934,7 @@
       <c r="D55" s="12"/>
       <c r="E55" s="23" t="n">
         <f aca="false">IF(B55="","",MAX(0,B55-$B$6))</f>
-        <v>137789000</v>
+        <v>129289000</v>
       </c>
       <c r="F55" s="11" t="s">
         <v>207</v>
@@ -4953,7 +4953,7 @@
       <c r="D56" s="12"/>
       <c r="E56" s="23" t="n">
         <f aca="false">IF(B56="","",MAX(0,B56-$B$6))</f>
-        <v>167789000</v>
+        <v>159289000</v>
       </c>
       <c r="F56" s="11" t="s">
         <v>207</v>
@@ -4972,7 +4972,7 @@
       <c r="D57" s="12"/>
       <c r="E57" s="23" t="n">
         <f aca="false">IF(B57="","",MAX(0,B57-$B$6))</f>
-        <v>197789000</v>
+        <v>189289000</v>
       </c>
       <c r="F57" s="11" t="s">
         <v>207</v>
@@ -4991,7 +4991,7 @@
       <c r="D58" s="12"/>
       <c r="E58" s="23" t="n">
         <f aca="false">IF(B58="","",MAX(0,B58-$B$6))</f>
-        <v>227789000</v>
+        <v>219289000</v>
       </c>
       <c r="F58" s="11" t="s">
         <v>207</v>
@@ -5010,7 +5010,7 @@
       <c r="D59" s="12"/>
       <c r="E59" s="23" t="n">
         <f aca="false">IF(B59="","",MAX(0,B59-$B$6))</f>
-        <v>257789000</v>
+        <v>249289000</v>
       </c>
       <c r="F59" s="11" t="s">
         <v>207</v>
@@ -5029,7 +5029,7 @@
       <c r="D60" s="12"/>
       <c r="E60" s="23" t="n">
         <f aca="false">IF(B60="","",MAX(0,B60-$B$6))</f>
-        <v>317789000</v>
+        <v>309289000</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>207</v>
@@ -5048,7 +5048,7 @@
       <c r="D61" s="12"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>392789000</v>
+        <v>384289000</v>
       </c>
       <c r="F61" s="11" t="s">
         <v>207</v>
@@ -5067,7 +5067,7 @@
       <c r="D62" s="12"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>467789000</v>
+        <v>459289000</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>207</v>
@@ -5086,7 +5086,7 @@
       <c r="D63" s="12"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>542789000</v>
+        <v>534289000</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>207</v>
@@ -5105,7 +5105,7 @@
       <c r="D64" s="12"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>617789000</v>
+        <v>609289000</v>
       </c>
       <c r="F64" s="11" t="s">
         <v>207</v>
@@ -5124,7 +5124,7 @@
       <c r="D65" s="12"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>692789000</v>
+        <v>684289000</v>
       </c>
       <c r="F65" s="11" t="s">
         <v>207</v>
@@ -5143,7 +5143,7 @@
       <c r="D66" s="12"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>767789000</v>
+        <v>759289000</v>
       </c>
       <c r="F66" s="11" t="s">
         <v>207</v>
@@ -5162,7 +5162,7 @@
       <c r="D67" s="12"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>917789000</v>
+        <v>909289000</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>207</v>
@@ -5181,7 +5181,7 @@
       <c r="D68" s="12"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>1067789000</v>
+        <v>1059289000</v>
       </c>
       <c r="F68" s="11" t="s">
         <v>207</v>
@@ -5200,7 +5200,7 @@
       <c r="D69" s="12"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>1217789000</v>
+        <v>1209289000</v>
       </c>
       <c r="F69" s="11" t="s">
         <v>207</v>
@@ -5219,7 +5219,7 @@
       <c r="D70" s="12"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1442789000</v>
+        <v>1434289000</v>
       </c>
       <c r="F70" s="11" t="s">
         <v>207</v>
@@ -5238,7 +5238,7 @@
       <c r="D71" s="12"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1817789000</v>
+        <v>1809289000</v>
       </c>
       <c r="F71" s="11" t="s">
         <v>207</v>
@@ -5257,7 +5257,7 @@
       <c r="D72" s="12"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>2192789000</v>
+        <v>2184289000</v>
       </c>
       <c r="F72" s="11" t="s">
         <v>207</v>
@@ -5276,7 +5276,7 @@
       <c r="D73" s="12"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2567789000</v>
+        <v>2559289000</v>
       </c>
       <c r="F73" s="11" t="s">
         <v>207</v>
@@ -5295,7 +5295,7 @@
       <c r="D74" s="12"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2942789000</v>
+        <v>2934289000</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>207</v>
@@ -5314,7 +5314,7 @@
       <c r="D75" s="12"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>3317789000</v>
+        <v>3309289000</v>
       </c>
       <c r="F75" s="11" t="s">
         <v>207</v>
@@ -5333,7 +5333,7 @@
       <c r="D76" s="12"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3692789000</v>
+        <v>3684289000</v>
       </c>
       <c r="F76" s="11" t="s">
         <v>207</v>
@@ -10451,7 +10451,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19966394.5132271</v>
+        <v>19986277.4313375</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Crossbones plan and correct training stock
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="549">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1203,10 +1203,22 @@
     <t xml:space="preserve">Iron Monger Iso-8 to T3 level 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Crossbones to level 85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unlocks T3 Iso-8 and his raid tasks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crossbones Iso-8 to T3 level 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimate based on Iron Monger</t>
+  </si>
+  <si>
     <t xml:space="preserve">Doctor Strange to level 101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planned</t>
   </si>
   <si>
     <t xml:space="preserve">Check cost in game</t>
@@ -4172,7 +4184,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>528126531.296779</v>
+        <v>528568817.036196</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7040,7 +7052,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:K91"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -7092,7 +7104,7 @@
         <v>315</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>6570000</v>
+        <v>9320000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>755800</v>
@@ -7110,7 +7122,7 @@
         <v>715</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>429</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7152,7 +7164,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>29420000</v>
+        <v>32170000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -7176,7 +7188,7 @@
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>619</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7184,32 +7196,32 @@
         <v>318</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$87,"Planned",B69:B87)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$69:$J$89,"Planned",B69:B89)</f>
+        <v>9791250</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$87,"Planned",C69:C87)</f>
+        <f aca="false">SUMIF($J$69:$J$89,"Planned",C69:C89)</f>
+        <v>2070000</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <f aca="false">SUMIF($J$69:$J$89,"Planned",D69:D89)</f>
+        <v>2640000</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <f aca="false">SUMIF($J$69:$J$89,"Planned",E69:E89)</f>
         <v>1710000</v>
       </c>
-      <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$87,"Planned",D69:D87)</f>
-        <v>2640000</v>
-      </c>
-      <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$87,"Planned",E69:E87)</f>
-        <v>1710000</v>
-      </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$87,"Planned",F69:F87)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$69:$J$89,"Planned",F69:F89)</f>
+        <v>1</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$87,"Planned",G69:G87)</f>
+        <f aca="false">SUMIF($J$69:$J$89,"Planned",G69:G89)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$87,"Planned",H69:H87)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$69:$J$89,"Planned",H69:H89)</f>
+        <v>979</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7218,11 +7230,11 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>29420000</v>
+        <v>22378750</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>3295800</v>
+        <v>2935800</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
@@ -7234,7 +7246,7 @@
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
@@ -7242,7 +7254,7 @@
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>619</v>
+        <v>215</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9003,7 +9015,9 @@
       <c r="A71" s="12" t="s">
         <v>390</v>
       </c>
-      <c r="B71" s="26"/>
+      <c r="B71" s="30" t="n">
+        <v>9791250</v>
+      </c>
       <c r="C71" s="30" t="n">
         <v>0</v>
       </c>
@@ -9013,11 +9027,17 @@
       <c r="E71" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F71" s="26"/>
-      <c r="G71" s="26"/>
-      <c r="H71" s="26"/>
+      <c r="F71" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="30" t="n">
+        <v>979</v>
+      </c>
       <c r="I71" s="30" t="n">
-        <v>3000000</v>
+        <v>55000000</v>
       </c>
       <c r="J71" s="11" t="s">
         <v>391</v>
@@ -9030,9 +9050,11 @@
       <c r="A72" s="12" t="s">
         <v>393</v>
       </c>
-      <c r="B72" s="26"/>
+      <c r="B72" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="C72" s="30" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
       <c r="D72" s="30" t="n">
         <v>0</v>
@@ -9040,22 +9062,28 @@
       <c r="E72" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F72" s="26"/>
-      <c r="G72" s="26"/>
-      <c r="H72" s="26"/>
+      <c r="F72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I72" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J72" s="11" t="s">
         <v>391</v>
       </c>
       <c r="K72" s="15" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B73" s="26"/>
       <c r="C73" s="30" t="n">
@@ -9077,12 +9105,12 @@
         <v>391</v>
       </c>
       <c r="K73" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B74" s="26"/>
       <c r="C74" s="30" t="n">
@@ -9104,12 +9132,12 @@
         <v>391</v>
       </c>
       <c r="K74" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B75" s="26"/>
       <c r="C75" s="30" t="n">
@@ -9121,70 +9149,60 @@
       <c r="E75" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F75" s="26"/>
+      <c r="G75" s="26"/>
+      <c r="H75" s="26"/>
       <c r="I75" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J75" s="11" t="s">
         <v>391</v>
       </c>
       <c r="K75" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>397</v>
-      </c>
-      <c r="B76" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>399</v>
+      </c>
+      <c r="B76" s="26"/>
       <c r="C76" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="D76" s="30" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="E76" s="30" t="n">
-        <v>1710000</v>
-      </c>
-      <c r="F76" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H76" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F76" s="26"/>
+      <c r="G76" s="26"/>
+      <c r="H76" s="26"/>
       <c r="I76" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J76" s="11" t="s">
         <v>391</v>
       </c>
       <c r="K76" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>399</v>
-      </c>
-      <c r="B77" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C77" s="26"/>
-      <c r="D77" s="26"/>
-      <c r="E77" s="26"/>
+        <v>400</v>
+      </c>
+      <c r="B77" s="26"/>
+      <c r="C77" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="F77" s="30" t="n">
         <v>0</v>
       </c>
@@ -9201,19 +9219,25 @@
         <v>391</v>
       </c>
       <c r="K77" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B78" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C78" s="26"/>
-      <c r="D78" s="26"/>
-      <c r="E78" s="26"/>
+      <c r="C78" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D78" s="30" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="E78" s="30" t="n">
+        <v>1710000</v>
+      </c>
       <c r="F78" s="30" t="n">
         <v>0</v>
       </c>
@@ -9227,15 +9251,15 @@
         <v>17000000</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="K78" s="15" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B79" s="30" t="n">
         <v>0</v>
@@ -9256,15 +9280,15 @@
         <v>17000000</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B80" s="30" t="n">
         <v>0</v>
@@ -9285,66 +9309,98 @@
         <v>17000000</v>
       </c>
       <c r="J80" s="11" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="K80" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" s="26"/>
+      <c r="D81" s="26"/>
+      <c r="E81" s="26"/>
+      <c r="F81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J81" s="11" t="s">
+        <v>405</v>
+      </c>
+      <c r="K81" s="15" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="B82" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" s="26"/>
+      <c r="D82" s="26"/>
+      <c r="E82" s="26"/>
+      <c r="F82" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J82" s="11" t="s">
+        <v>405</v>
+      </c>
+      <c r="K82" s="15" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="12" t="s">
+        <v>408</v>
+      </c>
+      <c r="B83" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="26"/>
-      <c r="G81" s="26"/>
-      <c r="H81" s="26"/>
-      <c r="I81" s="30" t="n">
+      <c r="C83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" s="26"/>
+      <c r="G83" s="26"/>
+      <c r="H83" s="26"/>
+      <c r="I83" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J81" s="11" t="s">
-        <v>401</v>
-      </c>
-      <c r="K81" s="15" t="s">
+      <c r="J83" s="11" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="12"/>
-      <c r="B82" s="30"/>
-      <c r="C82" s="30"/>
-      <c r="D82" s="30"/>
-      <c r="E82" s="30"/>
-      <c r="F82" s="30"/>
-      <c r="G82" s="30"/>
-      <c r="H82" s="30"/>
-      <c r="I82" s="30"/>
-      <c r="J82" s="11"/>
-      <c r="K82" s="12"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="12"/>
-      <c r="B83" s="30"/>
-      <c r="C83" s="30"/>
-      <c r="D83" s="30"/>
-      <c r="E83" s="30"/>
-      <c r="F83" s="30"/>
-      <c r="G83" s="30"/>
-      <c r="H83" s="30"/>
-      <c r="I83" s="30"/>
-      <c r="J83" s="11"/>
-      <c r="K83" s="12"/>
+      <c r="K83" s="15" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12"/>
@@ -9398,13 +9454,39 @@
       <c r="J87" s="11"/>
       <c r="K87" s="12"/>
     </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="12"/>
+      <c r="B88" s="30"/>
+      <c r="C88" s="30"/>
+      <c r="D88" s="30"/>
+      <c r="E88" s="30"/>
+      <c r="F88" s="30"/>
+      <c r="G88" s="30"/>
+      <c r="H88" s="30"/>
+      <c r="I88" s="30"/>
+      <c r="J88" s="11"/>
+      <c r="K88" s="12"/>
+    </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="16" t="s">
-        <v>406</v>
-      </c>
-      <c r="I89" s="20" t="n">
-        <f aca="false">SUMIF(J69:J87,"Planned",I69:I87)</f>
-        <v>63000000</v>
+      <c r="A89" s="12"/>
+      <c r="B89" s="30"/>
+      <c r="C89" s="30"/>
+      <c r="D89" s="30"/>
+      <c r="E89" s="30"/>
+      <c r="F89" s="30"/>
+      <c r="G89" s="30"/>
+      <c r="H89" s="30"/>
+      <c r="I89" s="30"/>
+      <c r="J89" s="11"/>
+      <c r="K89" s="12"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="16" t="s">
+        <v>410</v>
+      </c>
+      <c r="I91" s="20" t="n">
+        <f aca="false">SUMIF(J69:J89,"Planned",I69:I89)</f>
+        <v>118000000</v>
       </c>
     </row>
   </sheetData>
@@ -9413,7 +9495,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J69:J87">
+  <conditionalFormatting sqref="J69:J89">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
@@ -9428,7 +9510,7 @@
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J69:J87" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J69:J89" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9459,12 +9541,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9478,50 +9560,50 @@
         <v>308</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="E6" s="32" t="s">
         <v>387</v>
@@ -9536,16 +9618,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="E7" s="32" t="s">
         <v>387</v>
@@ -9560,16 +9642,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>428</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>424</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>420</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="E8" s="32" t="s">
         <v>387</v>
@@ -9584,16 +9666,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="E9" s="32" t="s">
         <v>387</v>
@@ -9608,16 +9690,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="E10" s="32" t="s">
         <v>387</v>
@@ -9632,16 +9714,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="E11" s="32" t="s">
         <v>387</v>
@@ -9656,16 +9738,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="E12" s="32" t="s">
         <v>387</v>
@@ -9680,16 +9762,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="E13" s="32" t="s">
         <v>387</v>
@@ -9704,16 +9786,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="E14" s="32" t="s">
         <v>387</v>
@@ -9728,16 +9810,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="E15" s="32" t="s">
         <v>387</v>
@@ -9752,16 +9834,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="E16" s="32" t="s">
         <v>387</v>
@@ -9776,16 +9858,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -9798,16 +9880,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="E18" s="32" t="s">
         <v>387</v>
@@ -9822,16 +9904,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
+        <v>447</v>
+      </c>
+      <c r="B19" s="13" t="s">
         <v>443</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>439</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="E19" s="32" t="s">
         <v>387</v>
@@ -9846,16 +9928,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E20" s="32" t="s">
         <v>387</v>
@@ -9870,21 +9952,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="E22" s="32" t="s">
         <v>387</v>
@@ -9899,16 +9981,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -9921,16 +10003,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -9943,16 +10025,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="E25" s="32" t="s">
         <v>387</v>
@@ -9967,16 +10049,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="E26" s="32" t="s">
         <v>387</v>
@@ -9991,16 +10073,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -10013,16 +10095,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -10035,21 +10117,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -10062,16 +10144,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -10084,16 +10166,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="B32" s="13" t="s">
         <v>470</v>
       </c>
-      <c r="B32" s="13" t="s">
-        <v>466</v>
-      </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -10106,16 +10188,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="E33" s="32" t="s">
         <v>387</v>
@@ -10130,16 +10212,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -10152,16 +10234,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
+        <v>481</v>
+      </c>
+      <c r="B35" s="13" t="s">
         <v>477</v>
       </c>
-      <c r="B35" s="13" t="s">
-        <v>473</v>
-      </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -10174,16 +10256,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -10196,16 +10278,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -10218,7 +10300,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -10255,7 +10337,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -10292,7 +10374,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
     </row>
   </sheetData>
@@ -10336,12 +10418,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10349,10 +10431,10 @@
         <v>155</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10363,13 +10445,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10380,7 +10462,7 @@
         <v>285572765</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -10430,7 +10512,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -10438,7 +10520,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -10447,11 +10529,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>19986277.4313375</v>
+        <v>20003015.1830075</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10462,19 +10544,19 @@
         <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10490,7 +10572,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10516,7 +10598,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10542,7 +10624,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10568,7 +10650,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10593,10 +10675,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10621,10 +10703,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10649,10 +10731,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10677,10 +10759,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10705,10 +10787,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10733,10 +10815,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -10762,7 +10844,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -10787,10 +10869,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -10815,10 +10897,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -10843,10 +10925,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -10874,7 +10956,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -10901,10 +10983,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -10931,10 +11013,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="D29" s="12" t="s">
         <v>518</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>514</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -10961,10 +11043,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -10985,10 +11067,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -11015,7 +11097,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -11043,10 +11125,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -11073,7 +11155,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -11101,10 +11183,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -11131,7 +11213,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -11159,10 +11241,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -11189,7 +11271,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -11217,10 +11299,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -11247,7 +11329,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -11275,10 +11357,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -11305,7 +11387,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -11333,10 +11415,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -11363,7 +11445,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -11391,7 +11473,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -11419,7 +11501,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -11447,7 +11529,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11475,7 +11557,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11503,7 +11585,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11531,7 +11613,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11559,7 +11641,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11587,7 +11669,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11615,7 +11697,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11643,7 +11725,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11665,7 +11747,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add premium battle pass rewards and update gold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="552">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1075,6 +1075,15 @@
   </si>
   <si>
     <t xml:space="preserve">Battle pass level 88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claimed Oct 11, in current stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battle pass level 95, premium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battle pass level 97, premium</t>
   </si>
   <si>
     <t xml:space="preserve">Battle pass level 97</t>
@@ -4184,7 +4193,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>528568817.036196</v>
+        <v>533769203.857946</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7052,7 +7061,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -7104,7 +7113,7 @@
         <v>315</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>9320000</v>
+        <v>18170000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>755800</v>
@@ -7130,32 +7139,32 @@
         <v>316</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
-        <v>22850000</v>
+        <f aca="false">SUMIFS(B13:B67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <v>32500000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
+        <f aca="false">SUMIFS(C13:C67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
         <v>4250000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
+        <f aca="false">SUMIFS(D13:D67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
         <v>3136000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
+        <f aca="false">SUMIFS(E13:E67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
         <v>2736000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
+        <f aca="false">SUMIFS(F13:F67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
+        <f aca="false">SUMIFS(G13:G67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H65,$I$13:$I$65,"Yes",$J$13:$J$65,"No")</f>
-        <v>190</v>
+        <f aca="false">SUMIFS(H13:H67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <v>990</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7164,7 +7173,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>32170000</v>
+        <v>50670000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -7188,7 +7197,7 @@
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1194</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7196,31 +7205,31 @@
         <v>318</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$89,"Planned",B69:B89)</f>
+        <f aca="false">SUMIF($J$71:$J$91,"Planned",B71:B91)</f>
         <v>9791250</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$89,"Planned",C69:C89)</f>
+        <f aca="false">SUMIF($J$71:$J$91,"Planned",C71:C91)</f>
         <v>2070000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$89,"Planned",D69:D89)</f>
+        <f aca="false">SUMIF($J$71:$J$91,"Planned",D71:D91)</f>
         <v>2640000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$89,"Planned",E69:E89)</f>
+        <f aca="false">SUMIF($J$71:$J$91,"Planned",E71:E91)</f>
         <v>1710000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$89,"Planned",F69:F89)</f>
+        <f aca="false">SUMIF($J$71:$J$91,"Planned",F71:F91)</f>
         <v>1</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$89,"Planned",G69:G89)</f>
+        <f aca="false">SUMIF($J$71:$J$91,"Planned",G71:G91)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$69:$J$89,"Planned",H69:H89)</f>
+        <f aca="false">SUMIF($J$71:$J$91,"Planned",H71:H91)</f>
         <v>979</v>
       </c>
     </row>
@@ -7230,7 +7239,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>22378750</v>
+        <v>40878750</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -7254,7 +7263,7 @@
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>215</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7952,7 +7961,7 @@
         <v>347</v>
       </c>
       <c r="B32" s="30" t="n">
-        <v>350000</v>
+        <v>0</v>
       </c>
       <c r="C32" s="30" t="n">
         <v>0</v>
@@ -7978,14 +7987,16 @@
       <c r="J32" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K32" s="15"/>
+      <c r="K32" s="15" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B33" s="30" t="n">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="C33" s="30" t="n">
         <v>0</v>
@@ -8003,7 +8014,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="30" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="I33" s="11" t="s">
         <v>249</v>
@@ -8015,19 +8026,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B34" s="30" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="C34" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="D34" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="E34" s="30" t="n">
-        <v>2600000</v>
+        <v>0</v>
       </c>
       <c r="F34" s="30" t="n">
         <v>0</v>
@@ -8044,25 +8055,23 @@
       <c r="J34" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K34" s="15" t="s">
-        <v>350</v>
-      </c>
+      <c r="K34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
         <v>351</v>
       </c>
       <c r="B35" s="30" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="C35" s="30" t="n">
-        <v>900000</v>
+        <v>0</v>
       </c>
       <c r="D35" s="30" t="n">
-        <v>1300000</v>
+        <v>0</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>1900000</v>
+        <v>0</v>
       </c>
       <c r="F35" s="30" t="n">
         <v>0</v>
@@ -8074,30 +8083,28 @@
         <v>0</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J35" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K35" s="15" t="s">
-        <v>352</v>
-      </c>
+      <c r="K35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B36" s="30" t="n">
         <v>0</v>
       </c>
       <c r="C36" s="30" t="n">
-        <v>950000</v>
+        <v>3000000</v>
       </c>
       <c r="D36" s="30" t="n">
-        <v>0</v>
+        <v>3000000</v>
       </c>
       <c r="E36" s="30" t="n">
-        <v>1900000</v>
+        <v>2600000</v>
       </c>
       <c r="F36" s="30" t="n">
         <v>0</v>
@@ -8109,12 +8116,14 @@
         <v>0</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J36" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K36" s="15"/>
+      <c r="K36" s="15" t="s">
+        <v>353</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
@@ -8124,10 +8133,10 @@
         <v>0</v>
       </c>
       <c r="C37" s="30" t="n">
-        <v>0</v>
+        <v>900000</v>
       </c>
       <c r="D37" s="30" t="n">
-        <v>1400000</v>
+        <v>1300000</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>1900000</v>
@@ -8147,23 +8156,25 @@
       <c r="J37" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K37" s="15"/>
+      <c r="K37" s="15" t="s">
+        <v>355</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B38" s="30" t="n">
-        <v>900000</v>
+        <v>0</v>
       </c>
       <c r="C38" s="30" t="n">
-        <v>0</v>
+        <v>950000</v>
       </c>
       <c r="D38" s="30" t="n">
         <v>0</v>
       </c>
       <c r="E38" s="30" t="n">
-        <v>0</v>
+        <v>1900000</v>
       </c>
       <c r="F38" s="30" t="n">
         <v>0</v>
@@ -8180,9 +8191,7 @@
       <c r="J38" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K38" s="15" t="s">
-        <v>356</v>
-      </c>
+      <c r="K38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
@@ -8195,19 +8204,19 @@
         <v>0</v>
       </c>
       <c r="D39" s="30" t="n">
-        <v>0</v>
+        <v>1400000</v>
       </c>
       <c r="E39" s="30" t="n">
-        <v>0</v>
+        <v>1900000</v>
       </c>
       <c r="F39" s="30" t="n">
         <v>0</v>
       </c>
       <c r="G39" s="30" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H39" s="30" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="I39" s="11" t="s">
         <v>253</v>
@@ -8215,16 +8224,14 @@
       <c r="J39" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K39" s="15" t="s">
-        <v>356</v>
-      </c>
+      <c r="K39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
         <v>358</v>
       </c>
       <c r="B40" s="30" t="n">
-        <v>3300000</v>
+        <v>900000</v>
       </c>
       <c r="C40" s="30" t="n">
         <v>0</v>
@@ -8245,10 +8252,10 @@
         <v>0</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="K40" s="15" t="s">
         <v>359</v>
@@ -8259,7 +8266,7 @@
         <v>360</v>
       </c>
       <c r="B41" s="30" t="n">
-        <v>3300000</v>
+        <v>0</v>
       </c>
       <c r="C41" s="30" t="n">
         <v>0</v>
@@ -8274,30 +8281,30 @@
         <v>0</v>
       </c>
       <c r="G41" s="30" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H41" s="30" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="J41" s="11" t="s">
         <v>253</v>
       </c>
       <c r="K41" s="15" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B42" s="30" t="n">
-        <v>0</v>
+        <v>3300000</v>
       </c>
       <c r="C42" s="30" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D42" s="30" t="n">
         <v>0</v>
@@ -8318,18 +8325,18 @@
         <v>249</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B43" s="30" t="n">
-        <v>0</v>
+        <v>3300000</v>
       </c>
       <c r="C43" s="30" t="n">
         <v>0</v>
@@ -8340,9 +8347,15 @@
       <c r="E43" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F43" s="30"/>
-      <c r="G43" s="30"/>
-      <c r="H43" s="30"/>
+      <c r="F43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I43" s="11" t="s">
         <v>249</v>
       </c>
@@ -8350,24 +8363,24 @@
         <v>253</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B44" s="30" t="n">
         <v>0</v>
       </c>
       <c r="C44" s="30" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D44" s="30" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="E44" s="30" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="F44" s="30" t="n">
         <v>0</v>
@@ -8385,15 +8398,15 @@
         <v>253</v>
       </c>
       <c r="K44" s="15" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B45" s="30" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C45" s="30" t="n">
         <v>0</v>
@@ -8404,15 +8417,9 @@
       <c r="E45" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F45" s="30"/>
+      <c r="G45" s="30"/>
+      <c r="H45" s="30"/>
       <c r="I45" s="11" t="s">
         <v>249</v>
       </c>
@@ -8420,24 +8427,24 @@
         <v>253</v>
       </c>
       <c r="K45" s="15" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B46" s="30" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C46" s="30" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="30" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="E46" s="30" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="F46" s="30" t="n">
         <v>0</v>
@@ -8455,12 +8462,12 @@
         <v>253</v>
       </c>
       <c r="K46" s="15" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B47" s="30" t="n">
         <v>750000</v>
@@ -8490,7 +8497,7 @@
         <v>253</v>
       </c>
       <c r="K47" s="15" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8525,12 +8532,12 @@
         <v>253</v>
       </c>
       <c r="K48" s="15" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B49" s="30" t="n">
         <v>750000</v>
@@ -8560,12 +8567,12 @@
         <v>253</v>
       </c>
       <c r="K49" s="15" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B50" s="30" t="n">
         <v>750000</v>
@@ -8595,12 +8602,12 @@
         <v>253</v>
       </c>
       <c r="K50" s="15" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B51" s="30" t="n">
         <v>750000</v>
@@ -8630,12 +8637,12 @@
         <v>253</v>
       </c>
       <c r="K51" s="15" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B52" s="30" t="n">
         <v>750000</v>
@@ -8665,18 +8672,18 @@
         <v>253</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B53" s="30" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C53" s="30" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D53" s="30" t="n">
         <v>0</v>
@@ -8700,7 +8707,7 @@
         <v>253</v>
       </c>
       <c r="K53" s="15" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8708,7 +8715,7 @@
         <v>380</v>
       </c>
       <c r="B54" s="30" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C54" s="30" t="n">
         <v>0</v>
@@ -8735,18 +8742,18 @@
         <v>253</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B55" s="30" t="n">
         <v>0</v>
       </c>
       <c r="C55" s="30" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D55" s="30" t="n">
         <v>0</v>
@@ -8764,40 +8771,84 @@
         <v>0</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J55" s="11" t="s">
         <v>253</v>
       </c>
       <c r="K55" s="15" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="12" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="12"/>
-      <c r="B56" s="30"/>
-      <c r="C56" s="30"/>
-      <c r="D56" s="30"/>
-      <c r="E56" s="30"/>
-      <c r="F56" s="30"/>
-      <c r="G56" s="30"/>
-      <c r="H56" s="30"/>
-      <c r="I56" s="11"/>
-      <c r="J56" s="11"/>
-      <c r="K56" s="12"/>
+      <c r="B56" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J56" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K56" s="15" t="s">
+        <v>384</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="12"/>
-      <c r="B57" s="30"/>
-      <c r="C57" s="30"/>
-      <c r="D57" s="30"/>
-      <c r="E57" s="30"/>
-      <c r="F57" s="30"/>
-      <c r="G57" s="30"/>
-      <c r="H57" s="30"/>
-      <c r="I57" s="11"/>
-      <c r="J57" s="11"/>
-      <c r="K57" s="12"/>
+      <c r="A57" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="B57" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J57" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K57" s="15" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12"/>
@@ -8903,158 +8954,116 @@
       <c r="J65" s="11"/>
       <c r="K65" s="12"/>
     </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="12"/>
+      <c r="B66" s="30"/>
+      <c r="C66" s="30"/>
+      <c r="D66" s="30"/>
+      <c r="E66" s="30"/>
+      <c r="F66" s="30"/>
+      <c r="G66" s="30"/>
+      <c r="H66" s="30"/>
+      <c r="I66" s="11"/>
+      <c r="J66" s="11"/>
+      <c r="K66" s="12"/>
+    </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="29" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3" t="s">
-        <v>385</v>
-      </c>
-      <c r="B68" s="3" t="s">
+      <c r="A67" s="12"/>
+      <c r="B67" s="30"/>
+      <c r="C67" s="30"/>
+      <c r="D67" s="30"/>
+      <c r="E67" s="30"/>
+      <c r="F67" s="30"/>
+      <c r="G67" s="30"/>
+      <c r="H67" s="30"/>
+      <c r="I67" s="11"/>
+      <c r="J67" s="11"/>
+      <c r="K67" s="12"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="29" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="B70" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C70" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="D68" s="3" t="s">
+      <c r="D70" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="E68" s="3" t="s">
+      <c r="E70" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="F68" s="3" t="s">
+      <c r="F70" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="G68" s="3" t="s">
+      <c r="G70" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="H68" s="3" t="s">
+      <c r="H70" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="I68" s="3" t="s">
+      <c r="I70" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J68" s="3" t="s">
+      <c r="J70" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K68" s="3" t="s">
+      <c r="K70" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="B69" s="30" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C69" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G69" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H69" s="30" t="n">
-        <v>183</v>
-      </c>
-      <c r="I69" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" s="11" t="s">
-        <v>387</v>
-      </c>
-      <c r="K69" s="15" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="12" t="s">
-        <v>389</v>
-      </c>
-      <c r="B70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C70" s="30" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" s="11" t="s">
-        <v>387</v>
-      </c>
-      <c r="K70" s="15"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="B71" s="30" t="n">
+        <v>1837500</v>
+      </c>
+      <c r="C71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G71" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" s="30" t="n">
+        <v>183</v>
+      </c>
+      <c r="I71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="11" t="s">
         <v>390</v>
       </c>
-      <c r="B71" s="30" t="n">
-        <v>9791250</v>
-      </c>
-      <c r="C71" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E71" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F71" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H71" s="30" t="n">
-        <v>979</v>
-      </c>
-      <c r="I71" s="30" t="n">
-        <v>55000000</v>
-      </c>
-      <c r="J71" s="11" t="s">
+      <c r="K71" s="15" t="s">
         <v>391</v>
-      </c>
-      <c r="K71" s="15" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B72" s="30" t="n">
         <v>0</v>
       </c>
       <c r="C72" s="30" t="n">
-        <v>360000</v>
+        <v>359800</v>
       </c>
       <c r="D72" s="30" t="n">
         <v>0</v>
@@ -9075,64 +9084,78 @@
         <v>0</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>391</v>
-      </c>
-      <c r="K72" s="15" t="s">
-        <v>394</v>
-      </c>
+        <v>390</v>
+      </c>
+      <c r="K72" s="15"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="B73" s="30" t="n">
+        <v>9791250</v>
+      </c>
+      <c r="C73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="30" t="n">
+        <v>979</v>
+      </c>
+      <c r="I73" s="30" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="J73" s="11" t="s">
+        <v>394</v>
+      </c>
+      <c r="K73" s="15" t="s">
         <v>395</v>
-      </c>
-      <c r="B73" s="26"/>
-      <c r="C73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="26"/>
-      <c r="G73" s="26"/>
-      <c r="H73" s="26"/>
-      <c r="I73" s="30" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J73" s="11" t="s">
-        <v>391</v>
-      </c>
-      <c r="K73" s="15" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="B74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" s="30" t="n">
+        <v>360000</v>
+      </c>
+      <c r="D74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" s="11" t="s">
+        <v>394</v>
+      </c>
+      <c r="K74" s="15" t="s">
         <v>397</v>
-      </c>
-      <c r="B74" s="26"/>
-      <c r="C74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F74" s="26"/>
-      <c r="G74" s="26"/>
-      <c r="H74" s="26"/>
-      <c r="I74" s="30" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J74" s="11" t="s">
-        <v>391</v>
-      </c>
-      <c r="K74" s="15" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9156,15 +9179,15 @@
         <v>3000000</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="K75" s="15" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B76" s="26"/>
       <c r="C76" s="30" t="n">
@@ -9183,15 +9206,15 @@
         <v>3000000</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="K76" s="15" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B77" s="26"/>
       <c r="C77" s="30" t="n">
@@ -9203,70 +9226,60 @@
       <c r="E77" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F77" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G77" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H77" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F77" s="26"/>
+      <c r="G77" s="26"/>
+      <c r="H77" s="26"/>
       <c r="I77" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="K77" s="15" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>401</v>
-      </c>
-      <c r="B78" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>402</v>
+      </c>
+      <c r="B78" s="26"/>
       <c r="C78" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="D78" s="30" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="E78" s="30" t="n">
-        <v>1710000</v>
-      </c>
-      <c r="F78" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G78" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H78" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F78" s="26"/>
+      <c r="G78" s="26"/>
+      <c r="H78" s="26"/>
       <c r="I78" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="K78" s="15" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
         <v>403</v>
       </c>
-      <c r="B79" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C79" s="26"/>
-      <c r="D79" s="26"/>
-      <c r="E79" s="26"/>
+      <c r="B79" s="26"/>
+      <c r="C79" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="F79" s="30" t="n">
         <v>0</v>
       </c>
@@ -9280,10 +9293,10 @@
         <v>17000000</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9293,9 +9306,15 @@
       <c r="B80" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C80" s="26"/>
-      <c r="D80" s="26"/>
-      <c r="E80" s="26"/>
+      <c r="C80" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D80" s="30" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="E80" s="30" t="n">
+        <v>1710000</v>
+      </c>
       <c r="F80" s="30" t="n">
         <v>0</v>
       </c>
@@ -9309,10 +9328,10 @@
         <v>17000000</v>
       </c>
       <c r="J80" s="11" t="s">
+        <v>394</v>
+      </c>
+      <c r="K80" s="15" t="s">
         <v>405</v>
-      </c>
-      <c r="K80" s="15" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9338,10 +9357,10 @@
         <v>17000000</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="K81" s="15" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9367,66 +9386,98 @@
         <v>17000000</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
+        <v>409</v>
+      </c>
+      <c r="B83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" s="26"/>
+      <c r="D83" s="26"/>
+      <c r="E83" s="26"/>
+      <c r="F83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J83" s="11" t="s">
         <v>408</v>
       </c>
-      <c r="B83" s="30" t="n">
+      <c r="K83" s="15" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="B84" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" s="26"/>
+      <c r="D84" s="26"/>
+      <c r="E84" s="26"/>
+      <c r="F84" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J84" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="K84" s="15" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="12" t="s">
+        <v>411</v>
+      </c>
+      <c r="B85" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C83" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D83" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E83" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F83" s="26"/>
-      <c r="G83" s="26"/>
-      <c r="H83" s="26"/>
-      <c r="I83" s="30" t="n">
+      <c r="C85" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="26"/>
+      <c r="G85" s="26"/>
+      <c r="H85" s="26"/>
+      <c r="I85" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J83" s="11" t="s">
-        <v>405</v>
-      </c>
-      <c r="K83" s="15" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="12"/>
-      <c r="B84" s="30"/>
-      <c r="C84" s="30"/>
-      <c r="D84" s="30"/>
-      <c r="E84" s="30"/>
-      <c r="F84" s="30"/>
-      <c r="G84" s="30"/>
-      <c r="H84" s="30"/>
-      <c r="I84" s="30"/>
-      <c r="J84" s="11"/>
-      <c r="K84" s="12"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="12"/>
-      <c r="B85" s="30"/>
-      <c r="C85" s="30"/>
-      <c r="D85" s="30"/>
-      <c r="E85" s="30"/>
-      <c r="F85" s="30"/>
-      <c r="G85" s="30"/>
-      <c r="H85" s="30"/>
-      <c r="I85" s="30"/>
-      <c r="J85" s="11"/>
-      <c r="K85" s="12"/>
+      <c r="J85" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="K85" s="15" t="s">
+        <v>412</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12"/>
@@ -9480,12 +9531,38 @@
       <c r="J89" s="11"/>
       <c r="K89" s="12"/>
     </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="12"/>
+      <c r="B90" s="30"/>
+      <c r="C90" s="30"/>
+      <c r="D90" s="30"/>
+      <c r="E90" s="30"/>
+      <c r="F90" s="30"/>
+      <c r="G90" s="30"/>
+      <c r="H90" s="30"/>
+      <c r="I90" s="30"/>
+      <c r="J90" s="11"/>
+      <c r="K90" s="12"/>
+    </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="16" t="s">
-        <v>410</v>
-      </c>
-      <c r="I91" s="20" t="n">
-        <f aca="false">SUMIF(J69:J89,"Planned",I69:I89)</f>
+      <c r="A91" s="12"/>
+      <c r="B91" s="30"/>
+      <c r="C91" s="30"/>
+      <c r="D91" s="30"/>
+      <c r="E91" s="30"/>
+      <c r="F91" s="30"/>
+      <c r="G91" s="30"/>
+      <c r="H91" s="30"/>
+      <c r="I91" s="30"/>
+      <c r="J91" s="11"/>
+      <c r="K91" s="12"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="16" t="s">
+        <v>413</v>
+      </c>
+      <c r="I93" s="20" t="n">
+        <f aca="false">SUMIF(J71:J91,"Planned",I71:I91)</f>
         <v>118000000</v>
       </c>
     </row>
@@ -9495,22 +9572,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J69:J89">
+  <conditionalFormatting sqref="J71:J91">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J65">
+  <conditionalFormatting sqref="J13:J67">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J65" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J67" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J69:J89" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J71:J91" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9541,12 +9618,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9560,53 +9637,53 @@
         <v>308</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -9618,19 +9695,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -9642,19 +9719,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -9666,19 +9743,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9690,19 +9767,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9714,19 +9791,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9738,19 +9815,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9762,19 +9839,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9786,19 +9863,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9810,19 +9887,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -9834,19 +9911,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -9858,16 +9935,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -9880,19 +9957,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -9904,19 +9981,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -9928,19 +10005,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -9952,24 +10029,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -9981,16 +10058,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -10003,16 +10080,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="B24" s="13" t="s">
         <v>456</v>
       </c>
-      <c r="B24" s="13" t="s">
-        <v>453</v>
-      </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -10025,19 +10102,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -10049,19 +10126,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -10073,16 +10150,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -10095,16 +10172,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -10117,21 +10194,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -10144,16 +10221,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -10166,16 +10243,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -10188,19 +10265,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -10212,16 +10289,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -10234,16 +10311,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -10256,16 +10333,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -10278,16 +10355,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -10300,7 +10377,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -10337,7 +10414,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -10374,7 +10451,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
   </sheetData>
@@ -10418,12 +10495,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10431,10 +10508,10 @@
         <v>155</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10445,13 +10522,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10462,7 +10539,7 @@
         <v>285572765</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -10512,7 +10589,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -10520,7 +10597,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -10529,11 +10606,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>20003015.1830075</v>
+        <v>20199817.2122427</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10544,19 +10621,19 @@
         <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10572,7 +10649,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10598,7 +10675,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10624,7 +10701,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10650,7 +10727,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10675,10 +10752,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10703,10 +10780,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10731,10 +10808,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10759,10 +10836,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10787,10 +10864,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10815,10 +10892,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -10844,7 +10921,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -10869,10 +10946,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -10897,10 +10974,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -10925,10 +11002,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -10956,7 +11033,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -10983,10 +11060,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
+        <v>524</v>
+      </c>
+      <c r="D28" s="12" t="s">
         <v>521</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>518</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -11013,10 +11090,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -11043,10 +11120,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -11067,10 +11144,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -11097,7 +11174,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -11125,10 +11202,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -11155,7 +11232,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -11183,10 +11260,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -11213,7 +11290,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -11241,10 +11318,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -11271,7 +11348,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -11299,10 +11376,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -11329,7 +11406,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -11357,10 +11434,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -11387,7 +11464,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -11415,10 +11492,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -11445,7 +11522,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -11473,7 +11550,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -11501,7 +11578,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -11529,7 +11606,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11557,7 +11634,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11585,7 +11662,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11613,7 +11690,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11641,7 +11718,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11669,7 +11746,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11697,7 +11774,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11725,7 +11802,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11747,7 +11824,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Count claimed battle pass ions and training
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="552">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1071,13 +1071,13 @@
     <t xml:space="preserve">Battle pass level 86</t>
   </si>
   <si>
+    <t xml:space="preserve">Claimed Oct 11, in current stock</t>
+  </si>
+  <si>
     <t xml:space="preserve">Battle pass level 87</t>
   </si>
   <si>
     <t xml:space="preserve">Battle pass level 88</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claimed Oct 11, in current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Battle pass level 95, premium</t>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>533769203.857946</v>
+        <v>533784657.608701</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7116,7 +7116,7 @@
         <v>18170000</v>
       </c>
       <c r="C5" s="26" t="n">
-        <v>755800</v>
+        <v>1505800</v>
       </c>
       <c r="D5" s="26" t="n">
         <v>4370000</v>
@@ -7131,7 +7131,7 @@
         <v>715</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>1004</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7144,7 +7144,7 @@
       </c>
       <c r="C6" s="27" t="n">
         <f aca="false">SUMIFS(C13:C67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
-        <v>4250000</v>
+        <v>3500000</v>
       </c>
       <c r="D6" s="27" t="n">
         <f aca="false">SUMIFS(D13:D67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
@@ -7164,7 +7164,7 @@
       </c>
       <c r="H6" s="27" t="n">
         <f aca="false">SUMIFS(H13:H67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
-        <v>990</v>
+        <v>940</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7898,7 +7898,7 @@
         <v>0</v>
       </c>
       <c r="C30" s="30" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="D30" s="30" t="n">
         <v>0</v>
@@ -7921,11 +7921,13 @@
       <c r="J30" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K30" s="15"/>
+      <c r="K30" s="15" t="s">
+        <v>346</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B31" s="30" t="n">
         <v>0</v>
@@ -7946,7 +7948,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="30" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I31" s="11" t="s">
         <v>249</v>
@@ -7954,11 +7956,13 @@
       <c r="J31" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="K31" s="15"/>
+      <c r="K31" s="15" t="s">
+        <v>346</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B32" s="30" t="n">
         <v>0</v>
@@ -7988,7 +7992,7 @@
         <v>253</v>
       </c>
       <c r="K32" s="15" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10610,7 +10614,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>20199817.2122427</v>
+        <v>20200402.0255994</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Count level 110 training orb
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1137,7 +1137,7 @@
     <t xml:space="preserve">Level 110 training orb</t>
   </si>
   <si>
-    <t xml:space="preserve">Pending claim. Enter amounts once opened</t>
+    <t xml:space="preserve">Claimed Oct 11: 231 orange, in current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Alliance War, Oct 13 to 14</t>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>533784657.608701</v>
+        <v>533860133.837249</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7131,7 +7131,7 @@
         <v>715</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>1054</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7197,7 +7197,7 @@
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1994</v>
+        <v>2225</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>1015</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8421,9 +8421,15 @@
       <c r="E45" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="30"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="30"/>
+      <c r="F45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I45" s="11" t="s">
         <v>249</v>
       </c>
@@ -10614,7 +10620,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>20200402.0255994</v>
+        <v>20203258.3294727</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add misc gold from basic orbs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="554">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1186,6 +1186,12 @@
   </si>
   <si>
     <t xml:space="preserve">Expected about Oct 15. Gives 2,000 gold orb fragments, one orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misc: 14 basic orbs, Oct 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received, in current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Gold orbs</t>
@@ -4193,7 +4199,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>533860133.837249</v>
+        <v>534005638.900451</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7061,7 +7067,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -7113,7 +7119,7 @@
         <v>315</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>18170000</v>
+        <v>18181000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>1505800</v>
@@ -7139,31 +7145,31 @@
         <v>316</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <f aca="false">SUMIFS(B13:B68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
         <v>32500000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <f aca="false">SUMIFS(C13:C68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
         <v>3500000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <f aca="false">SUMIFS(D13:D68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
         <v>3136000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <f aca="false">SUMIFS(E13:E68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
         <v>2736000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <f aca="false">SUMIFS(F13:F68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <f aca="false">SUMIFS(G13:G68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H67,$I$13:$I$67,"Yes",$J$13:$J$67,"No")</f>
+        <f aca="false">SUMIFS(H13:H68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
         <v>940</v>
       </c>
     </row>
@@ -7173,7 +7179,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>50670000</v>
+        <v>50681000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -7205,31 +7211,31 @@
         <v>318</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$71:$J$91,"Planned",B71:B91)</f>
+        <f aca="false">SUMIF($J$72:$J$92,"Planned",B72:B92)</f>
         <v>9791250</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$71:$J$91,"Planned",C71:C91)</f>
+        <f aca="false">SUMIF($J$72:$J$92,"Planned",C72:C92)</f>
         <v>2070000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$71:$J$91,"Planned",D71:D91)</f>
+        <f aca="false">SUMIF($J$72:$J$92,"Planned",D72:D92)</f>
         <v>2640000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$71:$J$91,"Planned",E71:E91)</f>
+        <f aca="false">SUMIF($J$72:$J$92,"Planned",E72:E92)</f>
         <v>1710000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$71:$J$91,"Planned",F71:F91)</f>
+        <f aca="false">SUMIF($J$72:$J$92,"Planned",F72:F92)</f>
         <v>1</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$71:$J$91,"Planned",G71:G91)</f>
+        <f aca="false">SUMIF($J$72:$J$92,"Planned",G72:G92)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$71:$J$91,"Planned",H71:H91)</f>
+        <f aca="false">SUMIF($J$72:$J$92,"Planned",H72:H92)</f>
         <v>979</v>
       </c>
     </row>
@@ -7239,7 +7245,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>40878750</v>
+        <v>40889750</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8830,7 +8836,7 @@
         <v>385</v>
       </c>
       <c r="B57" s="30" t="n">
-        <v>0</v>
+        <v>11000</v>
       </c>
       <c r="C57" s="30" t="n">
         <v>0</v>
@@ -8851,27 +8857,49 @@
         <v>0</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K57" s="15" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12"/>
-      <c r="B58" s="30"/>
-      <c r="C58" s="30"/>
-      <c r="D58" s="30"/>
-      <c r="E58" s="30"/>
-      <c r="F58" s="30"/>
-      <c r="G58" s="30"/>
-      <c r="H58" s="30"/>
-      <c r="I58" s="11"/>
-      <c r="J58" s="11"/>
-      <c r="K58" s="12"/>
+      <c r="A58" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="B58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J58" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K58" s="15" t="s">
+        <v>388</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12"/>
@@ -8990,123 +9018,103 @@
       <c r="J67" s="11"/>
       <c r="K67" s="12"/>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="29" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="B70" s="3" t="s">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="12"/>
+      <c r="B68" s="30"/>
+      <c r="C68" s="30"/>
+      <c r="D68" s="30"/>
+      <c r="E68" s="30"/>
+      <c r="F68" s="30"/>
+      <c r="G68" s="30"/>
+      <c r="H68" s="30"/>
+      <c r="I68" s="11"/>
+      <c r="J68" s="11"/>
+      <c r="K68" s="12"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="29" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="B71" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C71" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="D70" s="3" t="s">
+      <c r="D71" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="E71" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="F70" s="3" t="s">
+      <c r="F71" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="G70" s="3" t="s">
+      <c r="G71" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="H70" s="3" t="s">
+      <c r="H71" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="I70" s="3" t="s">
+      <c r="I71" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J70" s="3" t="s">
+      <c r="J71" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K70" s="3" t="s">
+      <c r="K71" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="12" t="s">
-        <v>389</v>
-      </c>
-      <c r="B71" s="30" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C71" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E71" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F71" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G71" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H71" s="30" t="n">
-        <v>183</v>
-      </c>
-      <c r="I71" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" s="11" t="s">
-        <v>390</v>
-      </c>
-      <c r="K71" s="15" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="B72" s="30" t="n">
+        <v>1837500</v>
+      </c>
+      <c r="C72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G72" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" s="30" t="n">
+        <v>183</v>
+      </c>
+      <c r="I72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" s="11" t="s">
         <v>392</v>
       </c>
-      <c r="B72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C72" s="30" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" s="11" t="s">
-        <v>390</v>
-      </c>
-      <c r="K72" s="15"/>
+      <c r="K72" s="15" t="s">
+        <v>393</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B73" s="30" t="n">
-        <v>9791250</v>
+        <v>0</v>
       </c>
       <c r="C73" s="30" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D73" s="30" t="n">
         <v>0</v>
@@ -9115,54 +9123,52 @@
         <v>0</v>
       </c>
       <c r="F73" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G73" s="30" t="n">
         <v>0</v>
       </c>
       <c r="H73" s="30" t="n">
-        <v>979</v>
+        <v>0</v>
       </c>
       <c r="I73" s="30" t="n">
-        <v>55000000</v>
+        <v>0</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>394</v>
-      </c>
-      <c r="K73" s="15" t="s">
-        <v>395</v>
-      </c>
+        <v>392</v>
+      </c>
+      <c r="K73" s="15"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="B74" s="30" t="n">
+        <v>9791250</v>
+      </c>
+      <c r="C74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="30" t="n">
+        <v>979</v>
+      </c>
+      <c r="I74" s="30" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="J74" s="11" t="s">
         <v>396</v>
-      </c>
-      <c r="B74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C74" s="30" t="n">
-        <v>360000</v>
-      </c>
-      <c r="D74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J74" s="11" t="s">
-        <v>394</v>
       </c>
       <c r="K74" s="15" t="s">
         <v>397</v>
@@ -9172,9 +9178,11 @@
       <c r="A75" s="12" t="s">
         <v>398</v>
       </c>
-      <c r="B75" s="26"/>
+      <c r="B75" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="C75" s="30" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
       <c r="D75" s="30" t="n">
         <v>0</v>
@@ -9182,14 +9190,20 @@
       <c r="E75" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F75" s="26"/>
-      <c r="G75" s="26"/>
-      <c r="H75" s="26"/>
+      <c r="F75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I75" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="K75" s="15" t="s">
         <v>399</v>
@@ -9216,15 +9230,15 @@
         <v>3000000</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="K76" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B77" s="26"/>
       <c r="C77" s="30" t="n">
@@ -9243,15 +9257,15 @@
         <v>3000000</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="K77" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B78" s="26"/>
       <c r="C78" s="30" t="n">
@@ -9270,15 +9284,15 @@
         <v>3000000</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="K78" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B79" s="26"/>
       <c r="C79" s="30" t="n">
@@ -9290,40 +9304,32 @@
       <c r="E79" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F79" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G79" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H79" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F79" s="26"/>
+      <c r="G79" s="26"/>
+      <c r="H79" s="26"/>
       <c r="I79" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>404</v>
-      </c>
-      <c r="B80" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>405</v>
+      </c>
+      <c r="B80" s="26"/>
       <c r="C80" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="D80" s="30" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="E80" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="F80" s="30" t="n">
         <v>0</v>
@@ -9338,10 +9344,10 @@
         <v>17000000</v>
       </c>
       <c r="J80" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="K80" s="15" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9351,9 +9357,15 @@
       <c r="B81" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C81" s="26"/>
-      <c r="D81" s="26"/>
-      <c r="E81" s="26"/>
+      <c r="C81" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D81" s="30" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="E81" s="30" t="n">
+        <v>1710000</v>
+      </c>
       <c r="F81" s="30" t="n">
         <v>0</v>
       </c>
@@ -9367,15 +9379,15 @@
         <v>17000000</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="K81" s="15" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B82" s="30" t="n">
         <v>0</v>
@@ -9396,10 +9408,10 @@
         <v>17000000</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9425,15 +9437,15 @@
         <v>17000000</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="K83" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B84" s="30" t="n">
         <v>0</v>
@@ -9454,53 +9466,69 @@
         <v>17000000</v>
       </c>
       <c r="J84" s="11" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="K84" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B85" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C85" s="26"/>
+      <c r="D85" s="26"/>
+      <c r="E85" s="26"/>
+      <c r="F85" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J85" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="K85" s="15" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="12" t="s">
+        <v>413</v>
+      </c>
+      <c r="B86" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C85" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D85" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E85" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F85" s="26"/>
-      <c r="G85" s="26"/>
-      <c r="H85" s="26"/>
-      <c r="I85" s="30" t="n">
+      <c r="C86" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="26"/>
+      <c r="G86" s="26"/>
+      <c r="H86" s="26"/>
+      <c r="I86" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J85" s="11" t="s">
-        <v>408</v>
-      </c>
-      <c r="K85" s="15" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="12"/>
-      <c r="B86" s="30"/>
-      <c r="C86" s="30"/>
-      <c r="D86" s="30"/>
-      <c r="E86" s="30"/>
-      <c r="F86" s="30"/>
-      <c r="G86" s="30"/>
-      <c r="H86" s="30"/>
-      <c r="I86" s="30"/>
-      <c r="J86" s="11"/>
-      <c r="K86" s="12"/>
+      <c r="J86" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="K86" s="15" t="s">
+        <v>414</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12"/>
@@ -9567,12 +9595,25 @@
       <c r="J91" s="11"/>
       <c r="K91" s="12"/>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="16" t="s">
-        <v>413</v>
-      </c>
-      <c r="I93" s="20" t="n">
-        <f aca="false">SUMIF(J71:J91,"Planned",I71:I91)</f>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="12"/>
+      <c r="B92" s="30"/>
+      <c r="C92" s="30"/>
+      <c r="D92" s="30"/>
+      <c r="E92" s="30"/>
+      <c r="F92" s="30"/>
+      <c r="G92" s="30"/>
+      <c r="H92" s="30"/>
+      <c r="I92" s="30"/>
+      <c r="J92" s="11"/>
+      <c r="K92" s="12"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="16" t="s">
+        <v>415</v>
+      </c>
+      <c r="I94" s="20" t="n">
+        <f aca="false">SUMIF(J72:J92,"Planned",I72:I92)</f>
         <v>118000000</v>
       </c>
     </row>
@@ -9582,22 +9623,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J71:J91">
+  <conditionalFormatting sqref="J72:J92">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J67">
+  <conditionalFormatting sqref="J13:J68">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J67" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J68" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J71:J91" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J72:J92" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9628,12 +9669,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9647,53 +9688,53 @@
         <v>308</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -9705,19 +9746,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
+        <v>431</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>429</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>427</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -9729,19 +9770,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -9753,19 +9794,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9777,19 +9818,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9801,19 +9842,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9825,19 +9866,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9849,19 +9890,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9873,19 +9914,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9897,19 +9938,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -9921,19 +9962,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -9945,16 +9986,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -9967,19 +10008,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
+        <v>450</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>448</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>446</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -9991,19 +10032,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -10015,19 +10056,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -10039,24 +10080,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -10068,16 +10109,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
+        <v>460</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>458</v>
       </c>
-      <c r="B23" s="13" t="s">
-        <v>456</v>
-      </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -10090,16 +10131,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
+        <v>461</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>458</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="15" t="s">
         <v>459</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>456</v>
-      </c>
-      <c r="C24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>457</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -10112,19 +10153,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -10136,19 +10177,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
+        <v>465</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>463</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>461</v>
-      </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -10160,16 +10201,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -10182,16 +10223,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -10204,21 +10245,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -10231,16 +10272,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
+        <v>477</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>475</v>
       </c>
-      <c r="B31" s="13" t="s">
-        <v>473</v>
-      </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -10253,16 +10294,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -10275,19 +10316,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -10299,16 +10340,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
+        <v>484</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>482</v>
       </c>
-      <c r="B34" s="13" t="s">
-        <v>480</v>
-      </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -10321,16 +10362,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -10343,16 +10384,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -10365,16 +10406,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -10387,7 +10428,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -10424,7 +10465,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -10461,7 +10502,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
   </sheetData>
@@ -10505,12 +10546,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10518,10 +10559,10 @@
         <v>155</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10532,13 +10573,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10549,7 +10590,7 @@
         <v>285572765</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -10599,7 +10640,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -10607,7 +10648,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -10616,11 +10657,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>20203258.3294727</v>
+        <v>20208764.7798293</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10631,19 +10672,19 @@
         <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10659,7 +10700,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10685,7 +10726,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10711,7 +10752,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10737,7 +10778,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10762,10 +10803,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10790,10 +10831,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10818,10 +10859,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10846,10 +10887,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10874,10 +10915,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10902,10 +10943,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -10931,7 +10972,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -10956,10 +10997,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -10984,10 +11025,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -11012,10 +11053,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="D26" s="12" t="s">
         <v>523</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>521</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -11043,7 +11084,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -11070,10 +11111,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -11100,10 +11141,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -11130,10 +11171,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -11154,10 +11195,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -11184,7 +11225,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -11212,10 +11253,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -11242,7 +11283,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -11270,10 +11311,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -11300,7 +11341,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -11328,10 +11369,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -11358,7 +11399,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -11386,10 +11427,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -11416,7 +11457,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -11444,10 +11485,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -11474,7 +11515,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -11502,10 +11543,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -11532,7 +11573,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -11560,7 +11601,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -11588,7 +11629,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -11616,7 +11657,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11644,7 +11685,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11672,7 +11713,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11700,7 +11741,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11728,7 +11769,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11756,7 +11797,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11784,7 +11825,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11812,7 +11853,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11834,7 +11875,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use a single Misc row for small random sources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1188,10 +1188,10 @@
     <t xml:space="preserve">Expected about Oct 15. Gives 2,000 gold orb fragments, one orb</t>
   </si>
   <si>
-    <t xml:space="preserve">Misc: 14 basic orbs, Oct 11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Received, in current stock</t>
+    <t xml:space="preserve">Misc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running total of random drops and other small sources. Already in current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Gold orbs</t>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>534005638.900451</v>
+        <v>534146027.097991</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10661,7 +10661,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>20208764.7798293</v>
+        <v>20214077.5935729</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add campaign missions row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="556">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1186,6 +1186,12 @@
   </si>
   <si>
     <t xml:space="preserve">Expected about Oct 15. Gives 2,000 gold orb fragments, one orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campaign missions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running total. Fixed rewards per mission. Already in current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Misc</t>
@@ -4199,7 +4205,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>534146027.097991</v>
+        <v>534245313.467777</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7067,7 +7073,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K94"/>
+  <dimension ref="A1:K95"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -7119,7 +7125,7 @@
         <v>315</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>18181000</v>
+        <v>18225475</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>1505800</v>
@@ -7131,10 +7137,10 @@
         <v>14390000</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>715</v>
+        <v>735</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>1285</v>
@@ -7145,31 +7151,31 @@
         <v>316</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
+        <f aca="false">SUMIFS(B13:B69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
         <v>32500000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
+        <f aca="false">SUMIFS(C13:C69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
         <v>3500000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
+        <f aca="false">SUMIFS(D13:D69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
         <v>3136000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
+        <f aca="false">SUMIFS(E13:E69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
         <v>2736000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
+        <f aca="false">SUMIFS(F13:F69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
+        <f aca="false">SUMIFS(G13:G69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H68,$I$13:$I$68,"Yes",$J$13:$J$68,"No")</f>
+        <f aca="false">SUMIFS(H13:H69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
         <v>940</v>
       </c>
     </row>
@@ -7179,7 +7185,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>50681000</v>
+        <v>50725475</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -7195,11 +7201,11 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>815</v>
+        <v>835</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
@@ -7211,31 +7217,31 @@
         <v>318</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$72:$J$92,"Planned",B72:B92)</f>
+        <f aca="false">SUMIF($J$73:$J$93,"Planned",B73:B93)</f>
         <v>9791250</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$72:$J$92,"Planned",C72:C92)</f>
+        <f aca="false">SUMIF($J$73:$J$93,"Planned",C73:C93)</f>
         <v>2070000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$72:$J$92,"Planned",D72:D92)</f>
+        <f aca="false">SUMIF($J$73:$J$93,"Planned",D73:D93)</f>
         <v>2640000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$72:$J$92,"Planned",E72:E92)</f>
+        <f aca="false">SUMIF($J$73:$J$93,"Planned",E73:E93)</f>
         <v>1710000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$72:$J$92,"Planned",F72:F92)</f>
+        <f aca="false">SUMIF($J$73:$J$93,"Planned",F73:F93)</f>
         <v>1</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$72:$J$92,"Planned",G72:G92)</f>
+        <f aca="false">SUMIF($J$73:$J$93,"Planned",G73:G93)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$72:$J$92,"Planned",H72:H92)</f>
+        <f aca="false">SUMIF($J$73:$J$93,"Planned",H73:H93)</f>
         <v>979</v>
       </c>
     </row>
@@ -7245,7 +7251,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>40889750</v>
+        <v>40934225</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -7261,11 +7267,11 @@
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>815</v>
+        <v>835</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
@@ -8836,7 +8842,7 @@
         <v>385</v>
       </c>
       <c r="B57" s="30" t="n">
-        <v>11000</v>
+        <v>44475</v>
       </c>
       <c r="C57" s="30" t="n">
         <v>0</v>
@@ -8848,10 +8854,10 @@
         <v>0</v>
       </c>
       <c r="F57" s="30" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G57" s="30" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H57" s="30" t="n">
         <v>0</v>
@@ -8871,7 +8877,7 @@
         <v>387</v>
       </c>
       <c r="B58" s="30" t="n">
-        <v>0</v>
+        <v>11000</v>
       </c>
       <c r="C58" s="30" t="n">
         <v>0</v>
@@ -8892,27 +8898,49 @@
         <v>0</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K58" s="15" t="s">
         <v>388</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12"/>
-      <c r="B59" s="30"/>
-      <c r="C59" s="30"/>
-      <c r="D59" s="30"/>
-      <c r="E59" s="30"/>
-      <c r="F59" s="30"/>
-      <c r="G59" s="30"/>
-      <c r="H59" s="30"/>
-      <c r="I59" s="11"/>
-      <c r="J59" s="11"/>
-      <c r="K59" s="12"/>
+      <c r="A59" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="B59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J59" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K59" s="15" t="s">
+        <v>390</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12"/>
@@ -9031,123 +9059,103 @@
       <c r="J68" s="11"/>
       <c r="K68" s="12"/>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="29" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3" t="s">
-        <v>390</v>
-      </c>
-      <c r="B71" s="3" t="s">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="12"/>
+      <c r="B69" s="30"/>
+      <c r="C69" s="30"/>
+      <c r="D69" s="30"/>
+      <c r="E69" s="30"/>
+      <c r="F69" s="30"/>
+      <c r="G69" s="30"/>
+      <c r="H69" s="30"/>
+      <c r="I69" s="11"/>
+      <c r="J69" s="11"/>
+      <c r="K69" s="12"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="29" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="B72" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C72" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="D71" s="3" t="s">
+      <c r="D72" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="E71" s="3" t="s">
+      <c r="E72" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="F71" s="3" t="s">
+      <c r="F72" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="G71" s="3" t="s">
+      <c r="G72" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="H71" s="3" t="s">
+      <c r="H72" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="I71" s="3" t="s">
+      <c r="I72" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J71" s="3" t="s">
+      <c r="J72" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K71" s="3" t="s">
+      <c r="K72" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="12" t="s">
-        <v>391</v>
-      </c>
-      <c r="B72" s="30" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F72" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G72" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H72" s="30" t="n">
-        <v>183</v>
-      </c>
-      <c r="I72" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" s="11" t="s">
-        <v>392</v>
-      </c>
-      <c r="K72" s="15" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="B73" s="30" t="n">
+        <v>1837500</v>
+      </c>
+      <c r="C73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G73" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" s="30" t="n">
+        <v>183</v>
+      </c>
+      <c r="I73" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="11" t="s">
         <v>394</v>
       </c>
-      <c r="B73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C73" s="30" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" s="11" t="s">
-        <v>392</v>
-      </c>
-      <c r="K73" s="15"/>
+      <c r="K73" s="15" t="s">
+        <v>395</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B74" s="30" t="n">
-        <v>9791250</v>
+        <v>0</v>
       </c>
       <c r="C74" s="30" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D74" s="30" t="n">
         <v>0</v>
@@ -9156,54 +9164,52 @@
         <v>0</v>
       </c>
       <c r="F74" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G74" s="30" t="n">
         <v>0</v>
       </c>
       <c r="H74" s="30" t="n">
-        <v>979</v>
+        <v>0</v>
       </c>
       <c r="I74" s="30" t="n">
-        <v>55000000</v>
+        <v>0</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>396</v>
-      </c>
-      <c r="K74" s="15" t="s">
-        <v>397</v>
-      </c>
+        <v>394</v>
+      </c>
+      <c r="K74" s="15"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
+        <v>397</v>
+      </c>
+      <c r="B75" s="30" t="n">
+        <v>9791250</v>
+      </c>
+      <c r="C75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="30" t="n">
+        <v>979</v>
+      </c>
+      <c r="I75" s="30" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="J75" s="11" t="s">
         <v>398</v>
-      </c>
-      <c r="B75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C75" s="30" t="n">
-        <v>360000</v>
-      </c>
-      <c r="D75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I75" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J75" s="11" t="s">
-        <v>396</v>
       </c>
       <c r="K75" s="15" t="s">
         <v>399</v>
@@ -9213,9 +9219,11 @@
       <c r="A76" s="12" t="s">
         <v>400</v>
       </c>
-      <c r="B76" s="26"/>
+      <c r="B76" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="C76" s="30" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
       <c r="D76" s="30" t="n">
         <v>0</v>
@@ -9223,14 +9231,20 @@
       <c r="E76" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F76" s="26"/>
-      <c r="G76" s="26"/>
-      <c r="H76" s="26"/>
+      <c r="F76" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I76" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="K76" s="15" t="s">
         <v>401</v>
@@ -9257,15 +9271,15 @@
         <v>3000000</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="K77" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B78" s="26"/>
       <c r="C78" s="30" t="n">
@@ -9284,15 +9298,15 @@
         <v>3000000</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="K78" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B79" s="26"/>
       <c r="C79" s="30" t="n">
@@ -9311,15 +9325,15 @@
         <v>3000000</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B80" s="26"/>
       <c r="C80" s="30" t="n">
@@ -9331,40 +9345,32 @@
       <c r="E80" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F80" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G80" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H80" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F80" s="26"/>
+      <c r="G80" s="26"/>
+      <c r="H80" s="26"/>
       <c r="I80" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J80" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="K80" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>406</v>
-      </c>
-      <c r="B81" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>407</v>
+      </c>
+      <c r="B81" s="26"/>
       <c r="C81" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="D81" s="30" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="E81" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="F81" s="30" t="n">
         <v>0</v>
@@ -9379,10 +9385,10 @@
         <v>17000000</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="K81" s="15" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9392,9 +9398,15 @@
       <c r="B82" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C82" s="26"/>
-      <c r="D82" s="26"/>
-      <c r="E82" s="26"/>
+      <c r="C82" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D82" s="30" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="E82" s="30" t="n">
+        <v>1710000</v>
+      </c>
       <c r="F82" s="30" t="n">
         <v>0</v>
       </c>
@@ -9408,15 +9420,15 @@
         <v>17000000</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B83" s="30" t="n">
         <v>0</v>
@@ -9437,10 +9449,10 @@
         <v>17000000</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="K83" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9466,15 +9478,15 @@
         <v>17000000</v>
       </c>
       <c r="J84" s="11" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="K84" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B85" s="30" t="n">
         <v>0</v>
@@ -9495,53 +9507,69 @@
         <v>17000000</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="K85" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B86" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" s="26"/>
+      <c r="D86" s="26"/>
+      <c r="E86" s="26"/>
+      <c r="F86" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J86" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="K86" s="15" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="12" t="s">
+        <v>415</v>
+      </c>
+      <c r="B87" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C86" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D86" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E86" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F86" s="26"/>
-      <c r="G86" s="26"/>
-      <c r="H86" s="26"/>
-      <c r="I86" s="30" t="n">
+      <c r="C87" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="26"/>
+      <c r="G87" s="26"/>
+      <c r="H87" s="26"/>
+      <c r="I87" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J86" s="11" t="s">
-        <v>410</v>
-      </c>
-      <c r="K86" s="15" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="12"/>
-      <c r="B87" s="30"/>
-      <c r="C87" s="30"/>
-      <c r="D87" s="30"/>
-      <c r="E87" s="30"/>
-      <c r="F87" s="30"/>
-      <c r="G87" s="30"/>
-      <c r="H87" s="30"/>
-      <c r="I87" s="30"/>
-      <c r="J87" s="11"/>
-      <c r="K87" s="12"/>
+      <c r="J87" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="K87" s="15" t="s">
+        <v>416</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12"/>
@@ -9608,12 +9636,25 @@
       <c r="J92" s="11"/>
       <c r="K92" s="12"/>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="16" t="s">
-        <v>415</v>
-      </c>
-      <c r="I94" s="20" t="n">
-        <f aca="false">SUMIF(J72:J92,"Planned",I72:I92)</f>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="12"/>
+      <c r="B93" s="30"/>
+      <c r="C93" s="30"/>
+      <c r="D93" s="30"/>
+      <c r="E93" s="30"/>
+      <c r="F93" s="30"/>
+      <c r="G93" s="30"/>
+      <c r="H93" s="30"/>
+      <c r="I93" s="30"/>
+      <c r="J93" s="11"/>
+      <c r="K93" s="12"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="16" t="s">
+        <v>417</v>
+      </c>
+      <c r="I95" s="20" t="n">
+        <f aca="false">SUMIF(J73:J93,"Planned",I73:I93)</f>
         <v>118000000</v>
       </c>
     </row>
@@ -9623,22 +9664,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J72:J92">
+  <conditionalFormatting sqref="J73:J93">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J68">
+  <conditionalFormatting sqref="J13:J69">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J68" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J69" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J72:J92" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J73:J93" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9669,12 +9710,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9688,53 +9729,53 @@
         <v>308</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -9746,19 +9787,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
+        <v>433</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>431</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>429</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -9770,19 +9811,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -9794,19 +9835,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9818,19 +9859,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9842,19 +9883,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9866,19 +9907,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9890,19 +9931,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9914,19 +9955,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9938,19 +9979,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -9962,19 +10003,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -9986,16 +10027,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -10008,19 +10049,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
+        <v>452</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>450</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>448</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -10032,19 +10073,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -10056,19 +10097,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -10080,24 +10121,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -10109,16 +10150,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
+        <v>462</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>460</v>
       </c>
-      <c r="B23" s="13" t="s">
-        <v>458</v>
-      </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -10131,16 +10172,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
+        <v>463</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>460</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="15" t="s">
         <v>461</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>458</v>
-      </c>
-      <c r="C24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>459</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -10153,19 +10194,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -10177,19 +10218,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
+        <v>467</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>465</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>463</v>
-      </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -10201,16 +10242,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -10223,16 +10264,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -10245,21 +10286,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -10272,16 +10313,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
+        <v>479</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>477</v>
       </c>
-      <c r="B31" s="13" t="s">
-        <v>475</v>
-      </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -10294,16 +10335,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -10316,19 +10357,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -10340,16 +10381,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
+        <v>486</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>484</v>
       </c>
-      <c r="B34" s="13" t="s">
-        <v>482</v>
-      </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -10362,16 +10403,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -10384,16 +10425,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -10406,16 +10447,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -10428,7 +10469,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -10465,7 +10506,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -10502,7 +10543,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
   </sheetData>
@@ -10546,12 +10587,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10559,10 +10600,10 @@
         <v>155</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10573,13 +10614,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10590,7 +10631,7 @@
         <v>285572765</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -10640,7 +10681,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -10648,7 +10689,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -10657,11 +10698,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>20214077.5935729</v>
+        <v>20217834.9610904</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10672,19 +10713,19 @@
         <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10700,7 +10741,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10726,7 +10767,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10752,7 +10793,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10778,7 +10819,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10803,10 +10844,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10831,10 +10872,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10859,10 +10900,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10887,10 +10928,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10915,10 +10956,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10943,10 +10984,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -10972,7 +11013,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -10997,10 +11038,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -11025,10 +11066,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -11053,10 +11094,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D26" s="12" t="s">
         <v>525</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>523</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -11084,7 +11125,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -11111,10 +11152,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -11141,10 +11182,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -11171,10 +11212,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -11195,10 +11236,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -11225,7 +11266,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -11253,10 +11294,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -11283,7 +11324,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -11311,10 +11352,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -11341,7 +11382,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -11369,10 +11410,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -11399,7 +11440,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -11427,10 +11468,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -11457,7 +11498,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -11485,10 +11526,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -11515,7 +11556,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -11543,10 +11584,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -11573,7 +11614,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -11601,7 +11642,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -11629,7 +11670,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -11657,7 +11698,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11685,7 +11726,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11713,7 +11754,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11741,7 +11782,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11769,7 +11810,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11797,7 +11838,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11825,7 +11866,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11853,7 +11894,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11875,7 +11916,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Iso Fest points and count milestones 15 and 16
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="554">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1092,10 +1092,13 @@
     <t xml:space="preserve">Iso Fest milestone 15</t>
   </si>
   <si>
-    <t xml:space="preserve">14.6 million points away. Set to Yes once scoring is clear</t>
+    <t xml:space="preserve">Reached Oct 11, ready to claim</t>
   </si>
   <si>
     <t xml:space="preserve">Iso Fest milestone 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About 16.7 million points away</t>
   </si>
   <si>
     <t xml:space="preserve">Iso Fest milestone 17</t>
@@ -4196,7 +4199,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>534300731.429624</v>
+        <v>534464107.246895</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7147,15 +7150,15 @@
       </c>
       <c r="C6" s="27" t="n">
         <f aca="false">SUMIFS(C13:C69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>3500000</v>
+        <v>5350000</v>
       </c>
       <c r="D6" s="27" t="n">
         <f aca="false">SUMIFS(D13:D69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>3136000</v>
+        <v>4436000</v>
       </c>
       <c r="E6" s="27" t="n">
         <f aca="false">SUMIFS(E13:E69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>2736000</v>
+        <v>6536000</v>
       </c>
       <c r="F6" s="27" t="n">
         <f aca="false">SUMIFS(F13:F69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
@@ -7180,15 +7183,15 @@
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>4646000</v>
+        <v>6496000</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>7506000</v>
+        <v>8806000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>17126000</v>
+        <v>20926000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -7246,15 +7249,15 @@
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>2936000</v>
+        <v>4786000</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>4866000</v>
+        <v>6166000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>15416000</v>
+        <v>19216000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -8158,7 +8161,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="J37" s="11" t="s">
         <v>251</v>
@@ -8193,16 +8196,18 @@
         <v>0</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="J38" s="11" t="s">
         <v>251</v>
       </c>
-      <c r="K38" s="15"/>
+      <c r="K38" s="15" t="s">
+        <v>355</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B39" s="30" t="n">
         <v>0</v>
@@ -8235,7 +8240,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B40" s="30" t="n">
         <v>900000</v>
@@ -8265,12 +8270,12 @@
         <v>251</v>
       </c>
       <c r="K40" s="15" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B41" s="30" t="n">
         <v>0</v>
@@ -8300,12 +8305,12 @@
         <v>251</v>
       </c>
       <c r="K41" s="15" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B42" s="30" t="n">
         <v>3300000</v>
@@ -8335,12 +8340,12 @@
         <v>247</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B43" s="30" t="n">
         <v>3300000</v>
@@ -8370,12 +8375,12 @@
         <v>251</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B44" s="30" t="n">
         <v>0</v>
@@ -8405,12 +8410,12 @@
         <v>251</v>
       </c>
       <c r="K44" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B45" s="30" t="n">
         <v>0</v>
@@ -8440,12 +8445,12 @@
         <v>251</v>
       </c>
       <c r="K45" s="15" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B46" s="30" t="n">
         <v>0</v>
@@ -8475,12 +8480,12 @@
         <v>251</v>
       </c>
       <c r="K46" s="15" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B47" s="30" t="n">
         <v>750000</v>
@@ -8510,12 +8515,12 @@
         <v>251</v>
       </c>
       <c r="K47" s="15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B48" s="30" t="n">
         <v>750000</v>
@@ -8545,12 +8550,12 @@
         <v>251</v>
       </c>
       <c r="K48" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B49" s="30" t="n">
         <v>750000</v>
@@ -8580,12 +8585,12 @@
         <v>251</v>
       </c>
       <c r="K49" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B50" s="30" t="n">
         <v>750000</v>
@@ -8615,12 +8620,12 @@
         <v>251</v>
       </c>
       <c r="K50" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B51" s="30" t="n">
         <v>750000</v>
@@ -8650,12 +8655,12 @@
         <v>251</v>
       </c>
       <c r="K51" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B52" s="30" t="n">
         <v>750000</v>
@@ -8685,12 +8690,12 @@
         <v>251</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B53" s="30" t="n">
         <v>750000</v>
@@ -8720,12 +8725,12 @@
         <v>251</v>
       </c>
       <c r="K53" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B54" s="30" t="n">
         <v>750000</v>
@@ -8755,12 +8760,12 @@
         <v>251</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B55" s="30" t="n">
         <v>0</v>
@@ -8790,12 +8795,12 @@
         <v>251</v>
       </c>
       <c r="K55" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B56" s="30" t="n">
         <v>0</v>
@@ -8825,12 +8830,12 @@
         <v>251</v>
       </c>
       <c r="K56" s="15" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B57" s="30" t="n">
         <v>44475</v>
@@ -8860,12 +8865,12 @@
         <v>247</v>
       </c>
       <c r="K57" s="15" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B58" s="30" t="n">
         <v>11000</v>
@@ -8895,12 +8900,12 @@
         <v>247</v>
       </c>
       <c r="K58" s="15" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B59" s="30" t="n">
         <v>0</v>
@@ -8930,7 +8935,7 @@
         <v>251</v>
       </c>
       <c r="K59" s="15" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9065,12 +9070,12 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="29" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>306</v>
@@ -9105,7 +9110,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B73" s="30" t="n">
         <v>1837500</v>
@@ -9132,15 +9137,15 @@
         <v>0</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K73" s="15" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B74" s="30" t="n">
         <v>0</v>
@@ -9167,13 +9172,13 @@
         <v>0</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K74" s="15"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B75" s="30" t="n">
         <v>9791250</v>
@@ -9200,15 +9205,15 @@
         <v>55000000</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K75" s="15" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B76" s="30" t="n">
         <v>0</v>
@@ -9235,15 +9240,15 @@
         <v>0</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="K76" s="15" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B77" s="26"/>
       <c r="C77" s="30" t="n">
@@ -9262,15 +9267,15 @@
         <v>3000000</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K77" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B78" s="26"/>
       <c r="C78" s="30" t="n">
@@ -9289,15 +9294,15 @@
         <v>3000000</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K78" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B79" s="26"/>
       <c r="C79" s="30" t="n">
@@ -9316,15 +9321,15 @@
         <v>3000000</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B80" s="26"/>
       <c r="C80" s="30" t="n">
@@ -9343,15 +9348,15 @@
         <v>3000000</v>
       </c>
       <c r="J80" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K80" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B81" s="26"/>
       <c r="C81" s="30" t="n">
@@ -9376,15 +9381,15 @@
         <v>17000000</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K81" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B82" s="30" t="n">
         <v>0</v>
@@ -9411,15 +9416,15 @@
         <v>17000000</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B83" s="30" t="n">
         <v>0</v>
@@ -9440,15 +9445,15 @@
         <v>17000000</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K83" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B84" s="30" t="n">
         <v>0</v>
@@ -9469,15 +9474,15 @@
         <v>17000000</v>
       </c>
       <c r="J84" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K84" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B85" s="30" t="n">
         <v>0</v>
@@ -9498,15 +9503,15 @@
         <v>17000000</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K85" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B86" s="30" t="n">
         <v>0</v>
@@ -9527,15 +9532,15 @@
         <v>17000000</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K86" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B87" s="30" t="n">
         <v>13000000</v>
@@ -9556,10 +9561,10 @@
         <v>8000000</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K87" s="15" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9642,7 +9647,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="16" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="I95" s="20" t="n">
         <f aca="false">SUMIF(J73:J93,"Planned",I73:I93)</f>
@@ -9701,12 +9706,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9720,53 +9725,53 @@
         <v>306</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -9778,19 +9783,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -9802,19 +9807,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -9826,19 +9831,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9850,19 +9855,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9874,19 +9879,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9898,19 +9903,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9922,19 +9927,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9946,19 +9951,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9970,19 +9975,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -9994,19 +9999,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -10018,16 +10023,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -10040,19 +10045,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -10064,19 +10069,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -10088,19 +10093,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -10112,24 +10117,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -10141,16 +10146,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
+        <v>460</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>458</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="15" t="s">
         <v>459</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>457</v>
-      </c>
-      <c r="C23" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>458</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -10163,16 +10168,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -10185,19 +10190,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -10209,19 +10214,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -10233,16 +10238,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -10255,16 +10260,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -10277,21 +10282,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -10304,16 +10309,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -10326,16 +10331,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -10348,19 +10353,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -10372,16 +10377,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -10394,16 +10399,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
+        <v>486</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>482</v>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="15" t="s">
         <v>485</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>481</v>
-      </c>
-      <c r="C35" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>484</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -10416,16 +10421,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -10438,16 +10443,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -10460,7 +10465,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -10497,7 +10502,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -10534,7 +10539,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
   </sheetData>
@@ -10578,12 +10583,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10591,10 +10596,10 @@
         <v>153</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10605,13 +10610,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10619,10 +10624,10 @@
         <v>156</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>285572765</v>
+        <v>308343695</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -10643,22 +10648,22 @@
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>161</v>
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>0</v>
+        <v>900000</v>
       </c>
       <c r="F7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
-        <v>0</v>
+        <v>1300000</v>
       </c>
       <c r="G7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>0</v>
+        <v>1900000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10667,12 +10672,12 @@
       </c>
       <c r="B8" s="20" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>14427235</v>
+        <v>16656305</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -10680,20 +10685,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>139427235</v>
+        <v>116656305</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>20219932.1833902</v>
+        <v>16922833.1482074</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10704,19 +10709,19 @@
         <v>166</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10732,7 +10737,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10758,7 +10763,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10784,7 +10789,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10810,7 +10815,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10835,10 +10840,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10863,10 +10868,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10891,10 +10896,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10919,10 +10924,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10947,10 +10952,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10975,10 +10980,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -11004,7 +11009,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -11029,10 +11034,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -11057,10 +11062,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
+        <v>524</v>
+      </c>
+      <c r="D25" s="12" t="s">
         <v>523</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>522</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -11085,10 +11090,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -11116,7 +11121,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -11132,7 +11137,7 @@
       </c>
       <c r="I27" s="23" t="n">
         <f aca="false">IF(B27="","",MAX(0,B27-$B$6))</f>
-        <v>14427235</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11143,10 +11148,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -11162,7 +11167,7 @@
       </c>
       <c r="I28" s="23" t="n">
         <f aca="false">IF(B28="","",MAX(0,B28-$B$6))</f>
-        <v>39427235</v>
+        <v>16656305</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11173,10 +11178,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -11192,7 +11197,7 @@
       </c>
       <c r="I29" s="23" t="n">
         <f aca="false">IF(B29="","",MAX(0,B29-$B$6))</f>
-        <v>64427235</v>
+        <v>41656305</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11203,10 +11208,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -11216,7 +11221,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>89427235</v>
+        <v>66656305</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11227,10 +11232,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -11246,7 +11251,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>114427235</v>
+        <v>91656305</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11257,7 +11262,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -11274,7 +11279,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>139427235</v>
+        <v>116656305</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11285,10 +11290,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -11304,7 +11309,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>164427235</v>
+        <v>141656305</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11315,7 +11320,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -11332,7 +11337,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>189427235</v>
+        <v>166656305</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11343,10 +11348,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -11362,7 +11367,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>214427235</v>
+        <v>191656305</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11373,7 +11378,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -11390,7 +11395,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>239427235</v>
+        <v>216656305</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11401,10 +11406,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -11420,7 +11425,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>264427235</v>
+        <v>241656305</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11431,7 +11436,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -11448,7 +11453,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>314427235</v>
+        <v>291656305</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11459,10 +11464,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -11478,7 +11483,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>364427235</v>
+        <v>341656305</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11489,7 +11494,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -11506,7 +11511,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>464427235</v>
+        <v>441656305</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11517,10 +11522,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -11536,7 +11541,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>614427235</v>
+        <v>591656305</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11547,7 +11552,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -11564,7 +11569,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>814427235</v>
+        <v>791656305</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11575,10 +11580,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -11594,7 +11599,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>1014427235</v>
+        <v>991656305</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11605,7 +11610,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -11622,7 +11627,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1214427235</v>
+        <v>1191656305</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11633,7 +11638,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -11650,7 +11655,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1414427235</v>
+        <v>1391656305</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11661,7 +11666,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -11678,7 +11683,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1614427235</v>
+        <v>1591656305</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11689,7 +11694,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11706,7 +11711,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1814427235</v>
+        <v>1791656305</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11717,7 +11722,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11734,7 +11739,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>2014427235</v>
+        <v>1991656305</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11745,7 +11750,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11762,7 +11767,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2214427235</v>
+        <v>2191656305</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11773,7 +11778,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11790,7 +11795,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2414427235</v>
+        <v>2391656305</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11801,7 +11806,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11818,7 +11823,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2614427235</v>
+        <v>2591656305</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11829,7 +11834,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11846,7 +11851,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2814427235</v>
+        <v>2791656305</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11857,7 +11862,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11874,7 +11879,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>3014427235</v>
+        <v>2991656305</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11885,7 +11890,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11902,12 +11907,12 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3214427235</v>
+        <v>3191656305</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Iron Vengeance after Iron Raider raids
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -648,10 +648,10 @@
     <t xml:space="preserve">Spider-Man Diamond 2</t>
   </si>
   <si>
+    <t xml:space="preserve">Yellowjacket Diamond 3</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not claimed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellowjacket Diamond 3</t>
   </si>
   <si>
     <t xml:space="preserve">Crossbones Diamond 3</t>
@@ -4133,14 +4133,14 @@
         <v>156</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>440711000</v>
+        <v>542501630</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>157</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>5987711000</v>
+        <v>5997501630</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6))+SUMPRODUCT((B13:B76="")*(F13:F76="Claimed"))</f>
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>159</v>
@@ -4165,14 +4165,14 @@
       </c>
       <c r="B8" s="16" t="n">
         <f aca="false">IFERROR(INDEX(A13:A76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),"All done")</f>
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>161</v>
       </c>
       <c r="E8" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6)*(F13:F76&lt;&gt;"Claimed"))</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B9" s="20" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>9289000</v>
+        <v>27498370</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3684289000</v>
+        <v>3582498370</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>534464107.246895</v>
+        <v>519788665.387178</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4867,7 +4867,7 @@
         <v>0</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>205</v>
+        <v>170</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4878,15 +4878,15 @@
         <v>450000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>9289000</v>
+        <v>0</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4902,10 +4902,10 @@
       <c r="D52" s="12"/>
       <c r="E52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>39289000</v>
+        <v>0</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4923,10 +4923,10 @@
       </c>
       <c r="E53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>69289000</v>
+        <v>0</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4942,10 +4942,10 @@
       <c r="D54" s="12"/>
       <c r="E54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>99289000</v>
+        <v>0</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4961,10 +4961,10 @@
       <c r="D55" s="12"/>
       <c r="E55" s="23" t="n">
         <f aca="false">IF(B55="","",MAX(0,B55-$B$6))</f>
-        <v>129289000</v>
+        <v>27498370</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4980,10 +4980,10 @@
       <c r="D56" s="12"/>
       <c r="E56" s="23" t="n">
         <f aca="false">IF(B56="","",MAX(0,B56-$B$6))</f>
-        <v>159289000</v>
+        <v>57498370</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4999,10 +4999,10 @@
       <c r="D57" s="12"/>
       <c r="E57" s="23" t="n">
         <f aca="false">IF(B57="","",MAX(0,B57-$B$6))</f>
-        <v>189289000</v>
+        <v>87498370</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5018,10 +5018,10 @@
       <c r="D58" s="12"/>
       <c r="E58" s="23" t="n">
         <f aca="false">IF(B58="","",MAX(0,B58-$B$6))</f>
-        <v>219289000</v>
+        <v>117498370</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5037,10 +5037,10 @@
       <c r="D59" s="12"/>
       <c r="E59" s="23" t="n">
         <f aca="false">IF(B59="","",MAX(0,B59-$B$6))</f>
-        <v>249289000</v>
+        <v>147498370</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5056,10 +5056,10 @@
       <c r="D60" s="12"/>
       <c r="E60" s="23" t="n">
         <f aca="false">IF(B60="","",MAX(0,B60-$B$6))</f>
-        <v>309289000</v>
+        <v>207498370</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5075,10 +5075,10 @@
       <c r="D61" s="12"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>384289000</v>
+        <v>282498370</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5094,10 +5094,10 @@
       <c r="D62" s="12"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>459289000</v>
+        <v>357498370</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5113,10 +5113,10 @@
       <c r="D63" s="12"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>534289000</v>
+        <v>432498370</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5132,10 +5132,10 @@
       <c r="D64" s="12"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>609289000</v>
+        <v>507498370</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5151,10 +5151,10 @@
       <c r="D65" s="12"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>684289000</v>
+        <v>582498370</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5170,10 +5170,10 @@
       <c r="D66" s="12"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>759289000</v>
+        <v>657498370</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5189,10 +5189,10 @@
       <c r="D67" s="12"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>909289000</v>
+        <v>807498370</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5208,10 +5208,10 @@
       <c r="D68" s="12"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>1059289000</v>
+        <v>957498370</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5227,10 +5227,10 @@
       <c r="D69" s="12"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>1209289000</v>
+        <v>1107498370</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5246,10 +5246,10 @@
       <c r="D70" s="12"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1434289000</v>
+        <v>1332498370</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5265,10 +5265,10 @@
       <c r="D71" s="12"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1809289000</v>
+        <v>1707498370</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5284,10 +5284,10 @@
       <c r="D72" s="12"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>2184289000</v>
+        <v>2082498370</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5303,10 +5303,10 @@
       <c r="D73" s="12"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2559289000</v>
+        <v>2457498370</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5322,10 +5322,10 @@
       <c r="D74" s="12"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2934289000</v>
+        <v>2832498370</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5341,10 +5341,10 @@
       <c r="D75" s="12"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>3309289000</v>
+        <v>3207498370</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5360,10 +5360,10 @@
       <c r="D76" s="12"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3684289000</v>
+        <v>3582498370</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6045,11 +6045,11 @@
         <v>15000000</v>
       </c>
       <c r="E21" s="24" t="n">
-        <v>3000000</v>
+        <v>9000000</v>
       </c>
       <c r="F21" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D21),MAX(0,D21-E21),0)</f>
-        <v>12000000</v>
+        <v>6000000</v>
       </c>
       <c r="G21" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D21),ROUNDUP(D21/C21,0),"No limit")</f>
@@ -6057,11 +6057,11 @@
       </c>
       <c r="H21" s="25" t="n">
         <f aca="false">IFERROR(INT(E21/C21),0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I21" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F21/C21,0),0)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J21" s="11" t="s">
         <v>247</v>
@@ -6081,11 +6081,11 @@
         <v>40000000</v>
       </c>
       <c r="E22" s="24" t="n">
-        <v>8000000</v>
+        <v>24000000</v>
       </c>
       <c r="F22" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D22),MAX(0,D22-E22),0)</f>
-        <v>32000000</v>
+        <v>16000000</v>
       </c>
       <c r="G22" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D22),ROUNDUP(D22/C22,0),"No limit")</f>
@@ -6093,11 +6093,11 @@
       </c>
       <c r="H22" s="25" t="n">
         <f aca="false">IFERROR(INT(E22/C22),0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I22" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F22/C22,0),0)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J22" s="11" t="s">
         <v>247</v>
@@ -6117,11 +6117,11 @@
         <v>15000000</v>
       </c>
       <c r="E23" s="24" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D23),MAX(0,D23-E23),0)</f>
-        <v>15000000</v>
+        <v>9000000</v>
       </c>
       <c r="G23" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D23),ROUNDUP(D23/C23,0),"No limit")</f>
@@ -6129,11 +6129,11 @@
       </c>
       <c r="H23" s="25" t="n">
         <f aca="false">IFERROR(INT(E23/C23),0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I23" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F23/C23,0),0)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J23" s="11" t="s">
         <v>247</v>
@@ -6153,11 +6153,11 @@
         <v>40000000</v>
       </c>
       <c r="E24" s="24" t="n">
-        <v>0</v>
+        <v>16000000</v>
       </c>
       <c r="F24" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D24),MAX(0,D24-E24),0)</f>
-        <v>40000000</v>
+        <v>24000000</v>
       </c>
       <c r="G24" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D24),ROUNDUP(D24/C24,0),"No limit")</f>
@@ -6165,11 +6165,11 @@
       </c>
       <c r="H24" s="25" t="n">
         <f aca="false">IFERROR(INT(E24/C24),0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I24" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F24/C24,0),0)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J24" s="11" t="s">
         <v>247</v>
@@ -6189,11 +6189,11 @@
         <v>40000000</v>
       </c>
       <c r="E25" s="24" t="n">
-        <v>8000000</v>
+        <v>24000000</v>
       </c>
       <c r="F25" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D25),MAX(0,D25-E25),0)</f>
-        <v>32000000</v>
+        <v>16000000</v>
       </c>
       <c r="G25" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D25),ROUNDUP(D25/C25,0),"No limit")</f>
@@ -6201,11 +6201,11 @@
       </c>
       <c r="H25" s="25" t="n">
         <f aca="false">IFERROR(INT(E25/C25),0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I25" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F25/C25,0),0)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J25" s="11" t="s">
         <v>247</v>
@@ -6261,11 +6261,11 @@
         <v>40000000</v>
       </c>
       <c r="E27" s="24" t="n">
-        <v>8000000</v>
+        <v>24000000</v>
       </c>
       <c r="F27" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D27),MAX(0,D27-E27),0)</f>
-        <v>32000000</v>
+        <v>16000000</v>
       </c>
       <c r="G27" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D27),ROUNDUP(D27/C27,0),"No limit")</f>
@@ -6273,11 +6273,11 @@
       </c>
       <c r="H27" s="25" t="n">
         <f aca="false">IFERROR(INT(E27/C27),0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I27" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F27/C27,0),0)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J27" s="11" t="s">
         <v>247</v>
@@ -6333,11 +6333,11 @@
         <v>40000000</v>
       </c>
       <c r="E29" s="24" t="n">
-        <v>0</v>
+        <v>16000000</v>
       </c>
       <c r="F29" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D29),MAX(0,D29-E29),0)</f>
-        <v>40000000</v>
+        <v>24000000</v>
       </c>
       <c r="G29" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D29),ROUNDUP(D29/C29,0),"No limit")</f>
@@ -6345,11 +6345,11 @@
       </c>
       <c r="H29" s="25" t="n">
         <f aca="false">IFERROR(INT(E29/C29),0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I29" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F29/C29,0),0)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J29" s="11" t="s">
         <v>247</v>
@@ -7009,7 +7009,7 @@
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>393123500</v>
+        <v>485123500</v>
       </c>
       <c r="F49" s="20"/>
     </row>
@@ -7020,7 +7020,7 @@
       <c r="E50" s="20"/>
       <c r="F50" s="20" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7508376500</v>
+        <v>7416376500</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7030,7 +7030,7 @@
       <c r="E51" s="20"/>
       <c r="F51" s="20" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5547000000</v>
+        <v>5455000000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>16922833.1482074</v>
+        <v>16925792.8096126</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11133,7 +11133,7 @@
         <v>1900000</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I27" s="23" t="n">
         <f aca="false">IF(B27="","",MAX(0,B27-$B$6))</f>
@@ -11163,7 +11163,7 @@
         <v>1900000</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I28" s="23" t="n">
         <f aca="false">IF(B28="","",MAX(0,B28-$B$6))</f>
@@ -11193,7 +11193,7 @@
         <v>1900000</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I29" s="23" t="n">
         <f aca="false">IF(B29="","",MAX(0,B29-$B$6))</f>
@@ -11217,7 +11217,7 @@
       <c r="F30" s="26"/>
       <c r="G30" s="26"/>
       <c r="H30" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
@@ -11247,7 +11247,7 @@
         <v>1900000</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
@@ -11275,7 +11275,7 @@
         <v>1900000</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
@@ -11305,7 +11305,7 @@
         <v>1900000</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
@@ -11333,7 +11333,7 @@
         <v>1900000</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
@@ -11363,7 +11363,7 @@
         <v>1900000</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
@@ -11391,7 +11391,7 @@
         <v>1900000</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
@@ -11421,7 +11421,7 @@
         <v>1900000</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
@@ -11449,7 +11449,7 @@
         <v>2000000</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
@@ -11479,7 +11479,7 @@
         <v>2000000</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
@@ -11507,7 +11507,7 @@
         <v>2000000</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
@@ -11537,7 +11537,7 @@
         <v>2000000</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
@@ -11565,7 +11565,7 @@
         <v>2000000</v>
       </c>
       <c r="H42" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
@@ -11595,7 +11595,7 @@
         <v>2000000</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
@@ -11623,7 +11623,7 @@
         <v>2700000</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
@@ -11651,7 +11651,7 @@
         <v>2700000</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
@@ -11679,7 +11679,7 @@
         <v>2700000</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
@@ -11707,7 +11707,7 @@
         <v>2700000</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
@@ -11735,7 +11735,7 @@
         <v>2700000</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
@@ -11763,7 +11763,7 @@
         <v>2700000</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
@@ -11791,7 +11791,7 @@
         <v>2700000</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
@@ -11819,7 +11819,7 @@
         <v>2700000</v>
       </c>
       <c r="H51" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
@@ -11847,7 +11847,7 @@
         <v>2700000</v>
       </c>
       <c r="H52" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
@@ -11875,7 +11875,7 @@
         <v>2700000</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
@@ -11903,7 +11903,7 @@
         <v>2700000</v>
       </c>
       <c r="H54" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>

</xml_diff>

<commit_message>
Mark claimed milestones and update ion stock
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="553">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -651,24 +651,24 @@
     <t xml:space="preserve">Yellowjacket Diamond 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Crossbones Diamond 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whiplash Diamond 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar and icon cut off, confirm in game</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ulysses Klaue Diamond 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iron Monger Diamond 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not claimed</t>
   </si>
   <si>
-    <t xml:space="preserve">Crossbones Diamond 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whiplash Diamond 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bar and icon cut off, confirm in game</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ulysses Klaue Diamond 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iron Monger Diamond 1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hulk Diamond 3</t>
   </si>
   <si>
@@ -1090,9 +1090,6 @@
   </si>
   <si>
     <t xml:space="preserve">Iso Fest milestone 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reached Oct 11, ready to claim</t>
   </si>
   <si>
     <t xml:space="preserve">Iso Fest milestone 16</t>
@@ -4172,7 +4169,7 @@
       </c>
       <c r="E8" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6)*(F13:F76&lt;&gt;"Claimed"))</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4199,7 +4196,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>519788665.387178</v>
+        <v>520036015.470375</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4886,7 +4883,7 @@
         <v>0</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>206</v>
+        <v>170</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4897,7 +4894,7 @@
         <v>480000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="23" t="n">
@@ -4905,7 +4902,7 @@
         <v>0</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>206</v>
+        <v>170</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4916,17 +4913,17 @@
         <v>510000000</v>
       </c>
       <c r="C53" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="D53" s="12" t="s">
         <v>208</v>
-      </c>
-      <c r="D53" s="12" t="s">
-        <v>209</v>
       </c>
       <c r="E53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
         <v>0</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>206</v>
+        <v>170</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4937,7 +4934,7 @@
         <v>540000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="23" t="n">
@@ -4945,7 +4942,7 @@
         <v>0</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>206</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4956,7 +4953,7 @@
         <v>570000000</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D55" s="12"/>
       <c r="E55" s="23" t="n">
@@ -4964,7 +4961,7 @@
         <v>27498370</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4983,7 +4980,7 @@
         <v>57498370</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5002,7 +4999,7 @@
         <v>87498370</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5021,7 +5018,7 @@
         <v>117498370</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5040,7 +5037,7 @@
         <v>147498370</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5059,7 +5056,7 @@
         <v>207498370</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5078,7 +5075,7 @@
         <v>282498370</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5097,7 +5094,7 @@
         <v>357498370</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5116,7 +5113,7 @@
         <v>432498370</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5135,7 +5132,7 @@
         <v>507498370</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5154,7 +5151,7 @@
         <v>582498370</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5173,7 +5170,7 @@
         <v>657498370</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5192,7 +5189,7 @@
         <v>807498370</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5211,7 +5208,7 @@
         <v>957498370</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5230,7 +5227,7 @@
         <v>1107498370</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5249,7 +5246,7 @@
         <v>1332498370</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5268,7 +5265,7 @@
         <v>1707498370</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5287,7 +5284,7 @@
         <v>2082498370</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5306,7 +5303,7 @@
         <v>2457498370</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5325,7 +5322,7 @@
         <v>2832498370</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5344,7 +5341,7 @@
         <v>3207498370</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5363,7 +5360,7 @@
         <v>3582498370</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7122,13 +7119,13 @@
         <v>8434225</v>
       </c>
       <c r="C5" s="26" t="n">
-        <v>1146000</v>
+        <v>2046000</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>4370000</v>
+        <v>5670000</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>14390000</v>
+        <v>16290000</v>
       </c>
       <c r="F5" s="26" t="n">
         <v>226</v>
@@ -7150,15 +7147,15 @@
       </c>
       <c r="C6" s="27" t="n">
         <f aca="false">SUMIFS(C13:C69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>5350000</v>
+        <v>4450000</v>
       </c>
       <c r="D6" s="27" t="n">
         <f aca="false">SUMIFS(D13:D69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>4436000</v>
+        <v>3136000</v>
       </c>
       <c r="E6" s="27" t="n">
         <f aca="false">SUMIFS(E13:E69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>6536000</v>
+        <v>4636000</v>
       </c>
       <c r="F6" s="27" t="n">
         <f aca="false">SUMIFS(F13:F69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
@@ -8143,13 +8140,13 @@
         <v>0</v>
       </c>
       <c r="C37" s="30" t="n">
-        <v>900000</v>
+        <v>0</v>
       </c>
       <c r="D37" s="30" t="n">
-        <v>1300000</v>
+        <v>0</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>1900000</v>
+        <v>0</v>
       </c>
       <c r="F37" s="30" t="n">
         <v>0</v>
@@ -8167,12 +8164,12 @@
         <v>251</v>
       </c>
       <c r="K37" s="15" t="s">
-        <v>353</v>
+        <v>344</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B38" s="30" t="n">
         <v>0</v>
@@ -8202,12 +8199,12 @@
         <v>251</v>
       </c>
       <c r="K38" s="15" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B39" s="30" t="n">
         <v>0</v>
@@ -8240,7 +8237,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B40" s="30" t="n">
         <v>900000</v>
@@ -8270,12 +8267,12 @@
         <v>251</v>
       </c>
       <c r="K40" s="15" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B41" s="30" t="n">
         <v>0</v>
@@ -8305,12 +8302,12 @@
         <v>251</v>
       </c>
       <c r="K41" s="15" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B42" s="30" t="n">
         <v>3300000</v>
@@ -8340,12 +8337,12 @@
         <v>247</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B43" s="30" t="n">
         <v>3300000</v>
@@ -8375,12 +8372,12 @@
         <v>251</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B44" s="30" t="n">
         <v>0</v>
@@ -8410,12 +8407,12 @@
         <v>251</v>
       </c>
       <c r="K44" s="15" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B45" s="30" t="n">
         <v>0</v>
@@ -8445,12 +8442,12 @@
         <v>251</v>
       </c>
       <c r="K45" s="15" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B46" s="30" t="n">
         <v>0</v>
@@ -8480,12 +8477,12 @@
         <v>251</v>
       </c>
       <c r="K46" s="15" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B47" s="30" t="n">
         <v>750000</v>
@@ -8515,12 +8512,12 @@
         <v>251</v>
       </c>
       <c r="K47" s="15" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B48" s="30" t="n">
         <v>750000</v>
@@ -8550,12 +8547,12 @@
         <v>251</v>
       </c>
       <c r="K48" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B49" s="30" t="n">
         <v>750000</v>
@@ -8585,12 +8582,12 @@
         <v>251</v>
       </c>
       <c r="K49" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B50" s="30" t="n">
         <v>750000</v>
@@ -8620,12 +8617,12 @@
         <v>251</v>
       </c>
       <c r="K50" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B51" s="30" t="n">
         <v>750000</v>
@@ -8655,12 +8652,12 @@
         <v>251</v>
       </c>
       <c r="K51" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B52" s="30" t="n">
         <v>750000</v>
@@ -8690,12 +8687,12 @@
         <v>251</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B53" s="30" t="n">
         <v>750000</v>
@@ -8725,12 +8722,12 @@
         <v>251</v>
       </c>
       <c r="K53" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B54" s="30" t="n">
         <v>750000</v>
@@ -8760,12 +8757,12 @@
         <v>251</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B55" s="30" t="n">
         <v>0</v>
@@ -8795,12 +8792,12 @@
         <v>251</v>
       </c>
       <c r="K55" s="15" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B56" s="30" t="n">
         <v>0</v>
@@ -8830,12 +8827,12 @@
         <v>251</v>
       </c>
       <c r="K56" s="15" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B57" s="30" t="n">
         <v>44475</v>
@@ -8865,12 +8862,12 @@
         <v>247</v>
       </c>
       <c r="K57" s="15" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B58" s="30" t="n">
         <v>11000</v>
@@ -8900,12 +8897,12 @@
         <v>247</v>
       </c>
       <c r="K58" s="15" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B59" s="30" t="n">
         <v>0</v>
@@ -8935,7 +8932,7 @@
         <v>251</v>
       </c>
       <c r="K59" s="15" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9070,12 +9067,12 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="29" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>306</v>
@@ -9110,7 +9107,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B73" s="30" t="n">
         <v>1837500</v>
@@ -9137,15 +9134,15 @@
         <v>0</v>
       </c>
       <c r="J73" s="11" t="s">
+        <v>392</v>
+      </c>
+      <c r="K73" s="15" t="s">
         <v>393</v>
-      </c>
-      <c r="K73" s="15" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B74" s="30" t="n">
         <v>0</v>
@@ -9172,13 +9169,13 @@
         <v>0</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="K74" s="15"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B75" s="30" t="n">
         <v>9791250</v>
@@ -9205,15 +9202,15 @@
         <v>55000000</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="K75" s="15" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B76" s="30" t="n">
         <v>0</v>
@@ -9240,15 +9237,15 @@
         <v>0</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="K76" s="15" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B77" s="26"/>
       <c r="C77" s="30" t="n">
@@ -9267,15 +9264,15 @@
         <v>3000000</v>
       </c>
       <c r="J77" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="K77" s="15" t="s">
         <v>400</v>
-      </c>
-      <c r="K77" s="15" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B78" s="26"/>
       <c r="C78" s="30" t="n">
@@ -9294,15 +9291,15 @@
         <v>3000000</v>
       </c>
       <c r="J78" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="K78" s="15" t="s">
         <v>400</v>
-      </c>
-      <c r="K78" s="15" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B79" s="26"/>
       <c r="C79" s="30" t="n">
@@ -9321,15 +9318,15 @@
         <v>3000000</v>
       </c>
       <c r="J79" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="K79" s="15" t="s">
         <v>400</v>
-      </c>
-      <c r="K79" s="15" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B80" s="26"/>
       <c r="C80" s="30" t="n">
@@ -9348,15 +9345,15 @@
         <v>3000000</v>
       </c>
       <c r="J80" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="K80" s="15" t="s">
         <v>400</v>
-      </c>
-      <c r="K80" s="15" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B81" s="26"/>
       <c r="C81" s="30" t="n">
@@ -9381,15 +9378,15 @@
         <v>17000000</v>
       </c>
       <c r="J81" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="K81" s="15" t="s">
         <v>400</v>
-      </c>
-      <c r="K81" s="15" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B82" s="30" t="n">
         <v>0</v>
@@ -9416,15 +9413,15 @@
         <v>17000000</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B83" s="30" t="n">
         <v>0</v>
@@ -9445,15 +9442,15 @@
         <v>17000000</v>
       </c>
       <c r="J83" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="K83" s="15" t="s">
         <v>400</v>
-      </c>
-      <c r="K83" s="15" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B84" s="30" t="n">
         <v>0</v>
@@ -9474,15 +9471,15 @@
         <v>17000000</v>
       </c>
       <c r="J84" s="11" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="K84" s="15" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B85" s="30" t="n">
         <v>0</v>
@@ -9503,15 +9500,15 @@
         <v>17000000</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="K85" s="15" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B86" s="30" t="n">
         <v>0</v>
@@ -9532,15 +9529,15 @@
         <v>17000000</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="K86" s="15" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B87" s="30" t="n">
         <v>13000000</v>
@@ -9561,10 +9558,10 @@
         <v>8000000</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="K87" s="15" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9647,7 +9644,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="16" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I95" s="20" t="n">
         <f aca="false">SUMIF(J73:J93,"Planned",I73:I93)</f>
@@ -9706,12 +9703,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9725,53 +9722,53 @@
         <v>306</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>422</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>424</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>425</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
+        <v>427</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>428</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>429</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -9783,19 +9780,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -9807,19 +9804,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -9831,19 +9828,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9855,19 +9852,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9879,19 +9876,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9903,19 +9900,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9927,19 +9924,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9951,19 +9948,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9975,19 +9972,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -9999,19 +9996,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -10023,16 +10020,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
+        <v>446</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>447</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>448</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -10045,19 +10042,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -10069,19 +10066,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -10093,19 +10090,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -10117,24 +10114,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
+        <v>456</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>457</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="C22" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="15" t="s">
         <v>458</v>
       </c>
-      <c r="C22" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>459</v>
-      </c>
       <c r="E22" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -10146,16 +10143,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B23" s="13" t="s">
+        <v>457</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="15" t="s">
         <v>458</v>
-      </c>
-      <c r="C23" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>459</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -10168,16 +10165,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B24" s="13" t="s">
+        <v>457</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="15" t="s">
         <v>458</v>
-      </c>
-      <c r="C24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>459</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -10190,19 +10187,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
+        <v>461</v>
+      </c>
+      <c r="B25" s="13" t="s">
         <v>462</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>463</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -10214,19 +10211,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>462</v>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="15" t="s">
         <v>465</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>463</v>
-      </c>
-      <c r="C26" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>466</v>
-      </c>
       <c r="E26" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -10238,16 +10235,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
+        <v>466</v>
+      </c>
+      <c r="B27" s="13" t="s">
         <v>467</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="C27" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="15" t="s">
         <v>468</v>
-      </c>
-      <c r="C27" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>469</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -10260,16 +10257,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
+        <v>469</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>470</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="C28" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="15" t="s">
         <v>471</v>
-      </c>
-      <c r="C28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>472</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -10282,21 +10279,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>474</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="C30" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="15" t="s">
         <v>475</v>
-      </c>
-      <c r="C30" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>476</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -10309,16 +10306,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
+        <v>476</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="C31" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="15" t="s">
         <v>477</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>475</v>
-      </c>
-      <c r="C31" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>478</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -10331,16 +10328,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
+        <v>478</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="C32" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="15" t="s">
         <v>479</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>475</v>
-      </c>
-      <c r="C32" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>480</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -10353,19 +10350,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
+        <v>480</v>
+      </c>
+      <c r="B33" s="13" t="s">
         <v>481</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="C33" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="15" t="s">
         <v>482</v>
       </c>
-      <c r="C33" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>483</v>
-      </c>
       <c r="E33" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -10377,16 +10374,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
+        <v>483</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>481</v>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="15" t="s">
         <v>484</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>482</v>
-      </c>
-      <c r="C34" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="15" t="s">
-        <v>485</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -10399,16 +10396,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -10421,16 +10418,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
+        <v>486</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="C36" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="15" t="s">
         <v>487</v>
-      </c>
-      <c r="B36" s="13" t="s">
-        <v>475</v>
-      </c>
-      <c r="C36" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>488</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -10443,16 +10440,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
+        <v>488</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="15" t="s">
         <v>489</v>
-      </c>
-      <c r="B37" s="13" t="s">
-        <v>475</v>
-      </c>
-      <c r="C37" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>490</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -10465,7 +10462,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E39" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
@@ -10502,7 +10499,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="E40" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
@@ -10539,7 +10536,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -10583,12 +10580,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10596,10 +10593,10 @@
         <v>153</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>495</v>
+      </c>
+      <c r="D4" s="16" t="s">
         <v>496</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10610,13 +10607,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
+        <v>497</v>
+      </c>
+      <c r="F5" s="16" t="s">
         <v>498</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="G5" s="16" t="s">
         <v>499</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10627,19 +10624,19 @@
         <v>308343695</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>3150000</v>
+        <v>2250000</v>
       </c>
       <c r="F6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
-        <v>5500000</v>
+        <v>4200000</v>
       </c>
       <c r="G6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>9500000</v>
+        <v>7600000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10655,15 +10652,15 @@
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>900000</v>
+        <v>0</v>
       </c>
       <c r="F7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
-        <v>1300000</v>
+        <v>0</v>
       </c>
       <c r="G7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>1900000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10677,7 +10674,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -10685,7 +10682,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -10694,11 +10691,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>16925792.8096126</v>
+        <v>16933847.239244</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10709,19 +10706,19 @@
         <v>166</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>498</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>499</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>500</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10737,7 +10734,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10763,7 +10760,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10789,7 +10786,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10815,7 +10812,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10840,10 +10837,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
+        <v>508</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>509</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>510</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10868,10 +10865,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
+        <v>510</v>
+      </c>
+      <c r="D18" s="12" t="s">
         <v>511</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>512</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10896,10 +10893,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
+        <v>512</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>513</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>514</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10924,10 +10921,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
+        <v>514</v>
+      </c>
+      <c r="D20" s="12" t="s">
         <v>515</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>516</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10952,10 +10949,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
+        <v>516</v>
+      </c>
+      <c r="D21" s="12" t="s">
         <v>517</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>518</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10980,10 +10977,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
+        <v>518</v>
+      </c>
+      <c r="D22" s="12" t="s">
         <v>519</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>520</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -11009,7 +11006,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -11034,10 +11031,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>522</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>523</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -11062,10 +11059,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -11090,10 +11087,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -11121,7 +11118,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -11133,7 +11130,7 @@
         <v>1900000</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>206</v>
+        <v>170</v>
       </c>
       <c r="I27" s="23" t="n">
         <f aca="false">IF(B27="","",MAX(0,B27-$B$6))</f>
@@ -11148,10 +11145,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -11163,7 +11160,7 @@
         <v>1900000</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I28" s="23" t="n">
         <f aca="false">IF(B28="","",MAX(0,B28-$B$6))</f>
@@ -11178,10 +11175,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -11193,7 +11190,7 @@
         <v>1900000</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I29" s="23" t="n">
         <f aca="false">IF(B29="","",MAX(0,B29-$B$6))</f>
@@ -11208,16 +11205,16 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="D30" s="12" t="s">
         <v>528</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>529</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
       <c r="G30" s="26"/>
       <c r="H30" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
@@ -11232,10 +11229,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -11247,7 +11244,7 @@
         <v>1900000</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
@@ -11262,7 +11259,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -11275,7 +11272,7 @@
         <v>1900000</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
@@ -11290,10 +11287,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -11305,7 +11302,7 @@
         <v>1900000</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
@@ -11320,7 +11317,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -11333,7 +11330,7 @@
         <v>1900000</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
@@ -11348,10 +11345,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -11363,7 +11360,7 @@
         <v>1900000</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
@@ -11378,7 +11375,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -11391,7 +11388,7 @@
         <v>1900000</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
@@ -11406,10 +11403,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -11421,7 +11418,7 @@
         <v>1900000</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
@@ -11436,7 +11433,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -11449,7 +11446,7 @@
         <v>2000000</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
@@ -11464,10 +11461,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -11479,7 +11476,7 @@
         <v>2000000</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
@@ -11494,7 +11491,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -11507,7 +11504,7 @@
         <v>2000000</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
@@ -11522,10 +11519,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -11537,7 +11534,7 @@
         <v>2000000</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
@@ -11552,7 +11549,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -11565,7 +11562,7 @@
         <v>2000000</v>
       </c>
       <c r="H42" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
@@ -11580,10 +11577,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -11595,7 +11592,7 @@
         <v>2000000</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
@@ -11610,7 +11607,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -11623,7 +11620,7 @@
         <v>2700000</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
@@ -11638,7 +11635,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -11651,7 +11648,7 @@
         <v>2700000</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
@@ -11666,7 +11663,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -11679,7 +11676,7 @@
         <v>2700000</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
@@ -11694,7 +11691,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11707,7 +11704,7 @@
         <v>2700000</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
@@ -11722,7 +11719,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11735,7 +11732,7 @@
         <v>2700000</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
@@ -11750,7 +11747,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11763,7 +11760,7 @@
         <v>2700000</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
@@ -11778,7 +11775,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11791,7 +11788,7 @@
         <v>2700000</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
@@ -11806,7 +11803,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11819,7 +11816,7 @@
         <v>2700000</v>
       </c>
       <c r="H51" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
@@ -11834,7 +11831,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11847,7 +11844,7 @@
         <v>2700000</v>
       </c>
       <c r="H52" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
@@ -11862,7 +11859,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11875,7 +11872,7 @@
         <v>2700000</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
@@ -11890,7 +11887,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11903,7 +11900,7 @@
         <v>2700000</v>
       </c>
       <c r="H54" s="11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
@@ -11912,7 +11909,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync Iron Vengeance scoring with in-game values
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -924,13 +924,13 @@
     <t xml:space="preserve">Upgrade an Amazing Avenger to T4 Level 3 Iso-8</t>
   </si>
   <si>
-    <t xml:space="preserve">Web store free claim</t>
+    <t xml:space="preserve">Web store free claim, Oct 12 onward</t>
   </si>
   <si>
     <t xml:space="preserve">Offers</t>
   </si>
   <si>
-    <t xml:space="preserve">Milestone points from select offers</t>
+    <t xml:space="preserve">Milestone points from select offers, includes free claims so far</t>
   </si>
   <si>
     <t xml:space="preserve">Unlimited</t>
@@ -4141,14 +4141,14 @@
         <v>158</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>542501630</v>
+        <v>558501630</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>159</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>5997501630</v>
+        <v>5988501630</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4189,7 +4189,7 @@
       </c>
       <c r="B9" s="20" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>27498370</v>
+        <v>11498370</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3582498370</v>
+        <v>3566498370</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>520855874.543334</v>
+        <v>518688875.910035</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4969,7 +4969,7 @@
       <c r="D55" s="12"/>
       <c r="E55" s="23" t="n">
         <f aca="false">IF(B55="","",MAX(0,B55-$B$6))</f>
-        <v>27498370</v>
+        <v>11498370</v>
       </c>
       <c r="F55" s="11" t="s">
         <v>213</v>
@@ -4988,7 +4988,7 @@
       <c r="D56" s="12"/>
       <c r="E56" s="23" t="n">
         <f aca="false">IF(B56="","",MAX(0,B56-$B$6))</f>
-        <v>57498370</v>
+        <v>41498370</v>
       </c>
       <c r="F56" s="11" t="s">
         <v>213</v>
@@ -5007,7 +5007,7 @@
       <c r="D57" s="12"/>
       <c r="E57" s="23" t="n">
         <f aca="false">IF(B57="","",MAX(0,B57-$B$6))</f>
-        <v>87498370</v>
+        <v>71498370</v>
       </c>
       <c r="F57" s="11" t="s">
         <v>213</v>
@@ -5026,7 +5026,7 @@
       <c r="D58" s="12"/>
       <c r="E58" s="23" t="n">
         <f aca="false">IF(B58="","",MAX(0,B58-$B$6))</f>
-        <v>117498370</v>
+        <v>101498370</v>
       </c>
       <c r="F58" s="11" t="s">
         <v>213</v>
@@ -5045,7 +5045,7 @@
       <c r="D59" s="12"/>
       <c r="E59" s="23" t="n">
         <f aca="false">IF(B59="","",MAX(0,B59-$B$6))</f>
-        <v>147498370</v>
+        <v>131498370</v>
       </c>
       <c r="F59" s="11" t="s">
         <v>213</v>
@@ -5064,7 +5064,7 @@
       <c r="D60" s="12"/>
       <c r="E60" s="23" t="n">
         <f aca="false">IF(B60="","",MAX(0,B60-$B$6))</f>
-        <v>207498370</v>
+        <v>191498370</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>213</v>
@@ -5083,7 +5083,7 @@
       <c r="D61" s="12"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>282498370</v>
+        <v>266498370</v>
       </c>
       <c r="F61" s="11" t="s">
         <v>213</v>
@@ -5102,7 +5102,7 @@
       <c r="D62" s="12"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>357498370</v>
+        <v>341498370</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>213</v>
@@ -5121,7 +5121,7 @@
       <c r="D63" s="12"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>432498370</v>
+        <v>416498370</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>213</v>
@@ -5140,7 +5140,7 @@
       <c r="D64" s="12"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>507498370</v>
+        <v>491498370</v>
       </c>
       <c r="F64" s="11" t="s">
         <v>213</v>
@@ -5159,7 +5159,7 @@
       <c r="D65" s="12"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>582498370</v>
+        <v>566498370</v>
       </c>
       <c r="F65" s="11" t="s">
         <v>213</v>
@@ -5178,7 +5178,7 @@
       <c r="D66" s="12"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>657498370</v>
+        <v>641498370</v>
       </c>
       <c r="F66" s="11" t="s">
         <v>213</v>
@@ -5197,7 +5197,7 @@
       <c r="D67" s="12"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>807498370</v>
+        <v>791498370</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>213</v>
@@ -5216,7 +5216,7 @@
       <c r="D68" s="12"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>957498370</v>
+        <v>941498370</v>
       </c>
       <c r="F68" s="11" t="s">
         <v>213</v>
@@ -5235,7 +5235,7 @@
       <c r="D69" s="12"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>1107498370</v>
+        <v>1091498370</v>
       </c>
       <c r="F69" s="11" t="s">
         <v>213</v>
@@ -5254,7 +5254,7 @@
       <c r="D70" s="12"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1332498370</v>
+        <v>1316498370</v>
       </c>
       <c r="F70" s="11" t="s">
         <v>213</v>
@@ -5273,7 +5273,7 @@
       <c r="D71" s="12"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1707498370</v>
+        <v>1691498370</v>
       </c>
       <c r="F71" s="11" t="s">
         <v>213</v>
@@ -5292,7 +5292,7 @@
       <c r="D72" s="12"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>2082498370</v>
+        <v>2066498370</v>
       </c>
       <c r="F72" s="11" t="s">
         <v>213</v>
@@ -5311,7 +5311,7 @@
       <c r="D73" s="12"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2457498370</v>
+        <v>2441498370</v>
       </c>
       <c r="F73" s="11" t="s">
         <v>213</v>
@@ -5330,7 +5330,7 @@
       <c r="D74" s="12"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2832498370</v>
+        <v>2816498370</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>213</v>
@@ -5349,7 +5349,7 @@
       <c r="D75" s="12"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>3207498370</v>
+        <v>3191498370</v>
       </c>
       <c r="F75" s="11" t="s">
         <v>213</v>
@@ -5368,7 +5368,7 @@
       <c r="D76" s="12"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3582498370</v>
+        <v>3566498370</v>
       </c>
       <c r="F76" s="11" t="s">
         <v>213</v>
@@ -5477,11 +5477,11 @@
         <v>40000000</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>12000000</v>
+        <v>16000000</v>
       </c>
       <c r="F5" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D5),MAX(0,D5-E5),0)</f>
-        <v>28000000</v>
+        <v>24000000</v>
       </c>
       <c r="G5" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D5),ROUNDUP(D5/C5,0),"No limit")</f>
@@ -5489,11 +5489,11 @@
       </c>
       <c r="H5" s="25" t="n">
         <f aca="false">IFERROR(INT(E5/C5),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I5" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F5/C5,0),0)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J5" s="11" t="s">
         <v>249</v>
@@ -5513,11 +5513,11 @@
         <v>40000000</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>8000000</v>
+        <v>12000000</v>
       </c>
       <c r="F6" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D6),MAX(0,D6-E6),0)</f>
-        <v>32000000</v>
+        <v>28000000</v>
       </c>
       <c r="G6" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D6),ROUNDUP(D6/C6,0),"No limit")</f>
@@ -5525,11 +5525,11 @@
       </c>
       <c r="H6" s="25" t="n">
         <f aca="false">IFERROR(INT(E6/C6),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F6/C6,0),0)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J6" s="11" t="s">
         <v>249</v>
@@ -5549,11 +5549,11 @@
         <v>1000000000</v>
       </c>
       <c r="E7" s="24" t="n">
-        <v>36023500</v>
+        <v>47651630</v>
       </c>
       <c r="F7" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D7),MAX(0,D7-E7),0)</f>
-        <v>963976500</v>
+        <v>952348370</v>
       </c>
       <c r="G7" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D7),ROUNDUP(D7/C7,0),"No limit")</f>
@@ -5561,11 +5561,11 @@
       </c>
       <c r="H7" s="25" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>36023500</v>
+        <v>47651630</v>
       </c>
       <c r="I7" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>963976500</v>
+        <v>952348370</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>253</v>
@@ -5585,11 +5585,11 @@
         <v>1000000000</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>2600000</v>
+        <v>3600000</v>
       </c>
       <c r="F8" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D8),MAX(0,D8-E8),0)</f>
-        <v>997400000</v>
+        <v>996400000</v>
       </c>
       <c r="G8" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D8),ROUNDUP(D8/C8,0),"No limit")</f>
@@ -5597,11 +5597,11 @@
       </c>
       <c r="H8" s="25" t="n">
         <f aca="false">IFERROR(INT(E8/C8),0)</f>
-        <v>650</v>
+        <v>900</v>
       </c>
       <c r="I8" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F8/C8,0),0)</f>
-        <v>249350</v>
+        <v>249100</v>
       </c>
       <c r="J8" s="11" t="s">
         <v>253</v>
@@ -6845,11 +6845,11 @@
         <v>85000000</v>
       </c>
       <c r="E43" s="24" t="n">
-        <v>0</v>
+        <v>17000000</v>
       </c>
       <c r="F43" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D43),MAX(0,D43-E43),0)</f>
-        <v>85000000</v>
+        <v>68000000</v>
       </c>
       <c r="G43" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D43),ROUNDUP(D43/C43,0),"No limit")</f>
@@ -6857,11 +6857,11 @@
       </c>
       <c r="H43" s="25" t="n">
         <f aca="false">IFERROR(INT(E43/C43),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I43" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F43/C43,0),0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J43" s="11" t="s">
         <v>249</v>
@@ -6950,10 +6950,10 @@
         <v>4500000</v>
       </c>
       <c r="D46" s="14" t="n">
-        <v>31500000</v>
+        <v>27000000</v>
       </c>
       <c r="E46" s="24" t="n">
-        <v>4500000</v>
+        <v>0</v>
       </c>
       <c r="F46" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D46),MAX(0,D46-E46),0)</f>
@@ -6961,11 +6961,11 @@
       </c>
       <c r="G46" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D46),ROUNDUP(D46/C46,0),"No limit")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H46" s="25" t="n">
         <f aca="false">IFERROR(INT(E46/C46),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I46" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F46/C46,0),0)</f>
@@ -6989,7 +6989,7 @@
         <v>300</v>
       </c>
       <c r="E47" s="24" t="n">
-        <v>0</v>
+        <v>40250000</v>
       </c>
       <c r="F47" s="25" t="n">
         <f aca="false">IF(ISNUMBER(D47),MAX(0,D47-E47),0)</f>
@@ -7001,7 +7001,7 @@
       </c>
       <c r="H47" s="25" t="n">
         <f aca="false">IFERROR(INT(E47/C47),0)</f>
-        <v>0</v>
+        <v>40250000</v>
       </c>
       <c r="I47" s="25" t="n">
         <f aca="false">IFERROR(ROUNDUP(F47/C47,0),0)</f>
@@ -7017,7 +7017,7 @@
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>485123500</v>
+        <v>558501630</v>
       </c>
       <c r="F49" s="20"/>
     </row>
@@ -7028,7 +7028,7 @@
       <c r="E50" s="20"/>
       <c r="F50" s="20" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7416376500</v>
+        <v>7378748370</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7038,7 +7038,7 @@
       <c r="E51" s="20"/>
       <c r="F51" s="20" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5455000000</v>
+        <v>5430000000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10712,7 +10712,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>16960544.1746998</v>
+        <v>16965752.2572045</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add 9 PM campaign runs and update gold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -4207,7 +4207,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>518688875.910035</v>
+        <v>524609676.304537</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7127,7 +7127,7 @@
         <v>315</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>8434225</v>
+        <v>11980000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>336000</v>
@@ -7142,7 +7142,7 @@
         <v>226</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>735</v>
+        <v>759</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>306</v>
@@ -7154,7 +7154,7 @@
       </c>
       <c r="B6" s="27" t="n">
         <f aca="false">SUMIFS(B13:B69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>32500000</v>
+        <v>29200000</v>
       </c>
       <c r="C6" s="27" t="n">
         <f aca="false">SUMIFS(C13:C69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
@@ -7187,7 +7187,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>40934225</v>
+        <v>41180000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -7207,7 +7207,7 @@
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>835</v>
+        <v>859</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>40934225</v>
+        <v>41180000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -7273,7 +7273,7 @@
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>835</v>
+        <v>859</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
@@ -8380,7 +8380,7 @@
         <v>249</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K43" s="15" t="s">
         <v>364</v>
@@ -8846,7 +8846,7 @@
         <v>385</v>
       </c>
       <c r="B57" s="30" t="n">
-        <v>44475</v>
+        <v>82475</v>
       </c>
       <c r="C57" s="30" t="n">
         <v>0</v>
@@ -8861,7 +8861,7 @@
         <v>10</v>
       </c>
       <c r="G57" s="30" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="H57" s="30" t="n">
         <v>0</v>
@@ -10712,7 +10712,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>16965752.2572045</v>
+        <v>17159415.2601599</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add VisionQuest rewards and daily
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="562">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1107,6 +1107,18 @@
     <t xml:space="preserve">Iso Fest milestone 17</t>
   </si>
   <si>
+    <t xml:space="preserve">VisionQuest level 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected about Oct 14. At level 15 now, +5 a day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VisionQuest levels 35 and 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected about Oct 15 and 16. Ion types read from icons</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Rush run</t>
   </si>
   <si>
@@ -1489,6 +1501,12 @@
   </si>
   <si>
     <t xml:space="preserve">100 campaign and 50 Iso-8 energy; enough fragments for one training orb and one energy orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VisionQuest: spend 10 surge energy in A.I. Avengers campaign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 levels. Resets about 6:40 PM</t>
   </si>
   <si>
     <t xml:space="preserve">Iron Vengeance: free web store milestone points</t>
@@ -4207,7 +4225,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>524609676.304537</v>
+        <v>524759892.696805</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7075,7 +7093,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K95"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -7153,31 +7171,31 @@
         <v>316</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
+        <f aca="false">SUMIFS(B13:B71,$I$13:$I$71,"Yes",$J$13:$J$71,"No")</f>
         <v>29200000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>4450000</v>
+        <f aca="false">SUMIFS(C13:C71,$I$13:$I$71,"Yes",$J$13:$J$71,"No")</f>
+        <v>4650000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>3136000</v>
+        <f aca="false">SUMIFS(D13:D71,$I$13:$I$71,"Yes",$J$13:$J$71,"No")</f>
+        <v>3886000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
-        <v>4636000</v>
+        <f aca="false">SUMIFS(E13:E71,$I$13:$I$71,"Yes",$J$13:$J$71,"No")</f>
+        <v>5386000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
+        <f aca="false">SUMIFS(F13:F71,$I$13:$I$71,"Yes",$J$13:$J$71,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
+        <f aca="false">SUMIFS(G13:G71,$I$13:$I$71,"Yes",$J$13:$J$71,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H69,$I$13:$I$69,"Yes",$J$13:$J$69,"No")</f>
+        <f aca="false">SUMIFS(H13:H71,$I$13:$I$71,"Yes",$J$13:$J$71,"No")</f>
         <v>940</v>
       </c>
     </row>
@@ -7191,15 +7209,15 @@
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>4786000</v>
+        <v>4986000</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>7096000</v>
+        <v>7846000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>18286000</v>
+        <v>19036000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -7219,31 +7237,31 @@
         <v>318</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$73:$J$93,"Planned",B73:B93)</f>
+        <f aca="false">SUMIF($J$75:$J$95,"Planned",B75:B95)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$73:$J$93,"Planned",C73:C93)</f>
+        <f aca="false">SUMIF($J$75:$J$95,"Planned",C75:C95)</f>
         <v>1710000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$73:$J$93,"Planned",D73:D93)</f>
+        <f aca="false">SUMIF($J$75:$J$95,"Planned",D75:D95)</f>
         <v>1710000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$73:$J$93,"Planned",E73:E93)</f>
+        <f aca="false">SUMIF($J$75:$J$95,"Planned",E75:E95)</f>
         <v>2640000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$73:$J$93,"Planned",F73:F93)</f>
+        <f aca="false">SUMIF($J$75:$J$95,"Planned",F75:F95)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$73:$J$93,"Planned",G73:G93)</f>
+        <f aca="false">SUMIF($J$75:$J$95,"Planned",G75:G95)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$73:$J$93,"Planned",H73:H93)</f>
+        <f aca="false">SUMIF($J$75:$J$95,"Planned",H75:H95)</f>
         <v>0</v>
       </c>
     </row>
@@ -7257,15 +7275,15 @@
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>3076000</v>
+        <v>3276000</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>5386000</v>
+        <v>6136000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>15646000</v>
+        <v>16396000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -8251,10 +8269,10 @@
         <v>358</v>
       </c>
       <c r="B40" s="30" t="n">
-        <v>900000</v>
+        <v>0</v>
       </c>
       <c r="C40" s="30" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="D40" s="30" t="n">
         <v>0</v>
@@ -8272,7 +8290,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J40" s="11" t="s">
         <v>253</v>
@@ -8292,36 +8310,36 @@
         <v>0</v>
       </c>
       <c r="D41" s="30" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="E41" s="30" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="F41" s="30" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="30" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H41" s="30" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J41" s="11" t="s">
         <v>253</v>
       </c>
       <c r="K41" s="15" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B42" s="30" t="n">
-        <v>3300000</v>
+        <v>900000</v>
       </c>
       <c r="C42" s="30" t="n">
         <v>0</v>
@@ -8342,48 +8360,48 @@
         <v>0</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="B43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="30" t="n">
+        <v>30</v>
+      </c>
+      <c r="H43" s="30" t="n">
+        <v>90</v>
+      </c>
+      <c r="I43" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J43" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K43" s="15" t="s">
         <v>363</v>
-      </c>
-      <c r="B43" s="30" t="n">
-        <v>3300000</v>
-      </c>
-      <c r="C43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="J43" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="K43" s="15" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8391,10 +8409,10 @@
         <v>365</v>
       </c>
       <c r="B44" s="30" t="n">
-        <v>0</v>
+        <v>3300000</v>
       </c>
       <c r="C44" s="30" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D44" s="30" t="n">
         <v>0</v>
@@ -8415,7 +8433,7 @@
         <v>249</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K44" s="15" t="s">
         <v>366</v>
@@ -8426,7 +8444,7 @@
         <v>367</v>
       </c>
       <c r="B45" s="30" t="n">
-        <v>0</v>
+        <v>3300000</v>
       </c>
       <c r="C45" s="30" t="n">
         <v>0</v>
@@ -8450,7 +8468,7 @@
         <v>249</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K45" s="15" t="s">
         <v>368</v>
@@ -8464,13 +8482,13 @@
         <v>0</v>
       </c>
       <c r="C46" s="30" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D46" s="30" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="E46" s="30" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="F46" s="30" t="n">
         <v>0</v>
@@ -8496,7 +8514,7 @@
         <v>371</v>
       </c>
       <c r="B47" s="30" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C47" s="30" t="n">
         <v>0</v>
@@ -8531,16 +8549,16 @@
         <v>373</v>
       </c>
       <c r="B48" s="30" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C48" s="30" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="30" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="E48" s="30" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="F48" s="30" t="n">
         <v>0</v>
@@ -8593,12 +8611,12 @@
         <v>253</v>
       </c>
       <c r="K49" s="15" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B50" s="30" t="n">
         <v>750000</v>
@@ -8628,12 +8646,12 @@
         <v>253</v>
       </c>
       <c r="K50" s="15" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B51" s="30" t="n">
         <v>750000</v>
@@ -8663,12 +8681,12 @@
         <v>253</v>
       </c>
       <c r="K51" s="15" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B52" s="30" t="n">
         <v>750000</v>
@@ -8698,12 +8716,12 @@
         <v>253</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B53" s="30" t="n">
         <v>750000</v>
@@ -8733,12 +8751,12 @@
         <v>253</v>
       </c>
       <c r="K53" s="15" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B54" s="30" t="n">
         <v>750000</v>
@@ -8768,18 +8786,18 @@
         <v>253</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B55" s="30" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C55" s="30" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D55" s="30" t="n">
         <v>0</v>
@@ -8803,15 +8821,15 @@
         <v>253</v>
       </c>
       <c r="K55" s="15" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B56" s="30" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C56" s="30" t="n">
         <v>0</v>
@@ -8838,7 +8856,7 @@
         <v>253</v>
       </c>
       <c r="K56" s="15" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8846,10 +8864,10 @@
         <v>385</v>
       </c>
       <c r="B57" s="30" t="n">
-        <v>82475</v>
+        <v>0</v>
       </c>
       <c r="C57" s="30" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D57" s="30" t="n">
         <v>0</v>
@@ -8858,10 +8876,10 @@
         <v>0</v>
       </c>
       <c r="F57" s="30" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G57" s="30" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="H57" s="30" t="n">
         <v>0</v>
@@ -8870,7 +8888,7 @@
         <v>249</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="K57" s="15" t="s">
         <v>386</v>
@@ -8881,7 +8899,7 @@
         <v>387</v>
       </c>
       <c r="B58" s="30" t="n">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="C58" s="30" t="n">
         <v>0</v>
@@ -8905,7 +8923,7 @@
         <v>249</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="K58" s="15" t="s">
         <v>388</v>
@@ -8916,7 +8934,7 @@
         <v>389</v>
       </c>
       <c r="B59" s="30" t="n">
-        <v>0</v>
+        <v>82475</v>
       </c>
       <c r="C59" s="30" t="n">
         <v>0</v>
@@ -8928,49 +8946,93 @@
         <v>0</v>
       </c>
       <c r="F59" s="30" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G59" s="30" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="H59" s="30" t="n">
         <v>0</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K59" s="15" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="12"/>
-      <c r="B60" s="30"/>
-      <c r="C60" s="30"/>
-      <c r="D60" s="30"/>
-      <c r="E60" s="30"/>
-      <c r="F60" s="30"/>
-      <c r="G60" s="30"/>
-      <c r="H60" s="30"/>
-      <c r="I60" s="11"/>
-      <c r="J60" s="11"/>
-      <c r="K60" s="12"/>
+      <c r="A60" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="B60" s="30" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C60" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J60" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="K60" s="15" t="s">
+        <v>392</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="12"/>
-      <c r="B61" s="30"/>
-      <c r="C61" s="30"/>
-      <c r="D61" s="30"/>
-      <c r="E61" s="30"/>
-      <c r="F61" s="30"/>
-      <c r="G61" s="30"/>
-      <c r="H61" s="30"/>
-      <c r="I61" s="11"/>
-      <c r="J61" s="11"/>
-      <c r="K61" s="12"/>
+      <c r="A61" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="B61" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C61" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J61" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="K61" s="15" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12"/>
@@ -9076,120 +9138,78 @@
       <c r="J69" s="11"/>
       <c r="K69" s="12"/>
     </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="12"/>
+      <c r="B70" s="30"/>
+      <c r="C70" s="30"/>
+      <c r="D70" s="30"/>
+      <c r="E70" s="30"/>
+      <c r="F70" s="30"/>
+      <c r="G70" s="30"/>
+      <c r="H70" s="30"/>
+      <c r="I70" s="11"/>
+      <c r="J70" s="11"/>
+      <c r="K70" s="12"/>
+    </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="29" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="B72" s="3" t="s">
+      <c r="A71" s="12"/>
+      <c r="B71" s="30"/>
+      <c r="C71" s="30"/>
+      <c r="D71" s="30"/>
+      <c r="E71" s="30"/>
+      <c r="F71" s="30"/>
+      <c r="G71" s="30"/>
+      <c r="H71" s="30"/>
+      <c r="I71" s="11"/>
+      <c r="J71" s="11"/>
+      <c r="K71" s="12"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="29" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="B74" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C74" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="D72" s="3" t="s">
+      <c r="D74" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="E72" s="3" t="s">
+      <c r="E74" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="F72" s="3" t="s">
+      <c r="F74" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="G72" s="3" t="s">
+      <c r="G74" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="H72" s="3" t="s">
+      <c r="H74" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="I72" s="3" t="s">
+      <c r="I74" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J72" s="3" t="s">
+      <c r="J74" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K72" s="3" t="s">
+      <c r="K74" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="12" t="s">
-        <v>393</v>
-      </c>
-      <c r="B73" s="30" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G73" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H73" s="30" t="n">
-        <v>183</v>
-      </c>
-      <c r="I73" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" s="11" t="s">
-        <v>394</v>
-      </c>
-      <c r="K73" s="15" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="12" t="s">
-        <v>396</v>
-      </c>
-      <c r="B74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C74" s="30" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I74" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J74" s="11" t="s">
-        <v>394</v>
-      </c>
-      <c r="K74" s="15"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
         <v>397</v>
       </c>
       <c r="B75" s="30" t="n">
-        <v>9791250</v>
+        <v>1837500</v>
       </c>
       <c r="C75" s="30" t="n">
         <v>0</v>
@@ -9201,27 +9221,27 @@
         <v>0</v>
       </c>
       <c r="F75" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G75" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="G75" s="30" t="n">
-        <v>0</v>
-      </c>
       <c r="H75" s="30" t="n">
-        <v>979</v>
+        <v>183</v>
       </c>
       <c r="I75" s="30" t="n">
-        <v>55000000</v>
+        <v>0</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="K75" s="15" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B76" s="30" t="n">
         <v>0</v>
@@ -9248,17 +9268,17 @@
         <v>0</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>394</v>
-      </c>
-      <c r="K76" s="15" t="s">
         <v>398</v>
       </c>
+      <c r="K76" s="15"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>400</v>
-      </c>
-      <c r="B77" s="26"/>
+        <v>401</v>
+      </c>
+      <c r="B77" s="30" t="n">
+        <v>9791250</v>
+      </c>
       <c r="C77" s="30" t="n">
         <v>0</v>
       </c>
@@ -9268,14 +9288,20 @@
       <c r="E77" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F77" s="26"/>
-      <c r="G77" s="26"/>
-      <c r="H77" s="26"/>
+      <c r="F77" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="30" t="n">
+        <v>979</v>
+      </c>
       <c r="I77" s="30" t="n">
-        <v>3000000</v>
+        <v>55000000</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="K77" s="15" t="s">
         <v>402</v>
@@ -9285,9 +9311,11 @@
       <c r="A78" s="12" t="s">
         <v>403</v>
       </c>
-      <c r="B78" s="26"/>
+      <c r="B78" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="C78" s="30" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D78" s="30" t="n">
         <v>0</v>
@@ -9295,14 +9323,20 @@
       <c r="E78" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F78" s="26"/>
-      <c r="G78" s="26"/>
-      <c r="H78" s="26"/>
+      <c r="F78" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I78" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="K78" s="15" t="s">
         <v>402</v>
@@ -9329,15 +9363,15 @@
         <v>3000000</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B80" s="26"/>
       <c r="C80" s="30" t="n">
@@ -9356,15 +9390,15 @@
         <v>3000000</v>
       </c>
       <c r="J80" s="11" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="K80" s="15" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B81" s="26"/>
       <c r="C81" s="30" t="n">
@@ -9376,75 +9410,59 @@
       <c r="E81" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H81" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F81" s="26"/>
+      <c r="G81" s="26"/>
+      <c r="H81" s="26"/>
       <c r="I81" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="K81" s="15" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>407</v>
-      </c>
-      <c r="B82" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>409</v>
+      </c>
+      <c r="B82" s="26"/>
       <c r="C82" s="30" t="n">
-        <v>1710500</v>
+        <v>0</v>
       </c>
       <c r="D82" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E82" s="30" t="n">
-        <v>2640000</v>
-      </c>
-      <c r="F82" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G82" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H82" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F82" s="26"/>
+      <c r="G82" s="26"/>
+      <c r="H82" s="26"/>
       <c r="I82" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>394</v>
+        <v>405</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>409</v>
-      </c>
-      <c r="B83" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>410</v>
+      </c>
+      <c r="B83" s="26"/>
       <c r="C83" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="D83" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E83" s="30" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F83" s="30" t="n">
         <v>0</v>
@@ -9459,10 +9477,10 @@
         <v>17000000</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="K83" s="15" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9472,9 +9490,15 @@
       <c r="B84" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C84" s="26"/>
-      <c r="D84" s="26"/>
-      <c r="E84" s="26"/>
+      <c r="C84" s="30" t="n">
+        <v>1710500</v>
+      </c>
+      <c r="D84" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E84" s="30" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F84" s="30" t="n">
         <v>0</v>
       </c>
@@ -9488,10 +9512,10 @@
         <v>17000000</v>
       </c>
       <c r="J84" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="K84" s="15" t="s">
         <v>412</v>
-      </c>
-      <c r="K84" s="15" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9501,9 +9525,15 @@
       <c r="B85" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C85" s="26"/>
-      <c r="D85" s="26"/>
-      <c r="E85" s="26"/>
+      <c r="C85" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D85" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E85" s="30" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F85" s="30" t="n">
         <v>0</v>
       </c>
@@ -9517,15 +9547,15 @@
         <v>17000000</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="K85" s="15" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B86" s="30" t="n">
         <v>0</v>
@@ -9546,66 +9576,98 @@
         <v>17000000</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="K86" s="15" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B87" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C87" s="26"/>
+      <c r="D87" s="26"/>
+      <c r="E87" s="26"/>
+      <c r="F87" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J87" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="K87" s="15" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="12" t="s">
+        <v>418</v>
+      </c>
+      <c r="B88" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C88" s="26"/>
+      <c r="D88" s="26"/>
+      <c r="E88" s="26"/>
+      <c r="F88" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J88" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="K88" s="15" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="12" t="s">
+        <v>419</v>
+      </c>
+      <c r="B89" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C87" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D87" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E87" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" s="26"/>
-      <c r="G87" s="26"/>
-      <c r="H87" s="26"/>
-      <c r="I87" s="30" t="n">
+      <c r="C89" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="26"/>
+      <c r="G89" s="26"/>
+      <c r="H89" s="26"/>
+      <c r="I89" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J87" s="11" t="s">
-        <v>412</v>
-      </c>
-      <c r="K87" s="15" t="s">
+      <c r="J89" s="11" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="12"/>
-      <c r="B88" s="30"/>
-      <c r="C88" s="30"/>
-      <c r="D88" s="30"/>
-      <c r="E88" s="30"/>
-      <c r="F88" s="30"/>
-      <c r="G88" s="30"/>
-      <c r="H88" s="30"/>
-      <c r="I88" s="30"/>
-      <c r="J88" s="11"/>
-      <c r="K88" s="12"/>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="12"/>
-      <c r="B89" s="30"/>
-      <c r="C89" s="30"/>
-      <c r="D89" s="30"/>
-      <c r="E89" s="30"/>
-      <c r="F89" s="30"/>
-      <c r="G89" s="30"/>
-      <c r="H89" s="30"/>
-      <c r="I89" s="30"/>
-      <c r="J89" s="11"/>
-      <c r="K89" s="12"/>
+      <c r="K89" s="15" t="s">
+        <v>420</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12"/>
@@ -9659,12 +9721,38 @@
       <c r="J93" s="11"/>
       <c r="K93" s="12"/>
     </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="12"/>
+      <c r="B94" s="30"/>
+      <c r="C94" s="30"/>
+      <c r="D94" s="30"/>
+      <c r="E94" s="30"/>
+      <c r="F94" s="30"/>
+      <c r="G94" s="30"/>
+      <c r="H94" s="30"/>
+      <c r="I94" s="30"/>
+      <c r="J94" s="11"/>
+      <c r="K94" s="12"/>
+    </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="16" t="s">
-        <v>417</v>
-      </c>
-      <c r="I95" s="20" t="n">
-        <f aca="false">SUMIF(J73:J93,"Planned",I73:I93)</f>
+      <c r="A95" s="12"/>
+      <c r="B95" s="30"/>
+      <c r="C95" s="30"/>
+      <c r="D95" s="30"/>
+      <c r="E95" s="30"/>
+      <c r="F95" s="30"/>
+      <c r="G95" s="30"/>
+      <c r="H95" s="30"/>
+      <c r="I95" s="30"/>
+      <c r="J95" s="11"/>
+      <c r="K95" s="12"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="16" t="s">
+        <v>421</v>
+      </c>
+      <c r="I97" s="20" t="n">
+        <f aca="false">SUMIF(J75:J95,"Planned",I75:I95)</f>
         <v>46000000</v>
       </c>
     </row>
@@ -9674,22 +9762,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J73:J93">
+  <conditionalFormatting sqref="J75:J95">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J69">
+  <conditionalFormatting sqref="J13:J71">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J69" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J71" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J73:J93" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J75:J95" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9709,7 +9797,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -9720,12 +9808,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9739,53 +9827,53 @@
         <v>308</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -9797,19 +9885,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -9821,19 +9909,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>439</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>435</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>431</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -9845,19 +9933,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -9869,19 +9957,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -9893,19 +9981,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -9917,19 +10005,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -9941,19 +10029,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -9965,19 +10053,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -9989,19 +10077,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -10013,19 +10101,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -10037,16 +10125,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -10059,19 +10147,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -10083,19 +10171,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
+        <v>458</v>
+      </c>
+      <c r="B19" s="13" t="s">
         <v>454</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>450</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -10107,19 +10195,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -10131,24 +10219,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -10160,16 +10248,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -10182,16 +10270,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -10204,19 +10292,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -10228,19 +10316,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -10252,16 +10340,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -10274,16 +10362,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -10296,21 +10384,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -10323,16 +10411,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -10345,16 +10433,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
+        <v>485</v>
+      </c>
+      <c r="B32" s="13" t="s">
         <v>481</v>
       </c>
-      <c r="B32" s="13" t="s">
-        <v>477</v>
-      </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -10367,19 +10455,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -10391,16 +10479,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -10413,16 +10501,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
+        <v>492</v>
+      </c>
+      <c r="B35" s="13" t="s">
         <v>488</v>
       </c>
-      <c r="B35" s="13" t="s">
-        <v>484</v>
-      </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -10435,16 +10523,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -10457,16 +10545,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -10477,93 +10565,115 @@
       <c r="K37" s="32"/>
       <c r="L37" s="32"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="16" t="s">
-        <v>493</v>
-      </c>
-      <c r="E39" s="20" t="n">
-        <f aca="false">SUMPRODUCT(($C$5:$C$37)*(E5:E37="Done"))</f>
-        <v>2400000</v>
-      </c>
-      <c r="F39" s="20" t="n">
-        <f aca="false">SUMPRODUCT(($C$5:$C$37)*(F5:F37="Done"))</f>
-        <v>0</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <f aca="false">SUMPRODUCT(($C$5:$C$37)*(G5:G37="Done"))</f>
-        <v>0</v>
-      </c>
-      <c r="H39" s="20" t="n">
-        <f aca="false">SUMPRODUCT(($C$5:$C$37)*(H5:H37="Done"))</f>
-        <v>0</v>
-      </c>
-      <c r="I39" s="20" t="n">
-        <f aca="false">SUMPRODUCT(($C$5:$C$37)*(I5:I37="Done"))</f>
-        <v>0</v>
-      </c>
-      <c r="J39" s="20" t="n">
-        <f aca="false">SUMPRODUCT(($C$5:$C$37)*(J5:J37="Done"))</f>
-        <v>0</v>
-      </c>
-      <c r="K39" s="20" t="n">
-        <f aca="false">SUMPRODUCT(($C$5:$C$37)*(K5:K37="Done"))</f>
-        <v>0</v>
-      </c>
-      <c r="L39" s="20" t="n">
-        <f aca="false">SUMPRODUCT(($C$5:$C$37)*(L5:L37="Done"))</f>
-        <v>0</v>
-      </c>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>497</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>481</v>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>498</v>
+      </c>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
+      <c r="L38" s="32"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>494</v>
-      </c>
-      <c r="E40" s="33" t="str">
-        <f aca="false">COUNTIFS($B$5:$B$37,"Required",E5:E37,"Done")&amp;" of 11"</f>
+        <v>499</v>
+      </c>
+      <c r="E40" s="20" t="n">
+        <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
+        <v>2400000</v>
+      </c>
+      <c r="F40" s="20" t="n">
+        <f aca="false">SUMPRODUCT(($C$5:$C$38)*(F5:F38="Done"))</f>
+        <v>0</v>
+      </c>
+      <c r="G40" s="20" t="n">
+        <f aca="false">SUMPRODUCT(($C$5:$C$38)*(G5:G38="Done"))</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="20" t="n">
+        <f aca="false">SUMPRODUCT(($C$5:$C$38)*(H5:H38="Done"))</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="20" t="n">
+        <f aca="false">SUMPRODUCT(($C$5:$C$38)*(I5:I38="Done"))</f>
+        <v>0</v>
+      </c>
+      <c r="J40" s="20" t="n">
+        <f aca="false">SUMPRODUCT(($C$5:$C$38)*(J5:J38="Done"))</f>
+        <v>0</v>
+      </c>
+      <c r="K40" s="20" t="n">
+        <f aca="false">SUMPRODUCT(($C$5:$C$38)*(K5:K38="Done"))</f>
+        <v>0</v>
+      </c>
+      <c r="L40" s="20" t="n">
+        <f aca="false">SUMPRODUCT(($C$5:$C$38)*(L5:L38="Done"))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="s">
+        <v>500</v>
+      </c>
+      <c r="E41" s="33" t="str">
+        <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
         <v>11 of 11</v>
       </c>
-      <c r="F40" s="33" t="str">
-        <f aca="false">COUNTIFS($B$5:$B$37,"Required",F5:F37,"Done")&amp;" of 11"</f>
+      <c r="F41" s="33" t="str">
+        <f aca="false">COUNTIFS($B$5:$B$38,"Required",F5:F38,"Done")&amp;" of 11"</f>
         <v>0 of 11</v>
       </c>
-      <c r="G40" s="33" t="str">
-        <f aca="false">COUNTIFS($B$5:$B$37,"Required",G5:G37,"Done")&amp;" of 11"</f>
+      <c r="G41" s="33" t="str">
+        <f aca="false">COUNTIFS($B$5:$B$38,"Required",G5:G38,"Done")&amp;" of 11"</f>
         <v>0 of 11</v>
       </c>
-      <c r="H40" s="33" t="str">
-        <f aca="false">COUNTIFS($B$5:$B$37,"Required",H5:H37,"Done")&amp;" of 11"</f>
+      <c r="H41" s="33" t="str">
+        <f aca="false">COUNTIFS($B$5:$B$38,"Required",H5:H38,"Done")&amp;" of 11"</f>
         <v>0 of 11</v>
       </c>
-      <c r="I40" s="33" t="str">
-        <f aca="false">COUNTIFS($B$5:$B$37,"Required",I5:I37,"Done")&amp;" of 11"</f>
+      <c r="I41" s="33" t="str">
+        <f aca="false">COUNTIFS($B$5:$B$38,"Required",I5:I38,"Done")&amp;" of 11"</f>
         <v>0 of 11</v>
       </c>
-      <c r="J40" s="33" t="str">
-        <f aca="false">COUNTIFS($B$5:$B$37,"Required",J5:J37,"Done")&amp;" of 11"</f>
+      <c r="J41" s="33" t="str">
+        <f aca="false">COUNTIFS($B$5:$B$38,"Required",J5:J38,"Done")&amp;" of 11"</f>
         <v>0 of 11</v>
       </c>
-      <c r="K40" s="33" t="str">
-        <f aca="false">COUNTIFS($B$5:$B$37,"Required",K5:K37,"Done")&amp;" of 11"</f>
+      <c r="K41" s="33" t="str">
+        <f aca="false">COUNTIFS($B$5:$B$38,"Required",K5:K38,"Done")&amp;" of 11"</f>
         <v>0 of 11</v>
       </c>
-      <c r="L40" s="33" t="str">
-        <f aca="false">COUNTIFS($B$5:$B$37,"Required",L5:L37,"Done")&amp;" of 11"</f>
+      <c r="L41" s="33" t="str">
+        <f aca="false">COUNTIFS($B$5:$B$38,"Required",L5:L38,"Done")&amp;" of 11"</f>
         <v>0 of 11</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
-        <v>495</v>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
+        <v>501</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E5:L37">
+  <conditionalFormatting sqref="E5:L38">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:L37" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:L38" type="list">
       <formula1>"Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -10597,12 +10707,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10610,10 +10720,10 @@
         <v>155</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10624,13 +10734,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10641,7 +10751,7 @@
         <v>308343695</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -10691,7 +10801,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -10699,7 +10809,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -10708,11 +10818,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>17159415.2601599</v>
+        <v>17164328.6617692</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10723,19 +10833,19 @@
         <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>507</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>500</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>501</v>
-      </c>
       <c r="G12" s="3" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -10751,7 +10861,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -10777,7 +10887,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -10803,7 +10913,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -10829,7 +10939,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -10854,10 +10964,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -10882,10 +10992,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -10910,10 +11020,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="12" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -10938,10 +11048,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="12" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -10966,10 +11076,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -10994,10 +11104,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="12" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -11023,7 +11133,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -11048,10 +11158,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="12" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -11076,10 +11186,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="12" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -11104,10 +11214,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="12" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -11135,7 +11245,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -11162,10 +11272,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -11192,10 +11302,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -11222,10 +11332,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -11246,10 +11356,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -11276,7 +11386,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -11304,10 +11414,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -11334,7 +11444,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -11362,10 +11472,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -11392,7 +11502,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -11420,10 +11530,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -11450,7 +11560,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -11478,10 +11588,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -11508,7 +11618,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -11536,10 +11646,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -11566,7 +11676,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -11594,10 +11704,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -11624,7 +11734,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -11652,7 +11762,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -11680,7 +11790,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -11708,7 +11818,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -11736,7 +11846,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -11764,7 +11874,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -11792,7 +11902,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -11820,7 +11930,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -11848,7 +11958,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -11876,7 +11986,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -11904,7 +12014,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -11926,7 +12036,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct training material stock
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -4225,7 +4225,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>524759892.696805</v>
+        <v>525413739.367938</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7157,13 +7157,13 @@
         <v>13650000</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G5" s="26" t="n">
         <v>759</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>306</v>
+        <v>492</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7221,7 +7221,7 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1246</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>1246</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>17164328.6617692</v>
+        <v>17185715.2757584</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Log Kyln cell 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="631">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -686,6 +686,15 @@
   </si>
   <si>
     <t xml:space="preserve">Score earned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cell 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cleared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immortal Weapons</t>
   </si>
   <si>
     <t xml:space="preserve">Type character names exactly as on the Tower Roster tab so team power fills in.</t>
@@ -4818,22 +4827,42 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11"/>
+      <c r="A33" s="11" t="s">
+        <v>218</v>
+      </c>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
+      <c r="D33" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>119</v>
+      </c>
       <c r="I33" s="24" t="n">
         <f aca="false">SUMIF('Tower Roster'!$A$5:$A$44,D33,'Tower Roster'!$C$5:$C$44)+SUMIF('Tower Roster'!$A$5:$A$44,E33,'Tower Roster'!$C$5:$C$44)+SUMIF('Tower Roster'!$A$5:$A$44,F33,'Tower Roster'!$C$5:$C$44)+SUMIF('Tower Roster'!$A$5:$A$44,G33,'Tower Roster'!$C$5:$C$44)+SUMIF('Tower Roster'!$A$5:$A$44,H33,'Tower Roster'!$C$5:$C$44)</f>
-        <v>0</v>
-      </c>
-      <c r="J33" s="11"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="11"/>
+        <v>4789170</v>
+      </c>
+      <c r="J33" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="K33" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="25" t="n">
+        <v>400</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11"/>
@@ -5539,7 +5568,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -5601,20 +5630,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5627,13 +5656,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B6" s="19" t="n">
         <v>558501630</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F51</f>
@@ -5642,14 +5671,14 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6))+SUMPRODUCT((B13:B76="")*(F13:F76="Claimed"))</f>
         <v>42</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E7" s="16" t="n">
         <f aca="false">IFERROR(INDEX(A13:A76,MATCH(E6,B13:B76,1)),37)</f>
@@ -5665,7 +5694,7 @@
         <v>43</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E8" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6)*(F13:F76&lt;&gt;"Claimed"))</f>
@@ -5683,7 +5712,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
@@ -5692,11 +5721,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>525563829.978157</v>
+        <v>525654635.46022</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5704,7 +5733,7 @@
         <v>159</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C12" s="21" t="s">
         <v>162</v>
@@ -5713,7 +5742,7 @@
         <v>13</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="F12" s="21" t="s">
         <v>12</v>
@@ -5725,7 +5754,7 @@
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="12" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="24" t="str">
@@ -5742,7 +5771,7 @@
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="12" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="24" t="str">
@@ -5759,7 +5788,7 @@
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="12" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="24" t="str">
@@ -5776,7 +5805,7 @@
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="12" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="24" t="str">
@@ -5793,7 +5822,7 @@
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="12" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="24" t="str">
@@ -5810,7 +5839,7 @@
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="12" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="24" t="str">
@@ -5827,7 +5856,7 @@
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="24" t="str">
@@ -5844,7 +5873,7 @@
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="12" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="24" t="str">
@@ -5861,7 +5890,7 @@
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="12" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D21" s="12"/>
       <c r="E21" s="24" t="str">
@@ -5878,7 +5907,7 @@
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="12" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="24" t="str">
@@ -5895,7 +5924,7 @@
       </c>
       <c r="B23" s="14"/>
       <c r="C23" s="12" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="24" t="str">
@@ -5912,7 +5941,7 @@
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="12" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="24" t="str">
@@ -5929,7 +5958,7 @@
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="12" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="24" t="str">
@@ -5946,7 +5975,7 @@
       </c>
       <c r="B26" s="14"/>
       <c r="C26" s="12" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="24" t="str">
@@ -5963,7 +5992,7 @@
       </c>
       <c r="B27" s="14"/>
       <c r="C27" s="12" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="24" t="str">
@@ -5980,7 +6009,7 @@
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="12" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="24" t="str">
@@ -5997,7 +6026,7 @@
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="12" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="24" t="str">
@@ -6014,7 +6043,7 @@
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="12" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="24" t="str">
@@ -6031,7 +6060,7 @@
       </c>
       <c r="B31" s="14"/>
       <c r="C31" s="12" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D31" s="12"/>
       <c r="E31" s="24" t="str">
@@ -6048,7 +6077,7 @@
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="12" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="24" t="str">
@@ -6065,7 +6094,7 @@
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="12" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D33" s="12"/>
       <c r="E33" s="24" t="str">
@@ -6082,7 +6111,7 @@
       </c>
       <c r="B34" s="14"/>
       <c r="C34" s="12" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="24" t="str">
@@ -6099,7 +6128,7 @@
       </c>
       <c r="B35" s="14"/>
       <c r="C35" s="12" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D35" s="12"/>
       <c r="E35" s="24" t="str">
@@ -6116,7 +6145,7 @@
       </c>
       <c r="B36" s="14"/>
       <c r="C36" s="12" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="24" t="str">
@@ -6133,7 +6162,7 @@
       </c>
       <c r="B37" s="14"/>
       <c r="C37" s="12" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D37" s="12"/>
       <c r="E37" s="24" t="str">
@@ -6150,7 +6179,7 @@
       </c>
       <c r="B38" s="14"/>
       <c r="C38" s="12" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="24" t="str">
@@ -6167,7 +6196,7 @@
       </c>
       <c r="B39" s="14"/>
       <c r="C39" s="12" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D39" s="12"/>
       <c r="E39" s="24" t="str">
@@ -6184,7 +6213,7 @@
       </c>
       <c r="B40" s="14"/>
       <c r="C40" s="12" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="24" t="str">
@@ -6201,7 +6230,7 @@
       </c>
       <c r="B41" s="14"/>
       <c r="C41" s="12" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D41" s="12"/>
       <c r="E41" s="24" t="str">
@@ -6219,7 +6248,7 @@
       <c r="B42" s="14"/>
       <c r="C42" s="12"/>
       <c r="D42" s="12" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E42" s="24" t="str">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
@@ -6236,7 +6265,7 @@
       <c r="B43" s="14"/>
       <c r="C43" s="12"/>
       <c r="D43" s="12" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E43" s="24" t="str">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
@@ -6253,7 +6282,7 @@
       <c r="B44" s="14"/>
       <c r="C44" s="12"/>
       <c r="D44" s="12" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E44" s="24" t="str">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
@@ -6270,7 +6299,7 @@
       <c r="B45" s="14"/>
       <c r="C45" s="12"/>
       <c r="D45" s="12" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E45" s="24" t="str">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
@@ -6286,7 +6315,7 @@
       </c>
       <c r="B46" s="14"/>
       <c r="C46" s="12" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="24" t="str">
@@ -6303,7 +6332,7 @@
       </c>
       <c r="B47" s="14"/>
       <c r="C47" s="12" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="24" t="str">
@@ -6320,7 +6349,7 @@
       </c>
       <c r="B48" s="14"/>
       <c r="C48" s="12" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="24" t="str">
@@ -6337,7 +6366,7 @@
       </c>
       <c r="B49" s="14"/>
       <c r="C49" s="12" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="24" t="str">
@@ -6356,7 +6385,7 @@
         <v>435000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="24" t="n">
@@ -6375,7 +6404,7 @@
         <v>450000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="24" t="n">
@@ -6394,7 +6423,7 @@
         <v>480000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="24" t="n">
@@ -6413,10 +6442,10 @@
         <v>510000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E53" s="24" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
@@ -6434,7 +6463,7 @@
         <v>540000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="24" t="n">
@@ -6453,7 +6482,7 @@
         <v>570000000</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="D55" s="12"/>
       <c r="E55" s="24" t="n">
@@ -6472,7 +6501,7 @@
         <v>600000000</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D56" s="12"/>
       <c r="E56" s="24" t="n">
@@ -6491,7 +6520,7 @@
         <v>630000000</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="D57" s="12"/>
       <c r="E57" s="24" t="n">
@@ -6510,7 +6539,7 @@
         <v>660000000</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D58" s="12"/>
       <c r="E58" s="24" t="n">
@@ -6529,7 +6558,7 @@
         <v>690000000</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="D59" s="12"/>
       <c r="E59" s="24" t="n">
@@ -6548,7 +6577,7 @@
         <v>750000000</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="D60" s="12"/>
       <c r="E60" s="24" t="n">
@@ -6567,7 +6596,7 @@
         <v>825000000</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D61" s="12"/>
       <c r="E61" s="24" t="n">
@@ -6586,7 +6615,7 @@
         <v>900000000</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D62" s="12"/>
       <c r="E62" s="24" t="n">
@@ -6605,7 +6634,7 @@
         <v>975000000</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="D63" s="12"/>
       <c r="E63" s="24" t="n">
@@ -6624,7 +6653,7 @@
         <v>1050000000</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="D64" s="12"/>
       <c r="E64" s="24" t="n">
@@ -6643,7 +6672,7 @@
         <v>1125000000</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="D65" s="12"/>
       <c r="E65" s="24" t="n">
@@ -6662,7 +6691,7 @@
         <v>1200000000</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D66" s="12"/>
       <c r="E66" s="24" t="n">
@@ -6681,7 +6710,7 @@
         <v>1350000000</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D67" s="12"/>
       <c r="E67" s="24" t="n">
@@ -6700,7 +6729,7 @@
         <v>1500000000</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D68" s="12"/>
       <c r="E68" s="24" t="n">
@@ -6719,7 +6748,7 @@
         <v>1650000000</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D69" s="12"/>
       <c r="E69" s="24" t="n">
@@ -6738,7 +6767,7 @@
         <v>1875000000</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D70" s="12"/>
       <c r="E70" s="24" t="n">
@@ -6757,7 +6786,7 @@
         <v>2250000000</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D71" s="12"/>
       <c r="E71" s="24" t="n">
@@ -6776,7 +6805,7 @@
         <v>2625000000</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D72" s="12"/>
       <c r="E72" s="24" t="n">
@@ -6795,7 +6824,7 @@
         <v>3000000000</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="D73" s="12"/>
       <c r="E73" s="24" t="n">
@@ -6814,7 +6843,7 @@
         <v>3375000000</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D74" s="12"/>
       <c r="E74" s="24" t="n">
@@ -6833,7 +6862,7 @@
         <v>3750000000</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D75" s="12"/>
       <c r="E75" s="24" t="n">
@@ -6852,7 +6881,7 @@
         <v>4125000000</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D76" s="12"/>
       <c r="E76" s="24" t="n">
@@ -6912,52 +6941,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="I4" s="21" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="J4" s="21" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>4000000</v>
@@ -6985,15 +7014,15 @@
         <v>6</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>4000000</v>
@@ -7021,15 +7050,15 @@
         <v>7</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="C7" s="14" t="n">
         <v>1</v>
@@ -7057,15 +7086,15 @@
         <v>952348370</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>4000</v>
@@ -7093,7 +7122,7 @@
         <v>249100</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7101,7 +7130,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>3000000</v>
@@ -7129,7 +7158,7 @@
         <v>4</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7137,7 +7166,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C10" s="14" t="n">
         <v>8000000</v>
@@ -7165,15 +7194,15 @@
         <v>5</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C11" s="14" t="n">
         <v>7000000</v>
@@ -7201,15 +7230,15 @@
         <v>0</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C12" s="14" t="n">
         <v>17000000</v>
@@ -7237,15 +7266,15 @@
         <v>0</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C13" s="14" t="n">
         <v>7000000</v>
@@ -7273,15 +7302,15 @@
         <v>0</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C14" s="14" t="n">
         <v>17000000</v>
@@ -7309,15 +7338,15 @@
         <v>5</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C15" s="14" t="n">
         <v>7000000</v>
@@ -7345,15 +7374,15 @@
         <v>0</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C16" s="14" t="n">
         <v>17000000</v>
@@ -7381,15 +7410,15 @@
         <v>5</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C17" s="14" t="n">
         <v>3000000</v>
@@ -7417,15 +7446,15 @@
         <v>0</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C18" s="14" t="n">
         <v>8000000</v>
@@ -7453,15 +7482,15 @@
         <v>0</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C19" s="14" t="n">
         <v>3000000</v>
@@ -7489,15 +7518,15 @@
         <v>0</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C20" s="14" t="n">
         <v>8000000</v>
@@ -7525,15 +7554,15 @@
         <v>0</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="C21" s="14" t="n">
         <v>3000000</v>
@@ -7561,15 +7590,15 @@
         <v>2</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C22" s="14" t="n">
         <v>8000000</v>
@@ -7597,15 +7626,15 @@
         <v>2</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="C23" s="14" t="n">
         <v>3000000</v>
@@ -7633,15 +7662,15 @@
         <v>3</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C24" s="14" t="n">
         <v>8000000</v>
@@ -7669,15 +7698,15 @@
         <v>3</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C25" s="14" t="n">
         <v>8000000</v>
@@ -7705,15 +7734,15 @@
         <v>2</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C26" s="14" t="n">
         <v>17000000</v>
@@ -7741,15 +7770,15 @@
         <v>5</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C27" s="14" t="n">
         <v>8000000</v>
@@ -7777,15 +7806,15 @@
         <v>2</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C28" s="14" t="n">
         <v>17000000</v>
@@ -7813,15 +7842,15 @@
         <v>5</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C29" s="14" t="n">
         <v>8000000</v>
@@ -7849,15 +7878,15 @@
         <v>3</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="C30" s="14" t="n">
         <v>17000000</v>
@@ -7885,15 +7914,15 @@
         <v>5</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C31" s="14" t="n">
         <v>40000000</v>
@@ -7921,15 +7950,15 @@
         <v>2</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="C32" s="14" t="n">
         <v>80000000</v>
@@ -7957,15 +7986,15 @@
         <v>2</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C33" s="14" t="n">
         <v>150000000</v>
@@ -7993,15 +8022,15 @@
         <v>2</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C34" s="14" t="n">
         <v>200000000</v>
@@ -8029,15 +8058,15 @@
         <v>1</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C35" s="14" t="n">
         <v>200000000</v>
@@ -8065,15 +8094,15 @@
         <v>1</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C36" s="14" t="n">
         <v>17000000</v>
@@ -8101,15 +8130,15 @@
         <v>5</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C37" s="14" t="n">
         <v>150000000</v>
@@ -8137,15 +8166,15 @@
         <v>5</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="C38" s="14" t="n">
         <v>17000000</v>
@@ -8173,15 +8202,15 @@
         <v>5</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C39" s="14" t="n">
         <v>50000000</v>
@@ -8209,15 +8238,15 @@
         <v>5</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="C40" s="14" t="n">
         <v>150000000</v>
@@ -8245,15 +8274,15 @@
         <v>5</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="C41" s="14" t="n">
         <v>17000000</v>
@@ -8281,15 +8310,15 @@
         <v>5</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C42" s="14" t="n">
         <v>150000000</v>
@@ -8317,15 +8346,15 @@
         <v>5</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="C43" s="14" t="n">
         <v>17000000</v>
@@ -8353,15 +8382,15 @@
         <v>4</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C44" s="14" t="n">
         <v>50000000</v>
@@ -8389,15 +8418,15 @@
         <v>5</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="C45" s="14" t="n">
         <v>150000000</v>
@@ -8425,15 +8454,15 @@
         <v>5</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C46" s="14" t="n">
         <v>4500000</v>
@@ -8461,21 +8490,21 @@
         <v>6</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="C47" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="E47" s="25" t="n">
         <v>40250000</v>
@@ -8497,12 +8526,12 @@
         <v>0</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="16" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">SUM(E5:E47)</f>
@@ -8512,7 +8541,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="16" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E50" s="20"/>
       <c r="F50" s="20" t="n">
@@ -8522,7 +8551,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="16" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="E51" s="20"/>
       <c r="F51" s="20" t="n">
@@ -8532,7 +8561,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="2" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -8577,43 +8606,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
         <v>11980000</v>
@@ -8639,7 +8668,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B6" s="28" t="n">
         <f aca="false">SUMIFS(B13:B75,$I$13:$I$75,"Yes",$J$13:$J$75,"No")</f>
@@ -8672,7 +8701,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
@@ -8705,7 +8734,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">SUMIF($J$79:$J$99,"Planned",B79:B99)</f>
@@ -8738,7 +8767,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
@@ -8771,44 +8800,44 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>13</v>
@@ -8816,7 +8845,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="B13" s="30" t="n">
         <v>100000</v>
@@ -8840,18 +8869,18 @@
         <v>0</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K13" s="15" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B14" s="30" t="n">
         <v>1600000</v>
@@ -8875,18 +8904,18 @@
         <v>0</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K14" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B15" s="30" t="n">
         <v>1600000</v>
@@ -8910,18 +8939,18 @@
         <v>0</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K15" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B16" s="30" t="n">
         <v>1600000</v>
@@ -8945,18 +8974,18 @@
         <v>0</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K16" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="B17" s="30" t="n">
         <v>1600000</v>
@@ -8980,18 +9009,18 @@
         <v>0</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B18" s="30" t="n">
         <v>1600000</v>
@@ -9015,18 +9044,18 @@
         <v>0</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B19" s="30" t="n">
         <v>1600000</v>
@@ -9050,18 +9079,18 @@
         <v>0</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K19" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B20" s="30" t="n">
         <v>1600000</v>
@@ -9085,18 +9114,18 @@
         <v>0</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B21" s="30" t="n">
         <v>100000</v>
@@ -9120,16 +9149,16 @@
         <v>0</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B22" s="30" t="n">
         <v>200000</v>
@@ -9153,16 +9182,16 @@
         <v>0</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B23" s="30" t="n">
         <v>0</v>
@@ -9186,18 +9215,18 @@
         <v>0</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K23" s="15" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B24" s="30" t="n">
         <v>150000</v>
@@ -9221,16 +9250,16 @@
         <v>15</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="K24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B25" s="30" t="n">
         <v>150000</v>
@@ -9254,16 +9283,16 @@
         <v>20</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="K25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B26" s="30" t="n">
         <v>200000</v>
@@ -9287,16 +9316,16 @@
         <v>25</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B27" s="30" t="n">
         <v>250000</v>
@@ -9320,16 +9349,16 @@
         <v>30</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B28" s="30" t="n">
         <v>300000</v>
@@ -9353,16 +9382,16 @@
         <v>40</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B29" s="30" t="n">
         <v>350000</v>
@@ -9386,16 +9415,16 @@
         <v>45</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B30" s="30" t="n">
         <v>0</v>
@@ -9419,18 +9448,18 @@
         <v>0</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K30" s="15" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B31" s="30" t="n">
         <v>0</v>
@@ -9454,18 +9483,18 @@
         <v>0</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K31" s="15" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B32" s="30" t="n">
         <v>0</v>
@@ -9489,18 +9518,18 @@
         <v>0</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K32" s="15" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="B33" s="30" t="n">
         <v>0</v>
@@ -9524,16 +9553,16 @@
         <v>800</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B34" s="30" t="n">
         <v>10000000</v>
@@ -9557,16 +9586,16 @@
         <v>0</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B35" s="30" t="n">
         <v>500000</v>
@@ -9590,16 +9619,16 @@
         <v>0</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B36" s="30" t="n">
         <v>0</v>
@@ -9623,18 +9652,18 @@
         <v>0</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K36" s="15" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B37" s="30" t="n">
         <v>0</v>
@@ -9658,18 +9687,18 @@
         <v>0</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K37" s="15" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B38" s="30" t="n">
         <v>0</v>
@@ -9693,18 +9722,18 @@
         <v>0</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K38" s="15" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="B39" s="30" t="n">
         <v>0</v>
@@ -9728,16 +9757,16 @@
         <v>0</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B40" s="30" t="n">
         <v>0</v>
@@ -9761,18 +9790,18 @@
         <v>0</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K40" s="15" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B41" s="30" t="n">
         <v>0</v>
@@ -9796,18 +9825,18 @@
         <v>0</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K41" s="15" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B42" s="30" t="n">
         <v>0</v>
@@ -9831,18 +9860,18 @@
         <v>500</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B43" s="30" t="n">
         <v>0</v>
@@ -9866,18 +9895,18 @@
         <v>500</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B44" s="30" t="n">
         <v>0</v>
@@ -9901,18 +9930,18 @@
         <v>1000</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K44" s="15" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B45" s="30" t="n">
         <v>0</v>
@@ -9936,18 +9965,18 @@
         <v>0</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K45" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B46" s="30" t="n">
         <v>900000</v>
@@ -9971,18 +10000,18 @@
         <v>0</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K46" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B47" s="30" t="n">
         <v>0</v>
@@ -10006,18 +10035,18 @@
         <v>90</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K47" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="B48" s="30" t="n">
         <v>3300000</v>
@@ -10041,18 +10070,18 @@
         <v>0</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="K48" s="15" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B49" s="30" t="n">
         <v>3300000</v>
@@ -10076,18 +10105,18 @@
         <v>0</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="K49" s="15" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B50" s="30" t="n">
         <v>0</v>
@@ -10111,18 +10140,18 @@
         <v>0</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K50" s="15" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="B51" s="30" t="n">
         <v>0</v>
@@ -10146,18 +10175,18 @@
         <v>0</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K51" s="15" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B52" s="30" t="n">
         <v>0</v>
@@ -10181,18 +10210,18 @@
         <v>0</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="B53" s="30" t="n">
         <v>750000</v>
@@ -10216,18 +10245,18 @@
         <v>0</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K53" s="15" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="B54" s="30" t="n">
         <v>750000</v>
@@ -10251,18 +10280,18 @@
         <v>0</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B55" s="30" t="n">
         <v>750000</v>
@@ -10286,18 +10315,18 @@
         <v>0</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K55" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B56" s="30" t="n">
         <v>750000</v>
@@ -10321,18 +10350,18 @@
         <v>0</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K56" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="B57" s="30" t="n">
         <v>750000</v>
@@ -10356,18 +10385,18 @@
         <v>0</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K57" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B58" s="30" t="n">
         <v>750000</v>
@@ -10391,18 +10420,18 @@
         <v>0</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K58" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="B59" s="30" t="n">
         <v>750000</v>
@@ -10426,18 +10455,18 @@
         <v>0</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K59" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B60" s="30" t="n">
         <v>750000</v>
@@ -10461,18 +10490,18 @@
         <v>0</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K60" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B61" s="30" t="n">
         <v>0</v>
@@ -10496,18 +10525,18 @@
         <v>0</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K61" s="15" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B62" s="30" t="n">
         <v>0</v>
@@ -10531,18 +10560,18 @@
         <v>0</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K62" s="15" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="B63" s="30" t="n">
         <v>82475</v>
@@ -10566,18 +10595,18 @@
         <v>0</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="K63" s="15" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B64" s="30" t="n">
         <v>11000</v>
@@ -10601,18 +10630,18 @@
         <v>0</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="K64" s="15" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="B65" s="30" t="n">
         <v>0</v>
@@ -10636,13 +10665,13 @@
         <v>0</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K65" s="15" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10777,33 +10806,33 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="23" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="H78" s="3" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="I78" s="3" t="s">
         <v>10</v>
@@ -10817,7 +10846,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B79" s="30" t="n">
         <v>1837500</v>
@@ -10844,15 +10873,15 @@
         <v>0</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="B80" s="30" t="n">
         <v>0</v>
@@ -10879,13 +10908,13 @@
         <v>0</v>
       </c>
       <c r="J80" s="11" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K80" s="15"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="B81" s="30" t="n">
         <v>9791250</v>
@@ -10912,15 +10941,15 @@
         <v>55000000</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K81" s="15" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="B82" s="30" t="n">
         <v>0</v>
@@ -10947,15 +10976,15 @@
         <v>0</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B83" s="27"/>
       <c r="C83" s="30" t="n">
@@ -10974,15 +11003,15 @@
         <v>3000000</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K83" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="B84" s="27"/>
       <c r="C84" s="30" t="n">
@@ -11001,15 +11030,15 @@
         <v>3000000</v>
       </c>
       <c r="J84" s="11" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K84" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="B85" s="27"/>
       <c r="C85" s="30" t="n">
@@ -11028,15 +11057,15 @@
         <v>3000000</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K85" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="B86" s="27"/>
       <c r="C86" s="30" t="n">
@@ -11055,15 +11084,15 @@
         <v>3000000</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K86" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B87" s="27"/>
       <c r="C87" s="30" t="n">
@@ -11088,15 +11117,15 @@
         <v>17000000</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K87" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B88" s="30" t="n">
         <v>0</v>
@@ -11123,15 +11152,15 @@
         <v>17000000</v>
       </c>
       <c r="J88" s="11" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="K88" s="15" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="B89" s="30" t="n">
         <v>0</v>
@@ -11158,15 +11187,15 @@
         <v>17000000</v>
       </c>
       <c r="J89" s="11" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K89" s="15" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="B90" s="30" t="n">
         <v>0</v>
@@ -11187,15 +11216,15 @@
         <v>17000000</v>
       </c>
       <c r="J90" s="11" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="K90" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B91" s="30" t="n">
         <v>0</v>
@@ -11216,15 +11245,15 @@
         <v>17000000</v>
       </c>
       <c r="J91" s="11" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="K91" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B92" s="30" t="n">
         <v>0</v>
@@ -11245,15 +11274,15 @@
         <v>17000000</v>
       </c>
       <c r="J92" s="11" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="K92" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="12" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="B93" s="30" t="n">
         <v>13000000</v>
@@ -11274,10 +11303,10 @@
         <v>8000000</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="K93" s="15" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11360,7 +11389,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="16" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="I101" s="20" t="n">
         <f aca="false">SUMIF(J79:J99,"Planned",I79:I99)</f>
@@ -11419,72 +11448,72 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -11496,19 +11525,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -11520,19 +11549,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -11544,19 +11573,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -11568,19 +11597,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -11592,19 +11621,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -11616,19 +11645,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -11640,19 +11669,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -11664,19 +11693,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -11688,19 +11717,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -11712,19 +11741,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C16" s="24" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -11736,16 +11765,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="C17" s="24" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -11758,19 +11787,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -11782,19 +11811,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="C19" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -11806,19 +11835,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="C20" s="24" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -11830,24 +11859,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="C22" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -11859,16 +11888,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="C23" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -11881,16 +11910,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
+        <v>536</v>
+      </c>
+      <c r="B24" s="13" t="s">
         <v>533</v>
       </c>
-      <c r="B24" s="13" t="s">
-        <v>530</v>
-      </c>
       <c r="C24" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -11903,19 +11932,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="C25" s="24" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -11927,19 +11956,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="C26" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -11951,16 +11980,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="C27" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -11973,16 +12002,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="C28" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -11995,21 +12024,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C30" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -12022,16 +12051,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C31" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -12044,16 +12073,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C32" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -12066,19 +12095,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C33" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -12090,16 +12119,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C34" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -12112,16 +12141,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C35" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -12134,16 +12163,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C36" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -12156,16 +12185,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C37" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -12178,16 +12207,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C38" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E38" s="32"/>
       <c r="F38" s="32"/>
@@ -12200,7 +12229,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="E40" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12237,7 +12266,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E41" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12274,7 +12303,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
   </sheetData>
@@ -12318,23 +12347,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12345,24 +12374,24 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B6" s="19" t="n">
         <v>308343695</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12386,7 +12415,7 @@
         <v>16</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12412,7 +12441,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -12420,7 +12449,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12429,11 +12458,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>17190624.5774776</v>
+        <v>17193594.7255043</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12441,28 +12470,28 @@
         <v>159</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12472,7 +12501,7 @@
       <c r="B13" s="27"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -12498,7 +12527,7 @@
       <c r="B14" s="27"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -12524,7 +12553,7 @@
       <c r="B15" s="27"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -12550,7 +12579,7 @@
       <c r="B16" s="27"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -12575,10 +12604,10 @@
       </c>
       <c r="B17" s="27"/>
       <c r="C17" s="12" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -12603,10 +12632,10 @@
       </c>
       <c r="B18" s="27"/>
       <c r="C18" s="12" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -12631,10 +12660,10 @@
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="12" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -12659,10 +12688,10 @@
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="12" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -12687,10 +12716,10 @@
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="12" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -12715,10 +12744,10 @@
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="12" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -12744,7 +12773,7 @@
       <c r="B23" s="27"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -12769,10 +12798,10 @@
       </c>
       <c r="B24" s="27"/>
       <c r="C24" s="12" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -12797,10 +12826,10 @@
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="12" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -12825,10 +12854,10 @@
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="12" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -12856,7 +12885,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -12883,10 +12912,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
+        <v>603</v>
+      </c>
+      <c r="D28" s="12" t="s">
         <v>600</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>597</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -12913,10 +12942,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -12943,10 +12972,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="E30" s="27"/>
       <c r="F30" s="27"/>
@@ -12967,10 +12996,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -12997,7 +13026,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -13025,10 +13054,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -13055,7 +13084,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -13083,10 +13112,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -13113,7 +13142,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -13141,10 +13170,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -13171,7 +13200,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -13199,10 +13228,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -13229,7 +13258,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -13257,10 +13286,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -13287,7 +13316,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -13315,10 +13344,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -13345,7 +13374,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -13373,7 +13402,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -13401,7 +13430,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -13429,7 +13458,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -13457,7 +13486,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -13485,7 +13514,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -13513,7 +13542,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -13541,7 +13570,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -13569,7 +13598,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -13597,7 +13626,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -13625,7 +13654,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -13647,7 +13676,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add morning campaign runs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5725,7 +5725,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>525654635.46022</v>
+        <v>552080687.146026</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8645,7 +8645,7 @@
         <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>11980000</v>
+        <v>12170000</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>336000</v>
@@ -8660,7 +8660,7 @@
         <v>227</v>
       </c>
       <c r="G5" s="27" t="n">
-        <v>759</v>
+        <v>807</v>
       </c>
       <c r="H5" s="27" t="n">
         <v>492</v>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
-        <v>41180000</v>
+        <v>41370000</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -8725,7 +8725,7 @@
       </c>
       <c r="G7" s="28" t="n">
         <f aca="false">G5+G6</f>
-        <v>859</v>
+        <v>907</v>
       </c>
       <c r="H7" s="28" t="n">
         <f aca="false">H5+H6</f>
@@ -8771,7 +8771,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>41180000</v>
+        <v>41370000</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -8791,7 +8791,7 @@
       </c>
       <c r="G9" s="29" t="n">
         <f aca="false">G7-G8</f>
-        <v>859</v>
+        <v>907</v>
       </c>
       <c r="H9" s="29" t="n">
         <f aca="false">H7-H8</f>
@@ -10574,7 +10574,7 @@
         <v>458</v>
       </c>
       <c r="B63" s="30" t="n">
-        <v>82475</v>
+        <v>168250</v>
       </c>
       <c r="C63" s="30" t="n">
         <v>0</v>
@@ -10589,7 +10589,7 @@
         <v>10</v>
       </c>
       <c r="G63" s="30" t="n">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="H63" s="30" t="n">
         <v>0</v>
@@ -10609,7 +10609,7 @@
         <v>460</v>
       </c>
       <c r="B64" s="30" t="n">
-        <v>11000</v>
+        <v>12000</v>
       </c>
       <c r="C64" s="30" t="n">
         <v>0</v>
@@ -12462,7 +12462,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>17193594.7255043</v>
+        <v>18057962.3055084</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Gold Rush Oct 12
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="634">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1327,13 +1327,22 @@
     <t xml:space="preserve">Kyln tower. Ion type read from icons, confirm</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Rush, Oct 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claimed, 900K in current stock</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Rush run</t>
   </si>
   <si>
+    <t xml:space="preserve">Runs Sundays, Mondays and other days. Set to Yes on days it runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training Day run</t>
+  </si>
+  <si>
     <t xml:space="preserve">Set to Yes on days it runs. Copy the row for more runs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Training Day run</t>
   </si>
   <si>
     <t xml:space="preserve">Level 110 gold orb, promo code Oct 11</t>
@@ -5725,7 +5734,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>552080687.146026</v>
+        <v>552133663.562459</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8593,7 +8602,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -8645,7 +8654,7 @@
         <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>12170000</v>
+        <v>13070000</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>336000</v>
@@ -8671,31 +8680,31 @@
         <v>378</v>
       </c>
       <c r="B6" s="28" t="n">
-        <f aca="false">SUMIFS(B13:B75,$I$13:$I$75,"Yes",$J$13:$J$75,"No")</f>
+        <f aca="false">SUMIFS(B13:B76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
         <v>29200000</v>
       </c>
       <c r="C6" s="28" t="n">
-        <f aca="false">SUMIFS(C13:C75,$I$13:$I$75,"Yes",$J$13:$J$75,"No")</f>
+        <f aca="false">SUMIFS(C13:C76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
         <v>4650000</v>
       </c>
       <c r="D6" s="28" t="n">
-        <f aca="false">SUMIFS(D13:D75,$I$13:$I$75,"Yes",$J$13:$J$75,"No")</f>
+        <f aca="false">SUMIFS(D13:D76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
         <v>3886000</v>
       </c>
       <c r="E6" s="28" t="n">
-        <f aca="false">SUMIFS(E13:E75,$I$13:$I$75,"Yes",$J$13:$J$75,"No")</f>
+        <f aca="false">SUMIFS(E13:E76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
         <v>5386000</v>
       </c>
       <c r="F6" s="28" t="n">
-        <f aca="false">SUMIFS(F13:F75,$I$13:$I$75,"Yes",$J$13:$J$75,"No")</f>
+        <f aca="false">SUMIFS(F13:F76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="28" t="n">
-        <f aca="false">SUMIFS(G13:G75,$I$13:$I$75,"Yes",$J$13:$J$75,"No")</f>
+        <f aca="false">SUMIFS(G13:G76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="28" t="n">
-        <f aca="false">SUMIFS(H13:H75,$I$13:$I$75,"Yes",$J$13:$J$75,"No")</f>
+        <f aca="false">SUMIFS(H13:H76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
         <v>940</v>
       </c>
     </row>
@@ -8705,7 +8714,7 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
-        <v>41370000</v>
+        <v>42270000</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -8737,31 +8746,31 @@
         <v>380</v>
       </c>
       <c r="B8" s="28" t="n">
-        <f aca="false">SUMIF($J$79:$J$99,"Planned",B79:B99)</f>
+        <f aca="false">SUMIF($J$80:$J$100,"Planned",B80:B100)</f>
         <v>0</v>
       </c>
       <c r="C8" s="28" t="n">
-        <f aca="false">SUMIF($J$79:$J$99,"Planned",C79:C99)</f>
+        <f aca="false">SUMIF($J$80:$J$100,"Planned",C80:C100)</f>
         <v>1710000</v>
       </c>
       <c r="D8" s="28" t="n">
-        <f aca="false">SUMIF($J$79:$J$99,"Planned",D79:D99)</f>
+        <f aca="false">SUMIF($J$80:$J$100,"Planned",D80:D100)</f>
         <v>1710000</v>
       </c>
       <c r="E8" s="28" t="n">
-        <f aca="false">SUMIF($J$79:$J$99,"Planned",E79:E99)</f>
+        <f aca="false">SUMIF($J$80:$J$100,"Planned",E80:E100)</f>
         <v>2640000</v>
       </c>
       <c r="F8" s="28" t="n">
-        <f aca="false">SUMIF($J$79:$J$99,"Planned",F79:F99)</f>
+        <f aca="false">SUMIF($J$80:$J$100,"Planned",F80:F100)</f>
         <v>0</v>
       </c>
       <c r="G8" s="28" t="n">
-        <f aca="false">SUMIF($J$79:$J$99,"Planned",G79:G99)</f>
+        <f aca="false">SUMIF($J$80:$J$100,"Planned",G80:G100)</f>
         <v>0</v>
       </c>
       <c r="H8" s="28" t="n">
-        <f aca="false">SUMIF($J$79:$J$99,"Planned",H79:H99)</f>
+        <f aca="false">SUMIF($J$80:$J$100,"Planned",H80:H100)</f>
         <v>0</v>
       </c>
     </row>
@@ -8771,7 +8780,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>41370000</v>
+        <v>42270000</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -9979,7 +9988,7 @@
         <v>431</v>
       </c>
       <c r="B46" s="30" t="n">
-        <v>900000</v>
+        <v>0</v>
       </c>
       <c r="C46" s="30" t="n">
         <v>0</v>
@@ -10000,7 +10009,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="J46" s="11" t="s">
         <v>315</v>
@@ -10014,7 +10023,7 @@
         <v>433</v>
       </c>
       <c r="B47" s="30" t="n">
-        <v>0</v>
+        <v>900000</v>
       </c>
       <c r="C47" s="30" t="n">
         <v>0</v>
@@ -10029,10 +10038,10 @@
         <v>0</v>
       </c>
       <c r="G47" s="30" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H47" s="30" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="I47" s="11" t="s">
         <v>315</v>
@@ -10041,15 +10050,15 @@
         <v>315</v>
       </c>
       <c r="K47" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B48" s="30" t="n">
-        <v>3300000</v>
+        <v>0</v>
       </c>
       <c r="C48" s="30" t="n">
         <v>0</v>
@@ -10064,24 +10073,24 @@
         <v>0</v>
       </c>
       <c r="G48" s="30" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H48" s="30" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="K48" s="15" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B49" s="30" t="n">
         <v>3300000</v>
@@ -10111,18 +10120,18 @@
         <v>311</v>
       </c>
       <c r="K49" s="15" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B50" s="30" t="n">
-        <v>0</v>
+        <v>3300000</v>
       </c>
       <c r="C50" s="30" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D50" s="30" t="n">
         <v>0</v>
@@ -10143,21 +10152,21 @@
         <v>311</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="K50" s="15" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B51" s="30" t="n">
         <v>0</v>
       </c>
       <c r="C51" s="30" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D51" s="30" t="n">
         <v>0</v>
@@ -10181,12 +10190,12 @@
         <v>315</v>
       </c>
       <c r="K51" s="15" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B52" s="30" t="n">
         <v>0</v>
@@ -10195,10 +10204,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="30" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="E52" s="30" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="F52" s="30" t="n">
         <v>0</v>
@@ -10216,24 +10225,24 @@
         <v>315</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B53" s="30" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C53" s="30" t="n">
         <v>0</v>
       </c>
       <c r="D53" s="30" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="E53" s="30" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="F53" s="30" t="n">
         <v>0</v>
@@ -10251,12 +10260,12 @@
         <v>315</v>
       </c>
       <c r="K53" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B54" s="30" t="n">
         <v>750000</v>
@@ -10286,12 +10295,12 @@
         <v>315</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B55" s="30" t="n">
         <v>750000</v>
@@ -10321,12 +10330,12 @@
         <v>315</v>
       </c>
       <c r="K55" s="15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B56" s="30" t="n">
         <v>750000</v>
@@ -10356,12 +10365,12 @@
         <v>315</v>
       </c>
       <c r="K56" s="15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B57" s="30" t="n">
         <v>750000</v>
@@ -10391,12 +10400,12 @@
         <v>315</v>
       </c>
       <c r="K57" s="15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B58" s="30" t="n">
         <v>750000</v>
@@ -10426,12 +10435,12 @@
         <v>315</v>
       </c>
       <c r="K58" s="15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B59" s="30" t="n">
         <v>750000</v>
@@ -10461,12 +10470,12 @@
         <v>315</v>
       </c>
       <c r="K59" s="15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B60" s="30" t="n">
         <v>750000</v>
@@ -10496,18 +10505,18 @@
         <v>315</v>
       </c>
       <c r="K60" s="15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B61" s="30" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C61" s="30" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D61" s="30" t="n">
         <v>0</v>
@@ -10531,18 +10540,18 @@
         <v>315</v>
       </c>
       <c r="K61" s="15" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B62" s="30" t="n">
         <v>0</v>
       </c>
       <c r="C62" s="30" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D62" s="30" t="n">
         <v>0</v>
@@ -10566,15 +10575,15 @@
         <v>315</v>
       </c>
       <c r="K62" s="15" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B63" s="30" t="n">
-        <v>168250</v>
+        <v>0</v>
       </c>
       <c r="C63" s="30" t="n">
         <v>0</v>
@@ -10586,10 +10595,10 @@
         <v>0</v>
       </c>
       <c r="F63" s="30" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G63" s="30" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="H63" s="30" t="n">
         <v>0</v>
@@ -10598,18 +10607,18 @@
         <v>311</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="K63" s="15" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B64" s="30" t="n">
-        <v>12000</v>
+        <v>168250</v>
       </c>
       <c r="C64" s="30" t="n">
         <v>0</v>
@@ -10621,10 +10630,10 @@
         <v>0</v>
       </c>
       <c r="F64" s="30" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G64" s="30" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="H64" s="30" t="n">
         <v>0</v>
@@ -10636,15 +10645,15 @@
         <v>311</v>
       </c>
       <c r="K64" s="15" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B65" s="30" t="n">
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="C65" s="30" t="n">
         <v>0</v>
@@ -10665,27 +10674,49 @@
         <v>0</v>
       </c>
       <c r="I65" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="J65" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="K65" s="15" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="12" t="s">
+        <v>465</v>
+      </c>
+      <c r="B66" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C66" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="11" t="s">
         <v>315</v>
       </c>
-      <c r="J65" s="11" t="s">
+      <c r="J66" s="11" t="s">
         <v>315</v>
       </c>
-      <c r="K65" s="15" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="12"/>
-      <c r="B66" s="30"/>
-      <c r="C66" s="30"/>
-      <c r="D66" s="30"/>
-      <c r="E66" s="30"/>
-      <c r="F66" s="30"/>
-      <c r="G66" s="30"/>
-      <c r="H66" s="30"/>
-      <c r="I66" s="11"/>
-      <c r="J66" s="11"/>
-      <c r="K66" s="12"/>
+      <c r="K66" s="15" t="s">
+        <v>466</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="12"/>
@@ -10804,79 +10835,57 @@
       <c r="J75" s="11"/>
       <c r="K75" s="12"/>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="23" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="B78" s="3" t="s">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="12"/>
+      <c r="B76" s="30"/>
+      <c r="C76" s="30"/>
+      <c r="D76" s="30"/>
+      <c r="E76" s="30"/>
+      <c r="F76" s="30"/>
+      <c r="G76" s="30"/>
+      <c r="H76" s="30"/>
+      <c r="I76" s="11"/>
+      <c r="J76" s="11"/>
+      <c r="K76" s="12"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="23" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="B79" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C79" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="D78" s="3" t="s">
+      <c r="D79" s="3" t="s">
         <v>372</v>
       </c>
-      <c r="E78" s="3" t="s">
+      <c r="E79" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="F78" s="3" t="s">
+      <c r="F79" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="G78" s="3" t="s">
+      <c r="G79" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="H78" s="3" t="s">
+      <c r="H79" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="I78" s="3" t="s">
+      <c r="I79" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J78" s="3" t="s">
+      <c r="J79" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K78" s="3" t="s">
+      <c r="K79" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="12" t="s">
-        <v>466</v>
-      </c>
-      <c r="B79" s="30" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C79" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D79" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E79" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G79" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H79" s="30" t="n">
-        <v>183</v>
-      </c>
-      <c r="I79" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J79" s="11" t="s">
-        <v>467</v>
-      </c>
-      <c r="K79" s="15" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10884,10 +10893,10 @@
         <v>469</v>
       </c>
       <c r="B80" s="30" t="n">
-        <v>0</v>
+        <v>1837500</v>
       </c>
       <c r="C80" s="30" t="n">
-        <v>359800</v>
+        <v>0</v>
       </c>
       <c r="D80" s="30" t="n">
         <v>0</v>
@@ -10896,66 +10905,66 @@
         <v>0</v>
       </c>
       <c r="F80" s="30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G80" s="30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H80" s="30" t="n">
-        <v>0</v>
+        <v>183</v>
       </c>
       <c r="I80" s="30" t="n">
         <v>0</v>
       </c>
       <c r="J80" s="11" t="s">
-        <v>467</v>
-      </c>
-      <c r="K80" s="15"/>
+        <v>470</v>
+      </c>
+      <c r="K80" s="15" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
+        <v>472</v>
+      </c>
+      <c r="B81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" s="30" t="n">
+        <v>359800</v>
+      </c>
+      <c r="D81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" s="11" t="s">
         <v>470</v>
       </c>
-      <c r="B81" s="30" t="n">
-        <v>9791250</v>
-      </c>
-      <c r="C81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G81" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H81" s="30" t="n">
-        <v>979</v>
-      </c>
-      <c r="I81" s="30" t="n">
-        <v>55000000</v>
-      </c>
-      <c r="J81" s="11" t="s">
-        <v>467</v>
-      </c>
-      <c r="K81" s="15" t="s">
-        <v>471</v>
-      </c>
+      <c r="K81" s="15"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B82" s="30" t="n">
-        <v>0</v>
+        <v>9791250</v>
       </c>
       <c r="C82" s="30" t="n">
-        <v>359800</v>
+        <v>0</v>
       </c>
       <c r="D82" s="30" t="n">
         <v>0</v>
@@ -10964,31 +10973,33 @@
         <v>0</v>
       </c>
       <c r="F82" s="30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G82" s="30" t="n">
         <v>0</v>
       </c>
       <c r="H82" s="30" t="n">
-        <v>0</v>
+        <v>979</v>
       </c>
       <c r="I82" s="30" t="n">
-        <v>0</v>
+        <v>55000000</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>473</v>
-      </c>
-      <c r="B83" s="27"/>
+        <v>475</v>
+      </c>
+      <c r="B83" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="C83" s="30" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D83" s="30" t="n">
         <v>0</v>
@@ -10996,17 +11007,23 @@
       <c r="E83" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F83" s="27"/>
-      <c r="G83" s="27"/>
-      <c r="H83" s="27"/>
+      <c r="F83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="I83" s="30" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J83" s="11" t="s">
+        <v>470</v>
+      </c>
+      <c r="K83" s="15" t="s">
         <v>474</v>
-      </c>
-      <c r="K83" s="15" t="s">
-        <v>475</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11030,15 +11047,15 @@
         <v>3000000</v>
       </c>
       <c r="J84" s="11" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="K84" s="15" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B85" s="27"/>
       <c r="C85" s="30" t="n">
@@ -11057,15 +11074,15 @@
         <v>3000000</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="K85" s="15" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B86" s="27"/>
       <c r="C86" s="30" t="n">
@@ -11084,15 +11101,15 @@
         <v>3000000</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="K86" s="15" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B87" s="27"/>
       <c r="C87" s="30" t="n">
@@ -11104,40 +11121,32 @@
       <c r="E87" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F87" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G87" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H87" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="F87" s="27"/>
+      <c r="G87" s="27"/>
+      <c r="H87" s="27"/>
       <c r="I87" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="K87" s="15" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>480</v>
-      </c>
-      <c r="B88" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>482</v>
+      </c>
+      <c r="B88" s="27"/>
       <c r="C88" s="30" t="n">
-        <v>1710500</v>
+        <v>0</v>
       </c>
       <c r="D88" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E88" s="30" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F88" s="30" t="n">
         <v>0</v>
@@ -11152,21 +11161,21 @@
         <v>17000000</v>
       </c>
       <c r="J88" s="11" t="s">
-        <v>467</v>
+        <v>477</v>
       </c>
       <c r="K88" s="15" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B89" s="30" t="n">
         <v>0</v>
       </c>
       <c r="C89" s="30" t="n">
-        <v>1710000</v>
+        <v>1710500</v>
       </c>
       <c r="D89" s="30" t="n">
         <v>1710000</v>
@@ -11187,22 +11196,28 @@
         <v>17000000</v>
       </c>
       <c r="J89" s="11" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="K89" s="15" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B90" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C90" s="27"/>
-      <c r="D90" s="27"/>
-      <c r="E90" s="27"/>
+      <c r="C90" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D90" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E90" s="30" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F90" s="30" t="n">
         <v>0</v>
       </c>
@@ -11216,15 +11231,15 @@
         <v>17000000</v>
       </c>
       <c r="J90" s="11" t="s">
-        <v>485</v>
+        <v>477</v>
       </c>
       <c r="K90" s="15" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B91" s="30" t="n">
         <v>0</v>
@@ -11245,15 +11260,15 @@
         <v>17000000</v>
       </c>
       <c r="J91" s="11" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="K91" s="15" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B92" s="30" t="n">
         <v>0</v>
@@ -11274,53 +11289,69 @@
         <v>17000000</v>
       </c>
       <c r="J92" s="11" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="K92" s="15" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="12" t="s">
+        <v>490</v>
+      </c>
+      <c r="B93" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" s="27"/>
+      <c r="D93" s="27"/>
+      <c r="E93" s="27"/>
+      <c r="F93" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J93" s="11" t="s">
         <v>488</v>
       </c>
-      <c r="B93" s="30" t="n">
+      <c r="K93" s="15" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="12" t="s">
+        <v>491</v>
+      </c>
+      <c r="B94" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C93" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D93" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E93" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F93" s="27"/>
-      <c r="G93" s="27"/>
-      <c r="H93" s="27"/>
-      <c r="I93" s="30" t="n">
+      <c r="C94" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" s="27"/>
+      <c r="G94" s="27"/>
+      <c r="H94" s="27"/>
+      <c r="I94" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J93" s="11" t="s">
-        <v>485</v>
-      </c>
-      <c r="K93" s="15" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="12"/>
-      <c r="B94" s="30"/>
-      <c r="C94" s="30"/>
-      <c r="D94" s="30"/>
-      <c r="E94" s="30"/>
-      <c r="F94" s="30"/>
-      <c r="G94" s="30"/>
-      <c r="H94" s="30"/>
-      <c r="I94" s="30"/>
-      <c r="J94" s="11"/>
-      <c r="K94" s="12"/>
+      <c r="J94" s="11" t="s">
+        <v>488</v>
+      </c>
+      <c r="K94" s="15" t="s">
+        <v>492</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12"/>
@@ -11387,12 +11418,25 @@
       <c r="J99" s="11"/>
       <c r="K99" s="12"/>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="16" t="s">
-        <v>490</v>
-      </c>
-      <c r="I101" s="20" t="n">
-        <f aca="false">SUMIF(J79:J99,"Planned",I79:I99)</f>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="12"/>
+      <c r="B100" s="30"/>
+      <c r="C100" s="30"/>
+      <c r="D100" s="30"/>
+      <c r="E100" s="30"/>
+      <c r="F100" s="30"/>
+      <c r="G100" s="30"/>
+      <c r="H100" s="30"/>
+      <c r="I100" s="30"/>
+      <c r="J100" s="11"/>
+      <c r="K100" s="12"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="16" t="s">
+        <v>493</v>
+      </c>
+      <c r="I102" s="20" t="n">
+        <f aca="false">SUMIF(J80:J100,"Planned",I80:I100)</f>
         <v>46000000</v>
       </c>
     </row>
@@ -11402,22 +11446,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J79:J99">
+  <conditionalFormatting sqref="J80:J100">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J75">
+  <conditionalFormatting sqref="J13:J76">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J75" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J76" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J79:J99" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J80:J100" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11448,12 +11492,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11467,53 +11511,53 @@
         <v>370</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
@@ -11525,19 +11569,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F7" s="32"/>
       <c r="G7" s="32"/>
@@ -11549,19 +11593,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>
@@ -11573,19 +11617,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F9" s="32"/>
       <c r="G9" s="32"/>
@@ -11597,19 +11641,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F10" s="32"/>
       <c r="G10" s="32"/>
@@ -11621,19 +11665,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F11" s="32"/>
       <c r="G11" s="32"/>
@@ -11645,19 +11689,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F12" s="32"/>
       <c r="G12" s="32"/>
@@ -11669,19 +11713,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F13" s="32"/>
       <c r="G13" s="32"/>
@@ -11693,19 +11737,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F14" s="32"/>
       <c r="G14" s="32"/>
@@ -11717,19 +11761,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15" s="32"/>
@@ -11741,19 +11785,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C16" s="24" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F16" s="32"/>
       <c r="G16" s="32"/>
@@ -11765,16 +11809,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C17" s="24" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -11787,19 +11831,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F18" s="32"/>
       <c r="G18" s="32"/>
@@ -11811,19 +11855,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C19" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F19" s="32"/>
       <c r="G19" s="32"/>
@@ -11835,19 +11879,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C20" s="24" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F20" s="32"/>
       <c r="G20" s="32"/>
@@ -11859,24 +11903,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="C22" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -11888,16 +11932,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="C23" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -11910,16 +11954,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
+        <v>539</v>
+      </c>
+      <c r="B24" s="13" t="s">
         <v>536</v>
       </c>
-      <c r="B24" s="13" t="s">
-        <v>533</v>
-      </c>
       <c r="C24" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -11932,19 +11976,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="C25" s="24" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="32"/>
@@ -11956,19 +12000,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="C26" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -11980,16 +12024,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="C27" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -12002,16 +12046,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="C28" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -12024,21 +12068,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="C30" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -12051,16 +12095,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="C31" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -12073,16 +12117,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="C32" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -12095,19 +12139,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="C33" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -12119,16 +12163,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="C34" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -12141,16 +12185,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="C35" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -12163,16 +12207,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="C36" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -12185,16 +12229,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="C37" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -12207,16 +12251,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="C38" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="E38" s="32"/>
       <c r="F38" s="32"/>
@@ -12229,7 +12273,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="E40" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12266,7 +12310,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="E41" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12303,7 +12347,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
     </row>
   </sheetData>
@@ -12347,12 +12391,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12360,10 +12404,10 @@
         <v>224</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12374,13 +12418,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12391,7 +12435,7 @@
         <v>308343695</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12441,7 +12485,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -12449,7 +12493,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12458,11 +12502,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>18057962.3055084</v>
+        <v>18059695.1080089</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12473,19 +12517,19 @@
         <v>233</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12501,7 +12545,7 @@
       <c r="B13" s="27"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -12527,7 +12571,7 @@
       <c r="B14" s="27"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -12553,7 +12597,7 @@
       <c r="B15" s="27"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -12579,7 +12623,7 @@
       <c r="B16" s="27"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -12604,10 +12648,10 @@
       </c>
       <c r="B17" s="27"/>
       <c r="C17" s="12" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -12632,10 +12676,10 @@
       </c>
       <c r="B18" s="27"/>
       <c r="C18" s="12" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -12660,10 +12704,10 @@
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="12" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -12688,10 +12732,10 @@
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="12" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -12716,10 +12760,10 @@
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="12" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -12744,10 +12788,10 @@
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="12" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -12773,7 +12817,7 @@
       <c r="B23" s="27"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -12798,10 +12842,10 @@
       </c>
       <c r="B24" s="27"/>
       <c r="C24" s="12" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -12826,10 +12870,10 @@
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="12" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -12854,10 +12898,10 @@
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="12" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -12885,7 +12929,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -12912,10 +12956,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
+        <v>606</v>
+      </c>
+      <c r="D28" s="12" t="s">
         <v>603</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>600</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -12942,10 +12986,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -12972,10 +13016,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="E30" s="27"/>
       <c r="F30" s="27"/>
@@ -12996,10 +13040,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -13026,7 +13070,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -13054,10 +13098,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -13084,7 +13128,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -13112,10 +13156,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -13142,7 +13186,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -13170,10 +13214,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -13200,7 +13244,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -13228,10 +13272,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -13258,7 +13302,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -13286,10 +13330,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -13316,7 +13360,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -13344,10 +13388,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -13374,7 +13418,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -13402,7 +13446,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -13430,7 +13474,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -13458,7 +13502,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -13486,7 +13530,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -13514,7 +13558,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -13542,7 +13586,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -13570,7 +13614,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -13598,7 +13642,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -13626,7 +13670,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -13654,7 +13698,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -13676,7 +13720,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add basic gold orbs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1432,7 +1432,7 @@
     <t xml:space="preserve">Gold orbs</t>
   </si>
   <si>
-    <t xml:space="preserve">Random amount. Enter what you get</t>
+    <t xml:space="preserve">Running total of basic gold orbs opened. Already in current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Planned upgrades</t>
@@ -5734,7 +5734,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>552133663.562459</v>
+        <v>552176552.000634</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8654,7 +8654,7 @@
         <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>13070000</v>
+        <v>13545000</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>336000</v>
@@ -8714,7 +8714,7 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
-        <v>42270000</v>
+        <v>42745000</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -8780,7 +8780,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>42270000</v>
+        <v>42745000</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -10688,7 +10688,7 @@
         <v>465</v>
       </c>
       <c r="B66" s="30" t="n">
-        <v>0</v>
+        <v>375000</v>
       </c>
       <c r="C66" s="30" t="n">
         <v>0</v>
@@ -12506,7 +12506,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>18059695.1080089</v>
+        <v>18061097.9395796</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Plan level 101s with real costs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="640">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1465,24 +1465,45 @@
     <t xml:space="preserve">Doctor Strange to level 101</t>
   </si>
   <si>
+    <t xml:space="preserve">Skipped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Astral team is low priority</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whiplash to level 101</t>
+  </si>
+  <si>
     <t xml:space="preserve">Planned</t>
   </si>
   <si>
+    <t xml:space="preserve">Expect about 1.65M gold and 164 orange, like Storm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storm to level 101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uncanny Avengers, from training screen Oct 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Second Uncanny Avenger to level 101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimate from Storm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Third Uncanny Avenger to level 101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimate from Storm. Needs battle pass level 95 orange</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whiplash to gear tier 20</t>
+  </si>
+  <si>
     <t xml:space="preserve">Check cost in game</t>
   </si>
   <si>
-    <t xml:space="preserve">Whiplash to level 101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellowjacket to level 101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ancient One to level 101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whiplash to gear tier 20</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hulk Iso-8 to T3 level 5</t>
   </si>
   <si>
@@ -1496,9 +1517,6 @@
   </si>
   <si>
     <t xml:space="preserve">Blade (Mighty) Iso-8 to T3 level 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skipped</t>
   </si>
   <si>
     <t xml:space="preserve">Spider-Woman (Julia) Iso-8 to T3 level 5</t>
@@ -5734,7 +5752,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>552245628.915153</v>
+        <v>552317272.231916</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8602,7 +8620,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K102"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -8654,7 +8672,7 @@
         <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>13554775</v>
+        <v>15270000</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>336000</v>
@@ -8672,7 +8690,7 @@
         <v>871</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>492</v>
+        <v>522</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8681,7 +8699,7 @@
       </c>
       <c r="B6" s="28" t="n">
         <f aca="false">SUMIFS(B13:B76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
-        <v>29200000</v>
+        <v>28750000</v>
       </c>
       <c r="C6" s="28" t="n">
         <f aca="false">SUMIFS(C13:C76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
@@ -8705,7 +8723,7 @@
       </c>
       <c r="H6" s="28" t="n">
         <f aca="false">SUMIFS(H13:H76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
-        <v>940</v>
+        <v>885</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8714,7 +8732,7 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
-        <v>42754775</v>
+        <v>44020000</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -8738,7 +8756,7 @@
       </c>
       <c r="H7" s="28" t="n">
         <f aca="false">H5+H6</f>
-        <v>1432</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8746,32 +8764,32 @@
         <v>380</v>
       </c>
       <c r="B8" s="28" t="n">
-        <f aca="false">SUMIF($J$80:$J$100,"Planned",B80:B100)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$80:$J$101,"Planned",B80:B101)</f>
+        <v>4950010</v>
       </c>
       <c r="C8" s="28" t="n">
-        <f aca="false">SUMIF($J$80:$J$100,"Planned",C80:C100)</f>
+        <f aca="false">SUMIF($J$80:$J$101,"Planned",C80:C101)</f>
         <v>1710000</v>
       </c>
       <c r="D8" s="28" t="n">
-        <f aca="false">SUMIF($J$80:$J$100,"Planned",D80:D100)</f>
+        <f aca="false">SUMIF($J$80:$J$101,"Planned",D80:D101)</f>
         <v>1710000</v>
       </c>
       <c r="E8" s="28" t="n">
-        <f aca="false">SUMIF($J$80:$J$100,"Planned",E80:E100)</f>
+        <f aca="false">SUMIF($J$80:$J$101,"Planned",E80:E101)</f>
         <v>2640000</v>
       </c>
       <c r="F8" s="28" t="n">
-        <f aca="false">SUMIF($J$80:$J$100,"Planned",F80:F100)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$80:$J$101,"Planned",F80:F101)</f>
+        <v>9</v>
       </c>
       <c r="G8" s="28" t="n">
-        <f aca="false">SUMIF($J$80:$J$100,"Planned",G80:G100)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$80:$J$101,"Planned",G80:G101)</f>
+        <v>3</v>
       </c>
       <c r="H8" s="28" t="n">
-        <f aca="false">SUMIF($J$80:$J$100,"Planned",H80:H100)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$80:$J$101,"Planned",H80:H101)</f>
+        <v>492</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8780,7 +8798,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>42754775</v>
+        <v>39069990</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -8796,15 +8814,15 @@
       </c>
       <c r="F9" s="29" t="n">
         <f aca="false">F7-F8</f>
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="G9" s="29" t="n">
         <f aca="false">G7-G8</f>
-        <v>971</v>
+        <v>968</v>
       </c>
       <c r="H9" s="29" t="n">
         <f aca="false">H7-H8</f>
-        <v>1432</v>
+        <v>915</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9328,7 +9346,7 @@
         <v>311</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="K26" s="15"/>
     </row>
@@ -9361,7 +9379,7 @@
         <v>311</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="K27" s="15"/>
     </row>
@@ -11074,17 +11092,19 @@
         <v>3000000</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="K85" s="15" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>480</v>
-      </c>
-      <c r="B86" s="27"/>
+        <v>482</v>
+      </c>
+      <c r="B86" s="30" t="n">
+        <v>1650010</v>
+      </c>
       <c r="C86" s="30" t="n">
         <v>0</v>
       </c>
@@ -11094,24 +11114,32 @@
       <c r="E86" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F86" s="27"/>
-      <c r="G86" s="27"/>
-      <c r="H86" s="27"/>
+      <c r="F86" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G86" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" s="30" t="n">
+        <v>164</v>
+      </c>
       <c r="I86" s="30" t="n">
         <v>3000000</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="K86" s="15" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>481</v>
-      </c>
-      <c r="B87" s="27"/>
+        <v>484</v>
+      </c>
+      <c r="B87" s="30" t="n">
+        <v>1650000</v>
+      </c>
       <c r="C87" s="30" t="n">
         <v>0</v>
       </c>
@@ -11121,24 +11149,32 @@
       <c r="E87" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F87" s="27"/>
-      <c r="G87" s="27"/>
-      <c r="H87" s="27"/>
+      <c r="F87" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G87" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" s="30" t="n">
+        <v>164</v>
+      </c>
       <c r="I87" s="30" t="n">
         <v>3000000</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="K87" s="15" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>482</v>
-      </c>
-      <c r="B88" s="27"/>
+        <v>486</v>
+      </c>
+      <c r="B88" s="30" t="n">
+        <v>1650000</v>
+      </c>
       <c r="C88" s="30" t="n">
         <v>0</v>
       </c>
@@ -11149,39 +11185,37 @@
         <v>0</v>
       </c>
       <c r="F88" s="30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G88" s="30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H88" s="30" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="I88" s="30" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J88" s="11" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="K88" s="15" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>483</v>
-      </c>
-      <c r="B89" s="30" t="n">
-        <v>0</v>
-      </c>
+        <v>488</v>
+      </c>
+      <c r="B89" s="27"/>
       <c r="C89" s="30" t="n">
-        <v>1710500</v>
+        <v>0</v>
       </c>
       <c r="D89" s="30" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E89" s="30" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F89" s="30" t="n">
         <v>0</v>
@@ -11196,21 +11230,21 @@
         <v>17000000</v>
       </c>
       <c r="J89" s="11" t="s">
-        <v>470</v>
+        <v>480</v>
       </c>
       <c r="K89" s="15" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B90" s="30" t="n">
         <v>0</v>
       </c>
       <c r="C90" s="30" t="n">
-        <v>1710000</v>
+        <v>1710500</v>
       </c>
       <c r="D90" s="30" t="n">
         <v>1710000</v>
@@ -11231,22 +11265,28 @@
         <v>17000000</v>
       </c>
       <c r="J90" s="11" t="s">
-        <v>477</v>
+        <v>470</v>
       </c>
       <c r="K90" s="15" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="B91" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="C91" s="27"/>
-      <c r="D91" s="27"/>
-      <c r="E91" s="27"/>
+      <c r="C91" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D91" s="30" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E91" s="30" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F91" s="30" t="n">
         <v>0</v>
       </c>
@@ -11260,15 +11300,15 @@
         <v>17000000</v>
       </c>
       <c r="J91" s="11" t="s">
-        <v>488</v>
+        <v>480</v>
       </c>
       <c r="K91" s="15" t="s">
-        <v>478</v>
+        <v>493</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="B92" s="30" t="n">
         <v>0</v>
@@ -11289,15 +11329,15 @@
         <v>17000000</v>
       </c>
       <c r="J92" s="11" t="s">
-        <v>488</v>
+        <v>477</v>
       </c>
       <c r="K92" s="15" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="12" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B93" s="30" t="n">
         <v>0</v>
@@ -11318,53 +11358,69 @@
         <v>17000000</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>488</v>
+        <v>477</v>
       </c>
       <c r="K93" s="15" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="12" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="B94" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" s="27"/>
+      <c r="D94" s="27"/>
+      <c r="E94" s="27"/>
+      <c r="F94" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" s="30" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J94" s="11" t="s">
+        <v>477</v>
+      </c>
+      <c r="K94" s="15" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="12" t="s">
+        <v>497</v>
+      </c>
+      <c r="B95" s="30" t="n">
         <v>13000000</v>
       </c>
-      <c r="C94" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D94" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E94" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F94" s="27"/>
-      <c r="G94" s="27"/>
-      <c r="H94" s="27"/>
-      <c r="I94" s="30" t="n">
+      <c r="C95" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" s="27"/>
+      <c r="G95" s="27"/>
+      <c r="H95" s="27"/>
+      <c r="I95" s="30" t="n">
         <v>8000000</v>
       </c>
-      <c r="J94" s="11" t="s">
-        <v>488</v>
-      </c>
-      <c r="K94" s="15" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="12"/>
-      <c r="B95" s="30"/>
-      <c r="C95" s="30"/>
-      <c r="D95" s="30"/>
-      <c r="E95" s="30"/>
-      <c r="F95" s="30"/>
-      <c r="G95" s="30"/>
-      <c r="H95" s="30"/>
-      <c r="I95" s="30"/>
-      <c r="J95" s="11"/>
-      <c r="K95" s="12"/>
+      <c r="J95" s="11" t="s">
+        <v>477</v>
+      </c>
+      <c r="K95" s="15" t="s">
+        <v>498</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="12"/>
@@ -11431,12 +11487,25 @@
       <c r="J100" s="11"/>
       <c r="K100" s="12"/>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="16" t="s">
-        <v>493</v>
-      </c>
-      <c r="I102" s="20" t="n">
-        <f aca="false">SUMIF(J80:J100,"Planned",I80:I100)</f>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="12"/>
+      <c r="B101" s="30"/>
+      <c r="C101" s="30"/>
+      <c r="D101" s="30"/>
+      <c r="E101" s="30"/>
+      <c r="F101" s="30"/>
+      <c r="G101" s="30"/>
+      <c r="H101" s="30"/>
+      <c r="I101" s="30"/>
+      <c r="J101" s="11"/>
+      <c r="K101" s="12"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="16" t="s">
+        <v>499</v>
+      </c>
+      <c r="I103" s="20" t="n">
+        <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
         <v>46000000</v>
       </c>
     </row>
@@ -11446,7 +11515,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J80:J100">
+  <conditionalFormatting sqref="J80:J101">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
@@ -11461,7 +11530,7 @@
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J80:J100" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J80:J101" type="list">
       <formula1>"Planned,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11492,12 +11561,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11511,50 +11580,50 @@
         <v>370</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="E6" s="32" t="s">
         <v>470</v>
@@ -11569,16 +11638,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="E7" s="32" t="s">
         <v>470</v>
@@ -11593,16 +11662,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="E8" s="32" t="s">
         <v>470</v>
@@ -11617,16 +11686,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
+        <v>519</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>513</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>507</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="E9" s="32" t="s">
         <v>470</v>
@@ -11641,16 +11710,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="E10" s="32" t="s">
         <v>470</v>
@@ -11665,16 +11734,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="E11" s="32" t="s">
         <v>470</v>
@@ -11689,16 +11758,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="E12" s="32" t="s">
         <v>470</v>
@@ -11713,16 +11782,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="E13" s="32" t="s">
         <v>470</v>
@@ -11737,16 +11806,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="E14" s="32" t="s">
         <v>470</v>
@@ -11761,16 +11830,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="E15" s="32" t="s">
         <v>470</v>
@@ -11785,16 +11854,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C16" s="24" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="E16" s="32" t="s">
         <v>470</v>
@@ -11809,16 +11878,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C17" s="24" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -11831,16 +11900,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="E18" s="32" t="s">
         <v>470</v>
@@ -11855,16 +11924,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C19" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="E19" s="32" t="s">
         <v>470</v>
@@ -11879,16 +11948,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
+        <v>538</v>
+      </c>
+      <c r="B20" s="13" t="s">
         <v>532</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>526</v>
       </c>
       <c r="C20" s="24" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="E20" s="32" t="s">
         <v>470</v>
@@ -11903,21 +11972,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="C22" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="E22" s="32" t="s">
         <v>470</v>
@@ -11932,16 +12001,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="C23" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -11954,16 +12023,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="C24" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -11976,16 +12045,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="C25" s="24" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="E25" s="32" t="s">
         <v>470</v>
@@ -12000,16 +12069,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="C26" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="E26" s="32" t="s">
         <v>470</v>
@@ -12024,16 +12093,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="C27" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -12046,16 +12115,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="C28" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -12068,21 +12137,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C30" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -12095,16 +12164,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C31" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -12117,16 +12186,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C32" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -12139,16 +12208,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="C33" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="E33" s="32" t="s">
         <v>470</v>
@@ -12163,16 +12232,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C34" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -12185,16 +12254,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="C35" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -12207,16 +12276,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
+        <v>572</v>
+      </c>
+      <c r="B36" s="13" t="s">
         <v>566</v>
       </c>
-      <c r="B36" s="13" t="s">
-        <v>560</v>
-      </c>
       <c r="C36" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -12229,16 +12298,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C37" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -12251,16 +12320,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C38" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="E38" s="32"/>
       <c r="F38" s="32"/>
@@ -12273,7 +12342,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E40" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12310,7 +12379,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="E41" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12347,7 +12416,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
     </row>
   </sheetData>
@@ -12391,12 +12460,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12404,10 +12473,10 @@
         <v>224</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12418,13 +12487,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12435,7 +12504,7 @@
         <v>308343695</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12485,7 +12554,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -12493,7 +12562,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12502,11 +12571,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>18063357.3768684</v>
+        <v>18065700.7440924</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12517,19 +12586,19 @@
         <v>233</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>585</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>496</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>578</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>579</v>
-      </c>
       <c r="G12" s="3" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12545,7 +12614,7 @@
       <c r="B13" s="27"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -12571,7 +12640,7 @@
       <c r="B14" s="27"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -12597,7 +12666,7 @@
       <c r="B15" s="27"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -12623,7 +12692,7 @@
       <c r="B16" s="27"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -12648,10 +12717,10 @@
       </c>
       <c r="B17" s="27"/>
       <c r="C17" s="12" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -12676,10 +12745,10 @@
       </c>
       <c r="B18" s="27"/>
       <c r="C18" s="12" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -12704,10 +12773,10 @@
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="12" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -12732,10 +12801,10 @@
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="12" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -12760,10 +12829,10 @@
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="12" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -12788,10 +12857,10 @@
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="12" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -12817,7 +12886,7 @@
       <c r="B23" s="27"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -12842,10 +12911,10 @@
       </c>
       <c r="B24" s="27"/>
       <c r="C24" s="12" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -12870,10 +12939,10 @@
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="12" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -12898,10 +12967,10 @@
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="12" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -12929,7 +12998,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -12956,10 +13025,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -12986,10 +13055,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -13016,10 +13085,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="E30" s="27"/>
       <c r="F30" s="27"/>
@@ -13040,10 +13109,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -13070,7 +13139,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -13098,10 +13167,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -13128,7 +13197,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -13156,10 +13225,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -13186,7 +13255,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -13214,10 +13283,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -13244,7 +13313,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -13272,10 +13341,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -13302,7 +13371,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -13330,10 +13399,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -13360,7 +13429,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -13388,10 +13457,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -13418,7 +13487,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -13446,7 +13515,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -13474,7 +13543,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -13502,7 +13571,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -13530,7 +13599,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -13558,7 +13627,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -13586,7 +13655,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -13614,7 +13683,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -13642,7 +13711,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -13670,7 +13739,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -13698,7 +13767,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -13720,7 +13789,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Log Oct 12 dailies and gold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="639">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1348,9 +1348,6 @@
     <t xml:space="preserve">Level 110 gold orb, promo code Oct 11</t>
   </si>
   <si>
-    <t xml:space="preserve">825K + 825K + 1.65M. Copy the row for each new orb</t>
-  </si>
-  <si>
     <t xml:space="preserve">Level 110 gold orb, Breaker of Nature level 120</t>
   </si>
   <si>
@@ -1771,7 +1768,7 @@
     <t xml:space="preserve">Objectives done, required</t>
   </si>
   <si>
-    <t xml:space="preserve">Oct 11 is filled in from your screenshots. The calendar and battle pass rows are left for you.</t>
+    <t xml:space="preserve">Oct 11 and Oct 12 are filled in from your screenshots. The calendar and battle pass rows are left for you.</t>
   </si>
   <si>
     <t xml:space="preserve">Iso Fest Milestones</t>
@@ -5752,7 +5749,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>552317272.231916</v>
+        <v>552405216.273781</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8672,7 +8669,7 @@
         <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>15270000</v>
+        <v>16720000</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>336000</v>
@@ -8699,7 +8696,7 @@
       </c>
       <c r="B6" s="28" t="n">
         <f aca="false">SUMIFS(B13:B76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
-        <v>28750000</v>
+        <v>27050000</v>
       </c>
       <c r="C6" s="28" t="n">
         <f aca="false">SUMIFS(C13:C76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
@@ -8732,7 +8729,7 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
-        <v>44020000</v>
+        <v>43770000</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -8798,7 +8795,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>39069990</v>
+        <v>38819990</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -8899,7 +8896,7 @@
         <v>311</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="K13" s="15" t="s">
         <v>388</v>
@@ -8934,7 +8931,7 @@
         <v>311</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="K14" s="15" t="s">
         <v>390</v>
@@ -10110,15 +10107,15 @@
       <c r="A49" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="B49" s="30" t="n">
+      <c r="B49" s="30" t="s">
+        <v>389</v>
+      </c>
+      <c r="C49" s="30" t="s">
+        <v>387</v>
+      </c>
+      <c r="D49" s="30" t="n">
         <v>3300000</v>
       </c>
-      <c r="C49" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="30" t="n">
-        <v>0</v>
-      </c>
       <c r="E49" s="30" t="n">
         <v>0</v>
       </c>
@@ -10131,19 +10128,19 @@
       <c r="H49" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I49" s="11" t="s">
-        <v>311</v>
+      <c r="I49" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="J49" s="11" t="s">
         <v>311</v>
       </c>
-      <c r="K49" s="15" t="s">
-        <v>438</v>
+      <c r="K49" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B50" s="30" t="n">
         <v>3300000</v>
@@ -10173,12 +10170,12 @@
         <v>311</v>
       </c>
       <c r="K50" s="15" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B51" s="30" t="n">
         <v>0</v>
@@ -10208,12 +10205,12 @@
         <v>315</v>
       </c>
       <c r="K51" s="15" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B52" s="30" t="n">
         <v>0</v>
@@ -10243,12 +10240,12 @@
         <v>315</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B53" s="30" t="n">
         <v>0</v>
@@ -10278,12 +10275,12 @@
         <v>315</v>
       </c>
       <c r="K53" s="15" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B54" s="30" t="n">
         <v>750000</v>
@@ -10313,12 +10310,12 @@
         <v>315</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B55" s="30" t="n">
         <v>750000</v>
@@ -10348,12 +10345,12 @@
         <v>315</v>
       </c>
       <c r="K55" s="15" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B56" s="30" t="n">
         <v>750000</v>
@@ -10383,12 +10380,12 @@
         <v>315</v>
       </c>
       <c r="K56" s="15" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B57" s="30" t="n">
         <v>750000</v>
@@ -10418,12 +10415,12 @@
         <v>315</v>
       </c>
       <c r="K57" s="15" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B58" s="30" t="n">
         <v>750000</v>
@@ -10453,12 +10450,12 @@
         <v>315</v>
       </c>
       <c r="K58" s="15" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B59" s="30" t="n">
         <v>750000</v>
@@ -10488,12 +10485,12 @@
         <v>315</v>
       </c>
       <c r="K59" s="15" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B60" s="30" t="n">
         <v>750000</v>
@@ -10523,12 +10520,12 @@
         <v>315</v>
       </c>
       <c r="K60" s="15" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B61" s="30" t="n">
         <v>750000</v>
@@ -10558,12 +10555,12 @@
         <v>315</v>
       </c>
       <c r="K61" s="15" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B62" s="30" t="n">
         <v>0</v>
@@ -10593,12 +10590,12 @@
         <v>315</v>
       </c>
       <c r="K62" s="15" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B63" s="30" t="n">
         <v>0</v>
@@ -10628,12 +10625,12 @@
         <v>315</v>
       </c>
       <c r="K63" s="15" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B64" s="30" t="n">
         <v>178025</v>
@@ -10663,12 +10660,12 @@
         <v>311</v>
       </c>
       <c r="K64" s="15" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B65" s="30" t="n">
         <v>12000</v>
@@ -10698,12 +10695,12 @@
         <v>311</v>
       </c>
       <c r="K65" s="15" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="12" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B66" s="30" t="n">
         <v>375000</v>
@@ -10733,7 +10730,7 @@
         <v>315</v>
       </c>
       <c r="K66" s="15" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10868,12 +10865,12 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="23" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>370</v>
@@ -10908,7 +10905,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B80" s="30" t="n">
         <v>1837500</v>
@@ -10935,15 +10932,15 @@
         <v>0</v>
       </c>
       <c r="J80" s="11" t="s">
+        <v>469</v>
+      </c>
+      <c r="K80" s="15" t="s">
         <v>470</v>
-      </c>
-      <c r="K80" s="15" t="s">
-        <v>471</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B81" s="30" t="n">
         <v>0</v>
@@ -10970,13 +10967,13 @@
         <v>0</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K81" s="15"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B82" s="30" t="n">
         <v>9791250</v>
@@ -11003,15 +11000,15 @@
         <v>55000000</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B83" s="30" t="n">
         <v>0</v>
@@ -11038,15 +11035,15 @@
         <v>0</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K83" s="15" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B84" s="27"/>
       <c r="C84" s="30" t="n">
@@ -11065,15 +11062,15 @@
         <v>3000000</v>
       </c>
       <c r="J84" s="11" t="s">
+        <v>476</v>
+      </c>
+      <c r="K84" s="15" t="s">
         <v>477</v>
-      </c>
-      <c r="K84" s="15" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B85" s="27"/>
       <c r="C85" s="30" t="n">
@@ -11092,15 +11089,15 @@
         <v>3000000</v>
       </c>
       <c r="J85" s="11" t="s">
+        <v>479</v>
+      </c>
+      <c r="K85" s="15" t="s">
         <v>480</v>
-      </c>
-      <c r="K85" s="15" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B86" s="30" t="n">
         <v>1650010</v>
@@ -11127,15 +11124,15 @@
         <v>3000000</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="K86" s="15" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B87" s="30" t="n">
         <v>1650000</v>
@@ -11162,15 +11159,15 @@
         <v>3000000</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="K87" s="15" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B88" s="30" t="n">
         <v>1650000</v>
@@ -11197,15 +11194,15 @@
         <v>3000000</v>
       </c>
       <c r="J88" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="K88" s="15" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B89" s="27"/>
       <c r="C89" s="30" t="n">
@@ -11230,15 +11227,15 @@
         <v>17000000</v>
       </c>
       <c r="J89" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="K89" s="15" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B90" s="30" t="n">
         <v>0</v>
@@ -11265,15 +11262,15 @@
         <v>17000000</v>
       </c>
       <c r="J90" s="11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K90" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B91" s="30" t="n">
         <v>0</v>
@@ -11300,15 +11297,15 @@
         <v>17000000</v>
       </c>
       <c r="J91" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="K91" s="15" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B92" s="30" t="n">
         <v>0</v>
@@ -11329,15 +11326,15 @@
         <v>17000000</v>
       </c>
       <c r="J92" s="11" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="K92" s="15" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="12" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B93" s="30" t="n">
         <v>0</v>
@@ -11358,15 +11355,15 @@
         <v>17000000</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="K93" s="15" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="12" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B94" s="30" t="n">
         <v>0</v>
@@ -11387,15 +11384,15 @@
         <v>17000000</v>
       </c>
       <c r="J94" s="11" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="K94" s="15" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B95" s="30" t="n">
         <v>13000000</v>
@@ -11416,10 +11413,10 @@
         <v>8000000</v>
       </c>
       <c r="J95" s="11" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="K95" s="15" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11502,7 +11499,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="16" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="I103" s="20" t="n">
         <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
@@ -11561,12 +11558,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11580,55 +11577,57 @@
         <v>370</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>502</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>503</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>504</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>505</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>506</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>507</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>508</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>509</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
+        <v>511</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>512</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>513</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F6" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G6" s="32"/>
       <c r="H6" s="32"/>
       <c r="I6" s="32"/>
@@ -11638,21 +11637,23 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F7" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G7" s="32"/>
       <c r="H7" s="32"/>
       <c r="I7" s="32"/>
@@ -11662,21 +11663,23 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F8" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F8" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G8" s="32"/>
       <c r="H8" s="32"/>
       <c r="I8" s="32"/>
@@ -11686,21 +11689,23 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F9" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G9" s="32"/>
       <c r="H9" s="32"/>
       <c r="I9" s="32"/>
@@ -11710,21 +11715,23 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F10" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G10" s="32"/>
       <c r="H10" s="32"/>
       <c r="I10" s="32"/>
@@ -11734,21 +11741,23 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F11" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F11" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G11" s="32"/>
       <c r="H11" s="32"/>
       <c r="I11" s="32"/>
@@ -11758,21 +11767,23 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F12" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F12" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G12" s="32"/>
       <c r="H12" s="32"/>
       <c r="I12" s="32"/>
@@ -11782,21 +11793,23 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F13" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G13" s="32"/>
       <c r="H13" s="32"/>
       <c r="I13" s="32"/>
@@ -11806,21 +11819,23 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F14" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F14" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G14" s="32"/>
       <c r="H14" s="32"/>
       <c r="I14" s="32"/>
@@ -11830,21 +11845,23 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F15" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F15" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G15" s="32"/>
       <c r="H15" s="32"/>
       <c r="I15" s="32"/>
@@ -11854,21 +11871,23 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C16" s="24" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F16" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F16" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G16" s="32"/>
       <c r="H16" s="32"/>
       <c r="I16" s="32"/>
@@ -11878,19 +11897,21 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
+        <v>530</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>531</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>532</v>
       </c>
       <c r="C17" s="24" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
+      <c r="F17" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G17" s="32"/>
       <c r="H17" s="32"/>
       <c r="I17" s="32"/>
@@ -11900,21 +11921,23 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F18" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G18" s="32"/>
       <c r="H18" s="32"/>
       <c r="I18" s="32"/>
@@ -11924,21 +11947,23 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C19" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F19" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F19" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G19" s="32"/>
       <c r="H19" s="32"/>
       <c r="I19" s="32"/>
@@ -11948,21 +11973,23 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C20" s="24" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F20" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G20" s="32"/>
       <c r="H20" s="32"/>
       <c r="I20" s="32"/>
@@ -11972,24 +11999,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
+        <v>540</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>541</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="C22" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="15" t="s">
         <v>542</v>
       </c>
-      <c r="C22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>543</v>
-      </c>
       <c r="E22" s="32" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
@@ -12001,16 +12028,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B23" s="13" t="s">
+        <v>541</v>
+      </c>
+      <c r="C23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="15" t="s">
         <v>542</v>
-      </c>
-      <c r="C23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>543</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -12023,16 +12050,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B24" s="13" t="s">
+        <v>541</v>
+      </c>
+      <c r="C24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="15" t="s">
         <v>542</v>
-      </c>
-      <c r="C24" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>543</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -12045,21 +12072,23 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
+        <v>545</v>
+      </c>
+      <c r="B25" s="13" t="s">
         <v>546</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>547</v>
       </c>
       <c r="C25" s="24" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>470</v>
-      </c>
-      <c r="F25" s="32"/>
+        <v>469</v>
+      </c>
+      <c r="F25" s="32" t="s">
+        <v>469</v>
+      </c>
       <c r="G25" s="32"/>
       <c r="H25" s="32"/>
       <c r="I25" s="32"/>
@@ -12069,19 +12098,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
+        <v>548</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>546</v>
+      </c>
+      <c r="C26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="15" t="s">
         <v>549</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>547</v>
-      </c>
-      <c r="C26" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>550</v>
-      </c>
       <c r="E26" s="32" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="32"/>
@@ -12093,16 +12122,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
+        <v>550</v>
+      </c>
+      <c r="B27" s="13" t="s">
         <v>551</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="C27" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="15" t="s">
         <v>552</v>
-      </c>
-      <c r="C27" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>553</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -12115,16 +12144,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>554</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="C28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="15" t="s">
         <v>555</v>
-      </c>
-      <c r="C28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>556</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -12137,21 +12166,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>558</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="C30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="15" t="s">
         <v>559</v>
-      </c>
-      <c r="C30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>560</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -12164,16 +12193,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
+        <v>560</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>558</v>
+      </c>
+      <c r="C31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="15" t="s">
         <v>561</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>559</v>
-      </c>
-      <c r="C31" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>562</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -12186,16 +12215,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
+        <v>562</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>558</v>
+      </c>
+      <c r="C32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="15" t="s">
         <v>563</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>559</v>
-      </c>
-      <c r="C32" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>564</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -12208,19 +12237,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
+        <v>564</v>
+      </c>
+      <c r="B33" s="13" t="s">
         <v>565</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="C33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="15" t="s">
         <v>566</v>
       </c>
-      <c r="C33" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>567</v>
-      </c>
       <c r="E33" s="32" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
@@ -12232,16 +12261,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
+        <v>567</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>558</v>
+      </c>
+      <c r="C34" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="15" t="s">
         <v>568</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>559</v>
-      </c>
-      <c r="C34" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="15" t="s">
-        <v>569</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -12254,16 +12283,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
+        <v>569</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>565</v>
+      </c>
+      <c r="C35" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="15" t="s">
         <v>570</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>566</v>
-      </c>
-      <c r="C35" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>571</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -12276,16 +12305,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C36" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -12298,16 +12327,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
+        <v>572</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>558</v>
+      </c>
+      <c r="C37" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="15" t="s">
         <v>573</v>
-      </c>
-      <c r="B37" s="13" t="s">
-        <v>559</v>
-      </c>
-      <c r="C37" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>574</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -12320,16 +12349,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
+        <v>574</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>558</v>
+      </c>
+      <c r="C38" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="15" t="s">
         <v>575</v>
-      </c>
-      <c r="B38" s="13" t="s">
-        <v>559</v>
-      </c>
-      <c r="C38" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="15" t="s">
-        <v>576</v>
       </c>
       <c r="E38" s="32"/>
       <c r="F38" s="32"/>
@@ -12342,7 +12371,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E40" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12350,7 +12379,7 @@
       </c>
       <c r="F40" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(F5:F38="Done"))</f>
-        <v>0</v>
+        <v>2500000</v>
       </c>
       <c r="G40" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(G5:G38="Done"))</f>
@@ -12379,7 +12408,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="E41" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12387,7 +12416,7 @@
       </c>
       <c r="F41" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",F5:F38,"Done")&amp;" of 11"</f>
-        <v>0 of 11</v>
+        <v>11 of 11</v>
       </c>
       <c r="G41" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",G5:G38,"Done")&amp;" of 11"</f>
@@ -12416,7 +12445,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
   </sheetData>
@@ -12460,12 +12489,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12473,10 +12502,10 @@
         <v>224</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>581</v>
+      </c>
+      <c r="D4" s="16" t="s">
         <v>582</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12487,13 +12516,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
+        <v>583</v>
+      </c>
+      <c r="F5" s="16" t="s">
         <v>584</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="G5" s="16" t="s">
         <v>585</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12504,7 +12533,7 @@
         <v>308343695</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12554,7 +12583,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -12562,7 +12591,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12571,11 +12600,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>18065700.7440924</v>
+        <v>18068577.2973275</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12586,19 +12615,19 @@
         <v>233</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>583</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>584</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>585</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>586</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12614,7 +12643,7 @@
       <c r="B13" s="27"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -12640,7 +12669,7 @@
       <c r="B14" s="27"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -12666,7 +12695,7 @@
       <c r="B15" s="27"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -12692,7 +12721,7 @@
       <c r="B16" s="27"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -12717,10 +12746,10 @@
       </c>
       <c r="B17" s="27"/>
       <c r="C17" s="12" t="s">
+        <v>594</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>595</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>596</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -12745,10 +12774,10 @@
       </c>
       <c r="B18" s="27"/>
       <c r="C18" s="12" t="s">
+        <v>596</v>
+      </c>
+      <c r="D18" s="12" t="s">
         <v>597</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>598</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -12773,10 +12802,10 @@
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="12" t="s">
+        <v>598</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>599</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>600</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -12801,10 +12830,10 @@
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="12" t="s">
+        <v>600</v>
+      </c>
+      <c r="D20" s="12" t="s">
         <v>601</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>602</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -12829,10 +12858,10 @@
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="12" t="s">
+        <v>602</v>
+      </c>
+      <c r="D21" s="12" t="s">
         <v>603</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>604</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -12857,10 +12886,10 @@
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="12" t="s">
+        <v>604</v>
+      </c>
+      <c r="D22" s="12" t="s">
         <v>605</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>606</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -12886,7 +12915,7 @@
       <c r="B23" s="27"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -12911,10 +12940,10 @@
       </c>
       <c r="B24" s="27"/>
       <c r="C24" s="12" t="s">
+        <v>607</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>608</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>609</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -12939,10 +12968,10 @@
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="12" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -12967,10 +12996,10 @@
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="12" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -12998,7 +13027,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -13025,10 +13054,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -13055,10 +13084,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -13085,10 +13114,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
+        <v>613</v>
+      </c>
+      <c r="D30" s="12" t="s">
         <v>614</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>615</v>
       </c>
       <c r="E30" s="27"/>
       <c r="F30" s="27"/>
@@ -13109,10 +13138,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -13139,7 +13168,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -13167,10 +13196,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -13197,7 +13226,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -13225,10 +13254,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -13255,7 +13284,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -13283,10 +13312,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -13313,7 +13342,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -13341,10 +13370,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -13371,7 +13400,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -13399,10 +13428,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -13429,7 +13458,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -13457,10 +13486,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -13487,7 +13516,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -13515,7 +13544,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -13543,7 +13572,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -13571,7 +13600,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -13599,7 +13628,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -13627,7 +13656,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -13655,7 +13684,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -13683,7 +13712,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -13711,7 +13740,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -13739,7 +13768,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -13767,7 +13796,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -13789,7 +13818,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Level Uncanny Avengers one at a time for tower cell 20
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="640">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1480,19 +1480,22 @@
     <t xml:space="preserve">Storm to level 101</t>
   </si>
   <si>
-    <t xml:space="preserve">Uncanny Avengers, from training screen Oct 12</t>
+    <t xml:space="preserve">First Uncanny Avenger. Then retry Spider-Man tower cell 20</t>
   </si>
   <si>
     <t xml:space="preserve">Second Uncanny Avenger to level 101</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimate from Storm</t>
+    <t xml:space="preserve">If needed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only if cell 20 still fails after Storm</t>
   </si>
   <si>
     <t xml:space="preserve">Third Uncanny Avenger to level 101</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimate from Storm. Needs battle pass level 95 orange</t>
+    <t xml:space="preserve">Only if cell 20 still fails. Needs battle pass level 95 orange</t>
   </si>
   <si>
     <t xml:space="preserve">Whiplash to gear tier 20</t>
@@ -5749,7 +5752,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>552405216.273781</v>
+        <v>553369423.586879</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8762,7 +8765,7 @@
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",B80:B101)</f>
-        <v>4950010</v>
+        <v>1650010</v>
       </c>
       <c r="C8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",C80:C101)</f>
@@ -8778,15 +8781,15 @@
       </c>
       <c r="F8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",F80:F101)</f>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",G80:G101)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",H80:H101)</f>
-        <v>492</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8795,7 +8798,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>38819990</v>
+        <v>42119990</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -8811,15 +8814,15 @@
       </c>
       <c r="F9" s="29" t="n">
         <f aca="false">F7-F8</f>
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="G9" s="29" t="n">
         <f aca="false">G7-G8</f>
-        <v>968</v>
+        <v>970</v>
       </c>
       <c r="H9" s="29" t="n">
         <f aca="false">H7-H8</f>
-        <v>915</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11159,15 +11162,15 @@
         <v>3000000</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="K87" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B88" s="30" t="n">
         <v>1650000</v>
@@ -11194,15 +11197,15 @@
         <v>3000000</v>
       </c>
       <c r="J88" s="11" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="K88" s="15" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B89" s="27"/>
       <c r="C89" s="30" t="n">
@@ -11230,12 +11233,12 @@
         <v>479</v>
       </c>
       <c r="K89" s="15" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B90" s="30" t="n">
         <v>0</v>
@@ -11265,12 +11268,12 @@
         <v>469</v>
       </c>
       <c r="K90" s="15" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B91" s="30" t="n">
         <v>0</v>
@@ -11300,12 +11303,12 @@
         <v>479</v>
       </c>
       <c r="K91" s="15" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B92" s="30" t="n">
         <v>0</v>
@@ -11329,12 +11332,12 @@
         <v>476</v>
       </c>
       <c r="K92" s="15" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="12" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B93" s="30" t="n">
         <v>0</v>
@@ -11358,12 +11361,12 @@
         <v>476</v>
       </c>
       <c r="K93" s="15" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="12" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B94" s="30" t="n">
         <v>0</v>
@@ -11387,12 +11390,12 @@
         <v>476</v>
       </c>
       <c r="K94" s="15" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B95" s="30" t="n">
         <v>13000000</v>
@@ -11416,7 +11419,7 @@
         <v>476</v>
       </c>
       <c r="K95" s="15" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11499,11 +11502,11 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="16" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="I103" s="20" t="n">
         <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
-        <v>46000000</v>
+        <v>40000000</v>
       </c>
     </row>
   </sheetData>
@@ -11528,7 +11531,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J80:J101" type="list">
-      <formula1>"Planned,Done,Skipped"</formula1>
+      <formula1>"Planned,If needed,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -11558,12 +11561,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11577,50 +11580,50 @@
         <v>370</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="E6" s="32" t="s">
         <v>469</v>
@@ -11637,16 +11640,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E7" s="32" t="s">
         <v>469</v>
@@ -11663,16 +11666,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E8" s="32" t="s">
         <v>469</v>
@@ -11689,16 +11692,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="E9" s="32" t="s">
         <v>469</v>
@@ -11715,16 +11718,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E10" s="32" t="s">
         <v>469</v>
@@ -11741,16 +11744,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E11" s="32" t="s">
         <v>469</v>
@@ -11767,16 +11770,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E12" s="32" t="s">
         <v>469</v>
@@ -11793,16 +11796,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E13" s="32" t="s">
         <v>469</v>
@@ -11819,16 +11822,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E14" s="32" t="s">
         <v>469</v>
@@ -11845,16 +11848,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E15" s="32" t="s">
         <v>469</v>
@@ -11871,16 +11874,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C16" s="24" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E16" s="32" t="s">
         <v>469</v>
@@ -11897,16 +11900,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C17" s="24" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32" t="s">
@@ -11921,16 +11924,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E18" s="32" t="s">
         <v>469</v>
@@ -11947,16 +11950,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C19" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="E19" s="32" t="s">
         <v>469</v>
@@ -11973,16 +11976,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C20" s="24" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="E20" s="32" t="s">
         <v>469</v>
@@ -11999,21 +12002,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C22" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E22" s="32" t="s">
         <v>469</v>
@@ -12028,16 +12031,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
+        <v>544</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>542</v>
+      </c>
+      <c r="C23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="15" t="s">
         <v>543</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>541</v>
-      </c>
-      <c r="C23" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>542</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
@@ -12050,16 +12053,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C24" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -12072,16 +12075,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C25" s="24" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="E25" s="32" t="s">
         <v>469</v>
@@ -12098,16 +12101,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C26" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="E26" s="32" t="s">
         <v>469</v>
@@ -12122,16 +12125,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C27" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
@@ -12144,16 +12147,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C28" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="E28" s="32"/>
       <c r="F28" s="32"/>
@@ -12166,21 +12169,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C30" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="32"/>
@@ -12193,16 +12196,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C31" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="E31" s="32"/>
       <c r="F31" s="32"/>
@@ -12215,16 +12218,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C32" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="32"/>
@@ -12237,16 +12240,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C33" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="E33" s="32" t="s">
         <v>469</v>
@@ -12261,16 +12264,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C34" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
@@ -12283,16 +12286,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C35" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
@@ -12305,16 +12308,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
+        <v>572</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>566</v>
+      </c>
+      <c r="C36" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="15" t="s">
         <v>571</v>
-      </c>
-      <c r="B36" s="13" t="s">
-        <v>565</v>
-      </c>
-      <c r="C36" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>570</v>
       </c>
       <c r="E36" s="32"/>
       <c r="F36" s="32"/>
@@ -12327,16 +12330,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C37" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -12349,16 +12352,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C38" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E38" s="32"/>
       <c r="F38" s="32"/>
@@ -12371,7 +12374,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E40" s="20" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12408,7 +12411,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="E41" s="33" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12445,7 +12448,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
   </sheetData>
@@ -12489,12 +12492,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12502,10 +12505,10 @@
         <v>224</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12516,13 +12519,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12533,7 +12536,7 @@
         <v>308343695</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12583,7 +12586,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B9" s="34" t="n">
         <v>20</v>
@@ -12591,7 +12594,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12600,11 +12603,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>18068577.2973275</v>
+        <v>18100115.4758211</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12615,19 +12618,19 @@
         <v>233</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12643,7 +12646,7 @@
       <c r="B13" s="27"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0</v>
@@ -12669,7 +12672,7 @@
       <c r="B14" s="27"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="E14" s="30" t="n">
         <v>0</v>
@@ -12695,7 +12698,7 @@
       <c r="B15" s="27"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0</v>
@@ -12721,7 +12724,7 @@
       <c r="B16" s="27"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0</v>
@@ -12746,10 +12749,10 @@
       </c>
       <c r="B17" s="27"/>
       <c r="C17" s="12" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="E17" s="30" t="n">
         <v>0</v>
@@ -12774,10 +12777,10 @@
       </c>
       <c r="B18" s="27"/>
       <c r="C18" s="12" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0</v>
@@ -12802,10 +12805,10 @@
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="12" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0</v>
@@ -12830,10 +12833,10 @@
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="12" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0</v>
@@ -12858,10 +12861,10 @@
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="12" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="E21" s="30" t="n">
         <v>0</v>
@@ -12886,10 +12889,10 @@
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="12" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="E22" s="30" t="n">
         <v>0</v>
@@ -12915,7 +12918,7 @@
       <c r="B23" s="27"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E23" s="30" t="n">
         <v>900000</v>
@@ -12940,10 +12943,10 @@
       </c>
       <c r="B24" s="27"/>
       <c r="C24" s="12" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E24" s="30" t="n">
         <v>900000</v>
@@ -12968,10 +12971,10 @@
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="12" t="s">
+        <v>610</v>
+      </c>
+      <c r="D25" s="12" t="s">
         <v>609</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>608</v>
       </c>
       <c r="E25" s="30" t="n">
         <v>0</v>
@@ -12996,10 +12999,10 @@
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="12" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E26" s="30" t="n">
         <v>900000</v>
@@ -13027,7 +13030,7 @@
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>900000</v>
@@ -13054,10 +13057,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>950000</v>
@@ -13084,10 +13087,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0</v>
@@ -13114,10 +13117,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="E30" s="27"/>
       <c r="F30" s="27"/>
@@ -13138,10 +13141,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0</v>
@@ -13168,7 +13171,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="30" t="n">
@@ -13196,10 +13199,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E33" s="30" t="n">
         <v>0</v>
@@ -13226,7 +13229,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="30" t="n">
@@ -13254,10 +13257,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E35" s="30" t="n">
         <v>0</v>
@@ -13284,7 +13287,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="30" t="n">
@@ -13312,10 +13315,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E37" s="30" t="n">
         <v>0</v>
@@ -13342,7 +13345,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="30" t="n">
@@ -13370,10 +13373,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E39" s="30" t="n">
         <v>0</v>
@@ -13400,7 +13403,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="D40" s="12"/>
       <c r="E40" s="30" t="n">
@@ -13428,10 +13431,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E41" s="30" t="n">
         <v>0</v>
@@ -13458,7 +13461,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="30" t="n">
@@ -13486,10 +13489,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E43" s="30" t="n">
         <v>0</v>
@@ -13516,7 +13519,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="30" t="n">
@@ -13544,7 +13547,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D45" s="12"/>
       <c r="E45" s="30" t="n">
@@ -13572,7 +13575,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="30" t="n">
@@ -13600,7 +13603,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="D47" s="12"/>
       <c r="E47" s="30" t="n">
@@ -13628,7 +13631,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="30" t="n">
@@ -13656,7 +13659,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="D49" s="12"/>
       <c r="E49" s="30" t="n">
@@ -13684,7 +13687,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D50" s="12"/>
       <c r="E50" s="30" t="n">
@@ -13712,7 +13715,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D51" s="12"/>
       <c r="E51" s="30" t="n">
@@ -13740,7 +13743,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="30" t="n">
@@ -13768,7 +13771,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D53" s="12"/>
       <c r="E53" s="30" t="n">
@@ -13796,7 +13799,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D54" s="12"/>
       <c r="E54" s="30" t="n">
@@ -13818,7 +13821,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Log Jocasta orbs and power core spending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1288,7 +1288,7 @@
     <t xml:space="preserve">Iso Fest milestone 16</t>
   </si>
   <si>
-    <t xml:space="preserve">About 16.7 million points away</t>
+    <t xml:space="preserve">Reached Oct 12, ready to claim</t>
   </si>
   <si>
     <t xml:space="preserve">Iso Fest milestone 17</t>
@@ -1423,7 +1423,7 @@
     <t xml:space="preserve">Misc</t>
   </si>
   <si>
-    <t xml:space="preserve">Running total of random drops and other small sources. Already in current stock</t>
+    <t xml:space="preserve">Running total of random drops and other small sources, including Jocasta orbs. Already in current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Gold orbs</t>
@@ -5686,14 +5686,14 @@
         <v>226</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>558501630</v>
+        <v>577001630</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>227</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>5988501630</v>
+        <v>6007001630</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6))+SUMPRODUCT((B13:B76="")*(F13:F76="Claimed"))</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>229</v>
@@ -5718,7 +5718,7 @@
       </c>
       <c r="B8" s="16" t="n">
         <f aca="false">IFERROR(INDEX(A13:A76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),"All done")</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>230</v>
@@ -5734,7 +5734,7 @@
       </c>
       <c r="B9" s="20" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>11498370</v>
+        <v>22998370</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5743,7 +5743,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3566498370</v>
+        <v>3547998370</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>553369423.586879</v>
+        <v>555276317.656699</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6514,10 +6514,10 @@
       <c r="D55" s="12"/>
       <c r="E55" s="24" t="n">
         <f aca="false">IF(B55="","",MAX(0,B55-$B$6))</f>
-        <v>11498370</v>
+        <v>0</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6533,7 +6533,7 @@
       <c r="D56" s="12"/>
       <c r="E56" s="24" t="n">
         <f aca="false">IF(B56="","",MAX(0,B56-$B$6))</f>
-        <v>41498370</v>
+        <v>22998370</v>
       </c>
       <c r="F56" s="11" t="s">
         <v>169</v>
@@ -6552,7 +6552,7 @@
       <c r="D57" s="12"/>
       <c r="E57" s="24" t="n">
         <f aca="false">IF(B57="","",MAX(0,B57-$B$6))</f>
-        <v>71498370</v>
+        <v>52998370</v>
       </c>
       <c r="F57" s="11" t="s">
         <v>169</v>
@@ -6571,7 +6571,7 @@
       <c r="D58" s="12"/>
       <c r="E58" s="24" t="n">
         <f aca="false">IF(B58="","",MAX(0,B58-$B$6))</f>
-        <v>101498370</v>
+        <v>82998370</v>
       </c>
       <c r="F58" s="11" t="s">
         <v>169</v>
@@ -6590,7 +6590,7 @@
       <c r="D59" s="12"/>
       <c r="E59" s="24" t="n">
         <f aca="false">IF(B59="","",MAX(0,B59-$B$6))</f>
-        <v>131498370</v>
+        <v>112998370</v>
       </c>
       <c r="F59" s="11" t="s">
         <v>169</v>
@@ -6609,7 +6609,7 @@
       <c r="D60" s="12"/>
       <c r="E60" s="24" t="n">
         <f aca="false">IF(B60="","",MAX(0,B60-$B$6))</f>
-        <v>191498370</v>
+        <v>172998370</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>169</v>
@@ -6628,7 +6628,7 @@
       <c r="D61" s="12"/>
       <c r="E61" s="24" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>266498370</v>
+        <v>247998370</v>
       </c>
       <c r="F61" s="11" t="s">
         <v>169</v>
@@ -6647,7 +6647,7 @@
       <c r="D62" s="12"/>
       <c r="E62" s="24" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>341498370</v>
+        <v>322998370</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>169</v>
@@ -6666,7 +6666,7 @@
       <c r="D63" s="12"/>
       <c r="E63" s="24" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>416498370</v>
+        <v>397998370</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>169</v>
@@ -6685,7 +6685,7 @@
       <c r="D64" s="12"/>
       <c r="E64" s="24" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>491498370</v>
+        <v>472998370</v>
       </c>
       <c r="F64" s="11" t="s">
         <v>169</v>
@@ -6704,7 +6704,7 @@
       <c r="D65" s="12"/>
       <c r="E65" s="24" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>566498370</v>
+        <v>547998370</v>
       </c>
       <c r="F65" s="11" t="s">
         <v>169</v>
@@ -6723,7 +6723,7 @@
       <c r="D66" s="12"/>
       <c r="E66" s="24" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>641498370</v>
+        <v>622998370</v>
       </c>
       <c r="F66" s="11" t="s">
         <v>169</v>
@@ -6742,7 +6742,7 @@
       <c r="D67" s="12"/>
       <c r="E67" s="24" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>791498370</v>
+        <v>772998370</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>169</v>
@@ -6761,7 +6761,7 @@
       <c r="D68" s="12"/>
       <c r="E68" s="24" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>941498370</v>
+        <v>922998370</v>
       </c>
       <c r="F68" s="11" t="s">
         <v>169</v>
@@ -6780,7 +6780,7 @@
       <c r="D69" s="12"/>
       <c r="E69" s="24" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>1091498370</v>
+        <v>1072998370</v>
       </c>
       <c r="F69" s="11" t="s">
         <v>169</v>
@@ -6799,7 +6799,7 @@
       <c r="D70" s="12"/>
       <c r="E70" s="24" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1316498370</v>
+        <v>1297998370</v>
       </c>
       <c r="F70" s="11" t="s">
         <v>169</v>
@@ -6818,7 +6818,7 @@
       <c r="D71" s="12"/>
       <c r="E71" s="24" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1691498370</v>
+        <v>1672998370</v>
       </c>
       <c r="F71" s="11" t="s">
         <v>169</v>
@@ -6837,7 +6837,7 @@
       <c r="D72" s="12"/>
       <c r="E72" s="24" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>2066498370</v>
+        <v>2047998370</v>
       </c>
       <c r="F72" s="11" t="s">
         <v>169</v>
@@ -6856,7 +6856,7 @@
       <c r="D73" s="12"/>
       <c r="E73" s="24" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2441498370</v>
+        <v>2422998370</v>
       </c>
       <c r="F73" s="11" t="s">
         <v>169</v>
@@ -6875,7 +6875,7 @@
       <c r="D74" s="12"/>
       <c r="E74" s="24" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2816498370</v>
+        <v>2797998370</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>169</v>
@@ -6894,7 +6894,7 @@
       <c r="D75" s="12"/>
       <c r="E75" s="24" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>3191498370</v>
+        <v>3172998370</v>
       </c>
       <c r="F75" s="11" t="s">
         <v>169</v>
@@ -6913,7 +6913,7 @@
       <c r="D76" s="12"/>
       <c r="E76" s="24" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3566498370</v>
+        <v>3547998370</v>
       </c>
       <c r="F76" s="11" t="s">
         <v>169</v>
@@ -7094,11 +7094,11 @@
         <v>1000000000</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>47651630</v>
+        <v>52651630</v>
       </c>
       <c r="F7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),MAX(0,D7-E7),0)</f>
-        <v>952348370</v>
+        <v>947348370</v>
       </c>
       <c r="G7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),ROUNDUP(D7/C7,0),"No limit")</f>
@@ -7106,11 +7106,11 @@
       </c>
       <c r="H7" s="22" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>47651630</v>
+        <v>52651630</v>
       </c>
       <c r="I7" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>952348370</v>
+        <v>947348370</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>315</v>
@@ -7130,11 +7130,11 @@
         <v>1000000000</v>
       </c>
       <c r="E8" s="25" t="n">
-        <v>3600000</v>
+        <v>17100000</v>
       </c>
       <c r="F8" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D8),MAX(0,D8-E8),0)</f>
-        <v>996400000</v>
+        <v>982900000</v>
       </c>
       <c r="G8" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D8),ROUNDUP(D8/C8,0),"No limit")</f>
@@ -7142,11 +7142,11 @@
       </c>
       <c r="H8" s="22" t="n">
         <f aca="false">IFERROR(INT(E8/C8),0)</f>
-        <v>900</v>
+        <v>4275</v>
       </c>
       <c r="I8" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F8/C8,0),0)</f>
-        <v>249100</v>
+        <v>245725</v>
       </c>
       <c r="J8" s="11" t="s">
         <v>315</v>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>558501630</v>
+        <v>577001630</v>
       </c>
       <c r="F49" s="20"/>
     </row>
@@ -8573,7 +8573,7 @@
       <c r="E50" s="20"/>
       <c r="F50" s="20" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7378748370</v>
+        <v>7360248370</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8672,7 +8672,7 @@
         <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>16720000</v>
+        <v>16828000</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>336000</v>
@@ -8732,7 +8732,7 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
-        <v>43770000</v>
+        <v>43878000</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -8798,7 +8798,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>42119990</v>
+        <v>42227990</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -10671,7 +10671,7 @@
         <v>462</v>
       </c>
       <c r="B65" s="30" t="n">
-        <v>12000</v>
+        <v>120000</v>
       </c>
       <c r="C65" s="30" t="n">
         <v>0</v>
@@ -12533,7 +12533,7 @@
         <v>226</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>308343695</v>
+        <v>325778995</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>587</v>
@@ -12557,14 +12557,14 @@
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>230</v>
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>0</v>
+        <v>950000</v>
       </c>
       <c r="F7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
@@ -12572,7 +12572,7 @@
       </c>
       <c r="G7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>0</v>
+        <v>1900000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12581,7 +12581,7 @@
       </c>
       <c r="B8" s="20" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>16656305</v>
+        <v>24221005</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12598,7 +12598,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>116656305</v>
+        <v>99221005</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12607,7 +12607,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>18100115.4758211</v>
+        <v>15528494.8366765</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13076,7 +13076,7 @@
       </c>
       <c r="I28" s="24" t="n">
         <f aca="false">IF(B28="","",MAX(0,B28-$B$6))</f>
-        <v>16656305</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13106,7 +13106,7 @@
       </c>
       <c r="I29" s="24" t="n">
         <f aca="false">IF(B29="","",MAX(0,B29-$B$6))</f>
-        <v>41656305</v>
+        <v>24221005</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="I30" s="24" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>66656305</v>
+        <v>49221005</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13160,7 +13160,7 @@
       </c>
       <c r="I31" s="24" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>91656305</v>
+        <v>74221005</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13188,7 +13188,7 @@
       </c>
       <c r="I32" s="24" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>116656305</v>
+        <v>99221005</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="I33" s="24" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>141656305</v>
+        <v>124221005</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13246,7 +13246,7 @@
       </c>
       <c r="I34" s="24" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>166656305</v>
+        <v>149221005</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="I35" s="24" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>191656305</v>
+        <v>174221005</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13304,7 +13304,7 @@
       </c>
       <c r="I36" s="24" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>216656305</v>
+        <v>199221005</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13334,7 +13334,7 @@
       </c>
       <c r="I37" s="24" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>241656305</v>
+        <v>224221005</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13362,7 +13362,7 @@
       </c>
       <c r="I38" s="24" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>291656305</v>
+        <v>274221005</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="I39" s="24" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>341656305</v>
+        <v>324221005</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13420,7 +13420,7 @@
       </c>
       <c r="I40" s="24" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>441656305</v>
+        <v>424221005</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13450,7 +13450,7 @@
       </c>
       <c r="I41" s="24" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>591656305</v>
+        <v>574221005</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13478,7 +13478,7 @@
       </c>
       <c r="I42" s="24" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>791656305</v>
+        <v>774221005</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="I43" s="24" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>991656305</v>
+        <v>974221005</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13536,7 +13536,7 @@
       </c>
       <c r="I44" s="24" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1191656305</v>
+        <v>1174221005</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="I45" s="24" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1391656305</v>
+        <v>1374221005</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13592,7 +13592,7 @@
       </c>
       <c r="I46" s="24" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1591656305</v>
+        <v>1574221005</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13620,7 +13620,7 @@
       </c>
       <c r="I47" s="24" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1791656305</v>
+        <v>1774221005</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="I48" s="24" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1991656305</v>
+        <v>1974221005</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13676,7 +13676,7 @@
       </c>
       <c r="I49" s="24" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2191656305</v>
+        <v>2174221005</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13704,7 +13704,7 @@
       </c>
       <c r="I50" s="24" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2391656305</v>
+        <v>2374221005</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13732,7 +13732,7 @@
       </c>
       <c r="I51" s="24" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2591656305</v>
+        <v>2574221005</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13760,7 +13760,7 @@
       </c>
       <c r="I52" s="24" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2791656305</v>
+        <v>2774221005</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="I53" s="24" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2991656305</v>
+        <v>2974221005</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13816,7 +13816,7 @@
       </c>
       <c r="I54" s="24" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3191656305</v>
+        <v>3174221005</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Storm leveled to 101
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1480,7 +1480,7 @@
     <t xml:space="preserve">Storm to level 101</t>
   </si>
   <si>
-    <t xml:space="preserve">First Uncanny Avenger. Then retry Spider-Man tower cell 20</t>
+    <t xml:space="preserve">Leveled Oct 12. Retry Spider-Man tower cell 20</t>
   </si>
   <si>
     <t xml:space="preserve">Second Uncanny Avenger to level 101</t>
@@ -5693,7 +5693,7 @@
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6007001630</v>
+        <v>6004001630</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>555276317.656699</v>
+        <v>556352310.953285</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7094,11 +7094,11 @@
         <v>1000000000</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>52651630</v>
+        <v>49651630</v>
       </c>
       <c r="F7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),MAX(0,D7-E7),0)</f>
-        <v>947348370</v>
+        <v>950348370</v>
       </c>
       <c r="G7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),ROUNDUP(D7/C7,0),"No limit")</f>
@@ -7106,11 +7106,11 @@
       </c>
       <c r="H7" s="22" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>52651630</v>
+        <v>49651630</v>
       </c>
       <c r="I7" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>947348370</v>
+        <v>950348370</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>315</v>
@@ -7166,11 +7166,11 @@
         <v>15000000</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>3000000</v>
+        <v>6000000</v>
       </c>
       <c r="F9" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D9),MAX(0,D9-E9),0)</f>
-        <v>12000000</v>
+        <v>9000000</v>
       </c>
       <c r="G9" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D9),ROUNDUP(D9/C9,0),"No limit")</f>
@@ -7178,11 +7178,11 @@
       </c>
       <c r="H9" s="22" t="n">
         <f aca="false">IFERROR(INT(E9/C9),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F9/C9,0),0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J9" s="11" t="s">
         <v>311</v>
@@ -8583,7 +8583,7 @@
       <c r="E51" s="20"/>
       <c r="F51" s="20" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5430000000</v>
+        <v>5427000000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8672,7 +8672,7 @@
         <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>16828000</v>
+        <v>13730000</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>336000</v>
@@ -8684,13 +8684,13 @@
         <v>13650000</v>
       </c>
       <c r="F5" s="27" t="n">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G5" s="27" t="n">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>522</v>
+        <v>358</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
-        <v>43878000</v>
+        <v>40780000</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
@@ -8748,15 +8748,15 @@
       </c>
       <c r="F7" s="28" t="n">
         <f aca="false">F5+F6</f>
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G7" s="28" t="n">
         <f aca="false">G5+G6</f>
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="H7" s="28" t="n">
         <f aca="false">H5+H6</f>
-        <v>1407</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",B80:B101)</f>
-        <v>1650010</v>
+        <v>0</v>
       </c>
       <c r="C8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",C80:C101)</f>
@@ -8781,15 +8781,15 @@
       </c>
       <c r="F8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",F80:F101)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",G80:G101)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",H80:H101)</f>
-        <v>164</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8798,7 +8798,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>42227990</v>
+        <v>40780000</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -11127,7 +11127,7 @@
         <v>3000000</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>479</v>
+        <v>469</v>
       </c>
       <c r="K86" s="15" t="s">
         <v>482</v>
@@ -11506,7 +11506,7 @@
       </c>
       <c r="I103" s="20" t="n">
         <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
-        <v>40000000</v>
+        <v>37000000</v>
       </c>
     </row>
   </sheetData>
@@ -12607,7 +12607,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>15528494.8366765</v>
+        <v>15558585.3607401</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Plan second Uncanny Avenger to 101
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1486,13 +1486,13 @@
     <t xml:space="preserve">Second Uncanny Avenger to level 101</t>
   </si>
   <si>
+    <t xml:space="preserve">Cell 20 failed with Storm. Level the weakest member next</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Third Uncanny Avenger to level 101</t>
+  </si>
+  <si>
     <t xml:space="preserve">If needed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only if cell 20 still fails after Storm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Third Uncanny Avenger to level 101</t>
   </si>
   <si>
     <t xml:space="preserve">Only if cell 20 still fails. Needs battle pass level 95 orange</t>
@@ -5752,7 +5752,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>556352310.953285</v>
+        <v>556874246.856147</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",B80:B101)</f>
-        <v>0</v>
+        <v>1650000</v>
       </c>
       <c r="C8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",C80:C101)</f>
@@ -8781,15 +8781,15 @@
       </c>
       <c r="F8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",F80:F101)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",G80:G101)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",H80:H101)</f>
-        <v>0</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8798,7 +8798,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7-B8</f>
-        <v>40780000</v>
+        <v>39130000</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
@@ -8814,15 +8814,15 @@
       </c>
       <c r="F9" s="29" t="n">
         <f aca="false">F7-F8</f>
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="G9" s="29" t="n">
         <f aca="false">G7-G8</f>
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="H9" s="29" t="n">
         <f aca="false">H7-H8</f>
-        <v>1243</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11162,15 +11162,15 @@
         <v>3000000</v>
       </c>
       <c r="J87" s="11" t="s">
+        <v>479</v>
+      </c>
+      <c r="K87" s="15" t="s">
         <v>484</v>
-      </c>
-      <c r="K87" s="15" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B88" s="30" t="n">
         <v>1650000</v>
@@ -11197,7 +11197,7 @@
         <v>3000000</v>
       </c>
       <c r="J88" s="11" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="K88" s="15" t="s">
         <v>487</v>
@@ -11506,7 +11506,7 @@
       </c>
       <c r="I103" s="20" t="n">
         <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
-        <v>37000000</v>
+        <v>40000000</v>
       </c>
     </row>
   </sheetData>
@@ -12607,7 +12607,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>15558585.3607401</v>
+        <v>15573181.4977898</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Beast to 101, Spider-Man iso cost, new stock
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="640">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1483,10 +1483,10 @@
     <t xml:space="preserve">Leveled Oct 12. Retry Spider-Man tower cell 20</t>
   </si>
   <si>
-    <t xml:space="preserve">Second Uncanny Avenger to level 101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cell 20 failed with Storm. Level the weakest member next</t>
+    <t xml:space="preserve">Beast to level 101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leveled Oct 12. Retry cell 20</t>
   </si>
   <si>
     <t xml:space="preserve">Third Uncanny Avenger to level 101</t>
@@ -1513,7 +1513,7 @@
     <t xml:space="preserve">Spider-Man Iso-8 to T3 level 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumed same as Hulk. Confirm with Quick Upgrade</t>
+    <t xml:space="preserve">Quick Upgrade cost Oct 12. Affordable now</t>
   </si>
   <si>
     <t xml:space="preserve">Blade (Mighty) Iso-8 to T3 level 5</t>
@@ -5686,14 +5686,14 @@
         <v>226</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>577001630</v>
+        <v>581651630</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>227</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6004001630</v>
+        <v>6002651630</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5734,7 +5734,7 @@
       </c>
       <c r="B9" s="20" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>22998370</v>
+        <v>18348370</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5743,7 +5743,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3547998370</v>
+        <v>3543348370</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>556874246.856147</v>
+        <v>557112913.759841</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6533,7 +6533,7 @@
       <c r="D56" s="12"/>
       <c r="E56" s="24" t="n">
         <f aca="false">IF(B56="","",MAX(0,B56-$B$6))</f>
-        <v>22998370</v>
+        <v>18348370</v>
       </c>
       <c r="F56" s="11" t="s">
         <v>169</v>
@@ -6552,7 +6552,7 @@
       <c r="D57" s="12"/>
       <c r="E57" s="24" t="n">
         <f aca="false">IF(B57="","",MAX(0,B57-$B$6))</f>
-        <v>52998370</v>
+        <v>48348370</v>
       </c>
       <c r="F57" s="11" t="s">
         <v>169</v>
@@ -6571,7 +6571,7 @@
       <c r="D58" s="12"/>
       <c r="E58" s="24" t="n">
         <f aca="false">IF(B58="","",MAX(0,B58-$B$6))</f>
-        <v>82998370</v>
+        <v>78348370</v>
       </c>
       <c r="F58" s="11" t="s">
         <v>169</v>
@@ -6590,7 +6590,7 @@
       <c r="D59" s="12"/>
       <c r="E59" s="24" t="n">
         <f aca="false">IF(B59="","",MAX(0,B59-$B$6))</f>
-        <v>112998370</v>
+        <v>108348370</v>
       </c>
       <c r="F59" s="11" t="s">
         <v>169</v>
@@ -6609,7 +6609,7 @@
       <c r="D60" s="12"/>
       <c r="E60" s="24" t="n">
         <f aca="false">IF(B60="","",MAX(0,B60-$B$6))</f>
-        <v>172998370</v>
+        <v>168348370</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>169</v>
@@ -6628,7 +6628,7 @@
       <c r="D61" s="12"/>
       <c r="E61" s="24" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>247998370</v>
+        <v>243348370</v>
       </c>
       <c r="F61" s="11" t="s">
         <v>169</v>
@@ -6647,7 +6647,7 @@
       <c r="D62" s="12"/>
       <c r="E62" s="24" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>322998370</v>
+        <v>318348370</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>169</v>
@@ -6666,7 +6666,7 @@
       <c r="D63" s="12"/>
       <c r="E63" s="24" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>397998370</v>
+        <v>393348370</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>169</v>
@@ -6685,7 +6685,7 @@
       <c r="D64" s="12"/>
       <c r="E64" s="24" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>472998370</v>
+        <v>468348370</v>
       </c>
       <c r="F64" s="11" t="s">
         <v>169</v>
@@ -6704,7 +6704,7 @@
       <c r="D65" s="12"/>
       <c r="E65" s="24" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>547998370</v>
+        <v>543348370</v>
       </c>
       <c r="F65" s="11" t="s">
         <v>169</v>
@@ -6723,7 +6723,7 @@
       <c r="D66" s="12"/>
       <c r="E66" s="24" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>622998370</v>
+        <v>618348370</v>
       </c>
       <c r="F66" s="11" t="s">
         <v>169</v>
@@ -6742,7 +6742,7 @@
       <c r="D67" s="12"/>
       <c r="E67" s="24" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>772998370</v>
+        <v>768348370</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>169</v>
@@ -6761,7 +6761,7 @@
       <c r="D68" s="12"/>
       <c r="E68" s="24" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>922998370</v>
+        <v>918348370</v>
       </c>
       <c r="F68" s="11" t="s">
         <v>169</v>
@@ -6780,7 +6780,7 @@
       <c r="D69" s="12"/>
       <c r="E69" s="24" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>1072998370</v>
+        <v>1068348370</v>
       </c>
       <c r="F69" s="11" t="s">
         <v>169</v>
@@ -6799,7 +6799,7 @@
       <c r="D70" s="12"/>
       <c r="E70" s="24" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1297998370</v>
+        <v>1293348370</v>
       </c>
       <c r="F70" s="11" t="s">
         <v>169</v>
@@ -6818,7 +6818,7 @@
       <c r="D71" s="12"/>
       <c r="E71" s="24" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1672998370</v>
+        <v>1668348370</v>
       </c>
       <c r="F71" s="11" t="s">
         <v>169</v>
@@ -6837,7 +6837,7 @@
       <c r="D72" s="12"/>
       <c r="E72" s="24" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>2047998370</v>
+        <v>2043348370</v>
       </c>
       <c r="F72" s="11" t="s">
         <v>169</v>
@@ -6856,7 +6856,7 @@
       <c r="D73" s="12"/>
       <c r="E73" s="24" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2422998370</v>
+        <v>2418348370</v>
       </c>
       <c r="F73" s="11" t="s">
         <v>169</v>
@@ -6875,7 +6875,7 @@
       <c r="D74" s="12"/>
       <c r="E74" s="24" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2797998370</v>
+        <v>2793348370</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>169</v>
@@ -6894,7 +6894,7 @@
       <c r="D75" s="12"/>
       <c r="E75" s="24" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>3172998370</v>
+        <v>3168348370</v>
       </c>
       <c r="F75" s="11" t="s">
         <v>169</v>
@@ -6913,7 +6913,7 @@
       <c r="D76" s="12"/>
       <c r="E76" s="24" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3547998370</v>
+        <v>3543348370</v>
       </c>
       <c r="F76" s="11" t="s">
         <v>169</v>
@@ -7094,11 +7094,11 @@
         <v>1000000000</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>49651630</v>
+        <v>51301630</v>
       </c>
       <c r="F7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),MAX(0,D7-E7),0)</f>
-        <v>950348370</v>
+        <v>948698370</v>
       </c>
       <c r="G7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),ROUNDUP(D7/C7,0),"No limit")</f>
@@ -7106,11 +7106,11 @@
       </c>
       <c r="H7" s="22" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>49651630</v>
+        <v>51301630</v>
       </c>
       <c r="I7" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>950348370</v>
+        <v>948698370</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>315</v>
@@ -7166,11 +7166,11 @@
         <v>15000000</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>6000000</v>
+        <v>9000000</v>
       </c>
       <c r="F9" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D9),MAX(0,D9-E9),0)</f>
-        <v>9000000</v>
+        <v>6000000</v>
       </c>
       <c r="G9" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D9),ROUNDUP(D9/C9,0),"No limit")</f>
@@ -7178,11 +7178,11 @@
       </c>
       <c r="H9" s="22" t="n">
         <f aca="false">IFERROR(INT(E9/C9),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F9/C9,0),0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="11" t="s">
         <v>311</v>
@@ -7670,11 +7670,11 @@
         <v>15000000</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>6000000</v>
+        <v>9000000</v>
       </c>
       <c r="F23" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D23),MAX(0,D23-E23),0)</f>
-        <v>9000000</v>
+        <v>6000000</v>
       </c>
       <c r="G23" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D23),ROUNDUP(D23/C23,0),"No limit")</f>
@@ -7682,11 +7682,11 @@
       </c>
       <c r="H23" s="22" t="n">
         <f aca="false">IFERROR(INT(E23/C23),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I23" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F23/C23,0),0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J23" s="11" t="s">
         <v>311</v>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>577001630</v>
+        <v>584651630</v>
       </c>
       <c r="F49" s="20"/>
     </row>
@@ -8573,7 +8573,7 @@
       <c r="E50" s="20"/>
       <c r="F50" s="20" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7360248370</v>
+        <v>7352598370</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8583,7 +8583,7 @@
       <c r="E51" s="20"/>
       <c r="F51" s="20" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5427000000</v>
+        <v>5421000000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8672,25 +8672,25 @@
         <v>377</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>13730000</v>
+        <v>12080000</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>336000</v>
+        <v>1530000</v>
       </c>
       <c r="D5" s="27" t="n">
         <v>3960000</v>
       </c>
       <c r="E5" s="27" t="n">
-        <v>13650000</v>
+        <v>15550000</v>
       </c>
       <c r="F5" s="27" t="n">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="G5" s="27" t="n">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>358</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8703,7 +8703,7 @@
       </c>
       <c r="C6" s="28" t="n">
         <f aca="false">SUMIFS(C13:C76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
-        <v>4650000</v>
+        <v>3700000</v>
       </c>
       <c r="D6" s="28" t="n">
         <f aca="false">SUMIFS(D13:D76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="E6" s="28" t="n">
         <f aca="false">SUMIFS(E13:E76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
-        <v>5386000</v>
+        <v>3486000</v>
       </c>
       <c r="F6" s="28" t="n">
         <f aca="false">SUMIFS(F13:F76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
@@ -8732,11 +8732,11 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B5+B6</f>
-        <v>40780000</v>
+        <v>39130000</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
-        <v>4986000</v>
+        <v>5230000</v>
       </c>
       <c r="D7" s="28" t="n">
         <f aca="false">D5+D6</f>
@@ -8748,15 +8748,15 @@
       </c>
       <c r="F7" s="28" t="n">
         <f aca="false">F5+F6</f>
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="G7" s="28" t="n">
         <f aca="false">G5+G6</f>
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="H7" s="28" t="n">
         <f aca="false">H5+H6</f>
-        <v>1243</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8765,31 +8765,31 @@
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",B80:B101)</f>
-        <v>1650000</v>
+        <v>0</v>
       </c>
       <c r="C8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",C80:C101)</f>
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="D8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",D80:D101)</f>
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="E8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",E80:E101)</f>
-        <v>2640000</v>
+        <v>2130000</v>
       </c>
       <c r="F8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",F80:F101)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",G80:G101)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",H80:H101)</f>
-        <v>164</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8802,15 +8802,15 @@
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
-        <v>3276000</v>
+        <v>3860000</v>
       </c>
       <c r="D9" s="29" t="n">
         <f aca="false">D7-D8</f>
-        <v>6136000</v>
+        <v>6476000</v>
       </c>
       <c r="E9" s="29" t="n">
         <f aca="false">E7-E8</f>
-        <v>16396000</v>
+        <v>16906000</v>
       </c>
       <c r="F9" s="29" t="n">
         <f aca="false">F7-F8</f>
@@ -9752,7 +9752,7 @@
         <v>311</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="K38" s="15" t="s">
         <v>418</v>
@@ -10114,13 +10114,13 @@
         <v>389</v>
       </c>
       <c r="C49" s="30" t="s">
+        <v>417</v>
+      </c>
+      <c r="D49" s="30" t="s">
         <v>387</v>
       </c>
-      <c r="D49" s="30" t="n">
+      <c r="E49" s="30" t="n">
         <v>3300000</v>
-      </c>
-      <c r="E49" s="30" t="n">
-        <v>0</v>
       </c>
       <c r="F49" s="30" t="n">
         <v>0</v>
@@ -11162,7 +11162,7 @@
         <v>3000000</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>479</v>
+        <v>469</v>
       </c>
       <c r="K87" s="15" t="s">
         <v>484</v>
@@ -11279,13 +11279,13 @@
         <v>0</v>
       </c>
       <c r="C91" s="30" t="n">
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="D91" s="30" t="n">
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="E91" s="30" t="n">
-        <v>2640000</v>
+        <v>2130000</v>
       </c>
       <c r="F91" s="30" t="n">
         <v>0</v>
@@ -11506,7 +11506,7 @@
       </c>
       <c r="I103" s="20" t="n">
         <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
-        <v>40000000</v>
+        <v>37000000</v>
       </c>
     </row>
   </sheetData>
@@ -12540,7 +12540,7 @@
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>2250000</v>
+        <v>1300000</v>
       </c>
       <c r="F6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="G6" s="20" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>7600000</v>
+        <v>5700000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12564,7 +12564,7 @@
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>950000</v>
+        <v>0</v>
       </c>
       <c r="F7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
@@ -12572,7 +12572,7 @@
       </c>
       <c r="G7" s="20" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>1900000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12607,7 +12607,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>15573181.4977898</v>
+        <v>15600301.6147948</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13072,7 +13072,7 @@
         <v>1900000</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="I28" s="24" t="n">
         <f aca="false">IF(B28="","",MAX(0,B28-$B$6))</f>

</xml_diff>

<commit_message>
Spider-Man T3L5, Iron Raider raid, IV at 649M
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1513,7 +1513,7 @@
     <t xml:space="preserve">Spider-Man Iso-8 to T3 level 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Quick Upgrade cost Oct 12. Affordable now</t>
+    <t xml:space="preserve">Done Oct 12, plus 500 ion 1 to unlock the T4 matrix</t>
   </si>
   <si>
     <t xml:space="preserve">Blade (Mighty) Iso-8 to T3 level 5</t>
@@ -5686,14 +5686,14 @@
         <v>226</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>581651630</v>
+        <v>649301650</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>227</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6002651630</v>
+        <v>6007301650</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6))+SUMPRODUCT((B13:B76="")*(F13:F76="Claimed"))</f>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>229</v>
@@ -5718,7 +5718,7 @@
       </c>
       <c r="B8" s="16" t="n">
         <f aca="false">IFERROR(INDEX(A13:A76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),"All done")</f>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>230</v>
@@ -5734,7 +5734,7 @@
       </c>
       <c r="B9" s="20" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>18348370</v>
+        <v>10698350</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5743,7 +5743,7 @@
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3543348370</v>
+        <v>3475698350</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>557112913.759841</v>
+        <v>548207240.6819</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6533,10 +6533,10 @@
       <c r="D56" s="12"/>
       <c r="E56" s="24" t="n">
         <f aca="false">IF(B56="","",MAX(0,B56-$B$6))</f>
-        <v>18348370</v>
+        <v>0</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6552,10 +6552,10 @@
       <c r="D57" s="12"/>
       <c r="E57" s="24" t="n">
         <f aca="false">IF(B57="","",MAX(0,B57-$B$6))</f>
-        <v>48348370</v>
+        <v>0</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6571,7 +6571,7 @@
       <c r="D58" s="12"/>
       <c r="E58" s="24" t="n">
         <f aca="false">IF(B58="","",MAX(0,B58-$B$6))</f>
-        <v>78348370</v>
+        <v>10698350</v>
       </c>
       <c r="F58" s="11" t="s">
         <v>169</v>
@@ -6590,7 +6590,7 @@
       <c r="D59" s="12"/>
       <c r="E59" s="24" t="n">
         <f aca="false">IF(B59="","",MAX(0,B59-$B$6))</f>
-        <v>108348370</v>
+        <v>40698350</v>
       </c>
       <c r="F59" s="11" t="s">
         <v>169</v>
@@ -6609,7 +6609,7 @@
       <c r="D60" s="12"/>
       <c r="E60" s="24" t="n">
         <f aca="false">IF(B60="","",MAX(0,B60-$B$6))</f>
-        <v>168348370</v>
+        <v>100698350</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>169</v>
@@ -6628,7 +6628,7 @@
       <c r="D61" s="12"/>
       <c r="E61" s="24" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>243348370</v>
+        <v>175698350</v>
       </c>
       <c r="F61" s="11" t="s">
         <v>169</v>
@@ -6647,7 +6647,7 @@
       <c r="D62" s="12"/>
       <c r="E62" s="24" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>318348370</v>
+        <v>250698350</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>169</v>
@@ -6666,7 +6666,7 @@
       <c r="D63" s="12"/>
       <c r="E63" s="24" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>393348370</v>
+        <v>325698350</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>169</v>
@@ -6685,7 +6685,7 @@
       <c r="D64" s="12"/>
       <c r="E64" s="24" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>468348370</v>
+        <v>400698350</v>
       </c>
       <c r="F64" s="11" t="s">
         <v>169</v>
@@ -6704,7 +6704,7 @@
       <c r="D65" s="12"/>
       <c r="E65" s="24" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>543348370</v>
+        <v>475698350</v>
       </c>
       <c r="F65" s="11" t="s">
         <v>169</v>
@@ -6723,7 +6723,7 @@
       <c r="D66" s="12"/>
       <c r="E66" s="24" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>618348370</v>
+        <v>550698350</v>
       </c>
       <c r="F66" s="11" t="s">
         <v>169</v>
@@ -6742,7 +6742,7 @@
       <c r="D67" s="12"/>
       <c r="E67" s="24" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>768348370</v>
+        <v>700698350</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>169</v>
@@ -6761,7 +6761,7 @@
       <c r="D68" s="12"/>
       <c r="E68" s="24" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>918348370</v>
+        <v>850698350</v>
       </c>
       <c r="F68" s="11" t="s">
         <v>169</v>
@@ -6780,7 +6780,7 @@
       <c r="D69" s="12"/>
       <c r="E69" s="24" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>1068348370</v>
+        <v>1000698350</v>
       </c>
       <c r="F69" s="11" t="s">
         <v>169</v>
@@ -6799,7 +6799,7 @@
       <c r="D70" s="12"/>
       <c r="E70" s="24" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1293348370</v>
+        <v>1225698350</v>
       </c>
       <c r="F70" s="11" t="s">
         <v>169</v>
@@ -6818,7 +6818,7 @@
       <c r="D71" s="12"/>
       <c r="E71" s="24" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1668348370</v>
+        <v>1600698350</v>
       </c>
       <c r="F71" s="11" t="s">
         <v>169</v>
@@ -6837,7 +6837,7 @@
       <c r="D72" s="12"/>
       <c r="E72" s="24" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>2043348370</v>
+        <v>1975698350</v>
       </c>
       <c r="F72" s="11" t="s">
         <v>169</v>
@@ -6856,7 +6856,7 @@
       <c r="D73" s="12"/>
       <c r="E73" s="24" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2418348370</v>
+        <v>2350698350</v>
       </c>
       <c r="F73" s="11" t="s">
         <v>169</v>
@@ -6875,7 +6875,7 @@
       <c r="D74" s="12"/>
       <c r="E74" s="24" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2793348370</v>
+        <v>2725698350</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>169</v>
@@ -6894,7 +6894,7 @@
       <c r="D75" s="12"/>
       <c r="E75" s="24" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>3168348370</v>
+        <v>3100698350</v>
       </c>
       <c r="F75" s="11" t="s">
         <v>169</v>
@@ -6913,7 +6913,7 @@
       <c r="D76" s="12"/>
       <c r="E76" s="24" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3543348370</v>
+        <v>3475698350</v>
       </c>
       <c r="F76" s="11" t="s">
         <v>169</v>
@@ -7094,11 +7094,11 @@
         <v>1000000000</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>51301630</v>
+        <v>55951650</v>
       </c>
       <c r="F7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),MAX(0,D7-E7),0)</f>
-        <v>948698370</v>
+        <v>944048350</v>
       </c>
       <c r="G7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),ROUNDUP(D7/C7,0),"No limit")</f>
@@ -7106,11 +7106,11 @@
       </c>
       <c r="H7" s="22" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>51301630</v>
+        <v>55951650</v>
       </c>
       <c r="I7" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>948698370</v>
+        <v>944048350</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>315</v>
@@ -7598,11 +7598,11 @@
         <v>15000000</v>
       </c>
       <c r="E21" s="25" t="n">
-        <v>9000000</v>
+        <v>12000000</v>
       </c>
       <c r="F21" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D21),MAX(0,D21-E21),0)</f>
-        <v>6000000</v>
+        <v>3000000</v>
       </c>
       <c r="G21" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D21),ROUNDUP(D21/C21,0),"No limit")</f>
@@ -7610,11 +7610,11 @@
       </c>
       <c r="H21" s="22" t="n">
         <f aca="false">IFERROR(INT(E21/C21),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I21" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F21/C21,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J21" s="11" t="s">
         <v>311</v>
@@ -7634,11 +7634,11 @@
         <v>40000000</v>
       </c>
       <c r="E22" s="25" t="n">
-        <v>24000000</v>
+        <v>32000000</v>
       </c>
       <c r="F22" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D22),MAX(0,D22-E22),0)</f>
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="G22" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D22),ROUNDUP(D22/C22,0),"No limit")</f>
@@ -7646,11 +7646,11 @@
       </c>
       <c r="H22" s="22" t="n">
         <f aca="false">IFERROR(INT(E22/C22),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I22" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F22/C22,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J22" s="11" t="s">
         <v>311</v>
@@ -7670,11 +7670,11 @@
         <v>15000000</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>9000000</v>
+        <v>12000000</v>
       </c>
       <c r="F23" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D23),MAX(0,D23-E23),0)</f>
-        <v>6000000</v>
+        <v>3000000</v>
       </c>
       <c r="G23" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D23),ROUNDUP(D23/C23,0),"No limit")</f>
@@ -7682,11 +7682,11 @@
       </c>
       <c r="H23" s="22" t="n">
         <f aca="false">IFERROR(INT(E23/C23),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I23" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F23/C23,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J23" s="11" t="s">
         <v>311</v>
@@ -7706,11 +7706,11 @@
         <v>40000000</v>
       </c>
       <c r="E24" s="25" t="n">
-        <v>16000000</v>
+        <v>24000000</v>
       </c>
       <c r="F24" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D24),MAX(0,D24-E24),0)</f>
-        <v>24000000</v>
+        <v>16000000</v>
       </c>
       <c r="G24" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D24),ROUNDUP(D24/C24,0),"No limit")</f>
@@ -7718,11 +7718,11 @@
       </c>
       <c r="H24" s="22" t="n">
         <f aca="false">IFERROR(INT(E24/C24),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I24" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F24/C24,0),0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J24" s="11" t="s">
         <v>311</v>
@@ -7742,11 +7742,11 @@
         <v>40000000</v>
       </c>
       <c r="E25" s="25" t="n">
-        <v>24000000</v>
+        <v>32000000</v>
       </c>
       <c r="F25" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D25),MAX(0,D25-E25),0)</f>
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="G25" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D25),ROUNDUP(D25/C25,0),"No limit")</f>
@@ -7754,11 +7754,11 @@
       </c>
       <c r="H25" s="22" t="n">
         <f aca="false">IFERROR(INT(E25/C25),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I25" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F25/C25,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J25" s="11" t="s">
         <v>311</v>
@@ -7814,11 +7814,11 @@
         <v>40000000</v>
       </c>
       <c r="E27" s="25" t="n">
-        <v>24000000</v>
+        <v>32000000</v>
       </c>
       <c r="F27" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D27),MAX(0,D27-E27),0)</f>
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="G27" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D27),ROUNDUP(D27/C27,0),"No limit")</f>
@@ -7826,11 +7826,11 @@
       </c>
       <c r="H27" s="22" t="n">
         <f aca="false">IFERROR(INT(E27/C27),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I27" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F27/C27,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J27" s="11" t="s">
         <v>311</v>
@@ -7886,11 +7886,11 @@
         <v>40000000</v>
       </c>
       <c r="E29" s="25" t="n">
-        <v>16000000</v>
+        <v>24000000</v>
       </c>
       <c r="F29" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D29),MAX(0,D29-E29),0)</f>
-        <v>24000000</v>
+        <v>16000000</v>
       </c>
       <c r="G29" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D29),ROUNDUP(D29/C29,0),"No limit")</f>
@@ -7898,11 +7898,11 @@
       </c>
       <c r="H29" s="22" t="n">
         <f aca="false">IFERROR(INT(E29/C29),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I29" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F29/C29,0),0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J29" s="11" t="s">
         <v>311</v>
@@ -8390,11 +8390,11 @@
         <v>85000000</v>
       </c>
       <c r="E43" s="25" t="n">
-        <v>17000000</v>
+        <v>34000000</v>
       </c>
       <c r="F43" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D43),MAX(0,D43-E43),0)</f>
-        <v>68000000</v>
+        <v>51000000</v>
       </c>
       <c r="G43" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D43),ROUNDUP(D43/C43,0),"No limit")</f>
@@ -8402,11 +8402,11 @@
       </c>
       <c r="H43" s="22" t="n">
         <f aca="false">IFERROR(INT(E43/C43),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I43" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F43/C43,0),0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J43" s="11" t="s">
         <v>311</v>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>584651630</v>
+        <v>652301650</v>
       </c>
       <c r="F49" s="20"/>
     </row>
@@ -8573,7 +8573,7 @@
       <c r="E50" s="20"/>
       <c r="F50" s="20" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7352598370</v>
+        <v>7284948350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8583,7 +8583,7 @@
       <c r="E51" s="20"/>
       <c r="F51" s="20" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5421000000</v>
+        <v>5358000000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8675,13 +8675,13 @@
         <v>12080000</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>1530000</v>
+        <v>159500</v>
       </c>
       <c r="D5" s="27" t="n">
-        <v>3960000</v>
+        <v>2590000</v>
       </c>
       <c r="E5" s="27" t="n">
-        <v>15550000</v>
+        <v>13420000</v>
       </c>
       <c r="F5" s="27" t="n">
         <v>221</v>
@@ -8736,15 +8736,15 @@
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C5+C6</f>
-        <v>5230000</v>
+        <v>3859500</v>
       </c>
       <c r="D7" s="28" t="n">
         <f aca="false">D5+D6</f>
-        <v>7846000</v>
+        <v>6476000</v>
       </c>
       <c r="E7" s="28" t="n">
         <f aca="false">E5+E6</f>
-        <v>19036000</v>
+        <v>16906000</v>
       </c>
       <c r="F7" s="28" t="n">
         <f aca="false">F5+F6</f>
@@ -8769,15 +8769,15 @@
       </c>
       <c r="C8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",C80:C101)</f>
-        <v>1370000</v>
+        <v>0</v>
       </c>
       <c r="D8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",D80:D101)</f>
-        <v>1370000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",E80:E101)</f>
-        <v>2130000</v>
+        <v>0</v>
       </c>
       <c r="F8" s="28" t="n">
         <f aca="false">SUMIF($J$80:$J$101,"Planned",F80:F101)</f>
@@ -8802,7 +8802,7 @@
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">C7-C8</f>
-        <v>3860000</v>
+        <v>3859500</v>
       </c>
       <c r="D9" s="29" t="n">
         <f aca="false">D7-D8</f>
@@ -11300,7 +11300,7 @@
         <v>17000000</v>
       </c>
       <c r="J91" s="11" t="s">
-        <v>479</v>
+        <v>469</v>
       </c>
       <c r="K91" s="15" t="s">
         <v>493</v>
@@ -11506,7 +11506,7 @@
       </c>
       <c r="I103" s="20" t="n">
         <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
-        <v>37000000</v>
+        <v>20000000</v>
       </c>
     </row>
   </sheetData>
@@ -12607,7 +12607,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>15600301.6147948</v>
+        <v>15649710.6454122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Sync scoring to 649M
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5752,7 +5752,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>548207240.6819</v>
+        <v>548219128.227808</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7094,11 +7094,11 @@
         <v>1000000000</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>55951650</v>
+        <v>52951650</v>
       </c>
       <c r="F7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),MAX(0,D7-E7),0)</f>
-        <v>944048350</v>
+        <v>947048350</v>
       </c>
       <c r="G7" s="22" t="n">
         <f aca="false">IF(ISNUMBER(D7),ROUNDUP(D7/C7,0),"No limit")</f>
@@ -7106,11 +7106,11 @@
       </c>
       <c r="H7" s="22" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>55951650</v>
+        <v>52951650</v>
       </c>
       <c r="I7" s="22" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>944048350</v>
+        <v>947048350</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>315</v>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>652301650</v>
+        <v>649301650</v>
       </c>
       <c r="F49" s="20"/>
     </row>
@@ -8573,7 +8573,7 @@
       <c r="E50" s="20"/>
       <c r="F50" s="20" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7284948350</v>
+        <v>7287948350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12607,7 +12607,7 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>15649710.6454122</v>
+        <v>15650049.9927477</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Jocasta blitz done, IV at 747M, Iso Fest at 348M
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -181,7 +181,7 @@
     <t xml:space="preserve">Main team; Diamond 4 at milestone 47</t>
   </si>
   <si>
-    <t xml:space="preserve">T3 L5 done Oct 12, T4 matrix unlocked. 3 diamonds</t>
+    <t xml:space="preserve">T3 L5 done Oct 12, T4 matrix unlocked. 4 diamonds</t>
   </si>
   <si>
     <t xml:space="preserve">Blade (Mighty)</t>
@@ -241,13 +241,13 @@
     <t xml:space="preserve">Blitz tasks in Iron Vengeance</t>
   </si>
   <si>
-    <t xml:space="preserve">Blitz twice with her for 80M points</t>
+    <t xml:space="preserve">Done. Hold until next blitz tier is reachable</t>
   </si>
   <si>
     <t xml:space="preserve">Power cores for more shards</t>
   </si>
   <si>
-    <t xml:space="preserve">Unlocked Oct 12, 1 of 55 shards to next star. Milestone 48 gives her 7 red stars</t>
+    <t xml:space="preserve">Blitzed twice Oct 12. 1 of 55 shards to next star. Milestone 48 gives her 7 red stars</t>
   </si>
   <si>
     <t xml:space="preserve">Doctor Strange</t>
@@ -3174,7 +3174,7 @@
         <v>69</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>80000000</v>
+        <v>0</v>
       </c>
       <c r="J16" s="7" t="s">
         <v>70</v>
@@ -5755,7 +5755,7 @@
         <v>234</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>666802650</v>
+        <v>746802650</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>235</v>
@@ -5771,7 +5771,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6))+SUMPRODUCT((B13:B76="")*(F13:F76="Claimed"))</f>
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>237</v>
@@ -5787,7 +5787,7 @@
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),"All done")</f>
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>238</v>
@@ -5803,7 +5803,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>23197350</v>
+        <v>3197350</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3458197350</v>
+        <v>3378197350</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5821,7 +5821,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>550168601.469724</v>
+        <v>537656223.555091</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6659,10 +6659,10 @@
       <c r="D59" s="11"/>
       <c r="E59" s="23" t="n">
         <f aca="false">IF(B59="","",MAX(0,B59-$B$6))</f>
-        <v>23197350</v>
+        <v>0</v>
       </c>
       <c r="F59" s="10" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6678,7 +6678,7 @@
       <c r="D60" s="11"/>
       <c r="E60" s="23" t="n">
         <f aca="false">IF(B60="","",MAX(0,B60-$B$6))</f>
-        <v>83197350</v>
+        <v>3197350</v>
       </c>
       <c r="F60" s="10" t="s">
         <v>177</v>
@@ -6697,7 +6697,7 @@
       <c r="D61" s="11"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>158197350</v>
+        <v>78197350</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>177</v>
@@ -6716,7 +6716,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>233197350</v>
+        <v>153197350</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>177</v>
@@ -6735,7 +6735,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>308197350</v>
+        <v>228197350</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>177</v>
@@ -6754,7 +6754,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>383197350</v>
+        <v>303197350</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>177</v>
@@ -6773,7 +6773,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>458197350</v>
+        <v>378197350</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>177</v>
@@ -6792,7 +6792,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>533197350</v>
+        <v>453197350</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>177</v>
@@ -6811,7 +6811,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>683197350</v>
+        <v>603197350</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>177</v>
@@ -6830,7 +6830,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>833197350</v>
+        <v>753197350</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>177</v>
@@ -6849,7 +6849,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>983197350</v>
+        <v>903197350</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>177</v>
@@ -6868,7 +6868,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1208197350</v>
+        <v>1128197350</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>177</v>
@@ -6887,7 +6887,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1583197350</v>
+        <v>1503197350</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>177</v>
@@ -6906,7 +6906,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1958197350</v>
+        <v>1878197350</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>177</v>
@@ -6925,7 +6925,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2333197350</v>
+        <v>2253197350</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>177</v>
@@ -6944,7 +6944,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2708197350</v>
+        <v>2628197350</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>177</v>
@@ -6963,7 +6963,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>3083197350</v>
+        <v>3003197350</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>177</v>
@@ -6982,7 +6982,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3458197350</v>
+        <v>3378197350</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>177</v>
@@ -8027,11 +8027,11 @@
         <v>80000000</v>
       </c>
       <c r="E31" s="24" t="n">
-        <v>0</v>
+        <v>80000000</v>
       </c>
       <c r="F31" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D31),MAX(0,D31-E31),0)</f>
-        <v>80000000</v>
+        <v>0</v>
       </c>
       <c r="G31" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D31),ROUNDUP(D31/C31,0),"No limit")</f>
@@ -8039,11 +8039,11 @@
       </c>
       <c r="H31" s="21" t="n">
         <f aca="false">IFERROR(INT(E31/C31),0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I31" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F31/C31,0),0)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J31" s="10" t="s">
         <v>319</v>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="E49" s="19" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>666802650</v>
+        <v>746802650</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -8642,7 +8642,7 @@
       <c r="E50" s="19"/>
       <c r="F50" s="19" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7270447350</v>
+        <v>7190447350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8652,7 +8652,7 @@
       <c r="E51" s="19"/>
       <c r="F51" s="19" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5358000000</v>
+        <v>5278000000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12602,7 +12602,7 @@
         <v>234</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>330153995</v>
+        <v>347958315</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>594</v>
@@ -12650,7 +12650,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>19846005</v>
+        <v>2041685</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12667,7 +12667,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>94846005</v>
+        <v>77041685</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12676,7 +12676,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>15089160.2513664</v>
+        <v>12261551.7161515</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13175,7 +13175,7 @@
       </c>
       <c r="I29" s="23" t="n">
         <f aca="false">IF(B29="","",MAX(0,B29-$B$6))</f>
-        <v>19846005</v>
+        <v>2041685</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13199,7 +13199,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>44846005</v>
+        <v>27041685</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13229,7 +13229,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>69846005</v>
+        <v>52041685</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13257,7 +13257,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>94846005</v>
+        <v>77041685</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>119846005</v>
+        <v>102041685</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13315,7 +13315,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>144846005</v>
+        <v>127041685</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13345,7 +13345,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>169846005</v>
+        <v>152041685</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13373,7 +13373,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>194846005</v>
+        <v>177041685</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13403,7 +13403,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>219846005</v>
+        <v>202041685</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13431,7 +13431,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>269846005</v>
+        <v>252041685</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>319846005</v>
+        <v>302041685</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>419846005</v>
+        <v>402041685</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13519,7 +13519,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>569846005</v>
+        <v>552041685</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13547,7 +13547,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>769846005</v>
+        <v>752041685</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13577,7 +13577,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>969846005</v>
+        <v>952041685</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1169846005</v>
+        <v>1152041685</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13633,7 +13633,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1369846005</v>
+        <v>1352041685</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13661,7 +13661,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1569846005</v>
+        <v>1552041685</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1769846005</v>
+        <v>1752041685</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1969846005</v>
+        <v>1952041685</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2169846005</v>
+        <v>2152041685</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13773,7 +13773,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2369846005</v>
+        <v>2352041685</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13801,7 +13801,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2569846005</v>
+        <v>2552041685</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13829,7 +13829,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2769846005</v>
+        <v>2752041685</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13857,7 +13857,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2969846005</v>
+        <v>2952041685</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13885,7 +13885,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3169846005</v>
+        <v>3152041685</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Prioritize Amazing Avengers, drop Uncanny Avengers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,12 +32,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1248" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1248" uniqueCount="646">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
   <si>
-    <t xml:space="preserve">Iron Raider goal: all five at gear tier 20 for Omega tower floors. Lower number means build first. Change Priority or Status anytime and sort by Priority. Blank yellow cells are details to fill in from the game.</t>
+    <t xml:space="preserve">Focus now: Amazing Avengers for Spider-Man tower cell 20. Iron Raider goal: all five at gear tier 20 for Omega tower floors. Lower number means build first. Change Priority or Status anytime and sort by Priority. Blank yellow cells are details to fill in from the game.</t>
   </si>
   <si>
     <t xml:space="preserve">Priority</t>
@@ -1513,10 +1513,7 @@
     <t xml:space="preserve">Third Uncanny Avenger to level 101</t>
   </si>
   <si>
-    <t xml:space="preserve">If needed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only if cell 20 still fails. Needs battle pass level 95 orange</t>
+    <t xml:space="preserve">Amazing Avengers carry cell 20 now</t>
   </si>
   <si>
     <t xml:space="preserve">Whiplash to gear tier 20</t>
@@ -2742,7 +2739,7 @@
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>14</v>
@@ -2780,7 +2777,7 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>22</v>
@@ -2818,7 +2815,7 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>27</v>
@@ -2856,7 +2853,7 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>32</v>
@@ -2894,7 +2891,7 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>36</v>
@@ -2932,7 +2929,7 @@
     </row>
     <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>40</v>
@@ -2970,7 +2967,7 @@
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>47</v>
@@ -3008,7 +3005,7 @@
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>50</v>
@@ -3044,7 +3041,7 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>56</v>
@@ -3082,7 +3079,7 @@
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>59</v>
@@ -5821,7 +5818,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>537656223.555091</v>
+        <v>538195003.702131</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11266,15 +11263,15 @@
         <v>3000000</v>
       </c>
       <c r="J88" s="10" t="s">
+        <v>483</v>
+      </c>
+      <c r="K88" s="14" t="s">
         <v>493</v>
-      </c>
-      <c r="K88" s="14" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B89" s="26"/>
       <c r="C89" s="29" t="n">
@@ -11302,12 +11299,12 @@
         <v>486</v>
       </c>
       <c r="K89" s="14" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="11" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B90" s="29" t="n">
         <v>0</v>
@@ -11337,12 +11334,12 @@
         <v>476</v>
       </c>
       <c r="K90" s="14" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B91" s="29" t="n">
         <v>0</v>
@@ -11372,12 +11369,12 @@
         <v>476</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="11" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B92" s="29" t="n">
         <v>0</v>
@@ -11401,12 +11398,12 @@
         <v>483</v>
       </c>
       <c r="K92" s="14" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B93" s="29" t="n">
         <v>0</v>
@@ -11430,12 +11427,12 @@
         <v>483</v>
       </c>
       <c r="K93" s="14" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B94" s="29" t="n">
         <v>0</v>
@@ -11459,12 +11456,12 @@
         <v>483</v>
       </c>
       <c r="K94" s="14" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B95" s="29" t="n">
         <v>13000000</v>
@@ -11488,7 +11485,7 @@
         <v>483</v>
       </c>
       <c r="K95" s="14" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11571,7 +11568,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="15" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="I103" s="19" t="n">
         <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
@@ -11630,12 +11627,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11649,50 +11646,50 @@
         <v>377</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>509</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>510</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>511</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>512</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>513</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>514</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>515</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>516</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
+        <v>518</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>519</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>520</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="E6" s="31" t="s">
         <v>476</v>
@@ -11709,16 +11706,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E7" s="31" t="s">
         <v>476</v>
@@ -11735,16 +11732,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E8" s="31" t="s">
         <v>476</v>
@@ -11761,16 +11758,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E9" s="31" t="s">
         <v>476</v>
@@ -11787,16 +11784,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E10" s="31" t="s">
         <v>476</v>
@@ -11813,16 +11810,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E11" s="31" t="s">
         <v>476</v>
@@ -11839,16 +11836,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E12" s="31" t="s">
         <v>476</v>
@@ -11865,16 +11862,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E13" s="31" t="s">
         <v>476</v>
@@ -11891,16 +11888,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="E14" s="31" t="s">
         <v>476</v>
@@ -11917,16 +11914,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E15" s="31" t="s">
         <v>476</v>
@@ -11943,16 +11940,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="E16" s="31" t="s">
         <v>476</v>
@@ -11969,16 +11966,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
+        <v>537</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>538</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>539</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
@@ -11993,16 +11990,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E18" s="31" t="s">
         <v>476</v>
@@ -12019,16 +12016,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="E19" s="31" t="s">
         <v>476</v>
@@ -12045,16 +12042,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="E20" s="31" t="s">
         <v>476</v>
@@ -12071,21 +12068,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
+        <v>547</v>
+      </c>
+      <c r="B22" s="12" t="s">
         <v>548</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="C22" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="14" t="s">
         <v>549</v>
-      </c>
-      <c r="C22" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>550</v>
       </c>
       <c r="E22" s="31" t="s">
         <v>476</v>
@@ -12100,16 +12097,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B23" s="12" t="s">
+        <v>548</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>549</v>
-      </c>
-      <c r="C23" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>550</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12122,16 +12119,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B24" s="12" t="s">
+        <v>548</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="14" t="s">
         <v>549</v>
-      </c>
-      <c r="C24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>550</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12144,16 +12141,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
+        <v>552</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>553</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>554</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="E25" s="31" t="s">
         <v>476</v>
@@ -12170,16 +12167,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
+        <v>555</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>553</v>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="14" t="s">
         <v>556</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>554</v>
-      </c>
-      <c r="C26" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="14" t="s">
-        <v>557</v>
       </c>
       <c r="E26" s="31" t="s">
         <v>476</v>
@@ -12194,16 +12191,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
+        <v>557</v>
+      </c>
+      <c r="B27" s="12" t="s">
         <v>558</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="C27" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="14" t="s">
         <v>559</v>
-      </c>
-      <c r="C27" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="14" t="s">
-        <v>560</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12216,16 +12213,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
+        <v>560</v>
+      </c>
+      <c r="B28" s="12" t="s">
         <v>561</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="C28" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="14" t="s">
         <v>562</v>
-      </c>
-      <c r="C28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>563</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12238,21 +12235,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
+        <v>564</v>
+      </c>
+      <c r="B30" s="12" t="s">
         <v>565</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="C30" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="14" t="s">
         <v>566</v>
-      </c>
-      <c r="C30" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>567</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12265,16 +12262,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
+        <v>567</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="C31" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="14" t="s">
         <v>568</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>566</v>
-      </c>
-      <c r="C31" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>569</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12287,16 +12284,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
+        <v>569</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="C32" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="14" t="s">
         <v>570</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>566</v>
-      </c>
-      <c r="C32" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>571</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12309,16 +12306,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
+        <v>571</v>
+      </c>
+      <c r="B33" s="12" t="s">
         <v>572</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="C33" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="14" t="s">
         <v>573</v>
-      </c>
-      <c r="C33" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>574</v>
       </c>
       <c r="E33" s="31" t="s">
         <v>476</v>
@@ -12333,16 +12330,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
+        <v>574</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="14" t="s">
         <v>575</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>566</v>
-      </c>
-      <c r="C34" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>576</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12355,16 +12352,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
+        <v>576</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>572</v>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="14" t="s">
         <v>577</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>573</v>
-      </c>
-      <c r="C35" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>578</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12377,16 +12374,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12399,16 +12396,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
+        <v>579</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="14" t="s">
         <v>580</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>566</v>
-      </c>
-      <c r="C37" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>581</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12421,16 +12418,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
+        <v>581</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="14" t="s">
         <v>582</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>566</v>
-      </c>
-      <c r="C38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>583</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12443,7 +12440,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12480,7 +12477,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12517,7 +12514,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
   </sheetData>
@@ -12561,12 +12558,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12574,10 +12571,10 @@
         <v>232</v>
       </c>
       <c r="B4" s="16" t="s">
+        <v>588</v>
+      </c>
+      <c r="D4" s="15" t="s">
         <v>589</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>590</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12588,13 +12585,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
+        <v>590</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="G5" s="15" t="s">
         <v>592</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12605,7 +12602,7 @@
         <v>347958315</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12655,7 +12652,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -12663,7 +12660,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12672,11 +12669,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>12261551.7161515</v>
+        <v>12273838.8889894</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12687,19 +12684,19 @@
         <v>241</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>591</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>592</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>593</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12715,7 +12712,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -12741,7 +12738,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -12767,7 +12764,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -12793,7 +12790,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -12818,10 +12815,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
+        <v>601</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>602</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>603</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -12846,10 +12843,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
+        <v>603</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>604</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>605</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -12874,10 +12871,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
+        <v>605</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>606</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>607</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -12902,10 +12899,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
+        <v>607</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>608</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>609</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -12930,10 +12927,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
+        <v>609</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>610</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>611</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -12958,10 +12955,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
+        <v>611</v>
+      </c>
+      <c r="D22" s="11" t="s">
         <v>612</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>613</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -12987,7 +12984,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13012,10 +13009,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
+        <v>614</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>615</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>616</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13040,10 +13037,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13068,10 +13065,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13099,7 +13096,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13126,10 +13123,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13156,10 +13153,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13186,10 +13183,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
+        <v>620</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>621</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>622</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13210,10 +13207,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13240,7 +13237,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13268,10 +13265,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13298,7 +13295,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13326,10 +13323,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13356,7 +13353,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13384,10 +13381,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13414,7 +13411,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13442,10 +13439,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13472,7 +13469,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13500,10 +13497,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13530,7 +13527,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13558,10 +13555,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -13588,7 +13585,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -13616,7 +13613,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -13644,7 +13641,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -13672,7 +13669,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -13700,7 +13697,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -13728,7 +13725,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -13756,7 +13753,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -13784,7 +13781,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -13812,7 +13809,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -13840,7 +13837,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -13868,7 +13865,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -13890,7 +13887,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Campaign rewards and basic training orb
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1250" uniqueCount="651">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1254" uniqueCount="653">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1394,6 +1394,12 @@
   </si>
   <si>
     <t xml:space="preserve">Pending claim. Also gives the level 110 training orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basic training orbs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running total of basic training orbs opened. Already in current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Level 110 training orb</t>
@@ -5837,7 +5843,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>538914595.922865</v>
+        <v>538952717.222715</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8705,7 +8711,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K103"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -8757,7 +8763,7 @@
         <v>389</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>12130000</v>
+        <v>12280000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>159500</v>
@@ -8772,10 +8778,10 @@
         <v>221</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>869</v>
+        <v>893</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>194</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8783,31 +8789,31 @@
         <v>390</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
+        <f aca="false">SUMIFS(B13:B77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
         <v>27050000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
+        <f aca="false">SUMIFS(C13:C77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
         <v>3700000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
+        <f aca="false">SUMIFS(D13:D77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
         <v>3886000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
+        <f aca="false">SUMIFS(E13:E77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
         <v>3486000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
+        <f aca="false">SUMIFS(F13:F77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
+        <f aca="false">SUMIFS(G13:G77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H76,$I$13:$I$76,"Yes",$J$13:$J$76,"No")</f>
+        <f aca="false">SUMIFS(H13:H77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
         <v>885</v>
       </c>
     </row>
@@ -8817,7 +8823,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>39180000</v>
+        <v>39330000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8837,11 +8843,11 @@
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>969</v>
+        <v>993</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1079</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8849,31 +8855,31 @@
         <v>392</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$80:$J$101,"Planned",B80:B101)</f>
+        <f aca="false">SUMIF($J$81:$J$102,"Planned",B81:B102)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$80:$J$101,"Planned",C80:C101)</f>
+        <f aca="false">SUMIF($J$81:$J$102,"Planned",C81:C102)</f>
         <v>0</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$80:$J$101,"Planned",D80:D101)</f>
+        <f aca="false">SUMIF($J$81:$J$102,"Planned",D81:D102)</f>
         <v>0</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$80:$J$101,"Planned",E80:E101)</f>
+        <f aca="false">SUMIF($J$81:$J$102,"Planned",E81:E102)</f>
         <v>0</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$80:$J$101,"Planned",F80:F101)</f>
+        <f aca="false">SUMIF($J$81:$J$102,"Planned",F81:F102)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$80:$J$101,"Planned",G80:G101)</f>
+        <f aca="false">SUMIF($J$81:$J$102,"Planned",G81:G102)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$80:$J$101,"Planned",H80:H101)</f>
+        <f aca="false">SUMIF($J$81:$J$102,"Planned",H81:H102)</f>
         <v>0</v>
       </c>
     </row>
@@ -8883,7 +8889,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>39180000</v>
+        <v>39330000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8903,11 +8909,11 @@
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>969</v>
+        <v>993</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>1079</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10319,13 +10325,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I52" s="10" t="s">
         <v>324</v>
       </c>
       <c r="J52" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K52" s="14" t="s">
         <v>455</v>
@@ -10342,10 +10348,10 @@
         <v>0</v>
       </c>
       <c r="D53" s="29" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="E53" s="29" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="F53" s="29" t="n">
         <v>0</v>
@@ -10371,16 +10377,16 @@
         <v>458</v>
       </c>
       <c r="B54" s="29" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C54" s="29" t="n">
         <v>0</v>
       </c>
       <c r="D54" s="29" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="E54" s="29" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="F54" s="29" t="n">
         <v>0</v>
@@ -10468,12 +10474,12 @@
         <v>328</v>
       </c>
       <c r="K56" s="14" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B57" s="29" t="n">
         <v>750000</v>
@@ -10503,12 +10509,12 @@
         <v>328</v>
       </c>
       <c r="K57" s="14" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B58" s="29" t="n">
         <v>750000</v>
@@ -10538,12 +10544,12 @@
         <v>328</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B59" s="29" t="n">
         <v>750000</v>
@@ -10573,12 +10579,12 @@
         <v>328</v>
       </c>
       <c r="K59" s="14" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B60" s="29" t="n">
         <v>750000</v>
@@ -10608,12 +10614,12 @@
         <v>328</v>
       </c>
       <c r="K60" s="14" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B61" s="29" t="n">
         <v>750000</v>
@@ -10643,18 +10649,18 @@
         <v>328</v>
       </c>
       <c r="K61" s="14" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B62" s="29" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C62" s="29" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D62" s="29" t="n">
         <v>0</v>
@@ -10678,7 +10684,7 @@
         <v>328</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10689,7 +10695,7 @@
         <v>0</v>
       </c>
       <c r="C63" s="29" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D63" s="29" t="n">
         <v>0</v>
@@ -10721,7 +10727,7 @@
         <v>472</v>
       </c>
       <c r="B64" s="29" t="n">
-        <v>178025</v>
+        <v>0</v>
       </c>
       <c r="C64" s="29" t="n">
         <v>0</v>
@@ -10733,10 +10739,10 @@
         <v>0</v>
       </c>
       <c r="F64" s="29" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G64" s="29" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="H64" s="29" t="n">
         <v>0</v>
@@ -10745,7 +10751,7 @@
         <v>324</v>
       </c>
       <c r="J64" s="10" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="K64" s="14" t="s">
         <v>473</v>
@@ -10756,7 +10762,7 @@
         <v>474</v>
       </c>
       <c r="B65" s="29" t="n">
-        <v>120000</v>
+        <v>225800</v>
       </c>
       <c r="C65" s="29" t="n">
         <v>0</v>
@@ -10768,10 +10774,10 @@
         <v>0</v>
       </c>
       <c r="F65" s="29" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G65" s="29" t="n">
-        <v>64</v>
+        <v>116</v>
       </c>
       <c r="H65" s="29" t="n">
         <v>0</v>
@@ -10791,7 +10797,7 @@
         <v>476</v>
       </c>
       <c r="B66" s="29" t="n">
-        <v>375000</v>
+        <v>120000</v>
       </c>
       <c r="C66" s="29" t="n">
         <v>0</v>
@@ -10806,33 +10812,55 @@
         <v>0</v>
       </c>
       <c r="G66" s="29" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="H66" s="29" t="n">
         <v>0</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="J66" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K66" s="14" t="s">
         <v>477</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="11"/>
-      <c r="B67" s="29"/>
-      <c r="C67" s="29"/>
-      <c r="D67" s="29"/>
-      <c r="E67" s="29"/>
-      <c r="F67" s="29"/>
-      <c r="G67" s="29"/>
-      <c r="H67" s="29"/>
-      <c r="I67" s="10"/>
-      <c r="J67" s="10"/>
-      <c r="K67" s="11"/>
+      <c r="A67" s="11" t="s">
+        <v>478</v>
+      </c>
+      <c r="B67" s="29" t="n">
+        <v>375000</v>
+      </c>
+      <c r="C67" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="J67" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="K67" s="14" t="s">
+        <v>479</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="11"/>
@@ -10951,123 +10979,103 @@
       <c r="J76" s="10"/>
       <c r="K76" s="11"/>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="22" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="3" t="s">
-        <v>479</v>
-      </c>
-      <c r="B79" s="3" t="s">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="11"/>
+      <c r="B77" s="29"/>
+      <c r="C77" s="29"/>
+      <c r="D77" s="29"/>
+      <c r="E77" s="29"/>
+      <c r="F77" s="29"/>
+      <c r="G77" s="29"/>
+      <c r="H77" s="29"/>
+      <c r="I77" s="10"/>
+      <c r="J77" s="10"/>
+      <c r="K77" s="11"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="22" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="B80" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="C80" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="D79" s="3" t="s">
+      <c r="D80" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="E79" s="3" t="s">
+      <c r="E80" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="F79" s="3" t="s">
+      <c r="F80" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="G79" s="3" t="s">
+      <c r="G80" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="H79" s="3" t="s">
+      <c r="H80" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="I79" s="3" t="s">
+      <c r="I80" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J79" s="3" t="s">
+      <c r="J80" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K79" s="3" t="s">
+      <c r="K80" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="11" t="s">
-        <v>480</v>
-      </c>
-      <c r="B80" s="29" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C80" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D80" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E80" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F80" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="G80" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H80" s="29" t="n">
-        <v>183</v>
-      </c>
-      <c r="I80" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J80" s="10" t="s">
-        <v>481</v>
-      </c>
-      <c r="K80" s="14" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
+        <v>482</v>
+      </c>
+      <c r="B81" s="29" t="n">
+        <v>1837500</v>
+      </c>
+      <c r="C81" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G81" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H81" s="29" t="n">
+        <v>183</v>
+      </c>
+      <c r="I81" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" s="10" t="s">
         <v>483</v>
       </c>
-      <c r="B81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C81" s="29" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J81" s="10" t="s">
-        <v>481</v>
-      </c>
-      <c r="K81" s="14"/>
+      <c r="K81" s="14" t="s">
+        <v>484</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="11" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B82" s="29" t="n">
-        <v>9791250</v>
+        <v>0</v>
       </c>
       <c r="C82" s="29" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D82" s="29" t="n">
         <v>0</v>
@@ -11076,33 +11084,31 @@
         <v>0</v>
       </c>
       <c r="F82" s="29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G82" s="29" t="n">
         <v>0</v>
       </c>
       <c r="H82" s="29" t="n">
-        <v>979</v>
+        <v>0</v>
       </c>
       <c r="I82" s="29" t="n">
-        <v>55000000</v>
+        <v>0</v>
       </c>
       <c r="J82" s="10" t="s">
-        <v>481</v>
-      </c>
-      <c r="K82" s="14" t="s">
-        <v>485</v>
-      </c>
+        <v>483</v>
+      </c>
+      <c r="K82" s="14"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
         <v>486</v>
       </c>
       <c r="B83" s="29" t="n">
-        <v>0</v>
+        <v>9791250</v>
       </c>
       <c r="C83" s="29" t="n">
-        <v>359800</v>
+        <v>0</v>
       </c>
       <c r="D83" s="29" t="n">
         <v>0</v>
@@ -11111,54 +11117,62 @@
         <v>0</v>
       </c>
       <c r="F83" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G83" s="29" t="n">
         <v>0</v>
       </c>
       <c r="H83" s="29" t="n">
-        <v>0</v>
+        <v>979</v>
       </c>
       <c r="I83" s="29" t="n">
-        <v>0</v>
+        <v>55000000</v>
       </c>
       <c r="J83" s="10" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="K83" s="14" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="s">
+        <v>488</v>
+      </c>
+      <c r="B84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" s="29" t="n">
+        <v>359800</v>
+      </c>
+      <c r="D84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="10" t="s">
+        <v>483</v>
+      </c>
+      <c r="K84" s="14" t="s">
         <v>487</v>
-      </c>
-      <c r="B84" s="26"/>
-      <c r="C84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F84" s="26"/>
-      <c r="G84" s="26"/>
-      <c r="H84" s="26"/>
-      <c r="I84" s="29" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J84" s="10" t="s">
-        <v>488</v>
-      </c>
-      <c r="K84" s="14" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B85" s="26"/>
       <c r="C85" s="29" t="n">
@@ -11177,19 +11191,17 @@
         <v>3000000</v>
       </c>
       <c r="J85" s="10" t="s">
+        <v>490</v>
+      </c>
+      <c r="K85" s="14" t="s">
         <v>491</v>
-      </c>
-      <c r="K85" s="14" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="s">
-        <v>493</v>
-      </c>
-      <c r="B86" s="29" t="n">
-        <v>1650010</v>
-      </c>
+        <v>492</v>
+      </c>
+      <c r="B86" s="26"/>
       <c r="C86" s="29" t="n">
         <v>0</v>
       </c>
@@ -11199,20 +11211,14 @@
       <c r="E86" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F86" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="G86" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H86" s="29" t="n">
-        <v>164</v>
-      </c>
+      <c r="F86" s="26"/>
+      <c r="G86" s="26"/>
+      <c r="H86" s="26"/>
       <c r="I86" s="29" t="n">
         <v>3000000</v>
       </c>
       <c r="J86" s="10" t="s">
-        <v>481</v>
+        <v>493</v>
       </c>
       <c r="K86" s="14" t="s">
         <v>494</v>
@@ -11223,7 +11229,7 @@
         <v>495</v>
       </c>
       <c r="B87" s="29" t="n">
-        <v>1650000</v>
+        <v>1650010</v>
       </c>
       <c r="C87" s="29" t="n">
         <v>0</v>
@@ -11247,7 +11253,7 @@
         <v>3000000</v>
       </c>
       <c r="J87" s="10" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="K87" s="14" t="s">
         <v>496</v>
@@ -11282,7 +11288,7 @@
         <v>3000000</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="K88" s="14" t="s">
         <v>498</v>
@@ -11292,7 +11298,9 @@
       <c r="A89" s="11" t="s">
         <v>499</v>
       </c>
-      <c r="B89" s="26"/>
+      <c r="B89" s="29" t="n">
+        <v>1650000</v>
+      </c>
       <c r="C89" s="29" t="n">
         <v>0</v>
       </c>
@@ -11303,19 +11311,19 @@
         <v>0</v>
       </c>
       <c r="F89" s="29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G89" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H89" s="29" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="I89" s="29" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J89" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="K89" s="14" t="s">
         <v>500</v>
@@ -11325,17 +11333,15 @@
       <c r="A90" s="11" t="s">
         <v>501</v>
       </c>
-      <c r="B90" s="29" t="n">
-        <v>0</v>
-      </c>
+      <c r="B90" s="26"/>
       <c r="C90" s="29" t="n">
-        <v>1710500</v>
+        <v>0</v>
       </c>
       <c r="D90" s="29" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E90" s="29" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F90" s="29" t="n">
         <v>0</v>
@@ -11350,7 +11356,7 @@
         <v>17000000</v>
       </c>
       <c r="J90" s="10" t="s">
-        <v>481</v>
+        <v>493</v>
       </c>
       <c r="K90" s="14" t="s">
         <v>502</v>
@@ -11364,13 +11370,13 @@
         <v>0</v>
       </c>
       <c r="C91" s="29" t="n">
-        <v>1370000</v>
+        <v>1710500</v>
       </c>
       <c r="D91" s="29" t="n">
-        <v>1370000</v>
+        <v>1710000</v>
       </c>
       <c r="E91" s="29" t="n">
-        <v>2130000</v>
+        <v>2640000</v>
       </c>
       <c r="F91" s="29" t="n">
         <v>0</v>
@@ -11385,7 +11391,7 @@
         <v>17000000</v>
       </c>
       <c r="J91" s="10" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="K91" s="14" t="s">
         <v>504</v>
@@ -11398,9 +11404,15 @@
       <c r="B92" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="C92" s="26"/>
-      <c r="D92" s="26"/>
-      <c r="E92" s="26"/>
+      <c r="C92" s="29" t="n">
+        <v>1370000</v>
+      </c>
+      <c r="D92" s="29" t="n">
+        <v>1370000</v>
+      </c>
+      <c r="E92" s="29" t="n">
+        <v>2130000</v>
+      </c>
       <c r="F92" s="29" t="n">
         <v>0</v>
       </c>
@@ -11414,15 +11426,15 @@
         <v>17000000</v>
       </c>
       <c r="J92" s="10" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="K92" s="14" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B93" s="29" t="n">
         <v>0</v>
@@ -11443,15 +11455,15 @@
         <v>17000000</v>
       </c>
       <c r="J93" s="10" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="K93" s="14" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B94" s="29" t="n">
         <v>0</v>
@@ -11472,53 +11484,69 @@
         <v>17000000</v>
       </c>
       <c r="J94" s="10" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="K94" s="14" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B95" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" s="26"/>
+      <c r="D95" s="26"/>
+      <c r="E95" s="26"/>
+      <c r="F95" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" s="29" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J95" s="10" t="s">
+        <v>490</v>
+      </c>
+      <c r="K95" s="14" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="11" t="s">
+        <v>510</v>
+      </c>
+      <c r="B96" s="29" t="n">
         <v>13000000</v>
       </c>
-      <c r="C95" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D95" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E95" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F95" s="26"/>
-      <c r="G95" s="26"/>
-      <c r="H95" s="26"/>
-      <c r="I95" s="29" t="n">
+      <c r="C96" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="26"/>
+      <c r="G96" s="26"/>
+      <c r="H96" s="26"/>
+      <c r="I96" s="29" t="n">
         <v>8000000</v>
       </c>
-      <c r="J95" s="10" t="s">
-        <v>488</v>
-      </c>
-      <c r="K95" s="14" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="11"/>
-      <c r="B96" s="29"/>
-      <c r="C96" s="29"/>
-      <c r="D96" s="29"/>
-      <c r="E96" s="29"/>
-      <c r="F96" s="29"/>
-      <c r="G96" s="29"/>
-      <c r="H96" s="29"/>
-      <c r="I96" s="29"/>
-      <c r="J96" s="10"/>
-      <c r="K96" s="11"/>
+      <c r="J96" s="10" t="s">
+        <v>490</v>
+      </c>
+      <c r="K96" s="14" t="s">
+        <v>511</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="11"/>
@@ -11585,12 +11613,25 @@
       <c r="J101" s="10"/>
       <c r="K101" s="11"/>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="15" t="s">
-        <v>510</v>
-      </c>
-      <c r="I103" s="19" t="n">
-        <f aca="false">SUMIF(J80:J101,"Planned",I80:I101)</f>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="11"/>
+      <c r="B102" s="29"/>
+      <c r="C102" s="29"/>
+      <c r="D102" s="29"/>
+      <c r="E102" s="29"/>
+      <c r="F102" s="29"/>
+      <c r="G102" s="29"/>
+      <c r="H102" s="29"/>
+      <c r="I102" s="29"/>
+      <c r="J102" s="10"/>
+      <c r="K102" s="11"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="15" t="s">
+        <v>512</v>
+      </c>
+      <c r="I104" s="19" t="n">
+        <f aca="false">SUMIF(J81:J102,"Planned",I81:I102)</f>
         <v>20000000</v>
       </c>
     </row>
@@ -11600,22 +11641,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J80:J101">
+  <conditionalFormatting sqref="J81:J102">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J76">
+  <conditionalFormatting sqref="J13:J77">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J76" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J77" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J80:J101" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J81:J102" type="list">
       <formula1>"Planned,If needed,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11646,12 +11687,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11665,56 +11706,56 @@
         <v>382</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G6" s="31"/>
       <c r="H6" s="31"/>
@@ -11725,22 +11766,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
+        <v>528</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>526</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>524</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G7" s="31"/>
       <c r="H7" s="31"/>
@@ -11751,22 +11792,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G8" s="31"/>
       <c r="H8" s="31"/>
@@ -11777,22 +11818,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G9" s="31"/>
       <c r="H9" s="31"/>
@@ -11803,22 +11844,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G10" s="31"/>
       <c r="H10" s="31"/>
@@ -11829,22 +11870,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G11" s="31"/>
       <c r="H11" s="31"/>
@@ -11855,22 +11896,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G12" s="31"/>
       <c r="H12" s="31"/>
@@ -11881,22 +11922,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G13" s="31"/>
       <c r="H13" s="31"/>
@@ -11907,22 +11948,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F14" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G14" s="31"/>
       <c r="H14" s="31"/>
@@ -11933,22 +11974,22 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G15" s="31"/>
       <c r="H15" s="31"/>
@@ -11959,22 +12000,22 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G16" s="31"/>
       <c r="H16" s="31"/>
@@ -11985,20 +12026,20 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G17" s="31"/>
       <c r="H17" s="31"/>
@@ -12009,22 +12050,22 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
+        <v>547</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>545</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>543</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F18" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G18" s="31"/>
       <c r="H18" s="31"/>
@@ -12035,22 +12076,22 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G19" s="31"/>
       <c r="H19" s="31"/>
@@ -12061,22 +12102,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G20" s="31"/>
       <c r="H20" s="31"/>
@@ -12087,24 +12128,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F22" s="31"/>
       <c r="G22" s="31"/>
@@ -12116,16 +12157,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
+        <v>557</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>555</v>
       </c>
-      <c r="B23" s="12" t="s">
-        <v>553</v>
-      </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12138,16 +12179,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
+        <v>558</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>555</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="14" t="s">
         <v>556</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>553</v>
-      </c>
-      <c r="C24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>554</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12160,22 +12201,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E25" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G25" s="31"/>
       <c r="H25" s="31"/>
@@ -12186,19 +12227,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
+        <v>562</v>
+      </c>
+      <c r="B26" s="12" t="s">
         <v>560</v>
       </c>
-      <c r="B26" s="12" t="s">
-        <v>558</v>
-      </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F26" s="31"/>
       <c r="G26" s="31"/>
@@ -12210,16 +12251,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12232,16 +12273,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12254,21 +12295,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12281,16 +12322,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
+        <v>574</v>
+      </c>
+      <c r="B31" s="12" t="s">
         <v>572</v>
       </c>
-      <c r="B31" s="12" t="s">
-        <v>570</v>
-      </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12303,16 +12344,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12325,19 +12366,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F33" s="31"/>
       <c r="G33" s="31"/>
@@ -12349,16 +12390,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12371,16 +12412,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12393,16 +12434,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12415,16 +12456,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12437,16 +12478,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12459,7 +12500,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12496,7 +12537,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12533,7 +12574,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
   </sheetData>
@@ -12577,12 +12618,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12590,10 +12631,10 @@
         <v>237</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12604,13 +12645,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12621,7 +12662,7 @@
         <v>347958315</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12671,7 +12712,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -12679,7 +12720,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12688,11 +12729,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>12290249.5908871</v>
+        <v>12291118.9694948</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12703,19 +12744,19 @@
         <v>246</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12731,7 +12772,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -12757,7 +12798,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -12783,7 +12824,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -12809,7 +12850,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -12834,10 +12875,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -12862,10 +12903,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -12890,10 +12931,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -12918,10 +12959,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -12946,10 +12987,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -12974,10 +13015,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -13003,7 +13044,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13028,10 +13069,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13056,10 +13097,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13084,10 +13125,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
+        <v>624</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>622</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>620</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13115,7 +13156,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13142,10 +13183,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13172,10 +13213,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13202,10 +13243,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13226,10 +13267,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13256,7 +13297,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13284,10 +13325,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13314,7 +13355,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13342,10 +13383,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13372,7 +13413,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13400,10 +13441,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13430,7 +13471,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13458,10 +13499,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13488,7 +13529,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13516,10 +13557,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13546,7 +13587,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13574,10 +13615,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -13604,7 +13645,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -13632,7 +13673,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -13660,7 +13701,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -13688,7 +13729,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -13716,7 +13757,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -13744,7 +13785,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -13772,7 +13813,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -13800,7 +13841,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -13828,7 +13869,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -13856,7 +13897,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -13884,7 +13925,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -13906,7 +13947,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Midday campaigns and dailies
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>538952717.222715</v>
+        <v>544865653.481514</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8763,7 +8763,7 @@
         <v>389</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>12280000</v>
+        <v>12320000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>159500</v>
@@ -8775,10 +8775,10 @@
         <v>13420000</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>221</v>
+        <v>253</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>893</v>
+        <v>909</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>226</v>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>39330000</v>
+        <v>39370000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8839,11 +8839,11 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
-        <v>221</v>
+        <v>253</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>993</v>
+        <v>1009</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
@@ -8889,7 +8889,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>39330000</v>
+        <v>39370000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8905,11 +8905,11 @@
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>221</v>
+        <v>253</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>993</v>
+        <v>1009</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
@@ -10762,7 +10762,7 @@
         <v>474</v>
       </c>
       <c r="B65" s="29" t="n">
-        <v>225800</v>
+        <v>260500</v>
       </c>
       <c r="C65" s="29" t="n">
         <v>0</v>
@@ -10774,10 +10774,10 @@
         <v>0</v>
       </c>
       <c r="F65" s="29" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="G65" s="29" t="n">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="H65" s="29" t="n">
         <v>0</v>
@@ -12064,9 +12064,7 @@
       <c r="E18" s="31" t="s">
         <v>483</v>
       </c>
-      <c r="F18" s="31" t="s">
-        <v>483</v>
-      </c>
+      <c r="F18" s="31"/>
       <c r="G18" s="31"/>
       <c r="H18" s="31"/>
       <c r="I18" s="31"/>
@@ -12147,7 +12145,9 @@
       <c r="E22" s="31" t="s">
         <v>483</v>
       </c>
-      <c r="F22" s="31"/>
+      <c r="F22" s="31" t="s">
+        <v>483</v>
+      </c>
       <c r="G22" s="31"/>
       <c r="H22" s="31"/>
       <c r="I22" s="31"/>
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(F5:F38="Done"))</f>
-        <v>2500000</v>
+        <v>2475000</v>
       </c>
       <c r="G40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(G5:G38="Done"))</f>
@@ -12733,7 +12733,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>12291118.9694948</v>
+        <v>12425966.796927</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Dailies reset at midnight
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1576,7 +1576,7 @@
     <t xml:space="preserve">Dailies</t>
   </si>
   <si>
-    <t xml:space="preserve">Mark each task Done from the dropdown. Objectives reset around 12:30 AM Eastern.</t>
+    <t xml:space="preserve">Mark each task Done from the dropdown. Objectives reset at midnight Eastern.</t>
   </si>
   <si>
     <t xml:space="preserve">Other reward</t>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>544865653.481514</v>
+        <v>545163258.382415</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12733,7 +12733,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>12425966.796927</v>
+        <v>12432753.8426547</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Spider-Man tower cell 20 cleared
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1254" uniqueCount="653">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1259" uniqueCount="655">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -388,7 +388,7 @@
     <t xml:space="preserve">Kingo</t>
   </si>
   <si>
-    <t xml:space="preserve">6 yellow, 4 red stars, 13 of 300 shards</t>
+    <t xml:space="preserve">6 yellow, 5 red stars, 68 of 300 shards</t>
   </si>
   <si>
     <t xml:space="preserve">6 6 6 4</t>
@@ -397,7 +397,7 @@
     <t xml:space="preserve">Spider-Man tower rewards</t>
   </si>
   <si>
-    <t xml:space="preserve">Gear tier 19, all six pieces ready for 20. Tower milestones give his shards, red stars and diamonds</t>
+    <t xml:space="preserve">Gear tier 19, all six pieces ready for 20. Spider-Man tower cell 20 cleared Oct 12. Later milestones give more shards, red stars and diamonds</t>
   </si>
   <si>
     <t xml:space="preserve">Super Skrull</t>
@@ -1384,6 +1384,9 @@
     <t xml:space="preserve">Level 110 gold orb, promo code Oct 11</t>
   </si>
   <si>
+    <t xml:space="preserve">Spider-Man tower milestone 10</t>
+  </si>
+  <si>
     <t xml:space="preserve">Level 110 gold orb, Breaker of Nature level 120</t>
   </si>
   <si>
@@ -1394,6 +1397,9 @@
   </si>
   <si>
     <t xml:space="preserve">Pending claim. Also gives the level 110 training orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cell 20 cleared Oct 12. In current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Basic training orbs</t>
@@ -5843,7 +5849,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>545163258.382415</v>
+        <v>556066703.886892</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8711,7 +8717,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K105"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -8763,7 +8769,7 @@
         <v>389</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>12320000</v>
+        <v>12350000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>159500</v>
@@ -8781,7 +8787,7 @@
         <v>909</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>226</v>
+        <v>726</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8789,31 +8795,31 @@
         <v>390</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
+        <f aca="false">SUMIFS(B13:B78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
         <v>27050000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
+        <f aca="false">SUMIFS(C13:C78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
         <v>3700000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
+        <f aca="false">SUMIFS(D13:D78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
         <v>3886000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
+        <f aca="false">SUMIFS(E13:E78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
         <v>3486000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
+        <f aca="false">SUMIFS(F13:F78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
+        <f aca="false">SUMIFS(G13:G78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H77,$I$13:$I$77,"Yes",$J$13:$J$77,"No")</f>
+        <f aca="false">SUMIFS(H13:H78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
         <v>885</v>
       </c>
     </row>
@@ -8823,7 +8829,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>39370000</v>
+        <v>39400000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8847,7 +8853,7 @@
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1111</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8855,31 +8861,31 @@
         <v>392</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$81:$J$102,"Planned",B81:B102)</f>
+        <f aca="false">SUMIF($J$82:$J$103,"Planned",B82:B103)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$81:$J$102,"Planned",C81:C102)</f>
+        <f aca="false">SUMIF($J$82:$J$103,"Planned",C82:C103)</f>
         <v>0</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$81:$J$102,"Planned",D81:D102)</f>
+        <f aca="false">SUMIF($J$82:$J$103,"Planned",D82:D103)</f>
         <v>0</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$81:$J$102,"Planned",E81:E102)</f>
+        <f aca="false">SUMIF($J$82:$J$103,"Planned",E82:E103)</f>
         <v>0</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$81:$J$102,"Planned",F81:F102)</f>
+        <f aca="false">SUMIF($J$82:$J$103,"Planned",F82:F103)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$81:$J$102,"Planned",G81:G102)</f>
+        <f aca="false">SUMIF($J$82:$J$103,"Planned",G82:G103)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$81:$J$102,"Planned",H81:H102)</f>
+        <f aca="false">SUMIF($J$82:$J$103,"Planned",H82:H103)</f>
         <v>0</v>
       </c>
     </row>
@@ -8889,7 +8895,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>39370000</v>
+        <v>39400000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8913,7 +8919,7 @@
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>1111</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10208,13 +10214,13 @@
         <v>429</v>
       </c>
       <c r="D49" s="29" t="s">
+        <v>450</v>
+      </c>
+      <c r="E49" s="29" t="s">
         <v>399</v>
       </c>
-      <c r="E49" s="29" t="n">
+      <c r="F49" s="29" t="n">
         <v>3300000</v>
-      </c>
-      <c r="F49" s="29" t="n">
-        <v>0</v>
       </c>
       <c r="G49" s="29" t="n">
         <v>0</v>
@@ -10234,7 +10240,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B50" s="29" t="n">
         <v>3300000</v>
@@ -10264,12 +10270,12 @@
         <v>324</v>
       </c>
       <c r="K50" s="14" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B51" s="29" t="n">
         <v>0</v>
@@ -10299,12 +10305,12 @@
         <v>328</v>
       </c>
       <c r="K51" s="14" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="B52" s="29" t="n">
         <v>0</v>
@@ -10325,7 +10331,7 @@
         <v>0</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>32</v>
+        <v>500</v>
       </c>
       <c r="I52" s="10" t="s">
         <v>324</v>
@@ -10360,13 +10366,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="29" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>324</v>
       </c>
       <c r="J53" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K53" s="14" t="s">
         <v>457</v>
@@ -10383,10 +10389,10 @@
         <v>0</v>
       </c>
       <c r="D54" s="29" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="E54" s="29" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="F54" s="29" t="n">
         <v>0</v>
@@ -10412,16 +10418,16 @@
         <v>460</v>
       </c>
       <c r="B55" s="29" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C55" s="29" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="29" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="E55" s="29" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="F55" s="29" t="n">
         <v>0</v>
@@ -10509,12 +10515,12 @@
         <v>328</v>
       </c>
       <c r="K57" s="14" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B58" s="29" t="n">
         <v>750000</v>
@@ -10544,12 +10550,12 @@
         <v>328</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B59" s="29" t="n">
         <v>750000</v>
@@ -10579,12 +10585,12 @@
         <v>328</v>
       </c>
       <c r="K59" s="14" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B60" s="29" t="n">
         <v>750000</v>
@@ -10614,12 +10620,12 @@
         <v>328</v>
       </c>
       <c r="K60" s="14" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B61" s="29" t="n">
         <v>750000</v>
@@ -10649,12 +10655,12 @@
         <v>328</v>
       </c>
       <c r="K61" s="14" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B62" s="29" t="n">
         <v>750000</v>
@@ -10684,18 +10690,18 @@
         <v>328</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B63" s="29" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C63" s="29" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D63" s="29" t="n">
         <v>0</v>
@@ -10719,7 +10725,7 @@
         <v>328</v>
       </c>
       <c r="K63" s="14" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10730,7 +10736,7 @@
         <v>0</v>
       </c>
       <c r="C64" s="29" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D64" s="29" t="n">
         <v>0</v>
@@ -10762,7 +10768,7 @@
         <v>474</v>
       </c>
       <c r="B65" s="29" t="n">
-        <v>260500</v>
+        <v>0</v>
       </c>
       <c r="C65" s="29" t="n">
         <v>0</v>
@@ -10774,10 +10780,10 @@
         <v>0</v>
       </c>
       <c r="F65" s="29" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="G65" s="29" t="n">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="H65" s="29" t="n">
         <v>0</v>
@@ -10786,7 +10792,7 @@
         <v>324</v>
       </c>
       <c r="J65" s="10" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="K65" s="14" t="s">
         <v>475</v>
@@ -10797,7 +10803,7 @@
         <v>476</v>
       </c>
       <c r="B66" s="29" t="n">
-        <v>120000</v>
+        <v>260500</v>
       </c>
       <c r="C66" s="29" t="n">
         <v>0</v>
@@ -10809,10 +10815,10 @@
         <v>0</v>
       </c>
       <c r="F66" s="29" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G66" s="29" t="n">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="H66" s="29" t="n">
         <v>0</v>
@@ -10832,7 +10838,7 @@
         <v>478</v>
       </c>
       <c r="B67" s="29" t="n">
-        <v>375000</v>
+        <v>120000</v>
       </c>
       <c r="C67" s="29" t="n">
         <v>0</v>
@@ -10847,33 +10853,55 @@
         <v>0</v>
       </c>
       <c r="G67" s="29" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="H67" s="29" t="n">
         <v>0</v>
       </c>
       <c r="I67" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="J67" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K67" s="14" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="11"/>
-      <c r="B68" s="29"/>
-      <c r="C68" s="29"/>
-      <c r="D68" s="29"/>
-      <c r="E68" s="29"/>
-      <c r="F68" s="29"/>
-      <c r="G68" s="29"/>
-      <c r="H68" s="29"/>
-      <c r="I68" s="10"/>
-      <c r="J68" s="10"/>
-      <c r="K68" s="11"/>
+      <c r="A68" s="11" t="s">
+        <v>480</v>
+      </c>
+      <c r="B68" s="29" t="n">
+        <v>375000</v>
+      </c>
+      <c r="C68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="J68" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="K68" s="14" t="s">
+        <v>481</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="11"/>
@@ -10992,123 +11020,103 @@
       <c r="J77" s="10"/>
       <c r="K77" s="11"/>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="22" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="B80" s="3" t="s">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="11"/>
+      <c r="B78" s="29"/>
+      <c r="C78" s="29"/>
+      <c r="D78" s="29"/>
+      <c r="E78" s="29"/>
+      <c r="F78" s="29"/>
+      <c r="G78" s="29"/>
+      <c r="H78" s="29"/>
+      <c r="I78" s="10"/>
+      <c r="J78" s="10"/>
+      <c r="K78" s="11"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="22" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="B81" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C81" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="D80" s="3" t="s">
+      <c r="D81" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="E80" s="3" t="s">
+      <c r="E81" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="F80" s="3" t="s">
+      <c r="F81" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="G80" s="3" t="s">
+      <c r="G81" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="H80" s="3" t="s">
+      <c r="H81" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="I80" s="3" t="s">
+      <c r="I81" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J80" s="3" t="s">
+      <c r="J81" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K80" s="3" t="s">
+      <c r="K81" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="11" t="s">
-        <v>482</v>
-      </c>
-      <c r="B81" s="29" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="G81" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H81" s="29" t="n">
-        <v>183</v>
-      </c>
-      <c r="I81" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J81" s="10" t="s">
-        <v>483</v>
-      </c>
-      <c r="K81" s="14" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="B82" s="29" t="n">
+        <v>1837500</v>
+      </c>
+      <c r="C82" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G82" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" s="29" t="n">
+        <v>183</v>
+      </c>
+      <c r="I82" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" s="10" t="s">
         <v>485</v>
       </c>
-      <c r="B82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C82" s="29" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J82" s="10" t="s">
-        <v>483</v>
-      </c>
-      <c r="K82" s="14"/>
+      <c r="K82" s="14" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B83" s="29" t="n">
-        <v>9791250</v>
+        <v>0</v>
       </c>
       <c r="C83" s="29" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D83" s="29" t="n">
         <v>0</v>
@@ -11117,33 +11125,31 @@
         <v>0</v>
       </c>
       <c r="F83" s="29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G83" s="29" t="n">
         <v>0</v>
       </c>
       <c r="H83" s="29" t="n">
-        <v>979</v>
+        <v>0</v>
       </c>
       <c r="I83" s="29" t="n">
-        <v>55000000</v>
+        <v>0</v>
       </c>
       <c r="J83" s="10" t="s">
-        <v>483</v>
-      </c>
-      <c r="K83" s="14" t="s">
-        <v>487</v>
-      </c>
+        <v>485</v>
+      </c>
+      <c r="K83" s="14"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="s">
         <v>488</v>
       </c>
       <c r="B84" s="29" t="n">
-        <v>0</v>
+        <v>9791250</v>
       </c>
       <c r="C84" s="29" t="n">
-        <v>359800</v>
+        <v>0</v>
       </c>
       <c r="D84" s="29" t="n">
         <v>0</v>
@@ -11152,54 +11158,62 @@
         <v>0</v>
       </c>
       <c r="F84" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G84" s="29" t="n">
         <v>0</v>
       </c>
       <c r="H84" s="29" t="n">
-        <v>0</v>
+        <v>979</v>
       </c>
       <c r="I84" s="29" t="n">
-        <v>0</v>
+        <v>55000000</v>
       </c>
       <c r="J84" s="10" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="K84" s="14" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
+        <v>490</v>
+      </c>
+      <c r="B85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C85" s="29" t="n">
+        <v>359800</v>
+      </c>
+      <c r="D85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="10" t="s">
+        <v>485</v>
+      </c>
+      <c r="K85" s="14" t="s">
         <v>489</v>
-      </c>
-      <c r="B85" s="26"/>
-      <c r="C85" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D85" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E85" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F85" s="26"/>
-      <c r="G85" s="26"/>
-      <c r="H85" s="26"/>
-      <c r="I85" s="29" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="J85" s="10" t="s">
-        <v>490</v>
-      </c>
-      <c r="K85" s="14" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B86" s="26"/>
       <c r="C86" s="29" t="n">
@@ -11218,19 +11232,17 @@
         <v>3000000</v>
       </c>
       <c r="J86" s="10" t="s">
+        <v>492</v>
+      </c>
+      <c r="K86" s="14" t="s">
         <v>493</v>
-      </c>
-      <c r="K86" s="14" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>495</v>
-      </c>
-      <c r="B87" s="29" t="n">
-        <v>1650010</v>
-      </c>
+        <v>494</v>
+      </c>
+      <c r="B87" s="26"/>
       <c r="C87" s="29" t="n">
         <v>0</v>
       </c>
@@ -11240,20 +11252,14 @@
       <c r="E87" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F87" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="G87" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H87" s="29" t="n">
-        <v>164</v>
-      </c>
+      <c r="F87" s="26"/>
+      <c r="G87" s="26"/>
+      <c r="H87" s="26"/>
       <c r="I87" s="29" t="n">
         <v>3000000</v>
       </c>
       <c r="J87" s="10" t="s">
-        <v>483</v>
+        <v>495</v>
       </c>
       <c r="K87" s="14" t="s">
         <v>496</v>
@@ -11264,7 +11270,7 @@
         <v>497</v>
       </c>
       <c r="B88" s="29" t="n">
-        <v>1650000</v>
+        <v>1650010</v>
       </c>
       <c r="C88" s="29" t="n">
         <v>0</v>
@@ -11288,7 +11294,7 @@
         <v>3000000</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="K88" s="14" t="s">
         <v>498</v>
@@ -11323,7 +11329,7 @@
         <v>3000000</v>
       </c>
       <c r="J89" s="10" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="K89" s="14" t="s">
         <v>500</v>
@@ -11333,7 +11339,9 @@
       <c r="A90" s="11" t="s">
         <v>501</v>
       </c>
-      <c r="B90" s="26"/>
+      <c r="B90" s="29" t="n">
+        <v>1650000</v>
+      </c>
       <c r="C90" s="29" t="n">
         <v>0</v>
       </c>
@@ -11344,19 +11352,19 @@
         <v>0</v>
       </c>
       <c r="F90" s="29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G90" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H90" s="29" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="I90" s="29" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J90" s="10" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="K90" s="14" t="s">
         <v>502</v>
@@ -11366,17 +11374,15 @@
       <c r="A91" s="11" t="s">
         <v>503</v>
       </c>
-      <c r="B91" s="29" t="n">
-        <v>0</v>
-      </c>
+      <c r="B91" s="26"/>
       <c r="C91" s="29" t="n">
-        <v>1710500</v>
+        <v>0</v>
       </c>
       <c r="D91" s="29" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E91" s="29" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F91" s="29" t="n">
         <v>0</v>
@@ -11391,7 +11397,7 @@
         <v>17000000</v>
       </c>
       <c r="J91" s="10" t="s">
-        <v>483</v>
+        <v>495</v>
       </c>
       <c r="K91" s="14" t="s">
         <v>504</v>
@@ -11405,13 +11411,13 @@
         <v>0</v>
       </c>
       <c r="C92" s="29" t="n">
-        <v>1370000</v>
+        <v>1710500</v>
       </c>
       <c r="D92" s="29" t="n">
-        <v>1370000</v>
+        <v>1710000</v>
       </c>
       <c r="E92" s="29" t="n">
-        <v>2130000</v>
+        <v>2640000</v>
       </c>
       <c r="F92" s="29" t="n">
         <v>0</v>
@@ -11426,7 +11432,7 @@
         <v>17000000</v>
       </c>
       <c r="J92" s="10" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="K92" s="14" t="s">
         <v>506</v>
@@ -11439,9 +11445,15 @@
       <c r="B93" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="C93" s="26"/>
-      <c r="D93" s="26"/>
-      <c r="E93" s="26"/>
+      <c r="C93" s="29" t="n">
+        <v>1370000</v>
+      </c>
+      <c r="D93" s="29" t="n">
+        <v>1370000</v>
+      </c>
+      <c r="E93" s="29" t="n">
+        <v>2130000</v>
+      </c>
       <c r="F93" s="29" t="n">
         <v>0</v>
       </c>
@@ -11455,15 +11467,15 @@
         <v>17000000</v>
       </c>
       <c r="J93" s="10" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="K93" s="14" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B94" s="29" t="n">
         <v>0</v>
@@ -11484,15 +11496,15 @@
         <v>17000000</v>
       </c>
       <c r="J94" s="10" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="K94" s="14" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B95" s="29" t="n">
         <v>0</v>
@@ -11513,53 +11525,69 @@
         <v>17000000</v>
       </c>
       <c r="J95" s="10" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="K95" s="14" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="11" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B96" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" s="26"/>
+      <c r="D96" s="26"/>
+      <c r="E96" s="26"/>
+      <c r="F96" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" s="29" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J96" s="10" t="s">
+        <v>492</v>
+      </c>
+      <c r="K96" s="14" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="11" t="s">
+        <v>512</v>
+      </c>
+      <c r="B97" s="29" t="n">
         <v>13000000</v>
       </c>
-      <c r="C96" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D96" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E96" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F96" s="26"/>
-      <c r="G96" s="26"/>
-      <c r="H96" s="26"/>
-      <c r="I96" s="29" t="n">
+      <c r="C97" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" s="26"/>
+      <c r="G97" s="26"/>
+      <c r="H97" s="26"/>
+      <c r="I97" s="29" t="n">
         <v>8000000</v>
       </c>
-      <c r="J96" s="10" t="s">
-        <v>490</v>
-      </c>
-      <c r="K96" s="14" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="11"/>
-      <c r="B97" s="29"/>
-      <c r="C97" s="29"/>
-      <c r="D97" s="29"/>
-      <c r="E97" s="29"/>
-      <c r="F97" s="29"/>
-      <c r="G97" s="29"/>
-      <c r="H97" s="29"/>
-      <c r="I97" s="29"/>
-      <c r="J97" s="10"/>
-      <c r="K97" s="11"/>
+      <c r="J97" s="10" t="s">
+        <v>492</v>
+      </c>
+      <c r="K97" s="14" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="11"/>
@@ -11626,12 +11654,25 @@
       <c r="J102" s="10"/>
       <c r="K102" s="11"/>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="15" t="s">
-        <v>512</v>
-      </c>
-      <c r="I104" s="19" t="n">
-        <f aca="false">SUMIF(J81:J102,"Planned",I81:I102)</f>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="11"/>
+      <c r="B103" s="29"/>
+      <c r="C103" s="29"/>
+      <c r="D103" s="29"/>
+      <c r="E103" s="29"/>
+      <c r="F103" s="29"/>
+      <c r="G103" s="29"/>
+      <c r="H103" s="29"/>
+      <c r="I103" s="29"/>
+      <c r="J103" s="10"/>
+      <c r="K103" s="11"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="15" t="s">
+        <v>514</v>
+      </c>
+      <c r="I105" s="19" t="n">
+        <f aca="false">SUMIF(J82:J103,"Planned",I82:I103)</f>
         <v>20000000</v>
       </c>
     </row>
@@ -11641,22 +11682,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J81:J102">
+  <conditionalFormatting sqref="J82:J103">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J77">
+  <conditionalFormatting sqref="J13:J78">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J77" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J78" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J81:J102" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J82:J103" type="list">
       <formula1>"Planned,If needed,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11687,12 +11728,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11706,56 +11747,56 @@
         <v>382</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G6" s="31"/>
       <c r="H6" s="31"/>
@@ -11766,22 +11807,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>528</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>526</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G7" s="31"/>
       <c r="H7" s="31"/>
@@ -11792,22 +11833,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G8" s="31"/>
       <c r="H8" s="31"/>
@@ -11818,22 +11859,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G9" s="31"/>
       <c r="H9" s="31"/>
@@ -11844,22 +11885,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G10" s="31"/>
       <c r="H10" s="31"/>
@@ -11870,22 +11911,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G11" s="31"/>
       <c r="H11" s="31"/>
@@ -11896,22 +11937,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G12" s="31"/>
       <c r="H12" s="31"/>
@@ -11922,22 +11963,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G13" s="31"/>
       <c r="H13" s="31"/>
@@ -11948,22 +11989,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F14" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G14" s="31"/>
       <c r="H14" s="31"/>
@@ -11974,22 +12015,22 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G15" s="31"/>
       <c r="H15" s="31"/>
@@ -12000,22 +12041,22 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G16" s="31"/>
       <c r="H16" s="31"/>
@@ -12026,20 +12067,20 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G17" s="31"/>
       <c r="H17" s="31"/>
@@ -12050,19 +12091,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
+        <v>549</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>547</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>545</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F18" s="31"/>
       <c r="G18" s="31"/>
@@ -12074,22 +12115,22 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G19" s="31"/>
       <c r="H19" s="31"/>
@@ -12100,22 +12141,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G20" s="31"/>
       <c r="H20" s="31"/>
@@ -12126,27 +12167,27 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F22" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G22" s="31"/>
       <c r="H22" s="31"/>
@@ -12157,16 +12198,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
+        <v>559</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>557</v>
       </c>
-      <c r="B23" s="12" t="s">
-        <v>555</v>
-      </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12179,16 +12220,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
+        <v>560</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>557</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="14" t="s">
         <v>558</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>555</v>
-      </c>
-      <c r="C24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>556</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12201,22 +12242,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="E25" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G25" s="31"/>
       <c r="H25" s="31"/>
@@ -12227,19 +12268,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
+        <v>564</v>
+      </c>
+      <c r="B26" s="12" t="s">
         <v>562</v>
       </c>
-      <c r="B26" s="12" t="s">
-        <v>560</v>
-      </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F26" s="31"/>
       <c r="G26" s="31"/>
@@ -12251,16 +12292,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12273,16 +12314,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12295,21 +12336,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12322,16 +12363,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
+        <v>576</v>
+      </c>
+      <c r="B31" s="12" t="s">
         <v>574</v>
       </c>
-      <c r="B31" s="12" t="s">
-        <v>572</v>
-      </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12344,16 +12385,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12366,19 +12407,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F33" s="31"/>
       <c r="G33" s="31"/>
@@ -12390,16 +12431,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12412,16 +12453,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12434,16 +12475,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12456,16 +12497,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12478,16 +12519,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12500,7 +12541,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12537,7 +12578,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12574,7 +12615,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
   </sheetData>
@@ -12618,12 +12659,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12631,10 +12672,10 @@
         <v>237</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12645,13 +12686,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12662,7 +12703,7 @@
         <v>347958315</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12712,7 +12753,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -12720,7 +12761,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12729,11 +12770,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>12432753.8426547</v>
+        <v>12681413.0296129</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12744,19 +12785,19 @@
         <v>246</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12772,7 +12813,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -12798,7 +12839,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -12824,7 +12865,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -12850,7 +12891,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -12875,10 +12916,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -12903,10 +12944,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -12931,10 +12972,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -12959,10 +13000,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -12987,10 +13028,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -13015,10 +13056,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -13044,7 +13085,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13069,10 +13110,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13097,10 +13138,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13125,10 +13166,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
+        <v>626</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>624</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>622</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13156,7 +13197,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13183,10 +13224,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13213,10 +13254,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13243,10 +13284,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13267,10 +13308,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13297,7 +13338,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13325,10 +13366,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13355,7 +13396,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13383,10 +13424,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13413,7 +13454,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13441,10 +13482,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13471,7 +13512,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13499,10 +13540,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13529,7 +13570,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13557,10 +13598,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13587,7 +13628,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13615,10 +13656,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -13645,7 +13686,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -13673,7 +13714,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -13701,7 +13742,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -13729,7 +13770,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -13757,7 +13798,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -13785,7 +13826,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -13813,7 +13854,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -13841,7 +13882,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -13869,7 +13910,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -13897,7 +13938,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -13925,7 +13966,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -13947,7 +13988,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Battle pass 100, Founding Force ions, Julia iso planned
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1259" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="659">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -208,10 +208,10 @@
     <t xml:space="preserve">Control</t>
   </si>
   <si>
-    <t xml:space="preserve">Psionic Webs to level 7, then Arachnid Swing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T4 ability materials</t>
+    <t xml:space="preserve">Iso-8 to T3 L5 now; Psionic Webs to level 7 with Scorpion event T4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purple ions, T4 ability materials</t>
   </si>
   <si>
     <t xml:space="preserve">Psionic Webs needs 240 T4s, Arachnid Swing 180. Have 47. Iso T3 L5 needs ion 1 from Founding Force</t>
@@ -1315,7 +1315,7 @@
     <t xml:space="preserve">Founding Force milestone 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Needs the battle pass level 100 token</t>
+    <t xml:space="preserve">Battle pass level 100 reached Oct 12</t>
   </si>
   <si>
     <t xml:space="preserve">Iso Fest milestone 15</t>
@@ -1330,6 +1330,9 @@
     <t xml:space="preserve">Iso Fest milestone 17</t>
   </si>
   <si>
+    <t xml:space="preserve">Reached Oct 12</t>
+  </si>
+  <si>
     <t xml:space="preserve">VisionQuest level 30</t>
   </si>
   <si>
@@ -1384,6 +1387,9 @@
     <t xml:space="preserve">Level 110 gold orb, promo code Oct 11</t>
   </si>
   <si>
+    <t xml:space="preserve">Moonlit Sigils store</t>
+  </si>
+  <si>
     <t xml:space="preserve">Spider-Man tower milestone 10</t>
   </si>
   <si>
@@ -1402,6 +1408,9 @@
     <t xml:space="preserve">Cell 20 cleared Oct 12. In current stock</t>
   </si>
   <si>
+    <t xml:space="preserve">Oct 12. In current stock</t>
+  </si>
+  <si>
     <t xml:space="preserve">Basic training orbs</t>
   </si>
   <si>
@@ -1565,6 +1574,9 @@
   </si>
   <si>
     <t xml:space="preserve">Spider-Woman (Julia) Iso-8 to T3 level 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimate from Hulk. Confirm with Quick Upgrade</t>
   </si>
   <si>
     <t xml:space="preserve">Rachel Cole-Alves Iso-8 to T3 level 5</t>
@@ -3092,7 +3104,7 @@
         <v>58</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>0</v>
+        <v>17000000</v>
       </c>
       <c r="J13" s="7" t="s">
         <v>59</v>
@@ -5783,14 +5795,14 @@
         <v>239</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>751302650</v>
+        <v>755302650</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>240</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6024802650</v>
+        <v>6028802650</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5831,7 +5843,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>73697350</v>
+        <v>69697350</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5840,7 +5852,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3373697350</v>
+        <v>3369697350</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5849,7 +5861,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>563356520.438897</v>
+        <v>564077484.596066</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6725,7 +6737,7 @@
       <c r="D61" s="11"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>73697350</v>
+        <v>69697350</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>182</v>
@@ -6744,7 +6756,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>148697350</v>
+        <v>144697350</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>182</v>
@@ -6763,7 +6775,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>223697350</v>
+        <v>219697350</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>182</v>
@@ -6782,7 +6794,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>298697350</v>
+        <v>294697350</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>182</v>
@@ -6801,7 +6813,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>373697350</v>
+        <v>369697350</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>182</v>
@@ -6820,7 +6832,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>448697350</v>
+        <v>444697350</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>182</v>
@@ -6839,7 +6851,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>598697350</v>
+        <v>594697350</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>182</v>
@@ -6858,7 +6870,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>748697350</v>
+        <v>744697350</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>182</v>
@@ -6877,7 +6889,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>898697350</v>
+        <v>894697350</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>182</v>
@@ -6896,7 +6908,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1123697350</v>
+        <v>1119697350</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>182</v>
@@ -6915,7 +6927,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1498697350</v>
+        <v>1494697350</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>182</v>
@@ -6934,7 +6946,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1873697350</v>
+        <v>1869697350</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>182</v>
@@ -6953,7 +6965,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2248697350</v>
+        <v>2244697350</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>182</v>
@@ -6972,7 +6984,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2623697350</v>
+        <v>2619697350</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>182</v>
@@ -6991,7 +7003,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2998697350</v>
+        <v>2994697350</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>182</v>
@@ -7010,7 +7022,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3373697350</v>
+        <v>3369697350</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>182</v>
@@ -8717,7 +8729,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -8769,16 +8781,16 @@
         <v>389</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>12350000</v>
+        <v>22850000</v>
       </c>
       <c r="C5" s="26" t="n">
-        <v>159500</v>
+        <v>3159500</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>2590000</v>
+        <v>6990000</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>13420000</v>
+        <v>17920000</v>
       </c>
       <c r="F5" s="26" t="n">
         <v>253</v>
@@ -8787,7 +8799,7 @@
         <v>909</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>726</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8795,32 +8807,32 @@
         <v>390</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
-        <v>27050000</v>
+        <f aca="false">SUMIFS(B13:B79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <v>16550000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
-        <v>3700000</v>
+        <f aca="false">SUMIFS(C13:C79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <v>700000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
-        <v>3886000</v>
+        <f aca="false">SUMIFS(D13:D79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <v>886000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
-        <v>3486000</v>
+        <f aca="false">SUMIFS(E13:E79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <v>886000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
+        <f aca="false">SUMIFS(F13:F79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
+        <f aca="false">SUMIFS(G13:G79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H78,$I$13:$I$78,"Yes",$J$13:$J$78,"No")</f>
-        <v>885</v>
+        <f aca="false">SUMIFS(H13:H79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8837,11 +8849,11 @@
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>6476000</v>
+        <v>7876000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>16906000</v>
+        <v>18806000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -8853,7 +8865,7 @@
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1611</v>
+        <v>1811</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8861,31 +8873,31 @@
         <v>392</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$82:$J$103,"Planned",B82:B103)</f>
+        <f aca="false">SUMIF($J$83:$J$104,"Planned",B83:B104)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$82:$J$103,"Planned",C82:C103)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$83:$J$104,"Planned",C83:C104)</f>
+        <v>1710000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$82:$J$103,"Planned",D82:D103)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$83:$J$104,"Planned",D83:D104)</f>
+        <v>1710000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$82:$J$103,"Planned",E82:E103)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$83:$J$104,"Planned",E83:E104)</f>
+        <v>2640000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$82:$J$103,"Planned",F82:F103)</f>
+        <f aca="false">SUMIF($J$83:$J$104,"Planned",F83:F104)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$82:$J$103,"Planned",G82:G103)</f>
+        <f aca="false">SUMIF($J$83:$J$104,"Planned",G83:G104)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$82:$J$103,"Planned",H82:H103)</f>
+        <f aca="false">SUMIF($J$83:$J$104,"Planned",H83:H104)</f>
         <v>0</v>
       </c>
     </row>
@@ -8899,15 +8911,15 @@
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>3859500</v>
+        <v>2149500</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>6476000</v>
+        <v>6166000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>16906000</v>
+        <v>16166000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -8919,7 +8931,7 @@
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>1611</v>
+        <v>1811</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9680,7 +9692,7 @@
         <v>324</v>
       </c>
       <c r="J33" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K33" s="14"/>
     </row>
@@ -9713,7 +9725,7 @@
         <v>324</v>
       </c>
       <c r="J34" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K34" s="14"/>
     </row>
@@ -9746,7 +9758,7 @@
         <v>324</v>
       </c>
       <c r="J35" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K35" s="14"/>
     </row>
@@ -9779,7 +9791,7 @@
         <v>324</v>
       </c>
       <c r="J36" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K36" s="14" t="s">
         <v>427</v>
@@ -9881,16 +9893,18 @@
         <v>0</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="J39" s="10" t="s">
-        <v>328</v>
-      </c>
-      <c r="K39" s="14"/>
+        <v>324</v>
+      </c>
+      <c r="K39" s="14" t="s">
+        <v>432</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B40" s="29" t="n">
         <v>0</v>
@@ -9920,12 +9934,12 @@
         <v>328</v>
       </c>
       <c r="K40" s="14" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B41" s="29" t="n">
         <v>0</v>
@@ -9955,12 +9969,12 @@
         <v>328</v>
       </c>
       <c r="K41" s="14" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B42" s="29" t="n">
         <v>0</v>
@@ -9990,12 +10004,12 @@
         <v>328</v>
       </c>
       <c r="K42" s="14" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B43" s="29" t="n">
         <v>0</v>
@@ -10025,12 +10039,12 @@
         <v>328</v>
       </c>
       <c r="K43" s="14" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B44" s="29" t="n">
         <v>0</v>
@@ -10060,12 +10074,12 @@
         <v>328</v>
       </c>
       <c r="K44" s="14" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B45" s="29" t="n">
         <v>0</v>
@@ -10095,12 +10109,12 @@
         <v>328</v>
       </c>
       <c r="K45" s="14" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B46" s="29" t="n">
         <v>0</v>
@@ -10130,12 +10144,12 @@
         <v>328</v>
       </c>
       <c r="K46" s="14" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B47" s="29" t="n">
         <v>900000</v>
@@ -10165,12 +10179,12 @@
         <v>328</v>
       </c>
       <c r="K47" s="14" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B48" s="29" t="n">
         <v>0</v>
@@ -10200,12 +10214,12 @@
         <v>328</v>
       </c>
       <c r="K48" s="14" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B49" s="29" t="s">
         <v>401</v>
@@ -10214,33 +10228,33 @@
         <v>429</v>
       </c>
       <c r="D49" s="29" t="s">
-        <v>450</v>
+        <v>431</v>
       </c>
       <c r="E49" s="29" t="s">
-        <v>399</v>
-      </c>
-      <c r="F49" s="29" t="n">
-        <v>3300000</v>
-      </c>
-      <c r="G49" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" s="10" t="n">
-        <v>0</v>
+        <v>426</v>
+      </c>
+      <c r="F49" s="29" t="s">
+        <v>423</v>
+      </c>
+      <c r="G49" s="29" t="s">
+        <v>424</v>
+      </c>
+      <c r="H49" s="29" t="s">
+        <v>425</v>
+      </c>
+      <c r="I49" s="10" t="s">
+        <v>451</v>
       </c>
       <c r="J49" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="K49" s="14" t="n">
-        <v>0</v>
+      <c r="K49" s="14" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B50" s="29" t="n">
         <v>3300000</v>
@@ -10270,12 +10284,12 @@
         <v>324</v>
       </c>
       <c r="K50" s="14" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B51" s="29" t="n">
         <v>0</v>
@@ -10305,12 +10319,12 @@
         <v>328</v>
       </c>
       <c r="K51" s="14" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B52" s="29" t="n">
         <v>0</v>
@@ -10340,12 +10354,12 @@
         <v>324</v>
       </c>
       <c r="K52" s="14" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="B53" s="29" t="n">
         <v>0</v>
@@ -10366,7 +10380,7 @@
         <v>0</v>
       </c>
       <c r="H53" s="29" t="n">
-        <v>32</v>
+        <v>200</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>324</v>
@@ -10375,12 +10389,12 @@
         <v>324</v>
       </c>
       <c r="K53" s="14" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B54" s="29" t="n">
         <v>0</v>
@@ -10401,21 +10415,21 @@
         <v>0</v>
       </c>
       <c r="H54" s="29" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I54" s="10" t="s">
         <v>324</v>
       </c>
       <c r="J54" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="K54" s="14" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B55" s="29" t="n">
         <v>0</v>
@@ -10424,10 +10438,10 @@
         <v>0</v>
       </c>
       <c r="D55" s="29" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="E55" s="29" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="F55" s="29" t="n">
         <v>0</v>
@@ -10445,24 +10459,24 @@
         <v>328</v>
       </c>
       <c r="K55" s="14" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B56" s="29" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C56" s="29" t="n">
         <v>0</v>
       </c>
       <c r="D56" s="29" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="E56" s="29" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="F56" s="29" t="n">
         <v>0</v>
@@ -10480,12 +10494,12 @@
         <v>328</v>
       </c>
       <c r="K56" s="14" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B57" s="29" t="n">
         <v>750000</v>
@@ -10515,12 +10529,12 @@
         <v>328</v>
       </c>
       <c r="K57" s="14" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B58" s="29" t="n">
         <v>750000</v>
@@ -10550,12 +10564,12 @@
         <v>328</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B59" s="29" t="n">
         <v>750000</v>
@@ -10585,12 +10599,12 @@
         <v>328</v>
       </c>
       <c r="K59" s="14" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B60" s="29" t="n">
         <v>750000</v>
@@ -10620,12 +10634,12 @@
         <v>328</v>
       </c>
       <c r="K60" s="14" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B61" s="29" t="n">
         <v>750000</v>
@@ -10655,12 +10669,12 @@
         <v>328</v>
       </c>
       <c r="K61" s="14" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B62" s="29" t="n">
         <v>750000</v>
@@ -10690,12 +10704,12 @@
         <v>328</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B63" s="29" t="n">
         <v>750000</v>
@@ -10725,18 +10739,18 @@
         <v>328</v>
       </c>
       <c r="K63" s="14" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="11" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B64" s="29" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C64" s="29" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D64" s="29" t="n">
         <v>0</v>
@@ -10760,18 +10774,18 @@
         <v>328</v>
       </c>
       <c r="K64" s="14" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B65" s="29" t="n">
         <v>0</v>
       </c>
       <c r="C65" s="29" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D65" s="29" t="n">
         <v>0</v>
@@ -10795,15 +10809,15 @@
         <v>328</v>
       </c>
       <c r="K65" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B66" s="29" t="n">
-        <v>260500</v>
+        <v>0</v>
       </c>
       <c r="C66" s="29" t="n">
         <v>0</v>
@@ -10815,10 +10829,10 @@
         <v>0</v>
       </c>
       <c r="F66" s="29" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="G66" s="29" t="n">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="H66" s="29" t="n">
         <v>0</v>
@@ -10827,18 +10841,18 @@
         <v>324</v>
       </c>
       <c r="J66" s="10" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="K66" s="14" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B67" s="29" t="n">
-        <v>120000</v>
+        <v>260500</v>
       </c>
       <c r="C67" s="29" t="n">
         <v>0</v>
@@ -10850,10 +10864,10 @@
         <v>0</v>
       </c>
       <c r="F67" s="29" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G67" s="29" t="n">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="H67" s="29" t="n">
         <v>0</v>
@@ -10865,56 +10879,78 @@
         <v>324</v>
       </c>
       <c r="K67" s="14" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B68" s="29" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="29" t="n">
+        <v>64</v>
+      </c>
+      <c r="H68" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="J68" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="K68" s="14" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="11" t="s">
+        <v>483</v>
+      </c>
+      <c r="B69" s="29" t="n">
         <v>375000</v>
       </c>
-      <c r="C68" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F68" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H68" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" s="10" t="s">
+      <c r="C69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="J68" s="10" t="s">
+      <c r="J69" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="K68" s="14" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="11"/>
-      <c r="B69" s="29"/>
-      <c r="C69" s="29"/>
-      <c r="D69" s="29"/>
-      <c r="E69" s="29"/>
-      <c r="F69" s="29"/>
-      <c r="G69" s="29"/>
-      <c r="H69" s="29"/>
-      <c r="I69" s="10"/>
-      <c r="J69" s="10"/>
-      <c r="K69" s="11"/>
+      <c r="K69" s="14" t="s">
+        <v>484</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="11"/>
@@ -11033,79 +11069,57 @@
       <c r="J78" s="10"/>
       <c r="K78" s="11"/>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="22" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="3" t="s">
-        <v>483</v>
-      </c>
-      <c r="B81" s="3" t="s">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="11"/>
+      <c r="B79" s="29"/>
+      <c r="C79" s="29"/>
+      <c r="D79" s="29"/>
+      <c r="E79" s="29"/>
+      <c r="F79" s="29"/>
+      <c r="G79" s="29"/>
+      <c r="H79" s="29"/>
+      <c r="I79" s="10"/>
+      <c r="J79" s="10"/>
+      <c r="K79" s="11"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="22" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="B82" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="C81" s="3" t="s">
+      <c r="C82" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="D81" s="3" t="s">
+      <c r="D82" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="E81" s="3" t="s">
+      <c r="E82" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="F81" s="3" t="s">
+      <c r="F82" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="G81" s="3" t="s">
+      <c r="G82" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="H81" s="3" t="s">
+      <c r="H82" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="I81" s="3" t="s">
+      <c r="I82" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J81" s="3" t="s">
+      <c r="J82" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K81" s="3" t="s">
+      <c r="K82" s="3" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="11" t="s">
-        <v>484</v>
-      </c>
-      <c r="B82" s="29" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F82" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="G82" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H82" s="29" t="n">
-        <v>183</v>
-      </c>
-      <c r="I82" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J82" s="10" t="s">
-        <v>485</v>
-      </c>
-      <c r="K82" s="14" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11113,10 +11127,10 @@
         <v>487</v>
       </c>
       <c r="B83" s="29" t="n">
-        <v>0</v>
+        <v>1837500</v>
       </c>
       <c r="C83" s="29" t="n">
-        <v>359800</v>
+        <v>0</v>
       </c>
       <c r="D83" s="29" t="n">
         <v>0</v>
@@ -11125,66 +11139,66 @@
         <v>0</v>
       </c>
       <c r="F83" s="29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G83" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H83" s="29" t="n">
-        <v>0</v>
+        <v>183</v>
       </c>
       <c r="I83" s="29" t="n">
         <v>0</v>
       </c>
       <c r="J83" s="10" t="s">
-        <v>485</v>
-      </c>
-      <c r="K83" s="14"/>
+        <v>488</v>
+      </c>
+      <c r="K83" s="14" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="s">
+        <v>490</v>
+      </c>
+      <c r="B84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" s="29" t="n">
+        <v>359800</v>
+      </c>
+      <c r="D84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="10" t="s">
         <v>488</v>
       </c>
-      <c r="B84" s="29" t="n">
-        <v>9791250</v>
-      </c>
-      <c r="C84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F84" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="G84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H84" s="29" t="n">
-        <v>979</v>
-      </c>
-      <c r="I84" s="29" t="n">
-        <v>55000000</v>
-      </c>
-      <c r="J84" s="10" t="s">
-        <v>485</v>
-      </c>
-      <c r="K84" s="14" t="s">
-        <v>489</v>
-      </c>
+      <c r="K84" s="14"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B85" s="29" t="n">
-        <v>0</v>
+        <v>9791250</v>
       </c>
       <c r="C85" s="29" t="n">
-        <v>359800</v>
+        <v>0</v>
       </c>
       <c r="D85" s="29" t="n">
         <v>0</v>
@@ -11193,31 +11207,33 @@
         <v>0</v>
       </c>
       <c r="F85" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G85" s="29" t="n">
         <v>0</v>
       </c>
       <c r="H85" s="29" t="n">
-        <v>0</v>
+        <v>979</v>
       </c>
       <c r="I85" s="29" t="n">
-        <v>0</v>
+        <v>55000000</v>
       </c>
       <c r="J85" s="10" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="K85" s="14" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="s">
-        <v>491</v>
-      </c>
-      <c r="B86" s="26"/>
+        <v>493</v>
+      </c>
+      <c r="B86" s="29" t="n">
+        <v>0</v>
+      </c>
       <c r="C86" s="29" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D86" s="29" t="n">
         <v>0</v>
@@ -11225,17 +11241,23 @@
       <c r="E86" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F86" s="26"/>
-      <c r="G86" s="26"/>
-      <c r="H86" s="26"/>
+      <c r="F86" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="29" t="n">
+        <v>0</v>
+      </c>
       <c r="I86" s="29" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J86" s="10" t="s">
+        <v>488</v>
+      </c>
+      <c r="K86" s="14" t="s">
         <v>492</v>
-      </c>
-      <c r="K86" s="14" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11269,9 +11291,7 @@
       <c r="A88" s="11" t="s">
         <v>497</v>
       </c>
-      <c r="B88" s="29" t="n">
-        <v>1650010</v>
-      </c>
+      <c r="B88" s="26"/>
       <c r="C88" s="29" t="n">
         <v>0</v>
       </c>
@@ -11281,31 +11301,25 @@
       <c r="E88" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F88" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="G88" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H88" s="29" t="n">
-        <v>164</v>
-      </c>
+      <c r="F88" s="26"/>
+      <c r="G88" s="26"/>
+      <c r="H88" s="26"/>
       <c r="I88" s="29" t="n">
         <v>3000000</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="K88" s="14" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B89" s="29" t="n">
-        <v>1650000</v>
+        <v>1650010</v>
       </c>
       <c r="C89" s="29" t="n">
         <v>0</v>
@@ -11329,15 +11343,15 @@
         <v>3000000</v>
       </c>
       <c r="J89" s="10" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="K89" s="14" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="11" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B90" s="29" t="n">
         <v>1650000</v>
@@ -11364,17 +11378,19 @@
         <v>3000000</v>
       </c>
       <c r="J90" s="10" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="K90" s="14" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>503</v>
-      </c>
-      <c r="B91" s="26"/>
+        <v>504</v>
+      </c>
+      <c r="B91" s="29" t="n">
+        <v>1650000</v>
+      </c>
       <c r="C91" s="29" t="n">
         <v>0</v>
       </c>
@@ -11385,39 +11401,37 @@
         <v>0</v>
       </c>
       <c r="F91" s="29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G91" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H91" s="29" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="I91" s="29" t="n">
-        <v>17000000</v>
+        <v>3000000</v>
       </c>
       <c r="J91" s="10" t="s">
         <v>495</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="11" t="s">
-        <v>505</v>
-      </c>
-      <c r="B92" s="29" t="n">
-        <v>0</v>
-      </c>
+        <v>506</v>
+      </c>
+      <c r="B92" s="26"/>
       <c r="C92" s="29" t="n">
-        <v>1710500</v>
+        <v>0</v>
       </c>
       <c r="D92" s="29" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E92" s="29" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F92" s="29" t="n">
         <v>0</v>
@@ -11432,27 +11446,27 @@
         <v>17000000</v>
       </c>
       <c r="J92" s="10" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="K92" s="14" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B93" s="29" t="n">
         <v>0</v>
       </c>
       <c r="C93" s="29" t="n">
-        <v>1370000</v>
+        <v>1710500</v>
       </c>
       <c r="D93" s="29" t="n">
-        <v>1370000</v>
+        <v>1710000</v>
       </c>
       <c r="E93" s="29" t="n">
-        <v>2130000</v>
+        <v>2640000</v>
       </c>
       <c r="F93" s="29" t="n">
         <v>0</v>
@@ -11467,22 +11481,28 @@
         <v>17000000</v>
       </c>
       <c r="J93" s="10" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="K93" s="14" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B94" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="C94" s="26"/>
-      <c r="D94" s="26"/>
-      <c r="E94" s="26"/>
+      <c r="C94" s="29" t="n">
+        <v>1370000</v>
+      </c>
+      <c r="D94" s="29" t="n">
+        <v>1370000</v>
+      </c>
+      <c r="E94" s="29" t="n">
+        <v>2130000</v>
+      </c>
       <c r="F94" s="29" t="n">
         <v>0</v>
       </c>
@@ -11496,15 +11516,15 @@
         <v>17000000</v>
       </c>
       <c r="J94" s="10" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="K94" s="14" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B95" s="29" t="n">
         <v>0</v>
@@ -11525,22 +11545,28 @@
         <v>17000000</v>
       </c>
       <c r="J95" s="10" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="K95" s="14" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="11" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B96" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="C96" s="26"/>
-      <c r="D96" s="26"/>
-      <c r="E96" s="26"/>
+      <c r="C96" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D96" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E96" s="29" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F96" s="29" t="n">
         <v>0</v>
       </c>
@@ -11554,53 +11580,69 @@
         <v>17000000</v>
       </c>
       <c r="J96" s="10" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="K96" s="14" t="s">
-        <v>504</v>
+        <v>514</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B97" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" s="26"/>
+      <c r="D97" s="26"/>
+      <c r="E97" s="26"/>
+      <c r="F97" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" s="29" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J97" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="K97" s="14" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="11" t="s">
+        <v>516</v>
+      </c>
+      <c r="B98" s="29" t="n">
         <v>13000000</v>
       </c>
-      <c r="C97" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D97" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E97" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F97" s="26"/>
-      <c r="G97" s="26"/>
-      <c r="H97" s="26"/>
-      <c r="I97" s="29" t="n">
+      <c r="C98" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" s="26"/>
+      <c r="G98" s="26"/>
+      <c r="H98" s="26"/>
+      <c r="I98" s="29" t="n">
         <v>8000000</v>
       </c>
-      <c r="J97" s="10" t="s">
-        <v>492</v>
-      </c>
-      <c r="K97" s="14" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="11"/>
-      <c r="B98" s="29"/>
-      <c r="C98" s="29"/>
-      <c r="D98" s="29"/>
-      <c r="E98" s="29"/>
-      <c r="F98" s="29"/>
-      <c r="G98" s="29"/>
-      <c r="H98" s="29"/>
-      <c r="I98" s="29"/>
-      <c r="J98" s="10"/>
-      <c r="K98" s="11"/>
+      <c r="J98" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="K98" s="14" t="s">
+        <v>517</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="11"/>
@@ -11667,13 +11709,26 @@
       <c r="J103" s="10"/>
       <c r="K103" s="11"/>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="15" t="s">
-        <v>514</v>
-      </c>
-      <c r="I105" s="19" t="n">
-        <f aca="false">SUMIF(J82:J103,"Planned",I82:I103)</f>
-        <v>20000000</v>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="11"/>
+      <c r="B104" s="29"/>
+      <c r="C104" s="29"/>
+      <c r="D104" s="29"/>
+      <c r="E104" s="29"/>
+      <c r="F104" s="29"/>
+      <c r="G104" s="29"/>
+      <c r="H104" s="29"/>
+      <c r="I104" s="29"/>
+      <c r="J104" s="10"/>
+      <c r="K104" s="11"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="I106" s="19" t="n">
+        <f aca="false">SUMIF(J83:J104,"Planned",I83:I104)</f>
+        <v>37000000</v>
       </c>
     </row>
   </sheetData>
@@ -11682,22 +11737,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J82:J103">
+  <conditionalFormatting sqref="J83:J104">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J78">
+  <conditionalFormatting sqref="J13:J79">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J78" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J79" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J82:J103" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J83:J104" type="list">
       <formula1>"Planned,If needed,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11728,12 +11783,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11747,56 +11802,56 @@
         <v>382</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G6" s="31"/>
       <c r="H6" s="31"/>
@@ -11807,22 +11862,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G7" s="31"/>
       <c r="H7" s="31"/>
@@ -11833,22 +11888,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
+        <v>536</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>532</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>528</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G8" s="31"/>
       <c r="H8" s="31"/>
@@ -11859,22 +11914,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G9" s="31"/>
       <c r="H9" s="31"/>
@@ -11885,22 +11940,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G10" s="31"/>
       <c r="H10" s="31"/>
@@ -11911,22 +11966,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G11" s="31"/>
       <c r="H11" s="31"/>
@@ -11937,22 +11992,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G12" s="31"/>
       <c r="H12" s="31"/>
@@ -11963,22 +12018,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G13" s="31"/>
       <c r="H13" s="31"/>
@@ -11989,22 +12044,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F14" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G14" s="31"/>
       <c r="H14" s="31"/>
@@ -12015,22 +12070,22 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G15" s="31"/>
       <c r="H15" s="31"/>
@@ -12041,22 +12096,22 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G16" s="31"/>
       <c r="H16" s="31"/>
@@ -12067,20 +12122,20 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G17" s="31"/>
       <c r="H17" s="31"/>
@@ -12091,19 +12146,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F18" s="31"/>
       <c r="G18" s="31"/>
@@ -12115,22 +12170,22 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
+        <v>555</v>
+      </c>
+      <c r="B19" s="12" t="s">
         <v>551</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>547</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G19" s="31"/>
       <c r="H19" s="31"/>
@@ -12141,22 +12196,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G20" s="31"/>
       <c r="H20" s="31"/>
@@ -12167,27 +12222,27 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F22" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G22" s="31"/>
       <c r="H22" s="31"/>
@@ -12198,16 +12253,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12220,16 +12275,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12242,22 +12297,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="E25" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G25" s="31"/>
       <c r="H25" s="31"/>
@@ -12268,19 +12323,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F26" s="31"/>
       <c r="G26" s="31"/>
@@ -12292,16 +12347,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12314,16 +12369,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12336,21 +12391,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12363,16 +12418,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12385,16 +12440,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
+        <v>582</v>
+      </c>
+      <c r="B32" s="12" t="s">
         <v>578</v>
       </c>
-      <c r="B32" s="12" t="s">
-        <v>574</v>
-      </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12407,19 +12462,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F33" s="31"/>
       <c r="G33" s="31"/>
@@ -12431,16 +12486,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12453,16 +12508,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
+        <v>589</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>585</v>
       </c>
-      <c r="B35" s="12" t="s">
-        <v>581</v>
-      </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12475,16 +12530,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12497,16 +12552,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12519,16 +12574,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12541,7 +12596,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12578,7 +12633,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12615,7 +12670,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
     </row>
   </sheetData>
@@ -12659,12 +12714,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12672,10 +12727,10 @@
         <v>237</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12686,13 +12741,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12700,10 +12755,10 @@
         <v>239</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>348958315</v>
+        <v>351958315</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12711,11 +12766,11 @@
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
-        <v>4200000</v>
+        <v>2800000</v>
       </c>
       <c r="G6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>5700000</v>
+        <v>3800000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12724,7 +12779,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>243</v>
@@ -12748,12 +12803,12 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>1041685</v>
+        <v>23041685</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -12761,20 +12816,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>76041685</v>
+        <v>73041685</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>12697813.3118306</v>
+        <v>12226964.5439335</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12785,19 +12840,19 @@
         <v>246</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12813,7 +12868,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -12839,7 +12894,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -12865,7 +12920,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -12891,7 +12946,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -12916,10 +12971,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -12944,10 +12999,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -12972,10 +13027,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -13000,10 +13055,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -13028,10 +13083,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -13056,10 +13111,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -13085,7 +13140,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13110,10 +13165,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13138,10 +13193,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13166,10 +13221,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13197,7 +13252,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13224,10 +13279,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13254,10 +13309,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
+        <v>632</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>628</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>624</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13269,11 +13324,11 @@
         <v>1900000</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="I29" s="23" t="n">
         <f aca="false">IF(B29="","",MAX(0,B29-$B$6))</f>
-        <v>1041685</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13284,10 +13339,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13297,7 +13352,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>26041685</v>
+        <v>23041685</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13308,10 +13363,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13327,7 +13382,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>51041685</v>
+        <v>48041685</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13338,7 +13393,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13355,7 +13410,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>76041685</v>
+        <v>73041685</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13366,10 +13421,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13385,7 +13440,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>101041685</v>
+        <v>98041685</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13396,7 +13451,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13413,7 +13468,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>126041685</v>
+        <v>123041685</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13424,10 +13479,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13443,7 +13498,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>151041685</v>
+        <v>148041685</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13454,7 +13509,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13471,7 +13526,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>176041685</v>
+        <v>173041685</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13482,10 +13537,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13501,7 +13556,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>201041685</v>
+        <v>198041685</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13512,7 +13567,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13529,7 +13584,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>251041685</v>
+        <v>248041685</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13540,10 +13595,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13559,7 +13614,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>301041685</v>
+        <v>298041685</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13570,7 +13625,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13587,7 +13642,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>401041685</v>
+        <v>398041685</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13598,10 +13653,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13617,7 +13672,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>551041685</v>
+        <v>548041685</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13628,7 +13683,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13645,7 +13700,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>751041685</v>
+        <v>748041685</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13656,10 +13711,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -13675,7 +13730,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>951041685</v>
+        <v>948041685</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13686,7 +13741,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -13703,7 +13758,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1151041685</v>
+        <v>1148041685</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13714,7 +13769,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -13731,7 +13786,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1351041685</v>
+        <v>1348041685</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13742,7 +13797,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -13759,7 +13814,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1551041685</v>
+        <v>1548041685</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13770,7 +13825,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -13787,7 +13842,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1751041685</v>
+        <v>1748041685</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13798,7 +13853,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -13815,7 +13870,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1951041685</v>
+        <v>1948041685</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13826,7 +13881,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -13843,7 +13898,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2151041685</v>
+        <v>2148041685</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13854,7 +13909,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -13871,7 +13926,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2351041685</v>
+        <v>2348041685</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13882,7 +13937,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -13899,7 +13954,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2551041685</v>
+        <v>2548041685</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13910,7 +13965,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -13927,7 +13982,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2751041685</v>
+        <v>2748041685</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13938,7 +13993,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -13955,7 +14010,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2951041685</v>
+        <v>2948041685</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13966,7 +14021,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -13983,12 +14038,12 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3151041685</v>
+        <v>3148041685</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Confirm Julia iso cost
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1570,7 +1570,7 @@
     <t xml:space="preserve">Spider-Woman (Julia) Iso-8 to T3 level 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimate from Hulk. Confirm with Quick Upgrade</t>
+    <t xml:space="preserve">Same cost as Hulk. Plus 500 ion 1 to unlock the T4 matrix</t>
   </si>
   <si>
     <t xml:space="preserve">Rachel Cole-Alves Iso-8 to T3 level 5</t>
@@ -5855,7 +5855,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>564240109.001267</v>
+        <v>564372213.432624</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12823,7 +12823,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>12230489.5916063</v>
+        <v>12233353.0884219</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Iso Fest at 386M
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5866,7 +5866,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>570186376.13673</v>
+        <v>572757086.217411</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12760,7 +12760,7 @@
         <v>238</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>351958315</v>
+        <v>386018715</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>605</v>
@@ -12784,7 +12784,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>242</v>
@@ -12808,7 +12808,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>23041685</v>
+        <v>13981285</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12825,7 +12825,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>73041685</v>
+        <v>38981285</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12834,7 +12834,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>12422049.8860974</v>
+        <v>6659356.60531975</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13357,7 +13357,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>23041685</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13387,7 +13387,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>48041685</v>
+        <v>13981285</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13415,7 +13415,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>73041685</v>
+        <v>38981285</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13445,7 +13445,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>98041685</v>
+        <v>63981285</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>123041685</v>
+        <v>88981285</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13503,7 +13503,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>148041685</v>
+        <v>113981285</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13531,7 +13531,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>173041685</v>
+        <v>138981285</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13561,7 +13561,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>198041685</v>
+        <v>163981285</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>248041685</v>
+        <v>213981285</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13619,7 +13619,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>298041685</v>
+        <v>263981285</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13647,7 +13647,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>398041685</v>
+        <v>363981285</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13677,7 +13677,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>548041685</v>
+        <v>513981285</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13705,7 +13705,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>748041685</v>
+        <v>713981285</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13735,7 +13735,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>948041685</v>
+        <v>913981285</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13763,7 +13763,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1148041685</v>
+        <v>1113981285</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13791,7 +13791,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1348041685</v>
+        <v>1313981285</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13819,7 +13819,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1548041685</v>
+        <v>1513981285</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13847,7 +13847,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1748041685</v>
+        <v>1713981285</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13875,7 +13875,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1948041685</v>
+        <v>1913981285</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13903,7 +13903,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2148041685</v>
+        <v>2113981285</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13931,7 +13931,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2348041685</v>
+        <v>2313981285</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13959,7 +13959,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2548041685</v>
+        <v>2513981285</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13987,7 +13987,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2748041685</v>
+        <v>2713981285</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14015,7 +14015,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2948041685</v>
+        <v>2913981285</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3148041685</v>
+        <v>3113981285</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Oct 13 dailies, gold orb, gold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1273" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1285" uniqueCount="661">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1396,27 +1396,27 @@
     <t xml:space="preserve">Breaker of Nature level 130</t>
   </si>
   <si>
+    <t xml:space="preserve">Level 110 gold orb, Breaker of Nature level 120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending claim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaker of Nature level 110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending claim. Also gives the level 110 training orb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spider-Man tower milestone 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cell 20 cleared Oct 12. In current stock</t>
+  </si>
+  <si>
     <t xml:space="preserve">Moonlit Sigils store</t>
   </si>
   <si>
-    <t xml:space="preserve">Level 110 gold orb, Breaker of Nature level 120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pending claim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Breaker of Nature level 110</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pending claim. Also gives the level 110 training orb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spider-Man tower milestone 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cell 20 cleared Oct 12. In current stock</t>
-  </si>
-  <si>
     <t xml:space="preserve">Oct 12. In current stock</t>
   </si>
   <si>
@@ -1834,7 +1834,7 @@
     <t xml:space="preserve">Objectives done, required</t>
   </si>
   <si>
-    <t xml:space="preserve">Oct 11 and Oct 12 are filled in from your screenshots. The calendar and battle pass rows are left for you.</t>
+    <t xml:space="preserve">Oct 11 to Oct 13 are filled in from your screenshots. The calendar and battle pass rows are left for you.</t>
   </si>
   <si>
     <t xml:space="preserve">Iso Fest Milestones</t>
@@ -5813,14 +5813,14 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>772302650</v>
+        <v>780302650</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6028802650</v>
+        <v>6036802650</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>52697350</v>
+        <v>44697350</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3352697350</v>
+        <v>3344697350</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5879,7 +5879,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>575254942.789311</v>
+        <v>614640319.024558</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6755,7 +6755,7 @@
       <c r="D61" s="11"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>52697350</v>
+        <v>44697350</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>185</v>
@@ -6774,7 +6774,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>127697350</v>
+        <v>119697350</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6793,7 +6793,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>202697350</v>
+        <v>194697350</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6812,7 +6812,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>277697350</v>
+        <v>269697350</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6831,7 +6831,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>352697350</v>
+        <v>344697350</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6850,7 +6850,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>427697350</v>
+        <v>419697350</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6869,7 +6869,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>577697350</v>
+        <v>569697350</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6888,7 +6888,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>727697350</v>
+        <v>719697350</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6907,7 +6907,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>877697350</v>
+        <v>869697350</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6926,7 +6926,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1102697350</v>
+        <v>1094697350</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6945,7 +6945,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1477697350</v>
+        <v>1469697350</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -6964,7 +6964,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1852697350</v>
+        <v>1844697350</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -6983,7 +6983,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2227697350</v>
+        <v>2219697350</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7002,7 +7002,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2602697350</v>
+        <v>2594697350</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7021,7 +7021,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2977697350</v>
+        <v>2969697350</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7040,7 +7040,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3352697350</v>
+        <v>3344697350</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -8799,7 +8799,7 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>27110000</v>
+        <v>28900000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>1699000</v>
@@ -8826,7 +8826,7 @@
       </c>
       <c r="B6" s="27" t="n">
         <f aca="false">SUMIFS(B13:B79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
-        <v>16550000</v>
+        <v>14950000</v>
       </c>
       <c r="C6" s="27" t="n">
         <f aca="false">SUMIFS(C13:C79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
@@ -8859,7 +8859,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>43660000</v>
+        <v>43850000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8925,7 +8925,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>43660000</v>
+        <v>43850000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -9096,7 +9096,7 @@
         <v>326</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="K15" s="14" t="s">
         <v>404</v>
@@ -10243,36 +10243,36 @@
         <v>403</v>
       </c>
       <c r="C49" s="29" t="s">
+        <v>405</v>
+      </c>
+      <c r="D49" s="29" t="s">
         <v>453</v>
       </c>
-      <c r="D49" s="29" t="s">
+      <c r="E49" s="29" t="s">
         <v>431</v>
       </c>
-      <c r="E49" s="29" t="s">
+      <c r="F49" s="29" t="s">
         <v>433</v>
       </c>
-      <c r="F49" s="29" t="s">
+      <c r="G49" s="29" t="s">
         <v>428</v>
       </c>
-      <c r="G49" s="29" t="s">
+      <c r="H49" s="29" t="s">
         <v>425</v>
       </c>
-      <c r="H49" s="29" t="s">
+      <c r="I49" s="10" t="s">
         <v>426</v>
-      </c>
-      <c r="I49" s="10" t="s">
-        <v>427</v>
       </c>
       <c r="J49" s="10" t="s">
         <v>326</v>
       </c>
       <c r="K49" s="14" t="s">
-        <v>454</v>
+        <v>427</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B50" s="29" t="n">
         <v>3300000</v>
@@ -10302,12 +10302,12 @@
         <v>326</v>
       </c>
       <c r="K50" s="14" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B51" s="29" t="n">
         <v>0</v>
@@ -10337,12 +10337,12 @@
         <v>330</v>
       </c>
       <c r="K51" s="14" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B52" s="29" t="n">
         <v>0</v>
@@ -10372,12 +10372,12 @@
         <v>326</v>
       </c>
       <c r="K52" s="14" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="B53" s="29" t="n">
         <v>0</v>
@@ -10940,7 +10940,7 @@
         <v>485</v>
       </c>
       <c r="B69" s="29" t="n">
-        <v>375000</v>
+        <v>455000</v>
       </c>
       <c r="C69" s="29" t="n">
         <v>0</v>
@@ -11871,7 +11871,9 @@
       <c r="F6" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G6" s="31"/>
+      <c r="G6" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H6" s="31"/>
       <c r="I6" s="31"/>
       <c r="J6" s="31"/>
@@ -11897,7 +11899,9 @@
       <c r="F7" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G7" s="31"/>
+      <c r="G7" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H7" s="31"/>
       <c r="I7" s="31"/>
       <c r="J7" s="31"/>
@@ -11923,7 +11927,9 @@
       <c r="F8" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G8" s="31"/>
+      <c r="G8" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H8" s="31"/>
       <c r="I8" s="31"/>
       <c r="J8" s="31"/>
@@ -11949,7 +11955,9 @@
       <c r="F9" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G9" s="31"/>
+      <c r="G9" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H9" s="31"/>
       <c r="I9" s="31"/>
       <c r="J9" s="31"/>
@@ -11975,7 +11983,9 @@
       <c r="F10" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G10" s="31"/>
+      <c r="G10" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H10" s="31"/>
       <c r="I10" s="31"/>
       <c r="J10" s="31"/>
@@ -12001,7 +12011,9 @@
       <c r="F11" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G11" s="31"/>
+      <c r="G11" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H11" s="31"/>
       <c r="I11" s="31"/>
       <c r="J11" s="31"/>
@@ -12027,7 +12039,9 @@
       <c r="F12" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G12" s="31"/>
+      <c r="G12" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H12" s="31"/>
       <c r="I12" s="31"/>
       <c r="J12" s="31"/>
@@ -12053,7 +12067,9 @@
       <c r="F13" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G13" s="31"/>
+      <c r="G13" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H13" s="31"/>
       <c r="I13" s="31"/>
       <c r="J13" s="31"/>
@@ -12079,7 +12095,9 @@
       <c r="F14" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G14" s="31"/>
+      <c r="G14" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H14" s="31"/>
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
@@ -12105,7 +12123,9 @@
       <c r="F15" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G15" s="31"/>
+      <c r="G15" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H15" s="31"/>
       <c r="I15" s="31"/>
       <c r="J15" s="31"/>
@@ -12131,7 +12151,9 @@
       <c r="F16" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G16" s="31"/>
+      <c r="G16" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H16" s="31"/>
       <c r="I16" s="31"/>
       <c r="J16" s="31"/>
@@ -12231,7 +12253,9 @@
       <c r="F20" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G20" s="31"/>
+      <c r="G20" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H20" s="31"/>
       <c r="I20" s="31"/>
       <c r="J20" s="31"/>
@@ -12626,7 +12650,7 @@
       </c>
       <c r="G40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(G5:G38="Done"))</f>
-        <v>0</v>
+        <v>1450000</v>
       </c>
       <c r="H40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(H5:H38="Done"))</f>
@@ -12663,7 +12687,7 @@
       </c>
       <c r="G41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",G5:G38,"Done")&amp;" of 11"</f>
-        <v>0 of 11</v>
+        <v>11 of 11</v>
       </c>
       <c r="H41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",H5:H38,"Done")&amp;" of 11"</f>
@@ -12847,7 +12871,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>6688398.79267416</v>
+        <v>7163419.28317224</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
IV 822M after raid, Iso Fest corrected
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5813,14 +5813,14 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>780302650</v>
+        <v>822502750</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6036802650</v>
+        <v>6033002750</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>44697350</v>
+        <v>2497250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3344697350</v>
+        <v>3302497250</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5879,7 +5879,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>614640319.024558</v>
+        <v>607076074.644587</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6755,7 +6755,7 @@
       <c r="D61" s="11"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>44697350</v>
+        <v>2497250</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>185</v>
@@ -6774,7 +6774,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>119697350</v>
+        <v>77497250</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6793,7 +6793,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>194697350</v>
+        <v>152497250</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6812,7 +6812,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>269697350</v>
+        <v>227497250</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6831,7 +6831,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>344697350</v>
+        <v>302497250</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6850,7 +6850,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>419697350</v>
+        <v>377497250</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6869,7 +6869,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>569697350</v>
+        <v>527497250</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6888,7 +6888,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>719697350</v>
+        <v>677497250</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6907,7 +6907,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>869697350</v>
+        <v>827497250</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6926,7 +6926,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1094697350</v>
+        <v>1052497250</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6945,7 +6945,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1469697350</v>
+        <v>1427497250</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -6964,7 +6964,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1844697350</v>
+        <v>1802497250</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -6983,7 +6983,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2219697350</v>
+        <v>2177497250</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7002,7 +7002,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2594697350</v>
+        <v>2552497250</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7021,7 +7021,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2969697350</v>
+        <v>2927497250</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7040,7 +7040,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3344697350</v>
+        <v>3302497250</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -7725,11 +7725,11 @@
         <v>15000000</v>
       </c>
       <c r="E21" s="24" t="n">
-        <v>12000000</v>
+        <v>15000000</v>
       </c>
       <c r="F21" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D21),MAX(0,D21-E21),0)</f>
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="G21" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D21),ROUNDUP(D21/C21,0),"No limit")</f>
@@ -7737,11 +7737,11 @@
       </c>
       <c r="H21" s="21" t="n">
         <f aca="false">IFERROR(INT(E21/C21),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I21" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F21/C21,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" s="10" t="s">
         <v>326</v>
@@ -7761,11 +7761,11 @@
         <v>40000000</v>
       </c>
       <c r="E22" s="24" t="n">
-        <v>32000000</v>
+        <v>40000000</v>
       </c>
       <c r="F22" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D22),MAX(0,D22-E22),0)</f>
-        <v>8000000</v>
+        <v>0</v>
       </c>
       <c r="G22" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D22),ROUNDUP(D22/C22,0),"No limit")</f>
@@ -7773,11 +7773,11 @@
       </c>
       <c r="H22" s="21" t="n">
         <f aca="false">IFERROR(INT(E22/C22),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I22" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F22/C22,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" s="10" t="s">
         <v>326</v>
@@ -7797,11 +7797,11 @@
         <v>15000000</v>
       </c>
       <c r="E23" s="24" t="n">
-        <v>12000000</v>
+        <v>15000000</v>
       </c>
       <c r="F23" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D23),MAX(0,D23-E23),0)</f>
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="G23" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D23),ROUNDUP(D23/C23,0),"No limit")</f>
@@ -7809,11 +7809,11 @@
       </c>
       <c r="H23" s="21" t="n">
         <f aca="false">IFERROR(INT(E23/C23),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I23" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F23/C23,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" s="10" t="s">
         <v>326</v>
@@ -7833,11 +7833,11 @@
         <v>40000000</v>
       </c>
       <c r="E24" s="24" t="n">
-        <v>24000000</v>
+        <v>32000000</v>
       </c>
       <c r="F24" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D24),MAX(0,D24-E24),0)</f>
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="G24" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D24),ROUNDUP(D24/C24,0),"No limit")</f>
@@ -7845,11 +7845,11 @@
       </c>
       <c r="H24" s="21" t="n">
         <f aca="false">IFERROR(INT(E24/C24),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I24" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F24/C24,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J24" s="10" t="s">
         <v>326</v>
@@ -7869,11 +7869,11 @@
         <v>40000000</v>
       </c>
       <c r="E25" s="24" t="n">
-        <v>32000000</v>
+        <v>40000000</v>
       </c>
       <c r="F25" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D25),MAX(0,D25-E25),0)</f>
-        <v>8000000</v>
+        <v>0</v>
       </c>
       <c r="G25" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D25),ROUNDUP(D25/C25,0),"No limit")</f>
@@ -7881,11 +7881,11 @@
       </c>
       <c r="H25" s="21" t="n">
         <f aca="false">IFERROR(INT(E25/C25),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I25" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F25/C25,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J25" s="10" t="s">
         <v>326</v>
@@ -7941,11 +7941,11 @@
         <v>40000000</v>
       </c>
       <c r="E27" s="24" t="n">
-        <v>32000000</v>
+        <v>40000000</v>
       </c>
       <c r="F27" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D27),MAX(0,D27-E27),0)</f>
-        <v>8000000</v>
+        <v>0</v>
       </c>
       <c r="G27" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D27),ROUNDUP(D27/C27,0),"No limit")</f>
@@ -7953,11 +7953,11 @@
       </c>
       <c r="H27" s="21" t="n">
         <f aca="false">IFERROR(INT(E27/C27),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I27" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F27/C27,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27" s="10" t="s">
         <v>326</v>
@@ -8013,11 +8013,11 @@
         <v>40000000</v>
       </c>
       <c r="E29" s="24" t="n">
-        <v>24000000</v>
+        <v>32000000</v>
       </c>
       <c r="F29" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D29),MAX(0,D29-E29),0)</f>
-        <v>16000000</v>
+        <v>8000000</v>
       </c>
       <c r="G29" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D29),ROUNDUP(D29/C29,0),"No limit")</f>
@@ -8025,11 +8025,11 @@
       </c>
       <c r="H29" s="21" t="n">
         <f aca="false">IFERROR(INT(E29/C29),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I29" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F29/C29,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J29" s="10" t="s">
         <v>326</v>
@@ -8689,7 +8689,7 @@
       </c>
       <c r="E49" s="19" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>768302650</v>
+        <v>814302650</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -8700,7 +8700,7 @@
       <c r="E50" s="19"/>
       <c r="F50" s="19" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7168947350</v>
+        <v>7122947350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8710,7 +8710,7 @@
       <c r="E51" s="19"/>
       <c r="F51" s="19" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5256500000</v>
+        <v>5210500000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12797,7 +12797,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>386018715</v>
+        <v>366068715</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>608</v>
@@ -12821,7 +12821,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>245</v>
@@ -12845,7 +12845,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>13981285</v>
+        <v>8931285</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12862,7 +12862,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>38981285</v>
+        <v>58931285</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12871,7 +12871,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>7163419.28317224</v>
+        <v>10832945.6550788</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13394,7 +13394,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>0</v>
+        <v>8931285</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13424,7 +13424,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>13981285</v>
+        <v>33931285</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13452,7 +13452,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>38981285</v>
+        <v>58931285</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>63981285</v>
+        <v>83931285</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>88981285</v>
+        <v>108931285</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13540,7 +13540,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>113981285</v>
+        <v>133931285</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13568,7 +13568,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>138981285</v>
+        <v>158931285</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13598,7 +13598,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>163981285</v>
+        <v>183931285</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13626,7 +13626,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>213981285</v>
+        <v>233931285</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13656,7 +13656,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>263981285</v>
+        <v>283931285</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13684,7 +13684,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>363981285</v>
+        <v>383931285</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13714,7 +13714,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>513981285</v>
+        <v>533931285</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13742,7 +13742,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>713981285</v>
+        <v>733931285</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13772,7 +13772,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>913981285</v>
+        <v>933931285</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13800,7 +13800,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1113981285</v>
+        <v>1133931285</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13828,7 +13828,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1313981285</v>
+        <v>1333931285</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13856,7 +13856,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1513981285</v>
+        <v>1533931285</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1713981285</v>
+        <v>1733931285</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13912,7 +13912,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1913981285</v>
+        <v>1933931285</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13940,7 +13940,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2113981285</v>
+        <v>2133931285</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2313981285</v>
+        <v>2333931285</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13996,7 +13996,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2513981285</v>
+        <v>2533931285</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14024,7 +14024,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2713981285</v>
+        <v>2733931285</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14052,7 +14052,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2913981285</v>
+        <v>2933931285</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14080,7 +14080,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3113981285</v>
+        <v>3133931285</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Oct 13 raids, campaign, training orb
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1285" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1286" uniqueCount="661">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>607076074.644587</v>
+        <v>607257731.940485</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8799,7 +8799,7 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>28900000</v>
+        <v>29340000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>1699000</v>
@@ -8814,10 +8814,10 @@
         <v>263</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>929</v>
+        <v>953</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>1837</v>
+        <v>1865</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>43850000</v>
+        <v>44290000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8879,11 +8879,11 @@
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>1029</v>
+        <v>1053</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1922</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8925,7 +8925,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>43850000</v>
+        <v>44290000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8945,11 +8945,11 @@
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>1029</v>
+        <v>1053</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>1922</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10433,7 +10433,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="29" t="n">
-        <v>143</v>
+        <v>171</v>
       </c>
       <c r="I54" s="10" t="s">
         <v>326</v>
@@ -10870,7 +10870,7 @@
         <v>481</v>
       </c>
       <c r="B67" s="29" t="n">
-        <v>304975</v>
+        <v>342975</v>
       </c>
       <c r="C67" s="29" t="n">
         <v>0</v>
@@ -10885,7 +10885,7 @@
         <v>52</v>
       </c>
       <c r="G67" s="29" t="n">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="H67" s="29" t="n">
         <v>0</v>
@@ -12177,7 +12177,9 @@
       <c r="F17" s="31" t="s">
         <v>490</v>
       </c>
-      <c r="G17" s="31"/>
+      <c r="G17" s="31" t="s">
+        <v>490</v>
+      </c>
       <c r="H17" s="31"/>
       <c r="I17" s="31"/>
       <c r="J17" s="31"/>
@@ -12650,7 +12652,7 @@
       </c>
       <c r="G40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(G5:G38="Done"))</f>
-        <v>1450000</v>
+        <v>1550000</v>
       </c>
       <c r="H40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(H5:H38="Done"))</f>
@@ -12871,7 +12873,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>10832945.6550788</v>
+        <v>10836187.2275217</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Training Day Oct 13, Gold Rush schedule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1286" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="664">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1378,10 +1378,19 @@
     <t xml:space="preserve">Claimed, 900K in current stock</t>
   </si>
   <si>
-    <t xml:space="preserve">Gold Rush run</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runs Sundays, Mondays and other days. Set to Yes on days it runs</t>
+    <t xml:space="preserve">Gold Rush, Thu Oct 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Mon, Thu, Sun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gold Rush, Sun Oct 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training Day, Oct 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three runs. In current stock</t>
   </si>
   <si>
     <t xml:space="preserve">Training Day run</t>
@@ -1735,7 +1744,7 @@
     <t xml:space="preserve">Free energy, 9 PM to midnight</t>
   </si>
   <si>
-    <t xml:space="preserve">Gold Rush, when available</t>
+    <t xml:space="preserve">Gold Rush, Mon Thu Sun</t>
   </si>
   <si>
     <t xml:space="preserve">Challenge</t>
@@ -5879,7 +5888,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>607257731.940485</v>
+        <v>607360867.062626</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8747,7 +8756,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K106"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -8814,10 +8823,10 @@
         <v>263</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>953</v>
+        <v>983</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>1865</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8825,31 +8834,31 @@
         <v>392</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">SUMIFS(B13:B79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
-        <v>14950000</v>
+        <f aca="false">SUMIFS(B13:B81,$I$13:$I$81,"Yes",$J$13:$J$81,"No")</f>
+        <v>16750000</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">SUMIFS(C13:C79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <f aca="false">SUMIFS(C13:C81,$I$13:$I$81,"Yes",$J$13:$J$81,"No")</f>
         <v>450000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">SUMIFS(D13:D79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <f aca="false">SUMIFS(D13:D81,$I$13:$I$81,"Yes",$J$13:$J$81,"No")</f>
         <v>886000</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">SUMIFS(E13:E79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <f aca="false">SUMIFS(E13:E81,$I$13:$I$81,"Yes",$J$13:$J$81,"No")</f>
         <v>886000</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">SUMIFS(F13:F79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <f aca="false">SUMIFS(F13:F81,$I$13:$I$81,"Yes",$J$13:$J$81,"No")</f>
         <v>0</v>
       </c>
       <c r="G6" s="27" t="n">
-        <f aca="false">SUMIFS(G13:G79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <f aca="false">SUMIFS(G13:G81,$I$13:$I$81,"Yes",$J$13:$J$81,"No")</f>
         <v>100</v>
       </c>
       <c r="H6" s="27" t="n">
-        <f aca="false">SUMIFS(H13:H79,$I$13:$I$79,"Yes",$J$13:$J$79,"No")</f>
+        <f aca="false">SUMIFS(H13:H81,$I$13:$I$81,"Yes",$J$13:$J$81,"No")</f>
         <v>85</v>
       </c>
     </row>
@@ -8859,7 +8868,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>44290000</v>
+        <v>46090000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8879,11 +8888,11 @@
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>1053</v>
+        <v>1083</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1950</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8891,31 +8900,31 @@
         <v>394</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$83:$J$104,"Planned",B83:B104)</f>
+        <f aca="false">SUMIF($J$85:$J$106,"Planned",B85:B106)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$83:$J$104,"Planned",C83:C104)</f>
+        <f aca="false">SUMIF($J$85:$J$106,"Planned",C85:C106)</f>
         <v>0</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$83:$J$104,"Planned",D83:D104)</f>
+        <f aca="false">SUMIF($J$85:$J$106,"Planned",D85:D106)</f>
         <v>0</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$83:$J$104,"Planned",E83:E104)</f>
+        <f aca="false">SUMIF($J$85:$J$106,"Planned",E85:E106)</f>
         <v>0</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$83:$J$104,"Planned",F83:F104)</f>
+        <f aca="false">SUMIF($J$85:$J$106,"Planned",F85:F106)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$83:$J$104,"Planned",G83:G104)</f>
+        <f aca="false">SUMIF($J$85:$J$106,"Planned",G85:G106)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$83:$J$104,"Planned",H83:H104)</f>
+        <f aca="false">SUMIF($J$85:$J$106,"Planned",H85:H106)</f>
         <v>0</v>
       </c>
     </row>
@@ -8925,7 +8934,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>44290000</v>
+        <v>46090000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8945,11 +8954,11 @@
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>1053</v>
+        <v>1083</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>1950</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10191,7 +10200,7 @@
         <v>0</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="J47" s="10" t="s">
         <v>330</v>
@@ -10205,7 +10214,7 @@
         <v>450</v>
       </c>
       <c r="B48" s="29" t="n">
-        <v>0</v>
+        <v>900000</v>
       </c>
       <c r="C48" s="29" t="n">
         <v>0</v>
@@ -10220,132 +10229,132 @@
         <v>0</v>
       </c>
       <c r="G48" s="29" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H48" s="29" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="J48" s="10" t="s">
         <v>330</v>
       </c>
       <c r="K48" s="14" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>452</v>
-      </c>
-      <c r="B49" s="29" t="s">
-        <v>403</v>
-      </c>
-      <c r="C49" s="29" t="s">
-        <v>405</v>
-      </c>
-      <c r="D49" s="29" t="s">
-        <v>453</v>
-      </c>
-      <c r="E49" s="29" t="s">
-        <v>431</v>
-      </c>
-      <c r="F49" s="29" t="s">
-        <v>433</v>
-      </c>
-      <c r="G49" s="29" t="s">
-        <v>428</v>
-      </c>
-      <c r="H49" s="29" t="s">
-        <v>425</v>
+        <v>451</v>
+      </c>
+      <c r="B49" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="H49" s="29" t="n">
+        <v>90</v>
       </c>
       <c r="I49" s="10" t="s">
-        <v>426</v>
+        <v>326</v>
       </c>
       <c r="J49" s="10" t="s">
         <v>326</v>
       </c>
       <c r="K49" s="14" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="B50" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="H50" s="29" t="n">
+        <v>90</v>
+      </c>
+      <c r="I50" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="J50" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="K50" s="14" t="s">
         <v>454</v>
-      </c>
-      <c r="B50" s="29" t="n">
-        <v>3300000</v>
-      </c>
-      <c r="C50" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I50" s="10" t="s">
-        <v>326</v>
-      </c>
-      <c r="J50" s="10" t="s">
-        <v>326</v>
-      </c>
-      <c r="K50" s="14" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="B51" s="29" t="s">
+        <v>403</v>
+      </c>
+      <c r="C51" s="29" t="s">
+        <v>405</v>
+      </c>
+      <c r="D51" s="29" t="s">
+        <v>451</v>
+      </c>
+      <c r="E51" s="29" t="s">
         <v>456</v>
       </c>
-      <c r="B51" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C51" s="29" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D51" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F51" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="29" t="n">
-        <v>0</v>
+      <c r="F51" s="29" t="s">
+        <v>431</v>
+      </c>
+      <c r="G51" s="29" t="s">
+        <v>433</v>
+      </c>
+      <c r="H51" s="29" t="s">
+        <v>428</v>
       </c>
       <c r="I51" s="10" t="s">
+        <v>425</v>
+      </c>
+      <c r="J51" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="J51" s="10" t="s">
-        <v>330</v>
-      </c>
       <c r="K51" s="14" t="s">
-        <v>457</v>
+        <v>426</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B52" s="29" t="n">
-        <v>0</v>
+        <v>3300000</v>
       </c>
       <c r="C52" s="29" t="n">
         <v>0</v>
@@ -10363,7 +10372,7 @@
         <v>0</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="I52" s="10" t="s">
         <v>326</v>
@@ -10372,18 +10381,18 @@
         <v>326</v>
       </c>
       <c r="K52" s="14" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B53" s="29" t="n">
         <v>0</v>
       </c>
       <c r="C53" s="29" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D53" s="29" t="n">
         <v>0</v>
@@ -10398,21 +10407,21 @@
         <v>0</v>
       </c>
       <c r="H53" s="29" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>326</v>
       </c>
       <c r="J53" s="10" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="K53" s="14" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B54" s="29" t="n">
         <v>0</v>
@@ -10433,7 +10442,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="29" t="n">
-        <v>171</v>
+        <v>500</v>
       </c>
       <c r="I54" s="10" t="s">
         <v>326</v>
@@ -10442,12 +10451,12 @@
         <v>326</v>
       </c>
       <c r="K54" s="14" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B55" s="29" t="n">
         <v>0</v>
@@ -10468,21 +10477,21 @@
         <v>0</v>
       </c>
       <c r="H55" s="29" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I55" s="10" t="s">
         <v>326</v>
       </c>
       <c r="J55" s="10" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="K55" s="14" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B56" s="29" t="n">
         <v>0</v>
@@ -10491,10 +10500,10 @@
         <v>0</v>
       </c>
       <c r="D56" s="29" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="E56" s="29" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="F56" s="29" t="n">
         <v>0</v>
@@ -10503,24 +10512,24 @@
         <v>0</v>
       </c>
       <c r="H56" s="29" t="n">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="I56" s="10" t="s">
         <v>326</v>
       </c>
       <c r="J56" s="10" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="K56" s="14" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B57" s="29" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C57" s="29" t="n">
         <v>0</v>
@@ -10547,24 +10556,24 @@
         <v>330</v>
       </c>
       <c r="K57" s="14" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B58" s="29" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="C58" s="29" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="29" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="E58" s="29" t="n">
-        <v>0</v>
+        <v>136000</v>
       </c>
       <c r="F58" s="29" t="n">
         <v>0</v>
@@ -10582,12 +10591,12 @@
         <v>330</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B59" s="29" t="n">
         <v>750000</v>
@@ -10617,7 +10626,7 @@
         <v>330</v>
       </c>
       <c r="K59" s="14" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10652,12 +10661,12 @@
         <v>330</v>
       </c>
       <c r="K60" s="14" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B61" s="29" t="n">
         <v>750000</v>
@@ -10687,12 +10696,12 @@
         <v>330</v>
       </c>
       <c r="K61" s="14" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B62" s="29" t="n">
         <v>750000</v>
@@ -10722,12 +10731,12 @@
         <v>330</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B63" s="29" t="n">
         <v>750000</v>
@@ -10757,12 +10766,12 @@
         <v>330</v>
       </c>
       <c r="K63" s="14" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B64" s="29" t="n">
         <v>750000</v>
@@ -10792,18 +10801,18 @@
         <v>330</v>
       </c>
       <c r="K64" s="14" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>453</v>
+        <v>479</v>
       </c>
       <c r="B65" s="29" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C65" s="29" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="D65" s="29" t="n">
         <v>0</v>
@@ -10824,18 +10833,18 @@
         <v>326</v>
       </c>
       <c r="J65" s="10" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="K65" s="14" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B66" s="29" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="C66" s="29" t="n">
         <v>0</v>
@@ -10862,18 +10871,18 @@
         <v>330</v>
       </c>
       <c r="K66" s="14" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>481</v>
+        <v>456</v>
       </c>
       <c r="B67" s="29" t="n">
-        <v>342975</v>
+        <v>0</v>
       </c>
       <c r="C67" s="29" t="n">
-        <v>0</v>
+        <v>250000</v>
       </c>
       <c r="D67" s="29" t="n">
         <v>0</v>
@@ -10882,10 +10891,10 @@
         <v>0</v>
       </c>
       <c r="F67" s="29" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="G67" s="29" t="n">
-        <v>176</v>
+        <v>0</v>
       </c>
       <c r="H67" s="29" t="n">
         <v>0</v>
@@ -10897,15 +10906,15 @@
         <v>326</v>
       </c>
       <c r="K67" s="14" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B68" s="29" t="n">
-        <v>120000</v>
+        <v>0</v>
       </c>
       <c r="C68" s="29" t="n">
         <v>0</v>
@@ -10920,7 +10929,7 @@
         <v>0</v>
       </c>
       <c r="G68" s="29" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="H68" s="29" t="n">
         <v>0</v>
@@ -10929,72 +10938,116 @@
         <v>326</v>
       </c>
       <c r="J68" s="10" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="K68" s="14" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="B69" s="29" t="n">
+        <v>342975</v>
+      </c>
+      <c r="C69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="29" t="n">
+        <v>52</v>
+      </c>
+      <c r="G69" s="29" t="n">
+        <v>176</v>
+      </c>
+      <c r="H69" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="J69" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="K69" s="14" t="s">
         <v>485</v>
       </c>
-      <c r="B69" s="29" t="n">
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="11" t="s">
+        <v>486</v>
+      </c>
+      <c r="B70" s="29" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C70" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="29" t="n">
+        <v>64</v>
+      </c>
+      <c r="H70" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="J70" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="K70" s="14" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="11" t="s">
+        <v>488</v>
+      </c>
+      <c r="B71" s="29" t="n">
         <v>455000</v>
       </c>
-      <c r="C69" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G69" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I69" s="10" t="s">
+      <c r="C71" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="J69" s="10" t="s">
+      <c r="J71" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="K69" s="14" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="11"/>
-      <c r="B70" s="29"/>
-      <c r="C70" s="29"/>
-      <c r="D70" s="29"/>
-      <c r="E70" s="29"/>
-      <c r="F70" s="29"/>
-      <c r="G70" s="29"/>
-      <c r="H70" s="29"/>
-      <c r="I70" s="10"/>
-      <c r="J70" s="10"/>
-      <c r="K70" s="11"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="11"/>
-      <c r="B71" s="29"/>
-      <c r="C71" s="29"/>
-      <c r="D71" s="29"/>
-      <c r="E71" s="29"/>
-      <c r="F71" s="29"/>
-      <c r="G71" s="29"/>
-      <c r="H71" s="29"/>
-      <c r="I71" s="10"/>
-      <c r="J71" s="10"/>
-      <c r="K71" s="11"/>
+      <c r="K71" s="14" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="11"/>
@@ -11100,144 +11153,102 @@
       <c r="J79" s="10"/>
       <c r="K79" s="11"/>
     </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="11"/>
+      <c r="B80" s="29"/>
+      <c r="C80" s="29"/>
+      <c r="D80" s="29"/>
+      <c r="E80" s="29"/>
+      <c r="F80" s="29"/>
+      <c r="G80" s="29"/>
+      <c r="H80" s="29"/>
+      <c r="I80" s="10"/>
+      <c r="J80" s="10"/>
+      <c r="K80" s="11"/>
+    </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="22" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="3" t="s">
-        <v>488</v>
-      </c>
-      <c r="B82" s="3" t="s">
+      <c r="A81" s="11"/>
+      <c r="B81" s="29"/>
+      <c r="C81" s="29"/>
+      <c r="D81" s="29"/>
+      <c r="E81" s="29"/>
+      <c r="F81" s="29"/>
+      <c r="G81" s="29"/>
+      <c r="H81" s="29"/>
+      <c r="I81" s="10"/>
+      <c r="J81" s="10"/>
+      <c r="K81" s="11"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="22" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B84" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="C82" s="3" t="s">
+      <c r="C84" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="D82" s="3" t="s">
+      <c r="D84" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="E82" s="3" t="s">
+      <c r="E84" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="F82" s="3" t="s">
+      <c r="F84" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="G82" s="3" t="s">
+      <c r="G84" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="H82" s="3" t="s">
+      <c r="H84" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="I82" s="3" t="s">
+      <c r="I84" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J82" s="3" t="s">
+      <c r="J84" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K82" s="3" t="s">
+      <c r="K84" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="11" t="s">
-        <v>489</v>
-      </c>
-      <c r="B83" s="29" t="n">
-        <v>1837500</v>
-      </c>
-      <c r="C83" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D83" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E83" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F83" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="G83" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H83" s="29" t="n">
-        <v>183</v>
-      </c>
-      <c r="I83" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J83" s="10" t="s">
-        <v>490</v>
-      </c>
-      <c r="K83" s="14" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="11" t="s">
-        <v>492</v>
-      </c>
-      <c r="B84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C84" s="29" t="n">
-        <v>359800</v>
-      </c>
-      <c r="D84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I84" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J84" s="10" t="s">
-        <v>490</v>
-      </c>
-      <c r="K84" s="14"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
+        <v>492</v>
+      </c>
+      <c r="B85" s="29" t="n">
+        <v>1837500</v>
+      </c>
+      <c r="C85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G85" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" s="29" t="n">
+        <v>183</v>
+      </c>
+      <c r="I85" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="10" t="s">
         <v>493</v>
-      </c>
-      <c r="B85" s="29" t="n">
-        <v>9791250</v>
-      </c>
-      <c r="C85" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D85" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E85" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F85" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="G85" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H85" s="29" t="n">
-        <v>979</v>
-      </c>
-      <c r="I85" s="29" t="n">
-        <v>55000000</v>
-      </c>
-      <c r="J85" s="10" t="s">
-        <v>490</v>
       </c>
       <c r="K85" s="14" t="s">
         <v>494</v>
@@ -11272,17 +11283,17 @@
         <v>0</v>
       </c>
       <c r="J86" s="10" t="s">
-        <v>490</v>
-      </c>
-      <c r="K86" s="14" t="s">
-        <v>494</v>
-      </c>
+        <v>493</v>
+      </c>
+      <c r="K86" s="14"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
         <v>496</v>
       </c>
-      <c r="B87" s="26"/>
+      <c r="B87" s="29" t="n">
+        <v>9791250</v>
+      </c>
       <c r="C87" s="29" t="n">
         <v>0</v>
       </c>
@@ -11292,26 +11303,34 @@
       <c r="E87" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F87" s="26"/>
-      <c r="G87" s="26"/>
-      <c r="H87" s="26"/>
+      <c r="F87" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="29" t="n">
+        <v>979</v>
+      </c>
       <c r="I87" s="29" t="n">
-        <v>3000000</v>
+        <v>55000000</v>
       </c>
       <c r="J87" s="10" t="s">
+        <v>493</v>
+      </c>
+      <c r="K87" s="14" t="s">
         <v>497</v>
-      </c>
-      <c r="K87" s="14" t="s">
-        <v>498</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="11" t="s">
-        <v>499</v>
-      </c>
-      <c r="B88" s="26"/>
+        <v>498</v>
+      </c>
+      <c r="B88" s="29" t="n">
+        <v>0</v>
+      </c>
       <c r="C88" s="29" t="n">
-        <v>0</v>
+        <v>359800</v>
       </c>
       <c r="D88" s="29" t="n">
         <v>0</v>
@@ -11319,26 +11338,30 @@
       <c r="E88" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F88" s="26"/>
-      <c r="G88" s="26"/>
-      <c r="H88" s="26"/>
+      <c r="F88" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="29" t="n">
+        <v>0</v>
+      </c>
       <c r="I88" s="29" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="K88" s="14" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>502</v>
-      </c>
-      <c r="B89" s="29" t="n">
-        <v>1650010</v>
-      </c>
+        <v>499</v>
+      </c>
+      <c r="B89" s="26"/>
       <c r="C89" s="29" t="n">
         <v>0</v>
       </c>
@@ -11348,32 +11371,24 @@
       <c r="E89" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F89" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="G89" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H89" s="29" t="n">
-        <v>164</v>
-      </c>
+      <c r="F89" s="26"/>
+      <c r="G89" s="26"/>
+      <c r="H89" s="26"/>
       <c r="I89" s="29" t="n">
         <v>3000000</v>
       </c>
       <c r="J89" s="10" t="s">
-        <v>490</v>
+        <v>500</v>
       </c>
       <c r="K89" s="14" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="11" t="s">
-        <v>504</v>
-      </c>
-      <c r="B90" s="29" t="n">
-        <v>1650000</v>
-      </c>
+        <v>502</v>
+      </c>
+      <c r="B90" s="26"/>
       <c r="C90" s="29" t="n">
         <v>0</v>
       </c>
@@ -11383,31 +11398,25 @@
       <c r="E90" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F90" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="G90" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H90" s="29" t="n">
-        <v>164</v>
-      </c>
+      <c r="F90" s="26"/>
+      <c r="G90" s="26"/>
+      <c r="H90" s="26"/>
       <c r="I90" s="29" t="n">
         <v>3000000</v>
       </c>
       <c r="J90" s="10" t="s">
-        <v>490</v>
+        <v>503</v>
       </c>
       <c r="K90" s="14" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B91" s="29" t="n">
-        <v>1650000</v>
+        <v>1650010</v>
       </c>
       <c r="C91" s="29" t="n">
         <v>0</v>
@@ -11431,95 +11440,95 @@
         <v>3000000</v>
       </c>
       <c r="J91" s="10" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="11" t="s">
+        <v>507</v>
+      </c>
+      <c r="B92" s="29" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="C92" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G92" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H92" s="29" t="n">
+        <v>164</v>
+      </c>
+      <c r="I92" s="29" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J92" s="10" t="s">
+        <v>493</v>
+      </c>
+      <c r="K92" s="14" t="s">
         <v>508</v>
-      </c>
-      <c r="B92" s="26"/>
-      <c r="C92" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D92" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E92" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F92" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G92" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H92" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I92" s="29" t="n">
-        <v>17000000</v>
-      </c>
-      <c r="J92" s="10" t="s">
-        <v>500</v>
-      </c>
-      <c r="K92" s="14" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
+        <v>509</v>
+      </c>
+      <c r="B93" s="29" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="C93" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G93" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H93" s="29" t="n">
+        <v>164</v>
+      </c>
+      <c r="I93" s="29" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J93" s="10" t="s">
+        <v>500</v>
+      </c>
+      <c r="K93" s="14" t="s">
         <v>510</v>
-      </c>
-      <c r="B93" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C93" s="29" t="n">
-        <v>1710500</v>
-      </c>
-      <c r="D93" s="29" t="n">
-        <v>1710000</v>
-      </c>
-      <c r="E93" s="29" t="n">
-        <v>2640000</v>
-      </c>
-      <c r="F93" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G93" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H93" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I93" s="29" t="n">
-        <v>17000000</v>
-      </c>
-      <c r="J93" s="10" t="s">
-        <v>490</v>
-      </c>
-      <c r="K93" s="14" t="s">
-        <v>511</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="s">
-        <v>512</v>
-      </c>
-      <c r="B94" s="29" t="n">
-        <v>0</v>
-      </c>
+        <v>511</v>
+      </c>
+      <c r="B94" s="26"/>
       <c r="C94" s="29" t="n">
-        <v>1370000</v>
+        <v>0</v>
       </c>
       <c r="D94" s="29" t="n">
-        <v>1370000</v>
+        <v>0</v>
       </c>
       <c r="E94" s="29" t="n">
-        <v>2130000</v>
+        <v>0</v>
       </c>
       <c r="F94" s="29" t="n">
         <v>0</v>
@@ -11534,22 +11543,28 @@
         <v>17000000</v>
       </c>
       <c r="J94" s="10" t="s">
-        <v>490</v>
+        <v>503</v>
       </c>
       <c r="K94" s="14" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B95" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="C95" s="26"/>
-      <c r="D95" s="26"/>
-      <c r="E95" s="26"/>
+      <c r="C95" s="29" t="n">
+        <v>1710500</v>
+      </c>
+      <c r="D95" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E95" s="29" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F95" s="29" t="n">
         <v>0</v>
       </c>
@@ -11563,10 +11578,10 @@
         <v>17000000</v>
       </c>
       <c r="J95" s="10" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="K95" s="14" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11577,13 +11592,13 @@
         <v>0</v>
       </c>
       <c r="C96" s="29" t="n">
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="D96" s="29" t="n">
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="E96" s="29" t="n">
-        <v>2640000</v>
+        <v>2130000</v>
       </c>
       <c r="F96" s="29" t="n">
         <v>0</v>
@@ -11598,7 +11613,7 @@
         <v>17000000</v>
       </c>
       <c r="J96" s="10" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="K96" s="14" t="s">
         <v>516</v>
@@ -11627,10 +11642,10 @@
         <v>17000000</v>
       </c>
       <c r="J97" s="10" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="K97" s="14" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11638,55 +11653,93 @@
         <v>518</v>
       </c>
       <c r="B98" s="29" t="n">
-        <v>13000000</v>
+        <v>0</v>
       </c>
       <c r="C98" s="29" t="n">
-        <v>0</v>
+        <v>1710000</v>
       </c>
       <c r="D98" s="29" t="n">
-        <v>0</v>
+        <v>1710000</v>
       </c>
       <c r="E98" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F98" s="26"/>
-      <c r="G98" s="26"/>
-      <c r="H98" s="26"/>
+        <v>2640000</v>
+      </c>
+      <c r="F98" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="29" t="n">
+        <v>0</v>
+      </c>
       <c r="I98" s="29" t="n">
-        <v>8000000</v>
+        <v>17000000</v>
       </c>
       <c r="J98" s="10" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="K98" s="14" t="s">
         <v>519</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="11"/>
-      <c r="B99" s="29"/>
-      <c r="C99" s="29"/>
-      <c r="D99" s="29"/>
-      <c r="E99" s="29"/>
-      <c r="F99" s="29"/>
-      <c r="G99" s="29"/>
-      <c r="H99" s="29"/>
-      <c r="I99" s="29"/>
-      <c r="J99" s="10"/>
-      <c r="K99" s="11"/>
+      <c r="A99" s="11" t="s">
+        <v>520</v>
+      </c>
+      <c r="B99" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" s="26"/>
+      <c r="D99" s="26"/>
+      <c r="E99" s="26"/>
+      <c r="F99" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" s="29" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J99" s="10" t="s">
+        <v>500</v>
+      </c>
+      <c r="K99" s="14" t="s">
+        <v>512</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="11"/>
-      <c r="B100" s="29"/>
-      <c r="C100" s="29"/>
-      <c r="D100" s="29"/>
-      <c r="E100" s="29"/>
-      <c r="F100" s="29"/>
-      <c r="G100" s="29"/>
-      <c r="H100" s="29"/>
-      <c r="I100" s="29"/>
-      <c r="J100" s="10"/>
-      <c r="K100" s="11"/>
+      <c r="A100" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B100" s="29" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="C100" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" s="26"/>
+      <c r="G100" s="26"/>
+      <c r="H100" s="26"/>
+      <c r="I100" s="29" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="J100" s="10" t="s">
+        <v>500</v>
+      </c>
+      <c r="K100" s="14" t="s">
+        <v>522</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="11"/>
@@ -11740,12 +11793,38 @@
       <c r="J104" s="10"/>
       <c r="K104" s="11"/>
     </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="11"/>
+      <c r="B105" s="29"/>
+      <c r="C105" s="29"/>
+      <c r="D105" s="29"/>
+      <c r="E105" s="29"/>
+      <c r="F105" s="29"/>
+      <c r="G105" s="29"/>
+      <c r="H105" s="29"/>
+      <c r="I105" s="29"/>
+      <c r="J105" s="10"/>
+      <c r="K105" s="11"/>
+    </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="15" t="s">
-        <v>520</v>
-      </c>
-      <c r="I106" s="19" t="n">
-        <f aca="false">SUMIF(J83:J104,"Planned",I83:I104)</f>
+      <c r="A106" s="11"/>
+      <c r="B106" s="29"/>
+      <c r="C106" s="29"/>
+      <c r="D106" s="29"/>
+      <c r="E106" s="29"/>
+      <c r="F106" s="29"/>
+      <c r="G106" s="29"/>
+      <c r="H106" s="29"/>
+      <c r="I106" s="29"/>
+      <c r="J106" s="10"/>
+      <c r="K106" s="11"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="15" t="s">
+        <v>523</v>
+      </c>
+      <c r="I108" s="19" t="n">
+        <f aca="false">SUMIF(J85:J106,"Planned",I85:I106)</f>
         <v>20000000</v>
       </c>
     </row>
@@ -11755,22 +11834,22 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J83:J104">
+  <conditionalFormatting sqref="J85:J106">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J13:J79">
+  <conditionalFormatting sqref="J13:J81">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J79" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:J81" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J83:J104" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J85:J106" type="list">
       <formula1>"Planned,If needed,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11801,12 +11880,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11820,59 +11899,59 @@
         <v>384</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H6" s="31"/>
       <c r="I6" s="31"/>
@@ -11882,25 +11961,25 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G7" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H7" s="31"/>
       <c r="I7" s="31"/>
@@ -11910,25 +11989,25 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H8" s="31"/>
       <c r="I8" s="31"/>
@@ -11938,25 +12017,25 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H9" s="31"/>
       <c r="I9" s="31"/>
@@ -11966,25 +12045,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H10" s="31"/>
       <c r="I10" s="31"/>
@@ -11994,25 +12073,25 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H11" s="31"/>
       <c r="I11" s="31"/>
@@ -12022,25 +12101,25 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H12" s="31"/>
       <c r="I12" s="31"/>
@@ -12050,25 +12129,25 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H13" s="31"/>
       <c r="I13" s="31"/>
@@ -12078,25 +12157,25 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F14" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G14" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H14" s="31"/>
       <c r="I14" s="31"/>
@@ -12106,25 +12185,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H15" s="31"/>
       <c r="I15" s="31"/>
@@ -12134,25 +12213,25 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G16" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H16" s="31"/>
       <c r="I16" s="31"/>
@@ -12162,23 +12241,23 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H17" s="31"/>
       <c r="I17" s="31"/>
@@ -12188,19 +12267,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F18" s="31"/>
       <c r="G18" s="31"/>
@@ -12212,22 +12291,22 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G19" s="31"/>
       <c r="H19" s="31"/>
@@ -12238,25 +12317,25 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="H20" s="31"/>
       <c r="I20" s="31"/>
@@ -12266,27 +12345,27 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F22" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G22" s="31"/>
       <c r="H22" s="31"/>
@@ -12297,16 +12376,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12319,16 +12398,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
+        <v>569</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>566</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>563</v>
-      </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12341,22 +12420,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="E25" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G25" s="31"/>
       <c r="H25" s="31"/>
@@ -12367,22 +12446,24 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
+      <c r="G26" s="31" t="s">
+        <v>493</v>
+      </c>
       <c r="H26" s="31"/>
       <c r="I26" s="31"/>
       <c r="J26" s="31"/>
@@ -12391,16 +12472,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12413,16 +12494,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12435,21 +12516,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12462,16 +12543,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12484,16 +12565,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12506,19 +12587,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F33" s="31"/>
       <c r="G33" s="31"/>
@@ -12530,16 +12611,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12552,16 +12633,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12574,16 +12655,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12596,16 +12677,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12618,16 +12699,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12640,7 +12721,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12677,7 +12758,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12714,7 +12795,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
     </row>
   </sheetData>
@@ -12758,12 +12839,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12771,10 +12852,10 @@
         <v>239</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12785,13 +12866,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12802,7 +12883,7 @@
         <v>366068715</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12852,7 +12933,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -12860,7 +12941,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12869,11 +12950,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>10836187.2275217</v>
+        <v>10838027.6190108</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12884,19 +12965,19 @@
         <v>248</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12912,7 +12993,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -12938,7 +13019,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -12964,7 +13045,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -12990,7 +13071,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -13015,10 +13096,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -13043,10 +13124,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -13071,10 +13152,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -13099,10 +13180,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -13127,10 +13208,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -13155,10 +13236,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -13184,7 +13265,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13209,10 +13290,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13237,10 +13318,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13265,10 +13346,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13296,7 +13377,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13323,10 +13404,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
+        <v>636</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>633</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>630</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13353,10 +13434,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13383,10 +13464,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13407,10 +13488,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13437,7 +13518,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13465,10 +13546,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13495,7 +13576,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13523,10 +13604,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13553,7 +13634,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13581,10 +13662,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13611,7 +13692,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13639,10 +13720,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13669,7 +13750,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13697,10 +13778,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13727,7 +13808,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13755,10 +13836,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -13785,7 +13866,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -13813,7 +13894,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -13841,7 +13922,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -13869,7 +13950,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -13897,7 +13978,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -13925,7 +14006,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -13953,7 +14034,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -13981,7 +14062,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -14009,7 +14090,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -14037,7 +14118,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -14065,7 +14146,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -14087,7 +14168,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Training stock from game, Jim GT10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5888,7 +5888,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>607360867.062626</v>
+        <v>607459880.711091</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8808,7 +8808,7 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>29340000</v>
+        <v>29100000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>1699000</v>
@@ -8820,13 +8820,13 @@
         <v>15280000</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>983</v>
+        <v>1051</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>1955</v>
+        <v>2221</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8868,7 +8868,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>46090000</v>
+        <v>45850000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8884,15 +8884,15 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>1083</v>
+        <v>1151</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>2040</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>46090000</v>
+        <v>45850000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8950,15 +8950,15 @@
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>1083</v>
+        <v>1151</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>2040</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>10838027.6190108</v>
+        <v>10839794.4725512</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Secondary classes, ions and event points
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5822,14 +5822,14 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>822502750</v>
+        <v>824545350</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6033002750</v>
+        <v>6035045350</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>2497250</v>
+        <v>454650</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5879,7 +5879,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3302497250</v>
+        <v>3300454650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>607459880.711091</v>
+        <v>607823325.89826</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6764,7 +6764,7 @@
       <c r="D61" s="11"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>2497250</v>
+        <v>454650</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>185</v>
@@ -6783,7 +6783,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>77497250</v>
+        <v>75454650</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6802,7 +6802,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>152497250</v>
+        <v>150454650</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6821,7 +6821,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>227497250</v>
+        <v>225454650</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6840,7 +6840,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>302497250</v>
+        <v>300454650</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6859,7 +6859,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>377497250</v>
+        <v>375454650</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6878,7 +6878,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>527497250</v>
+        <v>525454650</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6897,7 +6897,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>677497250</v>
+        <v>675454650</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6916,7 +6916,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>827497250</v>
+        <v>825454650</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6935,7 +6935,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1052497250</v>
+        <v>1050454650</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6954,7 +6954,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1427497250</v>
+        <v>1425454650</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -6973,7 +6973,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1802497250</v>
+        <v>1800454650</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -6992,7 +6992,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2177497250</v>
+        <v>2175454650</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7011,7 +7011,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2552497250</v>
+        <v>2550454650</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7030,7 +7030,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2927497250</v>
+        <v>2925454650</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7049,7 +7049,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3302497250</v>
+        <v>3300454650</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -8811,13 +8811,13 @@
         <v>29100000</v>
       </c>
       <c r="C5" s="26" t="n">
-        <v>1699000</v>
+        <v>2150000</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>5280000</v>
+        <v>5540000</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>15280000</v>
+        <v>15630000</v>
       </c>
       <c r="F5" s="26" t="n">
         <v>271</v>
@@ -8872,15 +8872,15 @@
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>2149000</v>
+        <v>2600000</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>6166000</v>
+        <v>6426000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>16166000</v>
+        <v>16516000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -8938,15 +8938,15 @@
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>2149000</v>
+        <v>2600000</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>6166000</v>
+        <v>6426000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>16166000</v>
+        <v>16516000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -12880,7 +12880,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>366068715</v>
+        <v>374935315</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>611</v>
@@ -12928,7 +12928,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>8931285</v>
+        <v>64685</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>58931285</v>
+        <v>50064685</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>10839794.4725512</v>
+        <v>9220088.32825916</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13477,7 +13477,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>8931285</v>
+        <v>64685</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>33931285</v>
+        <v>25064685</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>58931285</v>
+        <v>50064685</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13565,7 +13565,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>83931285</v>
+        <v>75064685</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13593,7 +13593,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>108931285</v>
+        <v>100064685</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>133931285</v>
+        <v>125064685</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>158931285</v>
+        <v>150064685</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13681,7 +13681,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>183931285</v>
+        <v>175064685</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13709,7 +13709,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>233931285</v>
+        <v>225064685</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13739,7 +13739,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>283931285</v>
+        <v>275064685</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13767,7 +13767,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>383931285</v>
+        <v>375064685</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13797,7 +13797,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>533931285</v>
+        <v>525064685</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>733931285</v>
+        <v>725064685</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13855,7 +13855,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>933931285</v>
+        <v>925064685</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13883,7 +13883,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1133931285</v>
+        <v>1125064685</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13911,7 +13911,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1333931285</v>
+        <v>1325064685</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13939,7 +13939,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1533931285</v>
+        <v>1525064685</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13967,7 +13967,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1733931285</v>
+        <v>1725064685</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13995,7 +13995,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1933931285</v>
+        <v>1925064685</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14023,7 +14023,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2133931285</v>
+        <v>2125064685</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14051,7 +14051,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2333931285</v>
+        <v>2325064685</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2533931285</v>
+        <v>2525064685</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14107,7 +14107,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2733931285</v>
+        <v>2725064685</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14135,7 +14135,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2933931285</v>
+        <v>2925064685</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14163,7 +14163,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3133931285</v>
+        <v>3125064685</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Hulk secondary, Iso Fest past milestone 18
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5888,7 +5888,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>607823325.89826</v>
+        <v>607879877.245242</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12880,7 +12880,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>374935315</v>
+        <v>376935315</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>611</v>
@@ -12904,7 +12904,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>245</v>
@@ -12928,7 +12928,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>64685</v>
+        <v>23064685</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>50064685</v>
+        <v>48064685</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>9220088.32825916</v>
+        <v>8852584.8571902</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13477,7 +13477,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>64685</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>25064685</v>
+        <v>23064685</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>50064685</v>
+        <v>48064685</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13565,7 +13565,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>75064685</v>
+        <v>73064685</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13593,7 +13593,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>100064685</v>
+        <v>98064685</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>125064685</v>
+        <v>123064685</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>150064685</v>
+        <v>148064685</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13681,7 +13681,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>175064685</v>
+        <v>173064685</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13709,7 +13709,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>225064685</v>
+        <v>223064685</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13739,7 +13739,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>275064685</v>
+        <v>273064685</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13767,7 +13767,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>375064685</v>
+        <v>373064685</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13797,7 +13797,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>525064685</v>
+        <v>523064685</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>725064685</v>
+        <v>723064685</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13855,7 +13855,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>925064685</v>
+        <v>923064685</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13883,7 +13883,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1125064685</v>
+        <v>1123064685</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13911,7 +13911,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1325064685</v>
+        <v>1323064685</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13939,7 +13939,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1525064685</v>
+        <v>1523064685</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13967,7 +13967,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1725064685</v>
+        <v>1723064685</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13995,7 +13995,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1925064685</v>
+        <v>1923064685</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14023,7 +14023,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2125064685</v>
+        <v>2123064685</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14051,7 +14051,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2325064685</v>
+        <v>2323064685</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2525064685</v>
+        <v>2523064685</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14107,7 +14107,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2725064685</v>
+        <v>2723064685</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14135,7 +14135,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2925064685</v>
+        <v>2923064685</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14163,7 +14163,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3125064685</v>
+        <v>3123064685</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Revert Iso Fest estimate to screenshot value
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5888,7 +5888,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>607879877.245242</v>
+        <v>608212087.410189</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12880,7 +12880,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>376935315</v>
+        <v>374935315</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>611</v>
@@ -12904,7 +12904,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>245</v>
@@ -12928,7 +12928,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>23064685</v>
+        <v>64685</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>48064685</v>
+        <v>50064685</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>8852584.8571902</v>
+        <v>9225985.46953892</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13477,7 +13477,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>0</v>
+        <v>64685</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>23064685</v>
+        <v>25064685</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>48064685</v>
+        <v>50064685</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13565,7 +13565,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>73064685</v>
+        <v>75064685</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13593,7 +13593,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>98064685</v>
+        <v>100064685</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>123064685</v>
+        <v>125064685</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>148064685</v>
+        <v>150064685</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13681,7 +13681,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>173064685</v>
+        <v>175064685</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13709,7 +13709,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>223064685</v>
+        <v>225064685</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13739,7 +13739,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>273064685</v>
+        <v>275064685</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13767,7 +13767,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>373064685</v>
+        <v>375064685</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13797,7 +13797,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>523064685</v>
+        <v>525064685</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>723064685</v>
+        <v>725064685</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13855,7 +13855,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>923064685</v>
+        <v>925064685</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13883,7 +13883,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1123064685</v>
+        <v>1125064685</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13911,7 +13911,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1323064685</v>
+        <v>1325064685</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13939,7 +13939,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1523064685</v>
+        <v>1525064685</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13967,7 +13967,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1723064685</v>
+        <v>1725064685</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13995,7 +13995,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1923064685</v>
+        <v>1925064685</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14023,7 +14023,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2123064685</v>
+        <v>2125064685</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14051,7 +14051,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2323064685</v>
+        <v>2325064685</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2523064685</v>
+        <v>2525064685</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14107,7 +14107,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2723064685</v>
+        <v>2725064685</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14135,7 +14135,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2923064685</v>
+        <v>2925064685</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14163,7 +14163,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3123064685</v>
+        <v>3125064685</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Blade T3L5, IV 841M, Iso Fest 391M
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="665">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -187,10 +187,28 @@
     <t xml:space="preserve">Blade (Mighty)</t>
   </si>
   <si>
+    <t xml:space="preserve">Healer and mid damage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only if Iso Fest ions come through</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spider-Woman (Julia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T3 L5 done Oct 12. Abilities on hold. Psionic Webs needs 240 T4s if wanted later</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rachel Cole-Alves</t>
+  </si>
+  <si>
     <t xml:space="preserve">T3 L4</t>
   </si>
   <si>
-    <t xml:space="preserve">Healer and mid damage</t>
+    <t xml:space="preserve">Speed from crits</t>
   </si>
   <si>
     <t xml:space="preserve">Iso-8 to T3 L5</t>
@@ -199,24 +217,6 @@
     <t xml:space="preserve">Purple ions</t>
   </si>
   <si>
-    <t xml:space="preserve">Only if Iso Fest ions come through</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spider-Woman (Julia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T3 L5 done Oct 12. Abilities on hold. Psionic Webs needs 240 T4s if wanted later</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rachel Cole-Alves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speed from crits</t>
-  </si>
-  <si>
     <t xml:space="preserve">5 yellow stars. Only if Iso Fest ions come through</t>
   </si>
   <si>
@@ -1586,6 +1586,9 @@
   </si>
   <si>
     <t xml:space="preserve">Blade (Mighty) Iso-8 to T3 level 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done Oct 13 with Healer secondary. Ion stock estimated after</t>
   </si>
   <si>
     <t xml:space="preserve">Spider-Woman (Julia) Iso-8 to T3 level 5</t>
@@ -3072,25 +3075,25 @@
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="H12" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L12" s="9" t="s">
         <v>52</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>17000000</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3098,7 +3101,7 @@
         <v>4</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>41</v>
@@ -3113,7 +3116,7 @@
         <v>42</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>44</v>
@@ -3128,7 +3131,7 @@
         <v>20</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3136,7 +3139,7 @@
         <v>5</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>41</v>
@@ -3144,19 +3147,19 @@
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="6" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="I14" s="8" t="n">
         <v>17000000</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>25</v>
@@ -3286,7 +3289,7 @@
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="6" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7" t="s">
@@ -3346,7 +3349,7 @@
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="6" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G20" s="7"/>
       <c r="H20" s="7" t="s">
@@ -3376,7 +3379,7 @@
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="6" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="7" t="s">
@@ -5822,7 +5825,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>824545350</v>
+        <v>841545350</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
@@ -5838,7 +5841,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6))+SUMPRODUCT((B13:B76="")*(F13:F76="Claimed"))</f>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>244</v>
@@ -5854,14 +5857,14 @@
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),"All done")</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>245</v>
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">SUMPRODUCT((B13:B76&lt;&gt;"")*(B13:B76&lt;=B6)*(F13:F76&lt;&gt;"Claimed"))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5870,7 +5873,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>454650</v>
+        <v>58454650</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5879,7 +5882,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3300454650</v>
+        <v>3283454650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5888,7 +5891,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>608212087.410189</v>
+        <v>607419603.761061</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6764,7 +6767,7 @@
       <c r="D61" s="11"/>
       <c r="E61" s="23" t="n">
         <f aca="false">IF(B61="","",MAX(0,B61-$B$6))</f>
-        <v>454650</v>
+        <v>0</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>185</v>
@@ -6783,7 +6786,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>75454650</v>
+        <v>58454650</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6802,7 +6805,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>150454650</v>
+        <v>133454650</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6821,7 +6824,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>225454650</v>
+        <v>208454650</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6840,7 +6843,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>300454650</v>
+        <v>283454650</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6859,7 +6862,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>375454650</v>
+        <v>358454650</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6878,7 +6881,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>525454650</v>
+        <v>508454650</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6897,7 +6900,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>675454650</v>
+        <v>658454650</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6916,7 +6919,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>825454650</v>
+        <v>808454650</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6935,7 +6938,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1050454650</v>
+        <v>1033454650</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6954,7 +6957,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1425454650</v>
+        <v>1408454650</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -6973,7 +6976,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1800454650</v>
+        <v>1783454650</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -6992,7 +6995,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2175454650</v>
+        <v>2158454650</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7011,7 +7014,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2550454650</v>
+        <v>2533454650</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7030,7 +7033,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2925454650</v>
+        <v>2908454650</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7049,7 +7052,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3300454650</v>
+        <v>3283454650</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -8526,11 +8529,11 @@
         <v>85000000</v>
       </c>
       <c r="E43" s="24" t="n">
-        <v>51000000</v>
+        <v>68000000</v>
       </c>
       <c r="F43" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D43),MAX(0,D43-E43),0)</f>
-        <v>34000000</v>
+        <v>17000000</v>
       </c>
       <c r="G43" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D43),ROUNDUP(D43/C43,0),"No limit")</f>
@@ -8538,11 +8541,11 @@
       </c>
       <c r="H43" s="21" t="n">
         <f aca="false">IFERROR(INT(E43/C43),0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I43" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F43/C43,0),0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J43" s="10" t="s">
         <v>326</v>
@@ -8698,7 +8701,7 @@
       </c>
       <c r="E49" s="19" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>814302650</v>
+        <v>831302650</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -8709,7 +8712,7 @@
       <c r="E50" s="19"/>
       <c r="F50" s="19" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7122947350</v>
+        <v>7105947350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8719,7 +8722,7 @@
       <c r="E51" s="19"/>
       <c r="F51" s="19" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5210500000</v>
+        <v>5193500000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8811,13 +8814,13 @@
         <v>29100000</v>
       </c>
       <c r="C5" s="26" t="n">
-        <v>2150000</v>
+        <v>440000</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>5540000</v>
+        <v>3830000</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>15630000</v>
+        <v>12990000</v>
       </c>
       <c r="F5" s="26" t="n">
         <v>271</v>
@@ -8872,15 +8875,15 @@
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>2600000</v>
+        <v>890000</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>6426000</v>
+        <v>4716000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>16516000</v>
+        <v>13876000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -8938,15 +8941,15 @@
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>2600000</v>
+        <v>890000</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>6426000</v>
+        <v>4716000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>16516000</v>
+        <v>13876000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -11626,9 +11629,15 @@
       <c r="B97" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="C97" s="26"/>
-      <c r="D97" s="26"/>
-      <c r="E97" s="26"/>
+      <c r="C97" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D97" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E97" s="29" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F97" s="29" t="n">
         <v>0</v>
       </c>
@@ -11642,15 +11651,15 @@
         <v>17000000</v>
       </c>
       <c r="J97" s="10" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="K97" s="14" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B98" s="29" t="n">
         <v>0</v>
@@ -11680,12 +11689,12 @@
         <v>493</v>
       </c>
       <c r="K98" s="14" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B99" s="29" t="n">
         <v>0</v>
@@ -11714,7 +11723,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B100" s="29" t="n">
         <v>13000000</v>
@@ -11738,7 +11747,7 @@
         <v>500</v>
       </c>
       <c r="K100" s="14" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11821,7 +11830,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="15" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="I108" s="19" t="n">
         <f aca="false">SUMIF(J85:J106,"Planned",I85:I106)</f>
@@ -11880,12 +11889,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11899,50 +11908,50 @@
         <v>384</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="E6" s="31" t="s">
         <v>493</v>
@@ -11961,16 +11970,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="E7" s="31" t="s">
         <v>493</v>
@@ -11989,16 +11998,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E8" s="31" t="s">
         <v>493</v>
@@ -12017,16 +12026,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E9" s="31" t="s">
         <v>493</v>
@@ -12045,16 +12054,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E10" s="31" t="s">
         <v>493</v>
@@ -12073,16 +12082,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E11" s="31" t="s">
         <v>493</v>
@@ -12101,16 +12110,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="E12" s="31" t="s">
         <v>493</v>
@@ -12129,16 +12138,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E13" s="31" t="s">
         <v>493</v>
@@ -12157,16 +12166,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="E14" s="31" t="s">
         <v>493</v>
@@ -12185,16 +12194,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E15" s="31" t="s">
         <v>493</v>
@@ -12213,16 +12222,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E16" s="31" t="s">
         <v>493</v>
@@ -12241,16 +12250,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
@@ -12267,16 +12276,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="E18" s="31" t="s">
         <v>493</v>
@@ -12291,16 +12300,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="E19" s="31" t="s">
         <v>493</v>
@@ -12317,16 +12326,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="E20" s="31" t="s">
         <v>493</v>
@@ -12345,21 +12354,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E22" s="31" t="s">
         <v>493</v>
@@ -12376,16 +12385,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
+        <v>569</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>567</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>568</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>566</v>
-      </c>
-      <c r="C23" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>567</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12398,16 +12407,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12420,16 +12429,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E25" s="31" t="s">
         <v>493</v>
@@ -12446,16 +12455,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E26" s="31" t="s">
         <v>493</v>
@@ -12472,16 +12481,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12494,16 +12503,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12516,21 +12525,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12543,16 +12552,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12565,16 +12574,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12587,16 +12596,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="E33" s="31" t="s">
         <v>493</v>
@@ -12611,16 +12620,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12633,16 +12642,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12655,16 +12664,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
+        <v>597</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>591</v>
+      </c>
+      <c r="C36" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="14" t="s">
         <v>596</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>590</v>
-      </c>
-      <c r="C36" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>595</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12677,16 +12686,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12699,16 +12708,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12721,7 +12730,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12758,7 +12767,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12795,7 +12804,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -12839,12 +12848,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12852,10 +12861,10 @@
         <v>239</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12866,13 +12875,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12880,10 +12889,10 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>374935315</v>
+        <v>391445215</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12904,7 +12913,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>245</v>
@@ -12928,12 +12937,12 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>64685</v>
+        <v>8554785</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -12941,20 +12950,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>50064685</v>
+        <v>33554785</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>9225985.46953892</v>
+        <v>6207435.89397831</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12965,19 +12974,19 @@
         <v>248</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -12993,7 +13002,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -13019,7 +13028,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -13045,7 +13054,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -13071,7 +13080,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -13096,10 +13105,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -13124,10 +13133,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -13152,10 +13161,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -13180,10 +13189,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -13208,10 +13217,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -13236,10 +13245,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -13265,7 +13274,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13290,10 +13299,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13318,10 +13327,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
+        <v>635</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>634</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>633</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13346,10 +13355,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13377,7 +13386,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13404,10 +13413,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13434,10 +13443,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13464,10 +13473,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13477,7 +13486,7 @@
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
-        <v>64685</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13488,10 +13497,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13507,7 +13516,7 @@
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>25064685</v>
+        <v>8554785</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13518,7 +13527,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13535,7 +13544,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>50064685</v>
+        <v>33554785</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13546,10 +13555,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13565,7 +13574,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>75064685</v>
+        <v>58554785</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13576,7 +13585,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13593,7 +13602,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>100064685</v>
+        <v>83554785</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13604,10 +13613,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13623,7 +13632,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>125064685</v>
+        <v>108554785</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13634,7 +13643,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13651,7 +13660,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>150064685</v>
+        <v>133554785</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13662,10 +13671,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13681,7 +13690,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>175064685</v>
+        <v>158554785</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13692,7 +13701,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13709,7 +13718,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>225064685</v>
+        <v>208554785</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13720,10 +13729,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13739,7 +13748,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>275064685</v>
+        <v>258554785</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13750,7 +13759,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13767,7 +13776,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>375064685</v>
+        <v>358554785</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13778,10 +13787,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13797,7 +13806,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>525064685</v>
+        <v>508554785</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13808,7 +13817,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13825,7 +13834,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>725064685</v>
+        <v>708554785</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13836,10 +13845,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -13855,7 +13864,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>925064685</v>
+        <v>908554785</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13866,7 +13875,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -13883,7 +13892,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1125064685</v>
+        <v>1108554785</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13894,7 +13903,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -13911,7 +13920,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1325064685</v>
+        <v>1308554785</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13922,7 +13931,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -13939,7 +13948,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1525064685</v>
+        <v>1508554785</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13950,7 +13959,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -13967,7 +13976,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1725064685</v>
+        <v>1708554785</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13978,7 +13987,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -13995,7 +14004,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1925064685</v>
+        <v>1908554785</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14006,7 +14015,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -14023,7 +14032,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2125064685</v>
+        <v>2108554785</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14034,7 +14043,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -14051,7 +14060,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2325064685</v>
+        <v>2308554785</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14062,7 +14071,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -14079,7 +14088,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2525064685</v>
+        <v>2508554785</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14090,7 +14099,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -14107,7 +14116,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2725064685</v>
+        <v>2708554785</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14118,7 +14127,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -14135,7 +14144,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2925064685</v>
+        <v>2908554785</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14146,7 +14155,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -14163,12 +14172,12 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3125064685</v>
+        <v>3108554785</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Symbiote secondaries, Iso Fest 403M, ion stock
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5891,7 +5891,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>607419603.761061</v>
+        <v>608316055.220006</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8811,16 +8811,16 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>29100000</v>
+        <v>28200000</v>
       </c>
       <c r="C5" s="26" t="n">
-        <v>440000</v>
+        <v>947600</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>3830000</v>
+        <v>6100000</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>12990000</v>
+        <v>14890000</v>
       </c>
       <c r="F5" s="26" t="n">
         <v>271</v>
@@ -8871,19 +8871,19 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>45850000</v>
+        <v>44950000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>890000</v>
+        <v>1397600</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>4716000</v>
+        <v>6986000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>13876000</v>
+        <v>15776000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -8937,19 +8937,19 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>45850000</v>
+        <v>44950000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>890000</v>
+        <v>1397600</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>4716000</v>
+        <v>6986000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>13876000</v>
+        <v>15776000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -12889,7 +12889,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>391445215</v>
+        <v>403693215</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>612</v>
@@ -12900,11 +12900,11 @@
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
-        <v>2800000</v>
+        <v>1400000</v>
       </c>
       <c r="G6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>3800000</v>
+        <v>1900000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12913,7 +12913,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>245</v>
@@ -12937,7 +12937,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>8554785</v>
+        <v>21306785</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>33554785</v>
+        <v>21306785</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12963,7 +12963,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>6207435.89397831</v>
+        <v>3947445.84607364</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13482,7 +13482,7 @@
       <c r="F30" s="26"/>
       <c r="G30" s="26"/>
       <c r="H30" s="10" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I30" s="23" t="n">
         <f aca="false">IF(B30="","",MAX(0,B30-$B$6))</f>
@@ -13512,11 +13512,11 @@
         <v>1900000</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I31" s="23" t="n">
         <f aca="false">IF(B31="","",MAX(0,B31-$B$6))</f>
-        <v>8554785</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13544,7 +13544,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>33554785</v>
+        <v>21306785</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>58554785</v>
+        <v>46306785</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13602,7 +13602,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>83554785</v>
+        <v>71306785</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13632,7 +13632,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>108554785</v>
+        <v>96306785</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>133554785</v>
+        <v>121306785</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13690,7 +13690,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>158554785</v>
+        <v>146306785</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13718,7 +13718,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>208554785</v>
+        <v>196306785</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13748,7 +13748,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>258554785</v>
+        <v>246306785</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>358554785</v>
+        <v>346306785</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13806,7 +13806,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>508554785</v>
+        <v>496306785</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13834,7 +13834,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>708554785</v>
+        <v>696306785</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13864,7 +13864,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>908554785</v>
+        <v>896306785</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13892,7 +13892,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1108554785</v>
+        <v>1096306785</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13920,7 +13920,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1308554785</v>
+        <v>1296306785</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1508554785</v>
+        <v>1496306785</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13976,7 +13976,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1708554785</v>
+        <v>1696306785</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14004,7 +14004,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1908554785</v>
+        <v>1896306785</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2108554785</v>
+        <v>2096306785</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14060,7 +14060,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2308554785</v>
+        <v>2296306785</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2508554785</v>
+        <v>2496306785</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14116,7 +14116,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2708554785</v>
+        <v>2696306785</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14144,7 +14144,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2908554785</v>
+        <v>2896306785</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3108554785</v>
+        <v>3096306785</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Iso-8 campaign auto wins
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5891,7 +5891,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>608316055.220006</v>
+        <v>624728540.017767</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8811,7 +8811,7 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>28200000</v>
+        <v>28219550</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>947600</v>
@@ -8871,7 +8871,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>44950000</v>
+        <v>44969550</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8937,7 +8937,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>44950000</v>
+        <v>44969550</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -10952,7 +10952,7 @@
         <v>484</v>
       </c>
       <c r="B69" s="29" t="n">
-        <v>342975</v>
+        <v>362525</v>
       </c>
       <c r="C69" s="29" t="n">
         <v>0</v>
@@ -12963,7 +12963,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>3947445.84607364</v>
+        <v>4053948.70402598</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Midday campaigns, Iso-8 daily done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="665">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1297" uniqueCount="665">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -5891,7 +5891,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>624728540.017767</v>
+        <v>630727525.406508</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8811,7 +8811,7 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>28219550</v>
+        <v>28260000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>947600</v>
@@ -8823,10 +8823,10 @@
         <v>14890000</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>271</v>
+        <v>303</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>1051</v>
+        <v>1067</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>2221</v>
@@ -8871,7 +8871,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>44969550</v>
+        <v>45010000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8887,11 +8887,11 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
-        <v>271</v>
+        <v>303</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>1151</v>
+        <v>1167</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
@@ -8937,7 +8937,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>44969550</v>
+        <v>45010000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8953,11 +8953,11 @@
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>271</v>
+        <v>303</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>1151</v>
+        <v>1167</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
@@ -10952,7 +10952,7 @@
         <v>484</v>
       </c>
       <c r="B69" s="29" t="n">
-        <v>362525</v>
+        <v>407000</v>
       </c>
       <c r="C69" s="29" t="n">
         <v>0</v>
@@ -10964,10 +10964,10 @@
         <v>0</v>
       </c>
       <c r="F69" s="29" t="n">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="G69" s="29" t="n">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="H69" s="29" t="n">
         <v>0</v>
@@ -12317,7 +12317,9 @@
       <c r="F19" s="31" t="s">
         <v>493</v>
       </c>
-      <c r="G19" s="31"/>
+      <c r="G19" s="31" t="s">
+        <v>493</v>
+      </c>
       <c r="H19" s="31"/>
       <c r="I19" s="31"/>
       <c r="J19" s="31"/>
@@ -12376,7 +12378,9 @@
       <c r="F22" s="31" t="s">
         <v>493</v>
       </c>
-      <c r="G22" s="31"/>
+      <c r="G22" s="31" t="s">
+        <v>493</v>
+      </c>
       <c r="H22" s="31"/>
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
@@ -12742,7 +12746,7 @@
       </c>
       <c r="G40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(G5:G38="Done"))</f>
-        <v>1550000</v>
+        <v>1575000</v>
       </c>
       <c r="H40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(H5:H38="Done"))</f>
@@ -12963,7 +12967,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>4053948.70402598</v>
+        <v>4092876.93473278</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Night Thrasher level 105 and gear tier 20
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1297" uniqueCount="665">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="669">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1571,6 +1571,18 @@
   </si>
   <si>
     <t xml:space="preserve">Check cost in game</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Night Thrasher to level 105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct 13, Daring Warriors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Night Thrasher to gear tier 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct 13. Used 75 of each crimson tech material</t>
   </si>
   <si>
     <t xml:space="preserve">Hulk Iso-8 to T3 level 5</t>
@@ -5891,7 +5903,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>630727525.406508</v>
+        <v>631360242.44754</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8759,7 +8771,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K110"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -8811,7 +8823,7 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>28260000</v>
+        <v>14400000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>947600</v>
@@ -8823,13 +8835,13 @@
         <v>14890000</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>2221</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8871,7 +8883,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>45010000</v>
+        <v>31150000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8887,15 +8899,15 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>2306</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8903,31 +8915,31 @@
         <v>394</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$106,"Planned",B85:B106)</f>
+        <f aca="false">SUMIF($J$85:$J$108,"Planned",B85:B108)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$106,"Planned",C85:C106)</f>
+        <f aca="false">SUMIF($J$85:$J$108,"Planned",C85:C108)</f>
         <v>0</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$106,"Planned",D85:D106)</f>
+        <f aca="false">SUMIF($J$85:$J$108,"Planned",D85:D108)</f>
         <v>0</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$106,"Planned",E85:E106)</f>
+        <f aca="false">SUMIF($J$85:$J$108,"Planned",E85:E108)</f>
         <v>0</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$106,"Planned",F85:F106)</f>
+        <f aca="false">SUMIF($J$85:$J$108,"Planned",F85:F108)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$106,"Planned",G85:G106)</f>
+        <f aca="false">SUMIF($J$85:$J$108,"Planned",G85:G108)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$106,"Planned",H85:H106)</f>
+        <f aca="false">SUMIF($J$85:$J$108,"Planned",H85:H108)</f>
         <v>0</v>
       </c>
     </row>
@@ -8937,7 +8949,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>45010000</v>
+        <v>31150000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8953,15 +8965,15 @@
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>2306</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11557,28 +11569,28 @@
         <v>513</v>
       </c>
       <c r="B95" s="29" t="n">
-        <v>0</v>
+        <v>9800000</v>
       </c>
       <c r="C95" s="29" t="n">
-        <v>1710500</v>
+        <v>0</v>
       </c>
       <c r="D95" s="29" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E95" s="29" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F95" s="29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G95" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H95" s="29" t="n">
-        <v>0</v>
+        <v>979</v>
       </c>
       <c r="I95" s="29" t="n">
-        <v>17000000</v>
+        <v>0</v>
       </c>
       <c r="J95" s="10" t="s">
         <v>493</v>
@@ -11592,16 +11604,16 @@
         <v>515</v>
       </c>
       <c r="B96" s="29" t="n">
-        <v>0</v>
+        <v>4092000</v>
       </c>
       <c r="C96" s="29" t="n">
-        <v>1370000</v>
+        <v>0</v>
       </c>
       <c r="D96" s="29" t="n">
-        <v>1370000</v>
+        <v>0</v>
       </c>
       <c r="E96" s="29" t="n">
-        <v>2130000</v>
+        <v>0</v>
       </c>
       <c r="F96" s="29" t="n">
         <v>0</v>
@@ -11613,7 +11625,7 @@
         <v>0</v>
       </c>
       <c r="I96" s="29" t="n">
-        <v>17000000</v>
+        <v>0</v>
       </c>
       <c r="J96" s="10" t="s">
         <v>493</v>
@@ -11630,7 +11642,7 @@
         <v>0</v>
       </c>
       <c r="C97" s="29" t="n">
-        <v>1710000</v>
+        <v>1710500</v>
       </c>
       <c r="D97" s="29" t="n">
         <v>1710000</v>
@@ -11665,13 +11677,13 @@
         <v>0</v>
       </c>
       <c r="C98" s="29" t="n">
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="D98" s="29" t="n">
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="E98" s="29" t="n">
-        <v>2640000</v>
+        <v>2130000</v>
       </c>
       <c r="F98" s="29" t="n">
         <v>0</v>
@@ -11699,9 +11711,15 @@
       <c r="B99" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="C99" s="26"/>
-      <c r="D99" s="26"/>
-      <c r="E99" s="26"/>
+      <c r="C99" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D99" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E99" s="29" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F99" s="29" t="n">
         <v>0</v>
       </c>
@@ -11715,66 +11733,104 @@
         <v>17000000</v>
       </c>
       <c r="J99" s="10" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="K99" s="14" t="s">
-        <v>512</v>
+        <v>522</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B100" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C100" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D100" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E100" s="29" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="F100" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" s="29" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J100" s="10" t="s">
+        <v>493</v>
+      </c>
+      <c r="K100" s="14" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="11" t="s">
+        <v>525</v>
+      </c>
+      <c r="B101" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C101" s="26"/>
+      <c r="D101" s="26"/>
+      <c r="E101" s="26"/>
+      <c r="F101" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" s="29" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J101" s="10" t="s">
+        <v>500</v>
+      </c>
+      <c r="K101" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="11" t="s">
+        <v>526</v>
+      </c>
+      <c r="B102" s="29" t="n">
         <v>13000000</v>
       </c>
-      <c r="C100" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D100" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E100" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F100" s="26"/>
-      <c r="G100" s="26"/>
-      <c r="H100" s="26"/>
-      <c r="I100" s="29" t="n">
+      <c r="C102" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" s="26"/>
+      <c r="G102" s="26"/>
+      <c r="H102" s="26"/>
+      <c r="I102" s="29" t="n">
         <v>8000000</v>
       </c>
-      <c r="J100" s="10" t="s">
+      <c r="J102" s="10" t="s">
         <v>500</v>
       </c>
-      <c r="K100" s="14" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="11"/>
-      <c r="B101" s="29"/>
-      <c r="C101" s="29"/>
-      <c r="D101" s="29"/>
-      <c r="E101" s="29"/>
-      <c r="F101" s="29"/>
-      <c r="G101" s="29"/>
-      <c r="H101" s="29"/>
-      <c r="I101" s="29"/>
-      <c r="J101" s="10"/>
-      <c r="K101" s="11"/>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="11"/>
-      <c r="B102" s="29"/>
-      <c r="C102" s="29"/>
-      <c r="D102" s="29"/>
-      <c r="E102" s="29"/>
-      <c r="F102" s="29"/>
-      <c r="G102" s="29"/>
-      <c r="H102" s="29"/>
-      <c r="I102" s="29"/>
-      <c r="J102" s="10"/>
-      <c r="K102" s="11"/>
+      <c r="K102" s="14" t="s">
+        <v>527</v>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="11"/>
@@ -11828,12 +11884,38 @@
       <c r="J106" s="10"/>
       <c r="K106" s="11"/>
     </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="11"/>
+      <c r="B107" s="29"/>
+      <c r="C107" s="29"/>
+      <c r="D107" s="29"/>
+      <c r="E107" s="29"/>
+      <c r="F107" s="29"/>
+      <c r="G107" s="29"/>
+      <c r="H107" s="29"/>
+      <c r="I107" s="29"/>
+      <c r="J107" s="10"/>
+      <c r="K107" s="11"/>
+    </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="15" t="s">
-        <v>524</v>
-      </c>
-      <c r="I108" s="19" t="n">
-        <f aca="false">SUMIF(J85:J106,"Planned",I85:I106)</f>
+      <c r="A108" s="11"/>
+      <c r="B108" s="29"/>
+      <c r="C108" s="29"/>
+      <c r="D108" s="29"/>
+      <c r="E108" s="29"/>
+      <c r="F108" s="29"/>
+      <c r="G108" s="29"/>
+      <c r="H108" s="29"/>
+      <c r="I108" s="29"/>
+      <c r="J108" s="10"/>
+      <c r="K108" s="11"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="15" t="s">
+        <v>528</v>
+      </c>
+      <c r="I110" s="19" t="n">
+        <f aca="false">SUMIF(J85:J108,"Planned",I85:I108)</f>
         <v>20000000</v>
       </c>
     </row>
@@ -11843,7 +11925,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J85:J106">
+  <conditionalFormatting sqref="J85:J108">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
@@ -11858,7 +11940,7 @@
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J85:J106" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J85:J108" type="list">
       <formula1>"Planned,If needed,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11889,12 +11971,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11908,50 +11990,50 @@
         <v>384</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="E6" s="31" t="s">
         <v>493</v>
@@ -11970,16 +12052,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="E7" s="31" t="s">
         <v>493</v>
@@ -11998,16 +12080,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
+        <v>546</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>542</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>538</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="E8" s="31" t="s">
         <v>493</v>
@@ -12026,16 +12108,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="E9" s="31" t="s">
         <v>493</v>
@@ -12054,16 +12136,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="E10" s="31" t="s">
         <v>493</v>
@@ -12082,16 +12164,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="E11" s="31" t="s">
         <v>493</v>
@@ -12110,16 +12192,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="E12" s="31" t="s">
         <v>493</v>
@@ -12138,16 +12220,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="E13" s="31" t="s">
         <v>493</v>
@@ -12166,16 +12248,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="E14" s="31" t="s">
         <v>493</v>
@@ -12194,16 +12276,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="E15" s="31" t="s">
         <v>493</v>
@@ -12222,16 +12304,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="E16" s="31" t="s">
         <v>493</v>
@@ -12250,16 +12332,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
@@ -12276,16 +12358,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="E18" s="31" t="s">
         <v>493</v>
@@ -12300,16 +12382,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="B19" s="12" t="s">
         <v>561</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>557</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="E19" s="31" t="s">
         <v>493</v>
@@ -12328,16 +12410,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="E20" s="31" t="s">
         <v>493</v>
@@ -12356,21 +12438,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="E22" s="31" t="s">
         <v>493</v>
@@ -12389,16 +12471,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12411,16 +12493,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12433,16 +12515,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="E25" s="31" t="s">
         <v>493</v>
@@ -12459,16 +12541,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E26" s="31" t="s">
         <v>493</v>
@@ -12485,16 +12567,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12507,16 +12589,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12529,21 +12611,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12556,16 +12638,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12578,16 +12660,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
+        <v>592</v>
+      </c>
+      <c r="B32" s="12" t="s">
         <v>588</v>
       </c>
-      <c r="B32" s="12" t="s">
-        <v>584</v>
-      </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12600,16 +12682,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="E33" s="31" t="s">
         <v>493</v>
@@ -12624,16 +12706,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12646,16 +12728,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
+        <v>599</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>595</v>
       </c>
-      <c r="B35" s="12" t="s">
-        <v>591</v>
-      </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12668,16 +12750,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12690,16 +12772,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12712,16 +12794,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12734,7 +12816,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12771,7 +12853,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12808,7 +12890,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
     </row>
   </sheetData>
@@ -12852,12 +12934,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12865,10 +12947,10 @@
         <v>239</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12879,13 +12961,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12896,7 +12978,7 @@
         <v>403693215</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12946,7 +13028,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -12954,7 +13036,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -12963,11 +13045,11 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>4092876.93473278</v>
+        <v>4096982.72288234</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12978,19 +13060,19 @@
         <v>248</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -13006,7 +13088,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -13032,7 +13114,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -13058,7 +13140,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -13084,7 +13166,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -13109,10 +13191,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -13137,10 +13219,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -13165,10 +13247,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -13193,10 +13275,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -13221,10 +13303,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -13249,10 +13331,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -13278,7 +13360,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13303,10 +13385,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13331,10 +13413,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13359,10 +13441,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13390,7 +13472,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13417,10 +13499,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13447,10 +13529,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
+        <v>642</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>638</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>634</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13477,10 +13559,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13501,10 +13583,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13531,7 +13613,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13559,10 +13641,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13589,7 +13671,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13617,10 +13699,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13647,7 +13729,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13675,10 +13757,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13705,7 +13787,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13733,10 +13815,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13763,7 +13845,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13791,10 +13873,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13821,7 +13903,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13849,10 +13931,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -13879,7 +13961,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -13907,7 +13989,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -13935,7 +14017,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -13963,7 +14045,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -13991,7 +14073,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -14019,7 +14101,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -14047,7 +14129,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -14075,7 +14157,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -14103,7 +14185,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -14131,7 +14213,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -14159,7 +14241,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -14181,7 +14263,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gold spent on Night Thrasher counted in both events
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5837,14 +5837,14 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>841545350</v>
+        <v>855437350</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6035045350</v>
+        <v>6048937350</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>58454650</v>
+        <v>44562650</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3283454650</v>
+        <v>3269562650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>631360242.44754</v>
+        <v>628712708.283145</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6798,7 +6798,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>58454650</v>
+        <v>44562650</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6817,7 +6817,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>133454650</v>
+        <v>119562650</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6836,7 +6836,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>208454650</v>
+        <v>194562650</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6855,7 +6855,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>283454650</v>
+        <v>269562650</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6874,7 +6874,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>358454650</v>
+        <v>344562650</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6893,7 +6893,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>508454650</v>
+        <v>494562650</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6912,7 +6912,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>658454650</v>
+        <v>644562650</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6931,7 +6931,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>808454650</v>
+        <v>794562650</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6950,7 +6950,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1033454650</v>
+        <v>1019562650</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6969,7 +6969,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1408454650</v>
+        <v>1394562650</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -6988,7 +6988,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1783454650</v>
+        <v>1769562650</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -7007,7 +7007,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2158454650</v>
+        <v>2144562650</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7026,7 +7026,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2533454650</v>
+        <v>2519562650</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7045,7 +7045,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2908454650</v>
+        <v>2894562650</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7064,7 +7064,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3283454650</v>
+        <v>3269562650</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -7245,11 +7245,11 @@
         <v>1000000000</v>
       </c>
       <c r="E7" s="24" t="n">
-        <v>52952650</v>
+        <v>66844650</v>
       </c>
       <c r="F7" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D7),MAX(0,D7-E7),0)</f>
-        <v>947047350</v>
+        <v>933155350</v>
       </c>
       <c r="G7" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D7),ROUNDUP(D7/C7,0),"No limit")</f>
@@ -7257,11 +7257,11 @@
       </c>
       <c r="H7" s="21" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>52952650</v>
+        <v>66844650</v>
       </c>
       <c r="I7" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>947047350</v>
+        <v>933155350</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>330</v>
@@ -8713,7 +8713,7 @@
       </c>
       <c r="E49" s="19" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>831302650</v>
+        <v>845194650</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -8724,7 +8724,7 @@
       <c r="E50" s="19"/>
       <c r="F50" s="19" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7105947350</v>
+        <v>7092055350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12975,7 +12975,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>403693215</v>
+        <v>417585215</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>616</v>
@@ -13023,7 +13023,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>21306785</v>
+        <v>7414785</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>21306785</v>
+        <v>7414785</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13049,7 +13049,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>4096982.72288234</v>
+        <v>1425808.30133719</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13630,7 +13630,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>21306785</v>
+        <v>7414785</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>46306785</v>
+        <v>32414785</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13688,7 +13688,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>71306785</v>
+        <v>57414785</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13718,7 +13718,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>96306785</v>
+        <v>82414785</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13746,7 +13746,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>121306785</v>
+        <v>107414785</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>146306785</v>
+        <v>132414785</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13804,7 +13804,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>196306785</v>
+        <v>182414785</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13834,7 +13834,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>246306785</v>
+        <v>232414785</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13862,7 +13862,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>346306785</v>
+        <v>332414785</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13892,7 +13892,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>496306785</v>
+        <v>482414785</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13920,7 +13920,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>696306785</v>
+        <v>682414785</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13950,7 +13950,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>896306785</v>
+        <v>882414785</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13978,7 +13978,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1096306785</v>
+        <v>1082414785</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14006,7 +14006,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1296306785</v>
+        <v>1282414785</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14034,7 +14034,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1496306785</v>
+        <v>1482414785</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14062,7 +14062,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1696306785</v>
+        <v>1682414785</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14090,7 +14090,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1896306785</v>
+        <v>1882414785</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14118,7 +14118,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2096306785</v>
+        <v>2082414785</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14146,7 +14146,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2296306785</v>
+        <v>2282414785</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2496306785</v>
+        <v>2482414785</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14202,7 +14202,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2696306785</v>
+        <v>2682414785</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14230,7 +14230,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2896306785</v>
+        <v>2882414785</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14258,7 +14258,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3096306785</v>
+        <v>3082414785</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Jim level 80 GT15, event points, Rachel planned
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="672">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1585,6 +1585,18 @@
     <t xml:space="preserve">Oct 13. Used 75 of each crimson tech material</t>
   </si>
   <si>
+    <t xml:space="preserve">Human Torch (Jim) to level 80 and gear tier 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct 13 for Breaker gear tier 15 task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rachel Cole-Alves Iso-8 to T3 level 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After claiming Iso Fest milestone 20</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hulk Iso-8 to T3 level 5</t>
   </si>
   <si>
@@ -1607,9 +1619,6 @@
   </si>
   <si>
     <t xml:space="preserve">Done Oct 12. Plus 500 ion 1 to unlock the T4 matrix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rachel Cole-Alves Iso-8 to T3 level 5</t>
   </si>
   <si>
     <t xml:space="preserve">One Amazing Avenger to level 110</t>
@@ -5837,14 +5846,14 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>855437350</v>
+        <v>866257350</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6048937350</v>
+        <v>6059757350</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5885,7 +5894,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>44562650</v>
+        <v>33742650</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5894,7 +5903,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3269562650</v>
+        <v>3258742650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5903,7 +5912,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>628712708.283145</v>
+        <v>628946055.252547</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6798,7 +6807,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>44562650</v>
+        <v>33742650</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6817,7 +6826,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>119562650</v>
+        <v>108742650</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6836,7 +6845,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>194562650</v>
+        <v>183742650</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6855,7 +6864,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>269562650</v>
+        <v>258742650</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6874,7 +6883,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>344562650</v>
+        <v>333742650</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6893,7 +6902,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>494562650</v>
+        <v>483742650</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6912,7 +6921,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>644562650</v>
+        <v>633742650</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6931,7 +6940,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>794562650</v>
+        <v>783742650</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6950,7 +6959,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1019562650</v>
+        <v>1008742650</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6969,7 +6978,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1394562650</v>
+        <v>1383742650</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -6988,7 +6997,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1769562650</v>
+        <v>1758742650</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -7007,7 +7016,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2144562650</v>
+        <v>2133742650</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7026,7 +7035,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2519562650</v>
+        <v>2508742650</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7045,7 +7054,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2894562650</v>
+        <v>2883742650</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7064,7 +7073,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3269562650</v>
+        <v>3258742650</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -8771,7 +8780,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K110"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -8823,7 +8832,7 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>14400000</v>
+        <v>13180000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>947600</v>
@@ -8835,13 +8844,13 @@
         <v>14890000</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>1242</v>
+        <v>560</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8883,7 +8892,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>31150000</v>
+        <v>29930000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8899,15 +8908,15 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">G5+G6</f>
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>1327</v>
+        <v>645</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8915,31 +8924,31 @@
         <v>394</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$108,"Planned",B85:B108)</f>
+        <f aca="false">SUMIF($J$85:$J$110,"Planned",B85:B110)</f>
         <v>0</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$108,"Planned",C85:C108)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$85:$J$110,"Planned",C85:C110)</f>
+        <v>1710000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$108,"Planned",D85:D108)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$85:$J$110,"Planned",D85:D110)</f>
+        <v>1710000</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$108,"Planned",E85:E108)</f>
-        <v>0</v>
+        <f aca="false">SUMIF($J$85:$J$110,"Planned",E85:E110)</f>
+        <v>2640000</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$108,"Planned",F85:F108)</f>
+        <f aca="false">SUMIF($J$85:$J$110,"Planned",F85:F110)</f>
         <v>0</v>
       </c>
       <c r="G8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$108,"Planned",G85:G108)</f>
+        <f aca="false">SUMIF($J$85:$J$110,"Planned",G85:G110)</f>
         <v>0</v>
       </c>
       <c r="H8" s="27" t="n">
-        <f aca="false">SUMIF($J$85:$J$108,"Planned",H85:H108)</f>
+        <f aca="false">SUMIF($J$85:$J$110,"Planned",H85:H110)</f>
         <v>0</v>
       </c>
     </row>
@@ -8949,31 +8958,31 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>31150000</v>
+        <v>29930000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>1397600</v>
+        <v>-312400</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>6986000</v>
+        <v>5276000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>15776000</v>
+        <v>13136000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">G7-G8</f>
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>1327</v>
+        <v>645</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11639,28 +11648,28 @@
         <v>517</v>
       </c>
       <c r="B97" s="29" t="n">
-        <v>0</v>
+        <v>7820000</v>
       </c>
       <c r="C97" s="29" t="n">
-        <v>1710500</v>
+        <v>0</v>
       </c>
       <c r="D97" s="29" t="n">
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E97" s="29" t="n">
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F97" s="29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G97" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H97" s="29" t="n">
-        <v>0</v>
+        <v>682</v>
       </c>
       <c r="I97" s="29" t="n">
-        <v>17000000</v>
+        <v>0</v>
       </c>
       <c r="J97" s="10" t="s">
         <v>493</v>
@@ -11677,13 +11686,13 @@
         <v>0</v>
       </c>
       <c r="C98" s="29" t="n">
-        <v>1370000</v>
+        <v>1710000</v>
       </c>
       <c r="D98" s="29" t="n">
-        <v>1370000</v>
+        <v>1710000</v>
       </c>
       <c r="E98" s="29" t="n">
-        <v>2130000</v>
+        <v>2640000</v>
       </c>
       <c r="F98" s="29" t="n">
         <v>0</v>
@@ -11698,7 +11707,7 @@
         <v>17000000</v>
       </c>
       <c r="J98" s="10" t="s">
-        <v>493</v>
+        <v>503</v>
       </c>
       <c r="K98" s="14" t="s">
         <v>520</v>
@@ -11712,7 +11721,7 @@
         <v>0</v>
       </c>
       <c r="C99" s="29" t="n">
-        <v>1710000</v>
+        <v>1710500</v>
       </c>
       <c r="D99" s="29" t="n">
         <v>1710000</v>
@@ -11747,13 +11756,13 @@
         <v>0</v>
       </c>
       <c r="C100" s="29" t="n">
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="D100" s="29" t="n">
-        <v>1710000</v>
+        <v>1370000</v>
       </c>
       <c r="E100" s="29" t="n">
-        <v>2640000</v>
+        <v>2130000</v>
       </c>
       <c r="F100" s="29" t="n">
         <v>0</v>
@@ -11781,9 +11790,15 @@
       <c r="B101" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="C101" s="26"/>
-      <c r="D101" s="26"/>
-      <c r="E101" s="26"/>
+      <c r="C101" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D101" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E101" s="29" t="n">
+        <v>2640000</v>
+      </c>
       <c r="F101" s="29" t="n">
         <v>0</v>
       </c>
@@ -11797,66 +11812,104 @@
         <v>17000000</v>
       </c>
       <c r="J101" s="10" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="K101" s="14" t="s">
-        <v>512</v>
+        <v>526</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B102" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C102" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="D102" s="29" t="n">
+        <v>1710000</v>
+      </c>
+      <c r="E102" s="29" t="n">
+        <v>2640000</v>
+      </c>
+      <c r="F102" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" s="29" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J102" s="10" t="s">
+        <v>493</v>
+      </c>
+      <c r="K102" s="14" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="11" t="s">
+        <v>519</v>
+      </c>
+      <c r="B103" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C103" s="26"/>
+      <c r="D103" s="26"/>
+      <c r="E103" s="26"/>
+      <c r="F103" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" s="29" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J103" s="10" t="s">
+        <v>500</v>
+      </c>
+      <c r="K103" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="11" t="s">
+        <v>529</v>
+      </c>
+      <c r="B104" s="29" t="n">
         <v>13000000</v>
       </c>
-      <c r="C102" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D102" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E102" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F102" s="26"/>
-      <c r="G102" s="26"/>
-      <c r="H102" s="26"/>
-      <c r="I102" s="29" t="n">
+      <c r="C104" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" s="26"/>
+      <c r="G104" s="26"/>
+      <c r="H104" s="26"/>
+      <c r="I104" s="29" t="n">
         <v>8000000</v>
       </c>
-      <c r="J102" s="10" t="s">
+      <c r="J104" s="10" t="s">
         <v>500</v>
       </c>
-      <c r="K102" s="14" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="11"/>
-      <c r="B103" s="29"/>
-      <c r="C103" s="29"/>
-      <c r="D103" s="29"/>
-      <c r="E103" s="29"/>
-      <c r="F103" s="29"/>
-      <c r="G103" s="29"/>
-      <c r="H103" s="29"/>
-      <c r="I103" s="29"/>
-      <c r="J103" s="10"/>
-      <c r="K103" s="11"/>
-    </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="11"/>
-      <c r="B104" s="29"/>
-      <c r="C104" s="29"/>
-      <c r="D104" s="29"/>
-      <c r="E104" s="29"/>
-      <c r="F104" s="29"/>
-      <c r="G104" s="29"/>
-      <c r="H104" s="29"/>
-      <c r="I104" s="29"/>
-      <c r="J104" s="10"/>
-      <c r="K104" s="11"/>
+      <c r="K104" s="14" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="11"/>
@@ -11910,13 +11963,39 @@
       <c r="J108" s="10"/>
       <c r="K108" s="11"/>
     </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="11"/>
+      <c r="B109" s="29"/>
+      <c r="C109" s="29"/>
+      <c r="D109" s="29"/>
+      <c r="E109" s="29"/>
+      <c r="F109" s="29"/>
+      <c r="G109" s="29"/>
+      <c r="H109" s="29"/>
+      <c r="I109" s="29"/>
+      <c r="J109" s="10"/>
+      <c r="K109" s="11"/>
+    </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="15" t="s">
-        <v>528</v>
-      </c>
-      <c r="I110" s="19" t="n">
-        <f aca="false">SUMIF(J85:J108,"Planned",I85:I108)</f>
-        <v>20000000</v>
+      <c r="A110" s="11"/>
+      <c r="B110" s="29"/>
+      <c r="C110" s="29"/>
+      <c r="D110" s="29"/>
+      <c r="E110" s="29"/>
+      <c r="F110" s="29"/>
+      <c r="G110" s="29"/>
+      <c r="H110" s="29"/>
+      <c r="I110" s="29"/>
+      <c r="J110" s="10"/>
+      <c r="K110" s="11"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="15" t="s">
+        <v>531</v>
+      </c>
+      <c r="I112" s="19" t="n">
+        <f aca="false">SUMIF(J85:J110,"Planned",I85:I110)</f>
+        <v>37000000</v>
       </c>
     </row>
   </sheetData>
@@ -11925,7 +12004,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J85:J108">
+  <conditionalFormatting sqref="J85:J110">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Done"</formula>
     </cfRule>
@@ -11940,7 +12019,7 @@
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J85:J108" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J85:J110" type="list">
       <formula1>"Planned,If needed,Done,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11971,12 +12050,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11990,50 +12069,50 @@
         <v>384</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="E6" s="31" t="s">
         <v>493</v>
@@ -12052,16 +12131,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="E7" s="31" t="s">
         <v>493</v>
@@ -12080,16 +12159,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="E8" s="31" t="s">
         <v>493</v>
@@ -12108,16 +12187,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="E9" s="31" t="s">
         <v>493</v>
@@ -12136,16 +12215,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="E10" s="31" t="s">
         <v>493</v>
@@ -12164,16 +12243,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="E11" s="31" t="s">
         <v>493</v>
@@ -12192,16 +12271,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="E12" s="31" t="s">
         <v>493</v>
@@ -12220,16 +12299,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="E13" s="31" t="s">
         <v>493</v>
@@ -12248,16 +12327,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="E14" s="31" t="s">
         <v>493</v>
@@ -12276,16 +12355,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="E15" s="31" t="s">
         <v>493</v>
@@ -12304,16 +12383,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="E16" s="31" t="s">
         <v>493</v>
@@ -12332,16 +12411,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
@@ -12358,16 +12437,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E18" s="31" t="s">
         <v>493</v>
@@ -12382,16 +12461,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E19" s="31" t="s">
         <v>493</v>
@@ -12410,16 +12489,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="E20" s="31" t="s">
         <v>493</v>
@@ -12438,21 +12517,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="E22" s="31" t="s">
         <v>493</v>
@@ -12471,16 +12550,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12493,16 +12572,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
+        <v>577</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>574</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>571</v>
-      </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12515,16 +12594,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="E25" s="31" t="s">
         <v>493</v>
@@ -12541,16 +12620,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E26" s="31" t="s">
         <v>493</v>
@@ -12567,16 +12646,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12589,16 +12668,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12611,21 +12690,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12638,16 +12717,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12660,16 +12739,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12682,16 +12761,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="E33" s="31" t="s">
         <v>493</v>
@@ -12706,16 +12785,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12728,16 +12807,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12750,16 +12829,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12772,16 +12851,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12794,16 +12873,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12816,7 +12895,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12853,7 +12932,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12890,7 +12969,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
     </row>
   </sheetData>
@@ -12934,12 +13013,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12947,10 +13026,10 @@
         <v>239</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12961,13 +13040,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12975,10 +13054,10 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>417585215</v>
+        <v>433710215</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
@@ -12999,22 +13078,22 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>245</v>
       </c>
       <c r="E7" s="19" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>0</v>
+        <v>1300000</v>
       </c>
       <c r="F7" s="19" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
-        <v>0</v>
+        <v>1400000</v>
       </c>
       <c r="G7" s="19" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>0</v>
+        <v>1900000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13023,12 +13102,12 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>7414785</v>
+        <v>16289785</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -13036,20 +13115,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
-        <v>7414785</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>1425808.30133719</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13060,19 +13139,19 @@
         <v>248</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -13088,7 +13167,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -13114,7 +13193,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -13140,7 +13219,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -13166,7 +13245,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -13191,10 +13270,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -13219,10 +13298,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -13247,10 +13326,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -13275,10 +13354,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -13303,10 +13382,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -13331,10 +13410,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -13360,7 +13439,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13385,10 +13464,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13413,10 +13492,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13441,10 +13520,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13472,7 +13551,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13499,10 +13578,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
+        <v>644</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>641</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>638</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13529,10 +13608,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13559,10 +13638,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13583,10 +13662,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13613,7 +13692,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13630,7 +13709,7 @@
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
-        <v>7414785</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13641,10 +13720,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13660,7 +13739,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>32414785</v>
+        <v>16289785</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13671,7 +13750,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13688,7 +13767,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>57414785</v>
+        <v>41289785</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13699,10 +13778,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13718,7 +13797,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>82414785</v>
+        <v>66289785</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13729,7 +13808,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13746,7 +13825,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>107414785</v>
+        <v>91289785</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13757,10 +13836,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13776,7 +13855,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>132414785</v>
+        <v>116289785</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13787,7 +13866,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13804,7 +13883,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>182414785</v>
+        <v>166289785</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13815,10 +13894,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13834,7 +13913,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>232414785</v>
+        <v>216289785</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13845,7 +13924,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13862,7 +13941,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>332414785</v>
+        <v>316289785</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13873,10 +13952,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13892,7 +13971,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>482414785</v>
+        <v>466289785</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13903,7 +13982,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13920,7 +13999,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>682414785</v>
+        <v>666289785</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13931,10 +14010,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -13950,7 +14029,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>882414785</v>
+        <v>866289785</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13961,7 +14040,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -13978,7 +14057,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1082414785</v>
+        <v>1066289785</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13989,7 +14068,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -14006,7 +14085,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1282414785</v>
+        <v>1266289785</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14017,7 +14096,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -14034,7 +14113,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1482414785</v>
+        <v>1466289785</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14045,7 +14124,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -14062,7 +14141,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1682414785</v>
+        <v>1666289785</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14073,7 +14152,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -14090,7 +14169,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1882414785</v>
+        <v>1866289785</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14101,7 +14180,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -14118,7 +14197,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2082414785</v>
+        <v>2066289785</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14129,7 +14208,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -14146,7 +14225,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2282414785</v>
+        <v>2266289785</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14157,7 +14236,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -14174,7 +14253,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2482414785</v>
+        <v>2466289785</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14185,7 +14264,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -14202,7 +14281,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2682414785</v>
+        <v>2666289785</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14213,7 +14292,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -14230,7 +14309,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2882414785</v>
+        <v>2866289785</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14241,7 +14320,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -14258,12 +14337,12 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3082414785</v>
+        <v>3066289785</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rachel T3L5, IV 883M, Iso Fest 443M
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="673">
   <si>
     <t xml:space="preserve">Build Priority</t>
   </si>
@@ -1402,6 +1402,9 @@
     <t xml:space="preserve">Level 110 gold orb, promo code Oct 11</t>
   </si>
   <si>
+    <t xml:space="preserve">Iso Fest milestone 20</t>
+  </si>
+  <si>
     <t xml:space="preserve">Breaker of Nature level 130</t>
   </si>
   <si>
@@ -1594,7 +1597,7 @@
     <t xml:space="preserve">Rachel Cole-Alves Iso-8 to T3 level 5</t>
   </si>
   <si>
-    <t xml:space="preserve">After claiming Iso Fest milestone 20</t>
+    <t xml:space="preserve">Done Oct 13. Ion stock estimated after</t>
   </si>
   <si>
     <t xml:space="preserve">Hulk Iso-8 to T3 level 5</t>
@@ -5846,7 +5849,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>866257350</v>
+        <v>883257350</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
@@ -5894,7 +5897,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>33742650</v>
+        <v>16742650</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5903,7 +5906,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3258742650</v>
+        <v>3241742650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5912,7 +5915,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>628946055.252547</v>
+        <v>625807021.377468</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6807,7 +6810,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>33742650</v>
+        <v>16742650</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6826,7 +6829,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>108742650</v>
+        <v>91742650</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6845,7 +6848,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>183742650</v>
+        <v>166742650</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6864,7 +6867,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>258742650</v>
+        <v>241742650</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6883,7 +6886,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>333742650</v>
+        <v>316742650</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6902,7 +6905,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>483742650</v>
+        <v>466742650</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6921,7 +6924,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>633742650</v>
+        <v>616742650</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6940,7 +6943,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>783742650</v>
+        <v>766742650</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6959,7 +6962,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>1008742650</v>
+        <v>991742650</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6978,7 +6981,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1383742650</v>
+        <v>1366742650</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -6997,7 +7000,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1758742650</v>
+        <v>1741742650</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -7016,7 +7019,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2133742650</v>
+        <v>2116742650</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7035,7 +7038,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2508742650</v>
+        <v>2491742650</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7054,7 +7057,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2883742650</v>
+        <v>2866742650</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7073,7 +7076,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3258742650</v>
+        <v>3241742650</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -8550,11 +8553,11 @@
         <v>85000000</v>
       </c>
       <c r="E43" s="24" t="n">
-        <v>68000000</v>
+        <v>85000000</v>
       </c>
       <c r="F43" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D43),MAX(0,D43-E43),0)</f>
-        <v>17000000</v>
+        <v>0</v>
       </c>
       <c r="G43" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D43),ROUNDUP(D43/C43,0),"No limit")</f>
@@ -8562,11 +8565,11 @@
       </c>
       <c r="H43" s="21" t="n">
         <f aca="false">IFERROR(INT(E43/C43),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I43" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F43/C43,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" s="10" t="s">
         <v>326</v>
@@ -8722,7 +8725,7 @@
       </c>
       <c r="E49" s="19" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>845194650</v>
+        <v>862194650</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -8733,7 +8736,7 @@
       <c r="E50" s="19"/>
       <c r="F50" s="19" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7092055350</v>
+        <v>7075055350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8743,7 +8746,7 @@
       <c r="E51" s="19"/>
       <c r="F51" s="19" t="n">
         <f aca="false">SUMIF(J5:J47,"Yes",F5:F47)</f>
-        <v>5193500000</v>
+        <v>5176500000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8835,13 +8838,13 @@
         <v>13180000</v>
       </c>
       <c r="C5" s="26" t="n">
-        <v>947600</v>
+        <v>537600</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>6100000</v>
+        <v>5790000</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>14890000</v>
+        <v>14150000</v>
       </c>
       <c r="F5" s="26" t="n">
         <v>297</v>
@@ -8896,15 +8899,15 @@
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
-        <v>1397600</v>
+        <v>987600</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>6986000</v>
+        <v>6676000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>15776000</v>
+        <v>15036000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -8929,15 +8932,15 @@
       </c>
       <c r="C8" s="27" t="n">
         <f aca="false">SUMIF($J$85:$J$110,"Planned",C85:C110)</f>
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="D8" s="27" t="n">
         <f aca="false">SUMIF($J$85:$J$110,"Planned",D85:D110)</f>
-        <v>1710000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="27" t="n">
         <f aca="false">SUMIF($J$85:$J$110,"Planned",E85:E110)</f>
-        <v>2640000</v>
+        <v>0</v>
       </c>
       <c r="F8" s="27" t="n">
         <f aca="false">SUMIF($J$85:$J$110,"Planned",F85:F110)</f>
@@ -8962,15 +8965,15 @@
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
-        <v>-312400</v>
+        <v>987600</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>5276000</v>
+        <v>6676000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>13136000</v>
+        <v>15036000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -10349,33 +10352,33 @@
         <v>405</v>
       </c>
       <c r="D51" s="29" t="s">
+        <v>456</v>
+      </c>
+      <c r="E51" s="29" t="s">
         <v>451</v>
       </c>
-      <c r="E51" s="29" t="s">
-        <v>456</v>
-      </c>
       <c r="F51" s="29" t="s">
+        <v>457</v>
+      </c>
+      <c r="G51" s="29" t="s">
         <v>431</v>
       </c>
-      <c r="G51" s="29" t="s">
+      <c r="H51" s="29" t="s">
         <v>433</v>
       </c>
-      <c r="H51" s="29" t="s">
+      <c r="I51" s="10" t="s">
         <v>428</v>
-      </c>
-      <c r="I51" s="10" t="s">
-        <v>425</v>
       </c>
       <c r="J51" s="10" t="s">
         <v>326</v>
       </c>
       <c r="K51" s="14" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B52" s="29" t="n">
         <v>3300000</v>
@@ -10405,12 +10408,12 @@
         <v>326</v>
       </c>
       <c r="K52" s="14" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B53" s="29" t="n">
         <v>0</v>
@@ -10440,12 +10443,12 @@
         <v>330</v>
       </c>
       <c r="K53" s="14" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B54" s="29" t="n">
         <v>0</v>
@@ -10475,12 +10478,12 @@
         <v>326</v>
       </c>
       <c r="K54" s="14" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B55" s="29" t="n">
         <v>0</v>
@@ -10510,12 +10513,12 @@
         <v>326</v>
       </c>
       <c r="K55" s="14" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B56" s="29" t="n">
         <v>0</v>
@@ -10545,12 +10548,12 @@
         <v>326</v>
       </c>
       <c r="K56" s="14" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B57" s="29" t="n">
         <v>0</v>
@@ -10580,12 +10583,12 @@
         <v>330</v>
       </c>
       <c r="K57" s="14" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B58" s="29" t="n">
         <v>0</v>
@@ -10615,12 +10618,12 @@
         <v>330</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B59" s="29" t="n">
         <v>750000</v>
@@ -10650,12 +10653,12 @@
         <v>330</v>
       </c>
       <c r="K59" s="14" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B60" s="29" t="n">
         <v>750000</v>
@@ -10685,12 +10688,12 @@
         <v>330</v>
       </c>
       <c r="K60" s="14" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B61" s="29" t="n">
         <v>750000</v>
@@ -10720,12 +10723,12 @@
         <v>330</v>
       </c>
       <c r="K61" s="14" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B62" s="29" t="n">
         <v>750000</v>
@@ -10755,12 +10758,12 @@
         <v>330</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B63" s="29" t="n">
         <v>750000</v>
@@ -10790,12 +10793,12 @@
         <v>330</v>
       </c>
       <c r="K63" s="14" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B64" s="29" t="n">
         <v>750000</v>
@@ -10825,12 +10828,12 @@
         <v>330</v>
       </c>
       <c r="K64" s="14" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B65" s="29" t="n">
         <v>750000</v>
@@ -10860,12 +10863,12 @@
         <v>330</v>
       </c>
       <c r="K65" s="14" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B66" s="29" t="n">
         <v>750000</v>
@@ -10895,12 +10898,12 @@
         <v>330</v>
       </c>
       <c r="K66" s="14" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B67" s="29" t="n">
         <v>0</v>
@@ -10930,12 +10933,12 @@
         <v>326</v>
       </c>
       <c r="K67" s="14" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B68" s="29" t="n">
         <v>0</v>
@@ -10965,12 +10968,12 @@
         <v>330</v>
       </c>
       <c r="K68" s="14" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B69" s="29" t="n">
         <v>407000</v>
@@ -11000,12 +11003,12 @@
         <v>326</v>
       </c>
       <c r="K69" s="14" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B70" s="29" t="n">
         <v>120000</v>
@@ -11035,12 +11038,12 @@
         <v>326</v>
       </c>
       <c r="K70" s="14" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B71" s="29" t="n">
         <v>455000</v>
@@ -11070,7 +11073,7 @@
         <v>330</v>
       </c>
       <c r="K71" s="14" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11205,12 +11208,12 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="22" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>384</v>
@@ -11245,7 +11248,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B85" s="29" t="n">
         <v>1837500</v>
@@ -11272,15 +11275,15 @@
         <v>0</v>
       </c>
       <c r="J85" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K85" s="14" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="11" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B86" s="29" t="n">
         <v>0</v>
@@ -11307,13 +11310,13 @@
         <v>0</v>
       </c>
       <c r="J86" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K86" s="14"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B87" s="29" t="n">
         <v>9791250</v>
@@ -11340,15 +11343,15 @@
         <v>55000000</v>
       </c>
       <c r="J87" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K87" s="14" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="11" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B88" s="29" t="n">
         <v>0</v>
@@ -11375,15 +11378,15 @@
         <v>0</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K88" s="14" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B89" s="26"/>
       <c r="C89" s="29" t="n">
@@ -11402,15 +11405,15 @@
         <v>3000000</v>
       </c>
       <c r="J89" s="10" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="K89" s="14" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="11" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B90" s="26"/>
       <c r="C90" s="29" t="n">
@@ -11429,15 +11432,15 @@
         <v>3000000</v>
       </c>
       <c r="J90" s="10" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K90" s="14" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B91" s="29" t="n">
         <v>1650010</v>
@@ -11464,15 +11467,15 @@
         <v>3000000</v>
       </c>
       <c r="J91" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B92" s="29" t="n">
         <v>1650000</v>
@@ -11499,15 +11502,15 @@
         <v>3000000</v>
       </c>
       <c r="J92" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K92" s="14" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B93" s="29" t="n">
         <v>1650000</v>
@@ -11534,15 +11537,15 @@
         <v>3000000</v>
       </c>
       <c r="J93" s="10" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="K93" s="14" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B94" s="26"/>
       <c r="C94" s="29" t="n">
@@ -11567,15 +11570,15 @@
         <v>17000000</v>
       </c>
       <c r="J94" s="10" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K94" s="14" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B95" s="29" t="n">
         <v>9800000</v>
@@ -11602,15 +11605,15 @@
         <v>0</v>
       </c>
       <c r="J95" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K95" s="14" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B96" s="29" t="n">
         <v>4092000</v>
@@ -11637,15 +11640,15 @@
         <v>0</v>
       </c>
       <c r="J96" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K96" s="14" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B97" s="29" t="n">
         <v>7820000</v>
@@ -11672,15 +11675,15 @@
         <v>0</v>
       </c>
       <c r="J97" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K97" s="14" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B98" s="29" t="n">
         <v>0</v>
@@ -11707,15 +11710,15 @@
         <v>17000000</v>
       </c>
       <c r="J98" s="10" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
       <c r="K98" s="14" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B99" s="29" t="n">
         <v>0</v>
@@ -11742,15 +11745,15 @@
         <v>17000000</v>
       </c>
       <c r="J99" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K99" s="14" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B100" s="29" t="n">
         <v>0</v>
@@ -11777,15 +11780,15 @@
         <v>17000000</v>
       </c>
       <c r="J100" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K100" s="14" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B101" s="29" t="n">
         <v>0</v>
@@ -11812,15 +11815,15 @@
         <v>17000000</v>
       </c>
       <c r="J101" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K101" s="14" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B102" s="29" t="n">
         <v>0</v>
@@ -11847,15 +11850,15 @@
         <v>17000000</v>
       </c>
       <c r="J102" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K102" s="14" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B103" s="29" t="n">
         <v>0</v>
@@ -11876,15 +11879,15 @@
         <v>17000000</v>
       </c>
       <c r="J103" s="10" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="K103" s="14" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="11" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B104" s="29" t="n">
         <v>13000000</v>
@@ -11905,10 +11908,10 @@
         <v>8000000</v>
       </c>
       <c r="J104" s="10" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="K104" s="14" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11991,11 +11994,11 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="15" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="I112" s="19" t="n">
         <f aca="false">SUMIF(J85:J110,"Planned",I85:I110)</f>
-        <v>37000000</v>
+        <v>20000000</v>
       </c>
     </row>
   </sheetData>
@@ -12050,12 +12053,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12069,59 +12072,59 @@
         <v>384</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H6" s="31"/>
       <c r="I6" s="31"/>
@@ -12131,25 +12134,25 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G7" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H7" s="31"/>
       <c r="I7" s="31"/>
@@ -12159,25 +12162,25 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H8" s="31"/>
       <c r="I8" s="31"/>
@@ -12187,25 +12190,25 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H9" s="31"/>
       <c r="I9" s="31"/>
@@ -12215,25 +12218,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H10" s="31"/>
       <c r="I10" s="31"/>
@@ -12243,25 +12246,25 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H11" s="31"/>
       <c r="I11" s="31"/>
@@ -12271,25 +12274,25 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H12" s="31"/>
       <c r="I12" s="31"/>
@@ -12299,25 +12302,25 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H13" s="31"/>
       <c r="I13" s="31"/>
@@ -12327,25 +12330,25 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F14" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G14" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H14" s="31"/>
       <c r="I14" s="31"/>
@@ -12355,25 +12358,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>50000</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H15" s="31"/>
       <c r="I15" s="31"/>
@@ -12383,25 +12386,25 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1000000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G16" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H16" s="31"/>
       <c r="I16" s="31"/>
@@ -12411,23 +12414,23 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>100000</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H17" s="31"/>
       <c r="I17" s="31"/>
@@ -12437,19 +12440,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F18" s="31"/>
       <c r="G18" s="31"/>
@@ -12461,25 +12464,25 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>25000</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H19" s="31"/>
       <c r="I19" s="31"/>
@@ -12489,25 +12492,25 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>75000</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H20" s="31"/>
       <c r="I20" s="31"/>
@@ -12517,30 +12520,30 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F22" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H22" s="31"/>
       <c r="I22" s="31"/>
@@ -12550,16 +12553,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
+        <v>577</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>575</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>576</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>574</v>
-      </c>
-      <c r="C23" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>575</v>
       </c>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
@@ -12572,16 +12575,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -12594,22 +12597,22 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>900000</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E25" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G25" s="31"/>
       <c r="H25" s="31"/>
@@ -12620,23 +12623,23 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F26" s="31"/>
       <c r="G26" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H26" s="31"/>
       <c r="I26" s="31"/>
@@ -12646,16 +12649,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E27" s="31"/>
       <c r="F27" s="31"/>
@@ -12668,16 +12671,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
@@ -12690,21 +12693,21 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
@@ -12717,16 +12720,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E31" s="31"/>
       <c r="F31" s="31"/>
@@ -12739,16 +12742,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="E32" s="31"/>
       <c r="F32" s="31"/>
@@ -12761,19 +12764,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F33" s="31"/>
       <c r="G33" s="31"/>
@@ -12785,16 +12788,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E34" s="31"/>
       <c r="F34" s="31"/>
@@ -12807,16 +12810,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -12829,16 +12832,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
+        <v>605</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>599</v>
+      </c>
+      <c r="C36" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="14" t="s">
         <v>604</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>598</v>
-      </c>
-      <c r="C36" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>603</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -12851,16 +12854,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
@@ -12873,16 +12876,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -12895,7 +12898,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="E40" s="19" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$38)*(E5:E38="Done"))</f>
@@ -12932,7 +12935,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E41" s="32" t="str">
         <f aca="false">COUNTIFS($B$5:$B$38,"Required",E5:E38,"Done")&amp;" of 11"</f>
@@ -12969,7 +12972,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
   </sheetData>
@@ -13013,12 +13016,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13026,10 +13029,10 @@
         <v>239</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13040,13 +13043,13 @@
         <v>46313.7083333333</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13054,22 +13057,22 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>433710215</v>
+        <v>442770515</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>1300000</v>
+        <v>0</v>
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
-        <v>1400000</v>
+        <v>0</v>
       </c>
       <c r="G6" s="19" t="n">
         <f aca="false">SUMPRODUCT((A13:A54&lt;=$B$9)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>1900000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13085,15 +13088,15 @@
       </c>
       <c r="E7" s="19" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*E13:E54)</f>
-        <v>1300000</v>
+        <v>0</v>
       </c>
       <c r="F7" s="19" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*F13:F54)</f>
-        <v>1400000</v>
+        <v>0</v>
       </c>
       <c r="G7" s="19" t="n">
         <f aca="false">SUMPRODUCT((B13:B54&lt;&gt;"")*(B13:B54&lt;=$B$6)*(H13:H54&lt;&gt;"Claimed")*G13:G54)</f>
-        <v>1900000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13102,12 +13105,12 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>16289785</v>
+        <v>7229485</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B9" s="33" t="n">
         <v>20</v>
@@ -13115,7 +13118,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,INDEX(B13:B54,B9)-B6)</f>
@@ -13124,7 +13127,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
@@ -13139,19 +13142,19 @@
         <v>248</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>12</v>
@@ -13167,7 +13170,7 @@
       <c r="B13" s="26"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>0</v>
@@ -13193,7 +13196,7 @@
       <c r="B14" s="26"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E14" s="29" t="n">
         <v>0</v>
@@ -13219,7 +13222,7 @@
       <c r="B15" s="26"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0</v>
@@ -13245,7 +13248,7 @@
       <c r="B16" s="26"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E16" s="29" t="n">
         <v>0</v>
@@ -13270,10 +13273,10 @@
       </c>
       <c r="B17" s="26"/>
       <c r="C17" s="11" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E17" s="29" t="n">
         <v>0</v>
@@ -13298,10 +13301,10 @@
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="11" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E18" s="29" t="n">
         <v>0</v>
@@ -13326,10 +13329,10 @@
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="11" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E19" s="29" t="n">
         <v>0</v>
@@ -13354,10 +13357,10 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="11" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="E20" s="29" t="n">
         <v>0</v>
@@ -13382,10 +13385,10 @@
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="11" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E21" s="29" t="n">
         <v>0</v>
@@ -13410,10 +13413,10 @@
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="11" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E22" s="29" t="n">
         <v>0</v>
@@ -13439,7 +13442,7 @@
       <c r="B23" s="26"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E23" s="29" t="n">
         <v>900000</v>
@@ -13464,10 +13467,10 @@
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="11" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E24" s="29" t="n">
         <v>900000</v>
@@ -13492,10 +13495,10 @@
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="11" t="s">
+        <v>643</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>642</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>641</v>
       </c>
       <c r="E25" s="29" t="n">
         <v>0</v>
@@ -13520,10 +13523,10 @@
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="11" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E26" s="29" t="n">
         <v>900000</v>
@@ -13551,7 +13554,7 @@
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E27" s="29" t="n">
         <v>900000</v>
@@ -13578,10 +13581,10 @@
         <v>325000000</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E28" s="29" t="n">
         <v>950000</v>
@@ -13608,10 +13611,10 @@
         <v>350000000</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E29" s="29" t="n">
         <v>0</v>
@@ -13638,10 +13641,10 @@
         <v>375000000</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E30" s="26"/>
       <c r="F30" s="26"/>
@@ -13662,10 +13665,10 @@
         <v>400000000</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E31" s="29" t="n">
         <v>0</v>
@@ -13692,7 +13695,7 @@
         <v>425000000</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="29" t="n">
@@ -13705,7 +13708,7 @@
         <v>1900000</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I32" s="23" t="n">
         <f aca="false">IF(B32="","",MAX(0,B32-$B$6))</f>
@@ -13720,10 +13723,10 @@
         <v>450000000</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E33" s="29" t="n">
         <v>0</v>
@@ -13739,7 +13742,7 @@
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>16289785</v>
+        <v>7229485</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13750,7 +13753,7 @@
         <v>475000000</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="29" t="n">
@@ -13767,7 +13770,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>41289785</v>
+        <v>32229485</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13778,10 +13781,10 @@
         <v>500000000</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E35" s="29" t="n">
         <v>0</v>
@@ -13797,7 +13800,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>66289785</v>
+        <v>57229485</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13808,7 +13811,7 @@
         <v>525000000</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="29" t="n">
@@ -13825,7 +13828,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>91289785</v>
+        <v>82229485</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13836,10 +13839,10 @@
         <v>550000000</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E37" s="29" t="n">
         <v>0</v>
@@ -13855,7 +13858,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>116289785</v>
+        <v>107229485</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13866,7 +13869,7 @@
         <v>600000000</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D38" s="11"/>
       <c r="E38" s="29" t="n">
@@ -13883,7 +13886,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>166289785</v>
+        <v>157229485</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13894,10 +13897,10 @@
         <v>650000000</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E39" s="29" t="n">
         <v>0</v>
@@ -13913,7 +13916,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>216289785</v>
+        <v>207229485</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13924,7 +13927,7 @@
         <v>750000000</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="29" t="n">
@@ -13941,7 +13944,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>316289785</v>
+        <v>307229485</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13952,10 +13955,10 @@
         <v>900000000</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E41" s="29" t="n">
         <v>0</v>
@@ -13971,7 +13974,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>466289785</v>
+        <v>457229485</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13982,7 +13985,7 @@
         <v>1100000000</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D42" s="11"/>
       <c r="E42" s="29" t="n">
@@ -13999,7 +14002,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>666289785</v>
+        <v>657229485</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14010,10 +14013,10 @@
         <v>1300000000</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E43" s="29" t="n">
         <v>0</v>
@@ -14029,7 +14032,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>866289785</v>
+        <v>857229485</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14040,7 +14043,7 @@
         <v>1500000000</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="29" t="n">
@@ -14057,7 +14060,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1066289785</v>
+        <v>1057229485</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14068,7 +14071,7 @@
         <v>1700000000</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="29" t="n">
@@ -14085,7 +14088,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1266289785</v>
+        <v>1257229485</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14096,7 +14099,7 @@
         <v>1900000000</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D46" s="11"/>
       <c r="E46" s="29" t="n">
@@ -14113,7 +14116,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1466289785</v>
+        <v>1457229485</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14124,7 +14127,7 @@
         <v>2100000000</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="29" t="n">
@@ -14141,7 +14144,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1666289785</v>
+        <v>1657229485</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14152,7 +14155,7 @@
         <v>2300000000</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="29" t="n">
@@ -14169,7 +14172,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1866289785</v>
+        <v>1857229485</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14180,7 +14183,7 @@
         <v>2500000000</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="29" t="n">
@@ -14197,7 +14200,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2066289785</v>
+        <v>2057229485</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14208,7 +14211,7 @@
         <v>2700000000</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="D50" s="11"/>
       <c r="E50" s="29" t="n">
@@ -14225,7 +14228,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2266289785</v>
+        <v>2257229485</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14236,7 +14239,7 @@
         <v>2900000000</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="29" t="n">
@@ -14253,7 +14256,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2466289785</v>
+        <v>2457229485</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14264,7 +14267,7 @@
         <v>3100000000</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D52" s="11"/>
       <c r="E52" s="29" t="n">
@@ -14281,7 +14284,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2666289785</v>
+        <v>2657229485</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14292,7 +14295,7 @@
         <v>3300000000</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="D53" s="11"/>
       <c r="E53" s="29" t="n">
@@ -14309,7 +14312,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2866289785</v>
+        <v>2857229485</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14320,7 +14323,7 @@
         <v>3500000000</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="29" t="n">
@@ -14337,12 +14340,12 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3066289785</v>
+        <v>3057229485</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Iso Fest milestone 21 claimed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5915,7 +5915,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>625807021.377468</v>
+        <v>627151929.932653</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13057,7 +13057,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>442770515</v>
+        <v>450220515</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>620</v>
@@ -13081,7 +13081,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IFERROR(INDEX(A13:A54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),"All done")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>245</v>
@@ -13105,7 +13105,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>7229485</v>
+        <v>24779485</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13738,11 +13738,11 @@
         <v>1900000</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I33" s="23" t="n">
         <f aca="false">IF(B33="","",MAX(0,B33-$B$6))</f>
-        <v>7229485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13770,7 +13770,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>32229485</v>
+        <v>24779485</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13800,7 +13800,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>57229485</v>
+        <v>49779485</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13828,7 +13828,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>82229485</v>
+        <v>74779485</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13858,7 +13858,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>107229485</v>
+        <v>99779485</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>157229485</v>
+        <v>149779485</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>207229485</v>
+        <v>199779485</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13944,7 +13944,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>307229485</v>
+        <v>299779485</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13974,7 +13974,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>457229485</v>
+        <v>449779485</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14002,7 +14002,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>657229485</v>
+        <v>649779485</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>857229485</v>
+        <v>849779485</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14060,7 +14060,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1057229485</v>
+        <v>1049779485</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1257229485</v>
+        <v>1249779485</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14116,7 +14116,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1457229485</v>
+        <v>1449779485</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14144,7 +14144,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1657229485</v>
+        <v>1649779485</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1857229485</v>
+        <v>1849779485</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14200,7 +14200,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2057229485</v>
+        <v>2049779485</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14228,7 +14228,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2257229485</v>
+        <v>2249779485</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14256,7 +14256,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2457229485</v>
+        <v>2449779485</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14284,7 +14284,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2657229485</v>
+        <v>2649779485</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14312,7 +14312,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2857229485</v>
+        <v>2849779485</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14340,7 +14340,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3057229485</v>
+        <v>3049779485</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Sync power core spending from Iso Fest task
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5849,14 +5849,14 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>883257350</v>
+        <v>883657350</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6059757350</v>
+        <v>6060157350</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5897,7 +5897,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>16742650</v>
+        <v>16342650</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3241742650</v>
+        <v>3241342650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5915,7 +5915,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>627151929.932653</v>
+        <v>627870703.837111</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6810,7 +6810,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>16742650</v>
+        <v>16342650</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6829,7 +6829,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>91742650</v>
+        <v>91342650</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6848,7 +6848,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>166742650</v>
+        <v>166342650</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6867,7 +6867,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>241742650</v>
+        <v>241342650</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6886,7 +6886,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>316742650</v>
+        <v>316342650</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6905,7 +6905,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>466742650</v>
+        <v>466342650</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6924,7 +6924,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>616742650</v>
+        <v>616342650</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6943,7 +6943,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>766742650</v>
+        <v>766342650</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6962,7 +6962,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>991742650</v>
+        <v>991342650</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6981,7 +6981,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1366742650</v>
+        <v>1366342650</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -7000,7 +7000,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1741742650</v>
+        <v>1741342650</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -7019,7 +7019,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2116742650</v>
+        <v>2116342650</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7038,7 +7038,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2491742650</v>
+        <v>2491342650</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7057,7 +7057,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2866742650</v>
+        <v>2866342650</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7076,7 +7076,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3241742650</v>
+        <v>3241342650</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -7293,11 +7293,11 @@
         <v>1000000000</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>34600000</v>
+        <v>39200000</v>
       </c>
       <c r="F8" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D8),MAX(0,D8-E8),0)</f>
-        <v>965400000</v>
+        <v>960800000</v>
       </c>
       <c r="G8" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D8),ROUNDUP(D8/C8,0),"No limit")</f>
@@ -7305,11 +7305,11 @@
       </c>
       <c r="H8" s="21" t="n">
         <f aca="false">IFERROR(INT(E8/C8),0)</f>
-        <v>8650</v>
+        <v>9800</v>
       </c>
       <c r="I8" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F8/C8,0),0)</f>
-        <v>241350</v>
+        <v>240200</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>330</v>
@@ -8725,7 +8725,7 @@
       </c>
       <c r="E49" s="19" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>862194650</v>
+        <v>866794650</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -8736,7 +8736,7 @@
       <c r="E50" s="19"/>
       <c r="F50" s="19" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7075055350</v>
+        <v>7070455350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13057,7 +13057,7 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>450220515</v>
+        <v>450320515</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>620</v>
@@ -13105,7 +13105,7 @@
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">IFERROR(INDEX(I13:I54,MATCH(TRUE(),INDEX(B13:B54&gt;B6,0),0)),0)</f>
-        <v>24779485</v>
+        <v>24679485</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13770,7 +13770,7 @@
       </c>
       <c r="I34" s="23" t="n">
         <f aca="false">IF(B34="","",MAX(0,B34-$B$6))</f>
-        <v>24779485</v>
+        <v>24679485</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13800,7 +13800,7 @@
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">IF(B35="","",MAX(0,B35-$B$6))</f>
-        <v>49779485</v>
+        <v>49679485</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13828,7 +13828,7 @@
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">IF(B36="","",MAX(0,B36-$B$6))</f>
-        <v>74779485</v>
+        <v>74679485</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13858,7 +13858,7 @@
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">IF(B37="","",MAX(0,B37-$B$6))</f>
-        <v>99779485</v>
+        <v>99679485</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">IF(B38="","",MAX(0,B38-$B$6))</f>
-        <v>149779485</v>
+        <v>149679485</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="I39" s="23" t="n">
         <f aca="false">IF(B39="","",MAX(0,B39-$B$6))</f>
-        <v>199779485</v>
+        <v>199679485</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13944,7 +13944,7 @@
       </c>
       <c r="I40" s="23" t="n">
         <f aca="false">IF(B40="","",MAX(0,B40-$B$6))</f>
-        <v>299779485</v>
+        <v>299679485</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13974,7 +13974,7 @@
       </c>
       <c r="I41" s="23" t="n">
         <f aca="false">IF(B41="","",MAX(0,B41-$B$6))</f>
-        <v>449779485</v>
+        <v>449679485</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14002,7 +14002,7 @@
       </c>
       <c r="I42" s="23" t="n">
         <f aca="false">IF(B42="","",MAX(0,B42-$B$6))</f>
-        <v>649779485</v>
+        <v>649679485</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="I43" s="23" t="n">
         <f aca="false">IF(B43="","",MAX(0,B43-$B$6))</f>
-        <v>849779485</v>
+        <v>849679485</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14060,7 +14060,7 @@
       </c>
       <c r="I44" s="23" t="n">
         <f aca="false">IF(B44="","",MAX(0,B44-$B$6))</f>
-        <v>1049779485</v>
+        <v>1049679485</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="I45" s="23" t="n">
         <f aca="false">IF(B45="","",MAX(0,B45-$B$6))</f>
-        <v>1249779485</v>
+        <v>1249679485</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14116,7 +14116,7 @@
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">IF(B46="","",MAX(0,B46-$B$6))</f>
-        <v>1449779485</v>
+        <v>1449679485</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14144,7 +14144,7 @@
       </c>
       <c r="I47" s="23" t="n">
         <f aca="false">IF(B47="","",MAX(0,B47-$B$6))</f>
-        <v>1649779485</v>
+        <v>1649679485</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="I48" s="23" t="n">
         <f aca="false">IF(B48="","",MAX(0,B48-$B$6))</f>
-        <v>1849779485</v>
+        <v>1849679485</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14200,7 +14200,7 @@
       </c>
       <c r="I49" s="23" t="n">
         <f aca="false">IF(B49="","",MAX(0,B49-$B$6))</f>
-        <v>2049779485</v>
+        <v>2049679485</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14228,7 +14228,7 @@
       </c>
       <c r="I50" s="23" t="n">
         <f aca="false">IF(B50="","",MAX(0,B50-$B$6))</f>
-        <v>2249779485</v>
+        <v>2249679485</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14256,7 +14256,7 @@
       </c>
       <c r="I51" s="23" t="n">
         <f aca="false">IF(B51="","",MAX(0,B51-$B$6))</f>
-        <v>2449779485</v>
+        <v>2449679485</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14284,7 +14284,7 @@
       </c>
       <c r="I52" s="23" t="n">
         <f aca="false">IF(B52="","",MAX(0,B52-$B$6))</f>
-        <v>2649779485</v>
+        <v>2649679485</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14312,7 +14312,7 @@
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">IF(B53="","",MAX(0,B53-$B$6))</f>
-        <v>2849779485</v>
+        <v>2849679485</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14340,7 +14340,7 @@
       </c>
       <c r="I54" s="23" t="n">
         <f aca="false">IF(B54="","",MAX(0,B54-$B$6))</f>
-        <v>3049779485</v>
+        <v>3049679485</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
IV power core count from game
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5915,7 +5915,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>627870703.837111</v>
+        <v>627897765.085204</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7293,11 +7293,11 @@
         <v>1000000000</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>39200000</v>
+        <v>36000000</v>
       </c>
       <c r="F8" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D8),MAX(0,D8-E8),0)</f>
-        <v>960800000</v>
+        <v>964000000</v>
       </c>
       <c r="G8" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D8),ROUNDUP(D8/C8,0),"No limit")</f>
@@ -7305,11 +7305,11 @@
       </c>
       <c r="H8" s="21" t="n">
         <f aca="false">IFERROR(INT(E8/C8),0)</f>
-        <v>9800</v>
+        <v>9000</v>
       </c>
       <c r="I8" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F8/C8,0),0)</f>
-        <v>240200</v>
+        <v>241000</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>330</v>
@@ -8725,7 +8725,7 @@
       </c>
       <c r="E49" s="19" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>866794650</v>
+        <v>863594650</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -8736,7 +8736,7 @@
       <c r="E50" s="19"/>
       <c r="F50" s="19" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7070455350</v>
+        <v>7073655350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Breaker 190 and 200 rewards, gold and training orbs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -1405,6 +1405,9 @@
     <t xml:space="preserve">Iso Fest milestone 20</t>
   </si>
   <si>
+    <t xml:space="preserve">Breaker of Nature level 140</t>
+  </si>
+  <si>
     <t xml:space="preserve">Breaker of Nature level 130</t>
   </si>
   <si>
@@ -1481,9 +1484,6 @@
   </si>
   <si>
     <t xml:space="preserve">Claimed Oct 12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Breaker of Nature level 140</t>
   </si>
   <si>
     <t xml:space="preserve">Expected about Oct 15. Gives 2,000 gold orb fragments, one orb</t>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>627897765.085204</v>
+        <v>635116161.437399</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8835,16 +8835,16 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>13180000</v>
+        <v>23080000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>537600</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>5790000</v>
+        <v>6540000</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>14150000</v>
+        <v>14350000</v>
       </c>
       <c r="F5" s="26" t="n">
         <v>297</v>
@@ -8853,7 +8853,7 @@
         <v>1065</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>560</v>
+        <v>791</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>29930000</v>
+        <v>39830000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8903,11 +8903,11 @@
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">D5+D6</f>
-        <v>6676000</v>
+        <v>7426000</v>
       </c>
       <c r="E7" s="27" t="n">
         <f aca="false">E5+E6</f>
-        <v>15036000</v>
+        <v>15236000</v>
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">F5+F6</f>
@@ -8919,7 +8919,7 @@
       </c>
       <c r="H7" s="27" t="n">
         <f aca="false">H5+H6</f>
-        <v>645</v>
+        <v>876</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8961,7 +8961,7 @@
       </c>
       <c r="B9" s="28" t="n">
         <f aca="false">B7-B8</f>
-        <v>29930000</v>
+        <v>39830000</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C7-C8</f>
@@ -8969,11 +8969,11 @@
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D7-D8</f>
-        <v>6676000</v>
+        <v>7426000</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E7-E8</f>
-        <v>15036000</v>
+        <v>15236000</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">F7-F8</f>
@@ -8985,7 +8985,7 @@
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">H7-H8</f>
-        <v>645</v>
+        <v>876</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10355,30 +10355,30 @@
         <v>456</v>
       </c>
       <c r="E51" s="29" t="s">
+        <v>457</v>
+      </c>
+      <c r="F51" s="29" t="s">
         <v>451</v>
       </c>
-      <c r="F51" s="29" t="s">
-        <v>457</v>
-      </c>
       <c r="G51" s="29" t="s">
+        <v>458</v>
+      </c>
+      <c r="H51" s="29" t="s">
         <v>431</v>
       </c>
-      <c r="H51" s="29" t="s">
+      <c r="I51" s="10" t="s">
         <v>433</v>
-      </c>
-      <c r="I51" s="10" t="s">
-        <v>428</v>
       </c>
       <c r="J51" s="10" t="s">
         <v>326</v>
       </c>
       <c r="K51" s="14" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B52" s="29" t="n">
         <v>3300000</v>
@@ -10408,12 +10408,12 @@
         <v>326</v>
       </c>
       <c r="K52" s="14" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B53" s="29" t="n">
         <v>0</v>
@@ -10443,12 +10443,12 @@
         <v>330</v>
       </c>
       <c r="K53" s="14" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B54" s="29" t="n">
         <v>0</v>
@@ -10478,12 +10478,12 @@
         <v>326</v>
       </c>
       <c r="K54" s="14" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B55" s="29" t="n">
         <v>0</v>
@@ -10513,12 +10513,12 @@
         <v>326</v>
       </c>
       <c r="K55" s="14" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B56" s="29" t="n">
         <v>0</v>
@@ -10548,12 +10548,12 @@
         <v>326</v>
       </c>
       <c r="K56" s="14" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B57" s="29" t="n">
         <v>0</v>
@@ -10583,12 +10583,12 @@
         <v>330</v>
       </c>
       <c r="K57" s="14" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B58" s="29" t="n">
         <v>0</v>
@@ -10618,12 +10618,12 @@
         <v>330</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B59" s="29" t="n">
         <v>750000</v>
@@ -10653,12 +10653,12 @@
         <v>330</v>
       </c>
       <c r="K59" s="14" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B60" s="29" t="n">
         <v>750000</v>
@@ -10688,12 +10688,12 @@
         <v>330</v>
       </c>
       <c r="K60" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B61" s="29" t="n">
         <v>750000</v>
@@ -10723,12 +10723,12 @@
         <v>330</v>
       </c>
       <c r="K61" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B62" s="29" t="n">
         <v>750000</v>
@@ -10758,12 +10758,12 @@
         <v>330</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B63" s="29" t="n">
         <v>750000</v>
@@ -10793,12 +10793,12 @@
         <v>330</v>
       </c>
       <c r="K63" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="11" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B64" s="29" t="n">
         <v>750000</v>
@@ -10828,12 +10828,12 @@
         <v>330</v>
       </c>
       <c r="K64" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B65" s="29" t="n">
         <v>750000</v>
@@ -10863,12 +10863,12 @@
         <v>330</v>
       </c>
       <c r="K65" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B66" s="29" t="n">
         <v>750000</v>
@@ -10898,12 +10898,12 @@
         <v>330</v>
       </c>
       <c r="K66" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B67" s="29" t="n">
         <v>0</v>
@@ -10933,12 +10933,12 @@
         <v>326</v>
       </c>
       <c r="K67" s="14" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="s">
-        <v>483</v>
+        <v>457</v>
       </c>
       <c r="B68" s="29" t="n">
         <v>0</v>
@@ -10965,7 +10965,7 @@
         <v>326</v>
       </c>
       <c r="J68" s="10" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="K68" s="14" t="s">
         <v>484</v>

</xml_diff>

<commit_message>
Night Thrasher ultimate maxed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Event_Tracker.xlsx
+++ b/Event_Tracker.xlsx
@@ -5849,14 +5849,14 @@
         <v>241</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>883657350</v>
+        <v>883882350</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>242</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">B6+Scoring!F51</f>
-        <v>6060157350</v>
+        <v>6060382350</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5897,7 +5897,7 @@
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">IFERROR(INDEX(E13:E76,MATCH(TRUE(),INDEX(B13:B76&gt;B6,0),0)),0)</f>
-        <v>16342650</v>
+        <v>16117650</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">MAX(0,B76-B6)</f>
-        <v>3241342650</v>
+        <v>3241117650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5915,7 +5915,7 @@
       </c>
       <c r="B11" s="19" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>635116161.437399</v>
+        <v>635176173.308457</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6810,7 +6810,7 @@
       <c r="D62" s="11"/>
       <c r="E62" s="23" t="n">
         <f aca="false">IF(B62="","",MAX(0,B62-$B$6))</f>
-        <v>16342650</v>
+        <v>16117650</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>185</v>
@@ -6829,7 +6829,7 @@
       <c r="D63" s="11"/>
       <c r="E63" s="23" t="n">
         <f aca="false">IF(B63="","",MAX(0,B63-$B$6))</f>
-        <v>91342650</v>
+        <v>91117650</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>185</v>
@@ -6848,7 +6848,7 @@
       <c r="D64" s="11"/>
       <c r="E64" s="23" t="n">
         <f aca="false">IF(B64="","",MAX(0,B64-$B$6))</f>
-        <v>166342650</v>
+        <v>166117650</v>
       </c>
       <c r="F64" s="10" t="s">
         <v>185</v>
@@ -6867,7 +6867,7 @@
       <c r="D65" s="11"/>
       <c r="E65" s="23" t="n">
         <f aca="false">IF(B65="","",MAX(0,B65-$B$6))</f>
-        <v>241342650</v>
+        <v>241117650</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>185</v>
@@ -6886,7 +6886,7 @@
       <c r="D66" s="11"/>
       <c r="E66" s="23" t="n">
         <f aca="false">IF(B66="","",MAX(0,B66-$B$6))</f>
-        <v>316342650</v>
+        <v>316117650</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>185</v>
@@ -6905,7 +6905,7 @@
       <c r="D67" s="11"/>
       <c r="E67" s="23" t="n">
         <f aca="false">IF(B67="","",MAX(0,B67-$B$6))</f>
-        <v>466342650</v>
+        <v>466117650</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>185</v>
@@ -6924,7 +6924,7 @@
       <c r="D68" s="11"/>
       <c r="E68" s="23" t="n">
         <f aca="false">IF(B68="","",MAX(0,B68-$B$6))</f>
-        <v>616342650</v>
+        <v>616117650</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>185</v>
@@ -6943,7 +6943,7 @@
       <c r="D69" s="11"/>
       <c r="E69" s="23" t="n">
         <f aca="false">IF(B69="","",MAX(0,B69-$B$6))</f>
-        <v>766342650</v>
+        <v>766117650</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>185</v>
@@ -6962,7 +6962,7 @@
       <c r="D70" s="11"/>
       <c r="E70" s="23" t="n">
         <f aca="false">IF(B70="","",MAX(0,B70-$B$6))</f>
-        <v>991342650</v>
+        <v>991117650</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>185</v>
@@ -6981,7 +6981,7 @@
       <c r="D71" s="11"/>
       <c r="E71" s="23" t="n">
         <f aca="false">IF(B71="","",MAX(0,B71-$B$6))</f>
-        <v>1366342650</v>
+        <v>1366117650</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>185</v>
@@ -7000,7 +7000,7 @@
       <c r="D72" s="11"/>
       <c r="E72" s="23" t="n">
         <f aca="false">IF(B72="","",MAX(0,B72-$B$6))</f>
-        <v>1741342650</v>
+        <v>1741117650</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>185</v>
@@ -7019,7 +7019,7 @@
       <c r="D73" s="11"/>
       <c r="E73" s="23" t="n">
         <f aca="false">IF(B73="","",MAX(0,B73-$B$6))</f>
-        <v>2116342650</v>
+        <v>2116117650</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>185</v>
@@ -7038,7 +7038,7 @@
       <c r="D74" s="11"/>
       <c r="E74" s="23" t="n">
         <f aca="false">IF(B74="","",MAX(0,B74-$B$6))</f>
-        <v>2491342650</v>
+        <v>2491117650</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>185</v>
@@ -7057,7 +7057,7 @@
       <c r="D75" s="11"/>
       <c r="E75" s="23" t="n">
         <f aca="false">IF(B75="","",MAX(0,B75-$B$6))</f>
-        <v>2866342650</v>
+        <v>2866117650</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>185</v>
@@ -7076,7 +7076,7 @@
       <c r="D76" s="11"/>
       <c r="E76" s="23" t="n">
         <f aca="false">IF(B76="","",MAX(0,B76-$B$6))</f>
-        <v>3241342650</v>
+        <v>3241117650</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>185</v>
@@ -7257,11 +7257,11 @@
         <v>1000000000</v>
       </c>
       <c r="E7" s="24" t="n">
-        <v>66844650</v>
+        <v>67069650</v>
       </c>
       <c r="F7" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D7),MAX(0,D7-E7),0)</f>
-        <v>933155350</v>
+        <v>932930350</v>
       </c>
       <c r="G7" s="21" t="n">
         <f aca="false">IF(ISNUMBER(D7),ROUNDUP(D7/C7,0),"No limit")</f>
@@ -7269,11 +7269,11 @@
       </c>
       <c r="H7" s="21" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>66844650</v>
+        <v>67069650</v>
       </c>
       <c r="I7" s="21" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>933155350</v>
+        <v>932930350</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>330</v>
@@ -8725,7 +8725,7 @@
       </c>
       <c r="E49" s="19" t="n">
         <f aca="false">SUM(E5:E47)</f>
-        <v>863594650</v>
+        <v>863819650</v>
       </c>
       <c r="F49" s="19"/>
     </row>
@@ -8736,7 +8736,7 @@
       <c r="E50" s="19"/>
       <c r="F50" s="19" t="n">
         <f aca="false">SUM(F5:F47)</f>
-        <v>7073655350</v>
+        <v>7073430350</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8835,7 +8835,7 @@
         <v>391</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>23080000</v>
+        <v>22855000</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>537600</v>
@@ -8895,7 +8895,7 @@
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">B5+B6</f>
-        <v>39830000</v>
+        <v>39605000</v>
       </c>
       <c r="C7" s="27" t="n">
         <f aca="false">C5+C6</f>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="B9" s="28" 